<commit_message>
[gameplay] Nouvelle rareté « Uncommon » (vert) entre Common et Rare
- items.js : ajout de la rareté uncommon (#4a9d52, vert) dans RARETES, avec un
  champ `rang` sur chaque rareté (ordre commun<uncommon<rare<epique<legendaire) ;
  prix de revente uncommon = 4 (entre commun 2 et rare 6).
- Nouvelle fonction rareteAuMoins(id, seuil) : compare par rang sans coder les
  noms en dur. Les confirmations de vente/jet passent de « != commun » à
  « >= rare » → un objet uncommon ne déclenche PAS de confirmation (cohérent avec
  l'intention « protéger les objets rare+ »), comportement des items existants
  inchangé.
- Tableau Excel régénéré : la rareté Uncommon apparaît dans la légende ; prête à
  être affectée à des items via l'onglet « Items ».

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJcbumK5KWRfGozDrLY2Kn
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -63,7 +63,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +78,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="009AA0A6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004A9D52"/>
       </patternFill>
     </fill>
     <fill>
@@ -152,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -175,14 +180,17 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -200,22 +208,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -584,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -675,19 +683,26 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rare  (rare)</t>
+          <t xml:space="preserve">  Uncommon  (uncommon)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Epic  (epique)</t>
+          <t xml:space="preserve">  Rare  (rare)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Epic  (epique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  Legendary  (legendaire)</t>
         </is>
@@ -724,1536 +739,1536 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>BRUTAL — Items par type (cartes ajoutées au deck)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Une ligne = une pièce d'équipement. Remplis les lignes vides pour proposer de nouveaux items.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Rareté</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Nb cartes</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Carte 1</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Qté</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>Carte 2</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>Qté</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>Carte 3</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
+      <c r="J3" s="11" t="inlineStr">
         <is>
           <t>Qté</t>
         </is>
       </c>
-      <c r="K3" s="10" t="inlineStr">
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>Carte 4</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr">
+      <c r="L3" s="11" t="inlineStr">
         <is>
           <t>Qté</t>
         </is>
       </c>
-      <c r="M3" s="10" t="inlineStr">
+      <c r="M3" s="11" t="inlineStr">
         <is>
           <t>Notes / nouvelles cartes</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Armes — une main   (5)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Rusty Axe</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>hache-rouillee</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="16" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Rusty Cleave</t>
         </is>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="16" t="n"/>
-      <c r="K5" s="16" t="n"/>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="16" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="17" t="n"/>
+      <c r="L5" s="17" t="n"/>
+      <c r="M5" s="17" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Forge Hammer</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>marteau-de-forge</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>Forge Smash</t>
         </is>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="16" t="n"/>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="16" t="n"/>
-      <c r="L6" s="16" t="n"/>
-      <c r="M6" s="16" t="n"/>
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="17" t="n"/>
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="17" t="n"/>
+      <c r="L6" s="17" t="n"/>
+      <c r="M6" s="17" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Miner's Pick</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>pioche-de-mineur</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Pickaxe Jab</t>
         </is>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="16" t="n"/>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="16" t="n"/>
+      <c r="G7" s="17" t="n"/>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="17" t="n"/>
+      <c r="L7" s="17" t="n"/>
+      <c r="M7" s="17" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Basilisk Fang</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>croc-de-basilic</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Venom Stab</t>
         </is>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="16" t="n"/>
-      <c r="J8" s="16" t="n"/>
-      <c r="K8" s="16" t="n"/>
-      <c r="L8" s="16" t="n"/>
-      <c r="M8" s="16" t="n"/>
+      <c r="G8" s="17" t="n"/>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
+      <c r="J8" s="17" t="n"/>
+      <c r="K8" s="17" t="n"/>
+      <c r="L8" s="17" t="n"/>
+      <c r="M8" s="17" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Magma Hammer</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>marteau-de-lave</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Lava Hammer</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="16" t="n"/>
-      <c r="I9" s="16" t="n"/>
-      <c r="J9" s="16" t="n"/>
-      <c r="K9" s="16" t="n"/>
-      <c r="L9" s="16" t="n"/>
-      <c r="M9" s="16" t="n"/>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n"/>
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="17" t="n"/>
+      <c r="L9" s="17" t="n"/>
+      <c r="M9" s="17" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="19" t="n"/>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="19" t="n"/>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="19" t="n"/>
-      <c r="M10" s="19" t="n"/>
+      <c r="A10" s="20" t="n"/>
+      <c r="B10" s="20" t="n"/>
+      <c r="C10" s="20" t="n"/>
+      <c r="D10" s="20" t="n"/>
+      <c r="E10" s="20" t="n"/>
+      <c r="F10" s="20" t="n"/>
+      <c r="G10" s="20" t="n"/>
+      <c r="H10" s="20" t="n"/>
+      <c r="I10" s="20" t="n"/>
+      <c r="J10" s="20" t="n"/>
+      <c r="K10" s="20" t="n"/>
+      <c r="L10" s="20" t="n"/>
+      <c r="M10" s="20" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="19" t="n"/>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
-      <c r="J11" s="19" t="n"/>
-      <c r="K11" s="19" t="n"/>
-      <c r="L11" s="19" t="n"/>
-      <c r="M11" s="19" t="n"/>
+      <c r="A11" s="20" t="n"/>
+      <c r="B11" s="20" t="n"/>
+      <c r="C11" s="20" t="n"/>
+      <c r="D11" s="20" t="n"/>
+      <c r="E11" s="20" t="n"/>
+      <c r="F11" s="20" t="n"/>
+      <c r="G11" s="20" t="n"/>
+      <c r="H11" s="20" t="n"/>
+      <c r="I11" s="20" t="n"/>
+      <c r="J11" s="20" t="n"/>
+      <c r="K11" s="20" t="n"/>
+      <c r="L11" s="20" t="n"/>
+      <c r="M11" s="20" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="19" t="n"/>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
-      <c r="J12" s="19" t="n"/>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" s="19" t="n"/>
-      <c r="M12" s="19" t="n"/>
+      <c r="A12" s="20" t="n"/>
+      <c r="B12" s="20" t="n"/>
+      <c r="C12" s="20" t="n"/>
+      <c r="D12" s="20" t="n"/>
+      <c r="E12" s="20" t="n"/>
+      <c r="F12" s="20" t="n"/>
+      <c r="G12" s="20" t="n"/>
+      <c r="H12" s="20" t="n"/>
+      <c r="I12" s="20" t="n"/>
+      <c r="J12" s="20" t="n"/>
+      <c r="K12" s="20" t="n"/>
+      <c r="L12" s="20" t="n"/>
+      <c r="M12" s="20" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="19" t="n"/>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="19" t="n"/>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="19" t="n"/>
-      <c r="J13" s="19" t="n"/>
-      <c r="K13" s="19" t="n"/>
-      <c r="L13" s="19" t="n"/>
-      <c r="M13" s="19" t="n"/>
+      <c r="A13" s="20" t="n"/>
+      <c r="B13" s="20" t="n"/>
+      <c r="C13" s="20" t="n"/>
+      <c r="D13" s="20" t="n"/>
+      <c r="E13" s="20" t="n"/>
+      <c r="F13" s="20" t="n"/>
+      <c r="G13" s="20" t="n"/>
+      <c r="H13" s="20" t="n"/>
+      <c r="I13" s="20" t="n"/>
+      <c r="J13" s="20" t="n"/>
+      <c r="K13" s="20" t="n"/>
+      <c r="L13" s="20" t="n"/>
+      <c r="M13" s="20" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="19" t="n"/>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
-      <c r="E14" s="19" t="n"/>
-      <c r="F14" s="19" t="n"/>
-      <c r="G14" s="19" t="n"/>
-      <c r="H14" s="19" t="n"/>
-      <c r="I14" s="19" t="n"/>
-      <c r="J14" s="19" t="n"/>
-      <c r="K14" s="19" t="n"/>
-      <c r="L14" s="19" t="n"/>
-      <c r="M14" s="19" t="n"/>
+      <c r="A14" s="20" t="n"/>
+      <c r="B14" s="20" t="n"/>
+      <c r="C14" s="20" t="n"/>
+      <c r="D14" s="20" t="n"/>
+      <c r="E14" s="20" t="n"/>
+      <c r="F14" s="20" t="n"/>
+      <c r="G14" s="20" t="n"/>
+      <c r="H14" s="20" t="n"/>
+      <c r="I14" s="20" t="n"/>
+      <c r="J14" s="20" t="n"/>
+      <c r="K14" s="20" t="n"/>
+      <c r="L14" s="20" t="n"/>
+      <c r="M14" s="20" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="19" t="n"/>
-      <c r="C15" s="19" t="n"/>
-      <c r="D15" s="19" t="n"/>
-      <c r="E15" s="19" t="n"/>
-      <c r="F15" s="19" t="n"/>
-      <c r="G15" s="19" t="n"/>
-      <c r="H15" s="19" t="n"/>
-      <c r="I15" s="19" t="n"/>
-      <c r="J15" s="19" t="n"/>
-      <c r="K15" s="19" t="n"/>
-      <c r="L15" s="19" t="n"/>
-      <c r="M15" s="19" t="n"/>
+      <c r="A15" s="20" t="n"/>
+      <c r="B15" s="20" t="n"/>
+      <c r="C15" s="20" t="n"/>
+      <c r="D15" s="20" t="n"/>
+      <c r="E15" s="20" t="n"/>
+      <c r="F15" s="20" t="n"/>
+      <c r="G15" s="20" t="n"/>
+      <c r="H15" s="20" t="n"/>
+      <c r="I15" s="20" t="n"/>
+      <c r="J15" s="20" t="n"/>
+      <c r="K15" s="20" t="n"/>
+      <c r="L15" s="20" t="n"/>
+      <c r="M15" s="20" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Armes — deux mains   (1)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>War Axe</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>hache-de-guerre</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>Pommel Strike</t>
         </is>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F18" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="16" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>Giant Swing</t>
         </is>
       </c>
-      <c r="H18" s="15" t="n">
+      <c r="H18" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="16" t="inlineStr">
+      <c r="I18" s="17" t="inlineStr">
         <is>
           <t>Cleave</t>
         </is>
       </c>
-      <c r="J18" s="15" t="n">
+      <c r="J18" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="K18" s="16" t="n"/>
-      <c r="L18" s="16" t="n"/>
-      <c r="M18" s="16" t="n"/>
+      <c r="K18" s="17" t="n"/>
+      <c r="L18" s="17" t="n"/>
+      <c r="M18" s="17" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="19" t="n"/>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="19" t="n"/>
-      <c r="E19" s="19" t="n"/>
-      <c r="F19" s="19" t="n"/>
-      <c r="G19" s="19" t="n"/>
-      <c r="H19" s="19" t="n"/>
-      <c r="I19" s="19" t="n"/>
-      <c r="J19" s="19" t="n"/>
-      <c r="K19" s="19" t="n"/>
-      <c r="L19" s="19" t="n"/>
-      <c r="M19" s="19" t="n"/>
+      <c r="A19" s="20" t="n"/>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
+      <c r="J19" s="20" t="n"/>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+      <c r="M19" s="20" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="19" t="n"/>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="19" t="n"/>
-      <c r="G20" s="19" t="n"/>
-      <c r="H20" s="19" t="n"/>
-      <c r="I20" s="19" t="n"/>
-      <c r="J20" s="19" t="n"/>
-      <c r="K20" s="19" t="n"/>
-      <c r="L20" s="19" t="n"/>
-      <c r="M20" s="19" t="n"/>
+      <c r="A20" s="20" t="n"/>
+      <c r="B20" s="20" t="n"/>
+      <c r="C20" s="20" t="n"/>
+      <c r="D20" s="20" t="n"/>
+      <c r="E20" s="20" t="n"/>
+      <c r="F20" s="20" t="n"/>
+      <c r="G20" s="20" t="n"/>
+      <c r="H20" s="20" t="n"/>
+      <c r="I20" s="20" t="n"/>
+      <c r="J20" s="20" t="n"/>
+      <c r="K20" s="20" t="n"/>
+      <c r="L20" s="20" t="n"/>
+      <c r="M20" s="20" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-      <c r="E21" s="19" t="n"/>
-      <c r="F21" s="19" t="n"/>
-      <c r="G21" s="19" t="n"/>
-      <c r="H21" s="19" t="n"/>
-      <c r="I21" s="19" t="n"/>
-      <c r="J21" s="19" t="n"/>
-      <c r="K21" s="19" t="n"/>
-      <c r="L21" s="19" t="n"/>
-      <c r="M21" s="19" t="n"/>
+      <c r="A21" s="20" t="n"/>
+      <c r="B21" s="20" t="n"/>
+      <c r="C21" s="20" t="n"/>
+      <c r="D21" s="20" t="n"/>
+      <c r="E21" s="20" t="n"/>
+      <c r="F21" s="20" t="n"/>
+      <c r="G21" s="20" t="n"/>
+      <c r="H21" s="20" t="n"/>
+      <c r="I21" s="20" t="n"/>
+      <c r="J21" s="20" t="n"/>
+      <c r="K21" s="20" t="n"/>
+      <c r="L21" s="20" t="n"/>
+      <c r="M21" s="20" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="19" t="n"/>
-      <c r="F22" s="19" t="n"/>
-      <c r="G22" s="19" t="n"/>
-      <c r="H22" s="19" t="n"/>
-      <c r="I22" s="19" t="n"/>
-      <c r="J22" s="19" t="n"/>
-      <c r="K22" s="19" t="n"/>
-      <c r="L22" s="19" t="n"/>
-      <c r="M22" s="19" t="n"/>
+      <c r="A22" s="20" t="n"/>
+      <c r="B22" s="20" t="n"/>
+      <c r="C22" s="20" t="n"/>
+      <c r="D22" s="20" t="n"/>
+      <c r="E22" s="20" t="n"/>
+      <c r="F22" s="20" t="n"/>
+      <c r="G22" s="20" t="n"/>
+      <c r="H22" s="20" t="n"/>
+      <c r="I22" s="20" t="n"/>
+      <c r="J22" s="20" t="n"/>
+      <c r="K22" s="20" t="n"/>
+      <c r="L22" s="20" t="n"/>
+      <c r="M22" s="20" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="19" t="n"/>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="19" t="n"/>
-      <c r="F23" s="19" t="n"/>
-      <c r="G23" s="19" t="n"/>
-      <c r="H23" s="19" t="n"/>
-      <c r="I23" s="19" t="n"/>
-      <c r="J23" s="19" t="n"/>
-      <c r="K23" s="19" t="n"/>
-      <c r="L23" s="19" t="n"/>
-      <c r="M23" s="19" t="n"/>
+      <c r="A23" s="20" t="n"/>
+      <c r="B23" s="20" t="n"/>
+      <c r="C23" s="20" t="n"/>
+      <c r="D23" s="20" t="n"/>
+      <c r="E23" s="20" t="n"/>
+      <c r="F23" s="20" t="n"/>
+      <c r="G23" s="20" t="n"/>
+      <c r="H23" s="20" t="n"/>
+      <c r="I23" s="20" t="n"/>
+      <c r="J23" s="20" t="n"/>
+      <c r="K23" s="20" t="n"/>
+      <c r="L23" s="20" t="n"/>
+      <c r="M23" s="20" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="19" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
-      <c r="G24" s="19" t="n"/>
-      <c r="H24" s="19" t="n"/>
-      <c r="I24" s="19" t="n"/>
-      <c r="J24" s="19" t="n"/>
-      <c r="K24" s="19" t="n"/>
-      <c r="L24" s="19" t="n"/>
-      <c r="M24" s="19" t="n"/>
+      <c r="A24" s="20" t="n"/>
+      <c r="B24" s="20" t="n"/>
+      <c r="C24" s="20" t="n"/>
+      <c r="D24" s="20" t="n"/>
+      <c r="E24" s="20" t="n"/>
+      <c r="F24" s="20" t="n"/>
+      <c r="G24" s="20" t="n"/>
+      <c r="H24" s="20" t="n"/>
+      <c r="I24" s="20" t="n"/>
+      <c r="J24" s="20" t="n"/>
+      <c r="K24" s="20" t="n"/>
+      <c r="L24" s="20" t="n"/>
+      <c r="M24" s="20" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Boucliers (main 2nde)   (1)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Tower Shield</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>bouclier-tour</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C27" s="19" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="D27" s="15" t="n">
+      <c r="D27" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>Shield Wall</t>
         </is>
       </c>
-      <c r="F27" s="15" t="n">
+      <c r="F27" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="16" t="inlineStr">
+      <c r="G27" s="17" t="inlineStr">
         <is>
           <t>Shield Bash</t>
         </is>
       </c>
-      <c r="H27" s="15" t="n">
+      <c r="H27" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I27" s="16" t="n"/>
-      <c r="J27" s="16" t="n"/>
-      <c r="K27" s="16" t="n"/>
-      <c r="L27" s="16" t="n"/>
-      <c r="M27" s="16" t="n"/>
+      <c r="I27" s="17" t="n"/>
+      <c r="J27" s="17" t="n"/>
+      <c r="K27" s="17" t="n"/>
+      <c r="L27" s="17" t="n"/>
+      <c r="M27" s="17" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="19" t="n"/>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="19" t="n"/>
-      <c r="E28" s="19" t="n"/>
-      <c r="F28" s="19" t="n"/>
-      <c r="G28" s="19" t="n"/>
-      <c r="H28" s="19" t="n"/>
-      <c r="I28" s="19" t="n"/>
-      <c r="J28" s="19" t="n"/>
-      <c r="K28" s="19" t="n"/>
-      <c r="L28" s="19" t="n"/>
-      <c r="M28" s="19" t="n"/>
+      <c r="A28" s="20" t="n"/>
+      <c r="B28" s="20" t="n"/>
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="20" t="n"/>
+      <c r="E28" s="20" t="n"/>
+      <c r="F28" s="20" t="n"/>
+      <c r="G28" s="20" t="n"/>
+      <c r="H28" s="20" t="n"/>
+      <c r="I28" s="20" t="n"/>
+      <c r="J28" s="20" t="n"/>
+      <c r="K28" s="20" t="n"/>
+      <c r="L28" s="20" t="n"/>
+      <c r="M28" s="20" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="19" t="n"/>
-      <c r="C29" s="19" t="n"/>
-      <c r="D29" s="19" t="n"/>
-      <c r="E29" s="19" t="n"/>
-      <c r="F29" s="19" t="n"/>
-      <c r="G29" s="19" t="n"/>
-      <c r="H29" s="19" t="n"/>
-      <c r="I29" s="19" t="n"/>
-      <c r="J29" s="19" t="n"/>
-      <c r="K29" s="19" t="n"/>
-      <c r="L29" s="19" t="n"/>
-      <c r="M29" s="19" t="n"/>
+      <c r="A29" s="20" t="n"/>
+      <c r="B29" s="20" t="n"/>
+      <c r="C29" s="20" t="n"/>
+      <c r="D29" s="20" t="n"/>
+      <c r="E29" s="20" t="n"/>
+      <c r="F29" s="20" t="n"/>
+      <c r="G29" s="20" t="n"/>
+      <c r="H29" s="20" t="n"/>
+      <c r="I29" s="20" t="n"/>
+      <c r="J29" s="20" t="n"/>
+      <c r="K29" s="20" t="n"/>
+      <c r="L29" s="20" t="n"/>
+      <c r="M29" s="20" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="19" t="n"/>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="19" t="n"/>
-      <c r="E30" s="19" t="n"/>
-      <c r="F30" s="19" t="n"/>
-      <c r="G30" s="19" t="n"/>
-      <c r="H30" s="19" t="n"/>
-      <c r="I30" s="19" t="n"/>
-      <c r="J30" s="19" t="n"/>
-      <c r="K30" s="19" t="n"/>
-      <c r="L30" s="19" t="n"/>
-      <c r="M30" s="19" t="n"/>
+      <c r="A30" s="20" t="n"/>
+      <c r="B30" s="20" t="n"/>
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="20" t="n"/>
+      <c r="E30" s="20" t="n"/>
+      <c r="F30" s="20" t="n"/>
+      <c r="G30" s="20" t="n"/>
+      <c r="H30" s="20" t="n"/>
+      <c r="I30" s="20" t="n"/>
+      <c r="J30" s="20" t="n"/>
+      <c r="K30" s="20" t="n"/>
+      <c r="L30" s="20" t="n"/>
+      <c r="M30" s="20" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="n"/>
-      <c r="B31" s="19" t="n"/>
-      <c r="C31" s="19" t="n"/>
-      <c r="D31" s="19" t="n"/>
-      <c r="E31" s="19" t="n"/>
-      <c r="F31" s="19" t="n"/>
-      <c r="G31" s="19" t="n"/>
-      <c r="H31" s="19" t="n"/>
-      <c r="I31" s="19" t="n"/>
-      <c r="J31" s="19" t="n"/>
-      <c r="K31" s="19" t="n"/>
-      <c r="L31" s="19" t="n"/>
-      <c r="M31" s="19" t="n"/>
+      <c r="A31" s="20" t="n"/>
+      <c r="B31" s="20" t="n"/>
+      <c r="C31" s="20" t="n"/>
+      <c r="D31" s="20" t="n"/>
+      <c r="E31" s="20" t="n"/>
+      <c r="F31" s="20" t="n"/>
+      <c r="G31" s="20" t="n"/>
+      <c r="H31" s="20" t="n"/>
+      <c r="I31" s="20" t="n"/>
+      <c r="J31" s="20" t="n"/>
+      <c r="K31" s="20" t="n"/>
+      <c r="L31" s="20" t="n"/>
+      <c r="M31" s="20" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="n"/>
-      <c r="B32" s="19" t="n"/>
-      <c r="C32" s="19" t="n"/>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="19" t="n"/>
-      <c r="F32" s="19" t="n"/>
-      <c r="G32" s="19" t="n"/>
-      <c r="H32" s="19" t="n"/>
-      <c r="I32" s="19" t="n"/>
-      <c r="J32" s="19" t="n"/>
-      <c r="K32" s="19" t="n"/>
-      <c r="L32" s="19" t="n"/>
-      <c r="M32" s="19" t="n"/>
+      <c r="A32" s="20" t="n"/>
+      <c r="B32" s="20" t="n"/>
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="20" t="n"/>
+      <c r="E32" s="20" t="n"/>
+      <c r="F32" s="20" t="n"/>
+      <c r="G32" s="20" t="n"/>
+      <c r="H32" s="20" t="n"/>
+      <c r="I32" s="20" t="n"/>
+      <c r="J32" s="20" t="n"/>
+      <c r="K32" s="20" t="n"/>
+      <c r="L32" s="20" t="n"/>
+      <c r="M32" s="20" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="n"/>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="19" t="n"/>
-      <c r="F33" s="19" t="n"/>
-      <c r="G33" s="19" t="n"/>
-      <c r="H33" s="19" t="n"/>
-      <c r="I33" s="19" t="n"/>
-      <c r="J33" s="19" t="n"/>
-      <c r="K33" s="19" t="n"/>
-      <c r="L33" s="19" t="n"/>
-      <c r="M33" s="19" t="n"/>
+      <c r="A33" s="20" t="n"/>
+      <c r="B33" s="20" t="n"/>
+      <c r="C33" s="20" t="n"/>
+      <c r="D33" s="20" t="n"/>
+      <c r="E33" s="20" t="n"/>
+      <c r="F33" s="20" t="n"/>
+      <c r="G33" s="20" t="n"/>
+      <c r="H33" s="20" t="n"/>
+      <c r="I33" s="20" t="n"/>
+      <c r="J33" s="20" t="n"/>
+      <c r="K33" s="20" t="n"/>
+      <c r="L33" s="20" t="n"/>
+      <c r="M33" s="20" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Armures   (3)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>Traveler's Garb</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>tenue-de-voyageur</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="C36" s="15" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D36" s="15" t="n">
+      <c r="D36" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="16" t="n"/>
-      <c r="F36" s="16" t="n"/>
-      <c r="G36" s="16" t="n"/>
-      <c r="H36" s="16" t="n"/>
-      <c r="I36" s="16" t="n"/>
-      <c r="J36" s="16" t="n"/>
-      <c r="K36" s="16" t="n"/>
-      <c r="L36" s="16" t="n"/>
-      <c r="M36" s="16" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="17" t="n"/>
+      <c r="G36" s="17" t="n"/>
+      <c r="H36" s="17" t="n"/>
+      <c r="I36" s="17" t="n"/>
+      <c r="J36" s="17" t="n"/>
+      <c r="K36" s="17" t="n"/>
+      <c r="L36" s="17" t="n"/>
+      <c r="M36" s="17" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>Onyx Guard Plate</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>plate-onyx</t>
         </is>
       </c>
-      <c r="C37" s="17" t="inlineStr">
+      <c r="C37" s="18" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="D37" s="15" t="n">
+      <c r="D37" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="E37" s="16" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>Onyx Armor</t>
         </is>
       </c>
-      <c r="F37" s="15" t="n">
+      <c r="F37" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G37" s="16" t="inlineStr">
+      <c r="G37" s="17" t="inlineStr">
         <is>
           <t>Dragon's Blaze</t>
         </is>
       </c>
-      <c r="H37" s="15" t="n">
+      <c r="H37" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I37" s="16" t="inlineStr">
+      <c r="I37" s="17" t="inlineStr">
         <is>
           <t>Onyx Breath</t>
         </is>
       </c>
-      <c r="J37" s="15" t="n">
+      <c r="J37" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="K37" s="16" t="n"/>
-      <c r="L37" s="16" t="n"/>
-      <c r="M37" s="16" t="n"/>
+      <c r="K37" s="17" t="n"/>
+      <c r="L37" s="17" t="n"/>
+      <c r="M37" s="17" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Forgemaster's Mail</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>maille-de-forge</t>
         </is>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="C38" s="18" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="D38" s="15" t="n">
+      <c r="D38" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="E38" s="16" t="inlineStr">
+      <c r="E38" s="17" t="inlineStr">
         <is>
           <t>Mail Armor</t>
         </is>
       </c>
-      <c r="F38" s="15" t="n">
+      <c r="F38" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G38" s="16" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr">
         <is>
           <t>Quench</t>
         </is>
       </c>
-      <c r="H38" s="15" t="n">
+      <c r="H38" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I38" s="16" t="n"/>
-      <c r="J38" s="16" t="n"/>
-      <c r="K38" s="16" t="n"/>
-      <c r="L38" s="16" t="n"/>
-      <c r="M38" s="16" t="n"/>
+      <c r="I38" s="17" t="n"/>
+      <c r="J38" s="17" t="n"/>
+      <c r="K38" s="17" t="n"/>
+      <c r="L38" s="17" t="n"/>
+      <c r="M38" s="17" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="n"/>
-      <c r="B39" s="19" t="n"/>
-      <c r="C39" s="19" t="n"/>
-      <c r="D39" s="19" t="n"/>
-      <c r="E39" s="19" t="n"/>
-      <c r="F39" s="19" t="n"/>
-      <c r="G39" s="19" t="n"/>
-      <c r="H39" s="19" t="n"/>
-      <c r="I39" s="19" t="n"/>
-      <c r="J39" s="19" t="n"/>
-      <c r="K39" s="19" t="n"/>
-      <c r="L39" s="19" t="n"/>
-      <c r="M39" s="19" t="n"/>
+      <c r="A39" s="20" t="n"/>
+      <c r="B39" s="20" t="n"/>
+      <c r="C39" s="20" t="n"/>
+      <c r="D39" s="20" t="n"/>
+      <c r="E39" s="20" t="n"/>
+      <c r="F39" s="20" t="n"/>
+      <c r="G39" s="20" t="n"/>
+      <c r="H39" s="20" t="n"/>
+      <c r="I39" s="20" t="n"/>
+      <c r="J39" s="20" t="n"/>
+      <c r="K39" s="20" t="n"/>
+      <c r="L39" s="20" t="n"/>
+      <c r="M39" s="20" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="n"/>
-      <c r="B40" s="19" t="n"/>
-      <c r="C40" s="19" t="n"/>
-      <c r="D40" s="19" t="n"/>
-      <c r="E40" s="19" t="n"/>
-      <c r="F40" s="19" t="n"/>
-      <c r="G40" s="19" t="n"/>
-      <c r="H40" s="19" t="n"/>
-      <c r="I40" s="19" t="n"/>
-      <c r="J40" s="19" t="n"/>
-      <c r="K40" s="19" t="n"/>
-      <c r="L40" s="19" t="n"/>
-      <c r="M40" s="19" t="n"/>
+      <c r="A40" s="20" t="n"/>
+      <c r="B40" s="20" t="n"/>
+      <c r="C40" s="20" t="n"/>
+      <c r="D40" s="20" t="n"/>
+      <c r="E40" s="20" t="n"/>
+      <c r="F40" s="20" t="n"/>
+      <c r="G40" s="20" t="n"/>
+      <c r="H40" s="20" t="n"/>
+      <c r="I40" s="20" t="n"/>
+      <c r="J40" s="20" t="n"/>
+      <c r="K40" s="20" t="n"/>
+      <c r="L40" s="20" t="n"/>
+      <c r="M40" s="20" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="n"/>
-      <c r="B41" s="19" t="n"/>
-      <c r="C41" s="19" t="n"/>
-      <c r="D41" s="19" t="n"/>
-      <c r="E41" s="19" t="n"/>
-      <c r="F41" s="19" t="n"/>
-      <c r="G41" s="19" t="n"/>
-      <c r="H41" s="19" t="n"/>
-      <c r="I41" s="19" t="n"/>
-      <c r="J41" s="19" t="n"/>
-      <c r="K41" s="19" t="n"/>
-      <c r="L41" s="19" t="n"/>
-      <c r="M41" s="19" t="n"/>
+      <c r="A41" s="20" t="n"/>
+      <c r="B41" s="20" t="n"/>
+      <c r="C41" s="20" t="n"/>
+      <c r="D41" s="20" t="n"/>
+      <c r="E41" s="20" t="n"/>
+      <c r="F41" s="20" t="n"/>
+      <c r="G41" s="20" t="n"/>
+      <c r="H41" s="20" t="n"/>
+      <c r="I41" s="20" t="n"/>
+      <c r="J41" s="20" t="n"/>
+      <c r="K41" s="20" t="n"/>
+      <c r="L41" s="20" t="n"/>
+      <c r="M41" s="20" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="19" t="n"/>
-      <c r="B42" s="19" t="n"/>
-      <c r="C42" s="19" t="n"/>
-      <c r="D42" s="19" t="n"/>
-      <c r="E42" s="19" t="n"/>
-      <c r="F42" s="19" t="n"/>
-      <c r="G42" s="19" t="n"/>
-      <c r="H42" s="19" t="n"/>
-      <c r="I42" s="19" t="n"/>
-      <c r="J42" s="19" t="n"/>
-      <c r="K42" s="19" t="n"/>
-      <c r="L42" s="19" t="n"/>
-      <c r="M42" s="19" t="n"/>
+      <c r="A42" s="20" t="n"/>
+      <c r="B42" s="20" t="n"/>
+      <c r="C42" s="20" t="n"/>
+      <c r="D42" s="20" t="n"/>
+      <c r="E42" s="20" t="n"/>
+      <c r="F42" s="20" t="n"/>
+      <c r="G42" s="20" t="n"/>
+      <c r="H42" s="20" t="n"/>
+      <c r="I42" s="20" t="n"/>
+      <c r="J42" s="20" t="n"/>
+      <c r="K42" s="20" t="n"/>
+      <c r="L42" s="20" t="n"/>
+      <c r="M42" s="20" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="19" t="n"/>
-      <c r="B43" s="19" t="n"/>
-      <c r="C43" s="19" t="n"/>
-      <c r="D43" s="19" t="n"/>
-      <c r="E43" s="19" t="n"/>
-      <c r="F43" s="19" t="n"/>
-      <c r="G43" s="19" t="n"/>
-      <c r="H43" s="19" t="n"/>
-      <c r="I43" s="19" t="n"/>
-      <c r="J43" s="19" t="n"/>
-      <c r="K43" s="19" t="n"/>
-      <c r="L43" s="19" t="n"/>
-      <c r="M43" s="19" t="n"/>
+      <c r="A43" s="20" t="n"/>
+      <c r="B43" s="20" t="n"/>
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="20" t="n"/>
+      <c r="E43" s="20" t="n"/>
+      <c r="F43" s="20" t="n"/>
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="20" t="n"/>
+      <c r="J43" s="20" t="n"/>
+      <c r="K43" s="20" t="n"/>
+      <c r="L43" s="20" t="n"/>
+      <c r="M43" s="20" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="19" t="n"/>
-      <c r="B44" s="19" t="n"/>
-      <c r="C44" s="19" t="n"/>
-      <c r="D44" s="19" t="n"/>
-      <c r="E44" s="19" t="n"/>
-      <c r="F44" s="19" t="n"/>
-      <c r="G44" s="19" t="n"/>
-      <c r="H44" s="19" t="n"/>
-      <c r="I44" s="19" t="n"/>
-      <c r="J44" s="19" t="n"/>
-      <c r="K44" s="19" t="n"/>
-      <c r="L44" s="19" t="n"/>
-      <c r="M44" s="19" t="n"/>
+      <c r="A44" s="20" t="n"/>
+      <c r="B44" s="20" t="n"/>
+      <c r="C44" s="20" t="n"/>
+      <c r="D44" s="20" t="n"/>
+      <c r="E44" s="20" t="n"/>
+      <c r="F44" s="20" t="n"/>
+      <c r="G44" s="20" t="n"/>
+      <c r="H44" s="20" t="n"/>
+      <c r="I44" s="20" t="n"/>
+      <c r="J44" s="20" t="n"/>
+      <c r="K44" s="20" t="n"/>
+      <c r="L44" s="20" t="n"/>
+      <c r="M44" s="20" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>Colliers   (1)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="12" t="inlineStr">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>Sapphire Amulet</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>collier-de-saphir</t>
         </is>
       </c>
-      <c r="C47" s="18" t="inlineStr">
+      <c r="C47" s="19" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="D47" s="15" t="n">
+      <c r="D47" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E47" s="16" t="inlineStr">
+      <c r="E47" s="17" t="inlineStr">
         <is>
           <t>Sapphire Surge</t>
         </is>
       </c>
-      <c r="F47" s="15" t="n">
+      <c r="F47" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G47" s="16" t="n"/>
-      <c r="H47" s="16" t="n"/>
-      <c r="I47" s="16" t="n"/>
-      <c r="J47" s="16" t="n"/>
-      <c r="K47" s="16" t="n"/>
-      <c r="L47" s="16" t="n"/>
-      <c r="M47" s="16" t="n"/>
+      <c r="G47" s="17" t="n"/>
+      <c r="H47" s="17" t="n"/>
+      <c r="I47" s="17" t="n"/>
+      <c r="J47" s="17" t="n"/>
+      <c r="K47" s="17" t="n"/>
+      <c r="L47" s="17" t="n"/>
+      <c r="M47" s="17" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="19" t="n"/>
-      <c r="B48" s="19" t="n"/>
-      <c r="C48" s="19" t="n"/>
-      <c r="D48" s="19" t="n"/>
-      <c r="E48" s="19" t="n"/>
-      <c r="F48" s="19" t="n"/>
-      <c r="G48" s="19" t="n"/>
-      <c r="H48" s="19" t="n"/>
-      <c r="I48" s="19" t="n"/>
-      <c r="J48" s="19" t="n"/>
-      <c r="K48" s="19" t="n"/>
-      <c r="L48" s="19" t="n"/>
-      <c r="M48" s="19" t="n"/>
+      <c r="A48" s="20" t="n"/>
+      <c r="B48" s="20" t="n"/>
+      <c r="C48" s="20" t="n"/>
+      <c r="D48" s="20" t="n"/>
+      <c r="E48" s="20" t="n"/>
+      <c r="F48" s="20" t="n"/>
+      <c r="G48" s="20" t="n"/>
+      <c r="H48" s="20" t="n"/>
+      <c r="I48" s="20" t="n"/>
+      <c r="J48" s="20" t="n"/>
+      <c r="K48" s="20" t="n"/>
+      <c r="L48" s="20" t="n"/>
+      <c r="M48" s="20" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="n"/>
-      <c r="B49" s="19" t="n"/>
-      <c r="C49" s="19" t="n"/>
-      <c r="D49" s="19" t="n"/>
-      <c r="E49" s="19" t="n"/>
-      <c r="F49" s="19" t="n"/>
-      <c r="G49" s="19" t="n"/>
-      <c r="H49" s="19" t="n"/>
-      <c r="I49" s="19" t="n"/>
-      <c r="J49" s="19" t="n"/>
-      <c r="K49" s="19" t="n"/>
-      <c r="L49" s="19" t="n"/>
-      <c r="M49" s="19" t="n"/>
+      <c r="A49" s="20" t="n"/>
+      <c r="B49" s="20" t="n"/>
+      <c r="C49" s="20" t="n"/>
+      <c r="D49" s="20" t="n"/>
+      <c r="E49" s="20" t="n"/>
+      <c r="F49" s="20" t="n"/>
+      <c r="G49" s="20" t="n"/>
+      <c r="H49" s="20" t="n"/>
+      <c r="I49" s="20" t="n"/>
+      <c r="J49" s="20" t="n"/>
+      <c r="K49" s="20" t="n"/>
+      <c r="L49" s="20" t="n"/>
+      <c r="M49" s="20" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="n"/>
-      <c r="B50" s="19" t="n"/>
-      <c r="C50" s="19" t="n"/>
-      <c r="D50" s="19" t="n"/>
-      <c r="E50" s="19" t="n"/>
-      <c r="F50" s="19" t="n"/>
-      <c r="G50" s="19" t="n"/>
-      <c r="H50" s="19" t="n"/>
-      <c r="I50" s="19" t="n"/>
-      <c r="J50" s="19" t="n"/>
-      <c r="K50" s="19" t="n"/>
-      <c r="L50" s="19" t="n"/>
-      <c r="M50" s="19" t="n"/>
+      <c r="A50" s="20" t="n"/>
+      <c r="B50" s="20" t="n"/>
+      <c r="C50" s="20" t="n"/>
+      <c r="D50" s="20" t="n"/>
+      <c r="E50" s="20" t="n"/>
+      <c r="F50" s="20" t="n"/>
+      <c r="G50" s="20" t="n"/>
+      <c r="H50" s="20" t="n"/>
+      <c r="I50" s="20" t="n"/>
+      <c r="J50" s="20" t="n"/>
+      <c r="K50" s="20" t="n"/>
+      <c r="L50" s="20" t="n"/>
+      <c r="M50" s="20" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="19" t="n"/>
-      <c r="B51" s="19" t="n"/>
-      <c r="C51" s="19" t="n"/>
-      <c r="D51" s="19" t="n"/>
-      <c r="E51" s="19" t="n"/>
-      <c r="F51" s="19" t="n"/>
-      <c r="G51" s="19" t="n"/>
-      <c r="H51" s="19" t="n"/>
-      <c r="I51" s="19" t="n"/>
-      <c r="J51" s="19" t="n"/>
-      <c r="K51" s="19" t="n"/>
-      <c r="L51" s="19" t="n"/>
-      <c r="M51" s="19" t="n"/>
+      <c r="A51" s="20" t="n"/>
+      <c r="B51" s="20" t="n"/>
+      <c r="C51" s="20" t="n"/>
+      <c r="D51" s="20" t="n"/>
+      <c r="E51" s="20" t="n"/>
+      <c r="F51" s="20" t="n"/>
+      <c r="G51" s="20" t="n"/>
+      <c r="H51" s="20" t="n"/>
+      <c r="I51" s="20" t="n"/>
+      <c r="J51" s="20" t="n"/>
+      <c r="K51" s="20" t="n"/>
+      <c r="L51" s="20" t="n"/>
+      <c r="M51" s="20" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="19" t="n"/>
-      <c r="B52" s="19" t="n"/>
-      <c r="C52" s="19" t="n"/>
-      <c r="D52" s="19" t="n"/>
-      <c r="E52" s="19" t="n"/>
-      <c r="F52" s="19" t="n"/>
-      <c r="G52" s="19" t="n"/>
-      <c r="H52" s="19" t="n"/>
-      <c r="I52" s="19" t="n"/>
-      <c r="J52" s="19" t="n"/>
-      <c r="K52" s="19" t="n"/>
-      <c r="L52" s="19" t="n"/>
-      <c r="M52" s="19" t="n"/>
+      <c r="A52" s="20" t="n"/>
+      <c r="B52" s="20" t="n"/>
+      <c r="C52" s="20" t="n"/>
+      <c r="D52" s="20" t="n"/>
+      <c r="E52" s="20" t="n"/>
+      <c r="F52" s="20" t="n"/>
+      <c r="G52" s="20" t="n"/>
+      <c r="H52" s="20" t="n"/>
+      <c r="I52" s="20" t="n"/>
+      <c r="J52" s="20" t="n"/>
+      <c r="K52" s="20" t="n"/>
+      <c r="L52" s="20" t="n"/>
+      <c r="M52" s="20" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="19" t="n"/>
-      <c r="B53" s="19" t="n"/>
-      <c r="C53" s="19" t="n"/>
-      <c r="D53" s="19" t="n"/>
-      <c r="E53" s="19" t="n"/>
-      <c r="F53" s="19" t="n"/>
-      <c r="G53" s="19" t="n"/>
-      <c r="H53" s="19" t="n"/>
-      <c r="I53" s="19" t="n"/>
-      <c r="J53" s="19" t="n"/>
-      <c r="K53" s="19" t="n"/>
-      <c r="L53" s="19" t="n"/>
-      <c r="M53" s="19" t="n"/>
+      <c r="A53" s="20" t="n"/>
+      <c r="B53" s="20" t="n"/>
+      <c r="C53" s="20" t="n"/>
+      <c r="D53" s="20" t="n"/>
+      <c r="E53" s="20" t="n"/>
+      <c r="F53" s="20" t="n"/>
+      <c r="G53" s="20" t="n"/>
+      <c r="H53" s="20" t="n"/>
+      <c r="I53" s="20" t="n"/>
+      <c r="J53" s="20" t="n"/>
+      <c r="K53" s="20" t="n"/>
+      <c r="L53" s="20" t="n"/>
+      <c r="M53" s="20" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t>Bagues   (2)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="inlineStr">
+      <c r="A56" s="13" t="inlineStr">
         <is>
           <t>Blood Ring</t>
         </is>
       </c>
-      <c r="B56" s="13" t="inlineStr">
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>bague-de-sang</t>
         </is>
       </c>
-      <c r="C56" s="17" t="inlineStr">
+      <c r="C56" s="18" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="D56" s="15" t="n">
+      <c r="D56" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E56" s="16" t="inlineStr">
+      <c r="E56" s="17" t="inlineStr">
         <is>
           <t>Bloodletting</t>
         </is>
       </c>
-      <c r="F56" s="15" t="n">
+      <c r="F56" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G56" s="16" t="n"/>
-      <c r="H56" s="16" t="n"/>
-      <c r="I56" s="16" t="n"/>
-      <c r="J56" s="16" t="n"/>
-      <c r="K56" s="16" t="n"/>
-      <c r="L56" s="16" t="n"/>
-      <c r="M56" s="16" t="n"/>
+      <c r="G56" s="17" t="n"/>
+      <c r="H56" s="17" t="n"/>
+      <c r="I56" s="17" t="n"/>
+      <c r="J56" s="17" t="n"/>
+      <c r="K56" s="17" t="n"/>
+      <c r="L56" s="17" t="n"/>
+      <c r="M56" s="17" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="inlineStr">
+      <c r="A57" s="13" t="inlineStr">
         <is>
           <t>Frost Ring</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>anneau-de-givre</t>
         </is>
       </c>
-      <c r="C57" s="17" t="inlineStr">
+      <c r="C57" s="18" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="D57" s="15" t="n">
+      <c r="D57" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E57" s="16" t="inlineStr">
+      <c r="E57" s="17" t="inlineStr">
         <is>
           <t>Frostbite</t>
         </is>
       </c>
-      <c r="F57" s="15" t="n">
+      <c r="F57" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G57" s="16" t="n"/>
-      <c r="H57" s="16" t="n"/>
-      <c r="I57" s="16" t="n"/>
-      <c r="J57" s="16" t="n"/>
-      <c r="K57" s="16" t="n"/>
-      <c r="L57" s="16" t="n"/>
-      <c r="M57" s="16" t="n"/>
+      <c r="G57" s="17" t="n"/>
+      <c r="H57" s="17" t="n"/>
+      <c r="I57" s="17" t="n"/>
+      <c r="J57" s="17" t="n"/>
+      <c r="K57" s="17" t="n"/>
+      <c r="L57" s="17" t="n"/>
+      <c r="M57" s="17" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="19" t="n"/>
-      <c r="B58" s="19" t="n"/>
-      <c r="C58" s="19" t="n"/>
-      <c r="D58" s="19" t="n"/>
-      <c r="E58" s="19" t="n"/>
-      <c r="F58" s="19" t="n"/>
-      <c r="G58" s="19" t="n"/>
-      <c r="H58" s="19" t="n"/>
-      <c r="I58" s="19" t="n"/>
-      <c r="J58" s="19" t="n"/>
-      <c r="K58" s="19" t="n"/>
-      <c r="L58" s="19" t="n"/>
-      <c r="M58" s="19" t="n"/>
+      <c r="A58" s="20" t="n"/>
+      <c r="B58" s="20" t="n"/>
+      <c r="C58" s="20" t="n"/>
+      <c r="D58" s="20" t="n"/>
+      <c r="E58" s="20" t="n"/>
+      <c r="F58" s="20" t="n"/>
+      <c r="G58" s="20" t="n"/>
+      <c r="H58" s="20" t="n"/>
+      <c r="I58" s="20" t="n"/>
+      <c r="J58" s="20" t="n"/>
+      <c r="K58" s="20" t="n"/>
+      <c r="L58" s="20" t="n"/>
+      <c r="M58" s="20" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="19" t="n"/>
-      <c r="B59" s="19" t="n"/>
-      <c r="C59" s="19" t="n"/>
-      <c r="D59" s="19" t="n"/>
-      <c r="E59" s="19" t="n"/>
-      <c r="F59" s="19" t="n"/>
-      <c r="G59" s="19" t="n"/>
-      <c r="H59" s="19" t="n"/>
-      <c r="I59" s="19" t="n"/>
-      <c r="J59" s="19" t="n"/>
-      <c r="K59" s="19" t="n"/>
-      <c r="L59" s="19" t="n"/>
-      <c r="M59" s="19" t="n"/>
+      <c r="A59" s="20" t="n"/>
+      <c r="B59" s="20" t="n"/>
+      <c r="C59" s="20" t="n"/>
+      <c r="D59" s="20" t="n"/>
+      <c r="E59" s="20" t="n"/>
+      <c r="F59" s="20" t="n"/>
+      <c r="G59" s="20" t="n"/>
+      <c r="H59" s="20" t="n"/>
+      <c r="I59" s="20" t="n"/>
+      <c r="J59" s="20" t="n"/>
+      <c r="K59" s="20" t="n"/>
+      <c r="L59" s="20" t="n"/>
+      <c r="M59" s="20" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="19" t="n"/>
-      <c r="B60" s="19" t="n"/>
-      <c r="C60" s="19" t="n"/>
-      <c r="D60" s="19" t="n"/>
-      <c r="E60" s="19" t="n"/>
-      <c r="F60" s="19" t="n"/>
-      <c r="G60" s="19" t="n"/>
-      <c r="H60" s="19" t="n"/>
-      <c r="I60" s="19" t="n"/>
-      <c r="J60" s="19" t="n"/>
-      <c r="K60" s="19" t="n"/>
-      <c r="L60" s="19" t="n"/>
-      <c r="M60" s="19" t="n"/>
+      <c r="A60" s="20" t="n"/>
+      <c r="B60" s="20" t="n"/>
+      <c r="C60" s="20" t="n"/>
+      <c r="D60" s="20" t="n"/>
+      <c r="E60" s="20" t="n"/>
+      <c r="F60" s="20" t="n"/>
+      <c r="G60" s="20" t="n"/>
+      <c r="H60" s="20" t="n"/>
+      <c r="I60" s="20" t="n"/>
+      <c r="J60" s="20" t="n"/>
+      <c r="K60" s="20" t="n"/>
+      <c r="L60" s="20" t="n"/>
+      <c r="M60" s="20" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="19" t="n"/>
-      <c r="B61" s="19" t="n"/>
-      <c r="C61" s="19" t="n"/>
-      <c r="D61" s="19" t="n"/>
-      <c r="E61" s="19" t="n"/>
-      <c r="F61" s="19" t="n"/>
-      <c r="G61" s="19" t="n"/>
-      <c r="H61" s="19" t="n"/>
-      <c r="I61" s="19" t="n"/>
-      <c r="J61" s="19" t="n"/>
-      <c r="K61" s="19" t="n"/>
-      <c r="L61" s="19" t="n"/>
-      <c r="M61" s="19" t="n"/>
+      <c r="A61" s="20" t="n"/>
+      <c r="B61" s="20" t="n"/>
+      <c r="C61" s="20" t="n"/>
+      <c r="D61" s="20" t="n"/>
+      <c r="E61" s="20" t="n"/>
+      <c r="F61" s="20" t="n"/>
+      <c r="G61" s="20" t="n"/>
+      <c r="H61" s="20" t="n"/>
+      <c r="I61" s="20" t="n"/>
+      <c r="J61" s="20" t="n"/>
+      <c r="K61" s="20" t="n"/>
+      <c r="L61" s="20" t="n"/>
+      <c r="M61" s="20" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="19" t="n"/>
-      <c r="B62" s="19" t="n"/>
-      <c r="C62" s="19" t="n"/>
-      <c r="D62" s="19" t="n"/>
-      <c r="E62" s="19" t="n"/>
-      <c r="F62" s="19" t="n"/>
-      <c r="G62" s="19" t="n"/>
-      <c r="H62" s="19" t="n"/>
-      <c r="I62" s="19" t="n"/>
-      <c r="J62" s="19" t="n"/>
-      <c r="K62" s="19" t="n"/>
-      <c r="L62" s="19" t="n"/>
-      <c r="M62" s="19" t="n"/>
+      <c r="A62" s="20" t="n"/>
+      <c r="B62" s="20" t="n"/>
+      <c r="C62" s="20" t="n"/>
+      <c r="D62" s="20" t="n"/>
+      <c r="E62" s="20" t="n"/>
+      <c r="F62" s="20" t="n"/>
+      <c r="G62" s="20" t="n"/>
+      <c r="H62" s="20" t="n"/>
+      <c r="I62" s="20" t="n"/>
+      <c r="J62" s="20" t="n"/>
+      <c r="K62" s="20" t="n"/>
+      <c r="L62" s="20" t="n"/>
+      <c r="M62" s="20" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="19" t="n"/>
-      <c r="B63" s="19" t="n"/>
-      <c r="C63" s="19" t="n"/>
-      <c r="D63" s="19" t="n"/>
-      <c r="E63" s="19" t="n"/>
-      <c r="F63" s="19" t="n"/>
-      <c r="G63" s="19" t="n"/>
-      <c r="H63" s="19" t="n"/>
-      <c r="I63" s="19" t="n"/>
-      <c r="J63" s="19" t="n"/>
-      <c r="K63" s="19" t="n"/>
-      <c r="L63" s="19" t="n"/>
-      <c r="M63" s="19" t="n"/>
+      <c r="A63" s="20" t="n"/>
+      <c r="B63" s="20" t="n"/>
+      <c r="C63" s="20" t="n"/>
+      <c r="D63" s="20" t="n"/>
+      <c r="E63" s="20" t="n"/>
+      <c r="F63" s="20" t="n"/>
+      <c r="G63" s="20" t="n"/>
+      <c r="H63" s="20" t="n"/>
+      <c r="I63" s="20" t="n"/>
+      <c r="J63" s="20" t="n"/>
+      <c r="K63" s="20" t="n"/>
+      <c r="L63" s="20" t="n"/>
+      <c r="M63" s="20" t="n"/>
     </row>
     <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="11" t="inlineStr">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>Gants   (1)</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="12" t="inlineStr">
+      <c r="A66" s="13" t="inlineStr">
         <is>
           <t>Miner's Gloves</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
+      <c r="B66" s="14" t="inlineStr">
         <is>
           <t>gants-de-mineur</t>
         </is>
       </c>
-      <c r="C66" s="14" t="inlineStr">
+      <c r="C66" s="15" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D66" s="15" t="n">
+      <c r="D66" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E66" s="16" t="n"/>
-      <c r="F66" s="16" t="n"/>
-      <c r="G66" s="16" t="n"/>
-      <c r="H66" s="16" t="n"/>
-      <c r="I66" s="16" t="n"/>
-      <c r="J66" s="16" t="n"/>
-      <c r="K66" s="16" t="n"/>
-      <c r="L66" s="16" t="n"/>
-      <c r="M66" s="16" t="n"/>
+      <c r="E66" s="17" t="n"/>
+      <c r="F66" s="17" t="n"/>
+      <c r="G66" s="17" t="n"/>
+      <c r="H66" s="17" t="n"/>
+      <c r="I66" s="17" t="n"/>
+      <c r="J66" s="17" t="n"/>
+      <c r="K66" s="17" t="n"/>
+      <c r="L66" s="17" t="n"/>
+      <c r="M66" s="17" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="19" t="n"/>
-      <c r="B67" s="19" t="n"/>
-      <c r="C67" s="19" t="n"/>
-      <c r="D67" s="19" t="n"/>
-      <c r="E67" s="19" t="n"/>
-      <c r="F67" s="19" t="n"/>
-      <c r="G67" s="19" t="n"/>
-      <c r="H67" s="19" t="n"/>
-      <c r="I67" s="19" t="n"/>
-      <c r="J67" s="19" t="n"/>
-      <c r="K67" s="19" t="n"/>
-      <c r="L67" s="19" t="n"/>
-      <c r="M67" s="19" t="n"/>
+      <c r="A67" s="20" t="n"/>
+      <c r="B67" s="20" t="n"/>
+      <c r="C67" s="20" t="n"/>
+      <c r="D67" s="20" t="n"/>
+      <c r="E67" s="20" t="n"/>
+      <c r="F67" s="20" t="n"/>
+      <c r="G67" s="20" t="n"/>
+      <c r="H67" s="20" t="n"/>
+      <c r="I67" s="20" t="n"/>
+      <c r="J67" s="20" t="n"/>
+      <c r="K67" s="20" t="n"/>
+      <c r="L67" s="20" t="n"/>
+      <c r="M67" s="20" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="19" t="n"/>
-      <c r="B68" s="19" t="n"/>
-      <c r="C68" s="19" t="n"/>
-      <c r="D68" s="19" t="n"/>
-      <c r="E68" s="19" t="n"/>
-      <c r="F68" s="19" t="n"/>
-      <c r="G68" s="19" t="n"/>
-      <c r="H68" s="19" t="n"/>
-      <c r="I68" s="19" t="n"/>
-      <c r="J68" s="19" t="n"/>
-      <c r="K68" s="19" t="n"/>
-      <c r="L68" s="19" t="n"/>
-      <c r="M68" s="19" t="n"/>
+      <c r="A68" s="20" t="n"/>
+      <c r="B68" s="20" t="n"/>
+      <c r="C68" s="20" t="n"/>
+      <c r="D68" s="20" t="n"/>
+      <c r="E68" s="20" t="n"/>
+      <c r="F68" s="20" t="n"/>
+      <c r="G68" s="20" t="n"/>
+      <c r="H68" s="20" t="n"/>
+      <c r="I68" s="20" t="n"/>
+      <c r="J68" s="20" t="n"/>
+      <c r="K68" s="20" t="n"/>
+      <c r="L68" s="20" t="n"/>
+      <c r="M68" s="20" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="19" t="n"/>
-      <c r="B69" s="19" t="n"/>
-      <c r="C69" s="19" t="n"/>
-      <c r="D69" s="19" t="n"/>
-      <c r="E69" s="19" t="n"/>
-      <c r="F69" s="19" t="n"/>
-      <c r="G69" s="19" t="n"/>
-      <c r="H69" s="19" t="n"/>
-      <c r="I69" s="19" t="n"/>
-      <c r="J69" s="19" t="n"/>
-      <c r="K69" s="19" t="n"/>
-      <c r="L69" s="19" t="n"/>
-      <c r="M69" s="19" t="n"/>
+      <c r="A69" s="20" t="n"/>
+      <c r="B69" s="20" t="n"/>
+      <c r="C69" s="20" t="n"/>
+      <c r="D69" s="20" t="n"/>
+      <c r="E69" s="20" t="n"/>
+      <c r="F69" s="20" t="n"/>
+      <c r="G69" s="20" t="n"/>
+      <c r="H69" s="20" t="n"/>
+      <c r="I69" s="20" t="n"/>
+      <c r="J69" s="20" t="n"/>
+      <c r="K69" s="20" t="n"/>
+      <c r="L69" s="20" t="n"/>
+      <c r="M69" s="20" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="19" t="n"/>
-      <c r="B70" s="19" t="n"/>
-      <c r="C70" s="19" t="n"/>
-      <c r="D70" s="19" t="n"/>
-      <c r="E70" s="19" t="n"/>
-      <c r="F70" s="19" t="n"/>
-      <c r="G70" s="19" t="n"/>
-      <c r="H70" s="19" t="n"/>
-      <c r="I70" s="19" t="n"/>
-      <c r="J70" s="19" t="n"/>
-      <c r="K70" s="19" t="n"/>
-      <c r="L70" s="19" t="n"/>
-      <c r="M70" s="19" t="n"/>
+      <c r="A70" s="20" t="n"/>
+      <c r="B70" s="20" t="n"/>
+      <c r="C70" s="20" t="n"/>
+      <c r="D70" s="20" t="n"/>
+      <c r="E70" s="20" t="n"/>
+      <c r="F70" s="20" t="n"/>
+      <c r="G70" s="20" t="n"/>
+      <c r="H70" s="20" t="n"/>
+      <c r="I70" s="20" t="n"/>
+      <c r="J70" s="20" t="n"/>
+      <c r="K70" s="20" t="n"/>
+      <c r="L70" s="20" t="n"/>
+      <c r="M70" s="20" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="19" t="n"/>
-      <c r="B71" s="19" t="n"/>
-      <c r="C71" s="19" t="n"/>
-      <c r="D71" s="19" t="n"/>
-      <c r="E71" s="19" t="n"/>
-      <c r="F71" s="19" t="n"/>
-      <c r="G71" s="19" t="n"/>
-      <c r="H71" s="19" t="n"/>
-      <c r="I71" s="19" t="n"/>
-      <c r="J71" s="19" t="n"/>
-      <c r="K71" s="19" t="n"/>
-      <c r="L71" s="19" t="n"/>
-      <c r="M71" s="19" t="n"/>
+      <c r="A71" s="20" t="n"/>
+      <c r="B71" s="20" t="n"/>
+      <c r="C71" s="20" t="n"/>
+      <c r="D71" s="20" t="n"/>
+      <c r="E71" s="20" t="n"/>
+      <c r="F71" s="20" t="n"/>
+      <c r="G71" s="20" t="n"/>
+      <c r="H71" s="20" t="n"/>
+      <c r="I71" s="20" t="n"/>
+      <c r="J71" s="20" t="n"/>
+      <c r="K71" s="20" t="n"/>
+      <c r="L71" s="20" t="n"/>
+      <c r="M71" s="20" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="19" t="n"/>
-      <c r="B72" s="19" t="n"/>
-      <c r="C72" s="19" t="n"/>
-      <c r="D72" s="19" t="n"/>
-      <c r="E72" s="19" t="n"/>
-      <c r="F72" s="19" t="n"/>
-      <c r="G72" s="19" t="n"/>
-      <c r="H72" s="19" t="n"/>
-      <c r="I72" s="19" t="n"/>
-      <c r="J72" s="19" t="n"/>
-      <c r="K72" s="19" t="n"/>
-      <c r="L72" s="19" t="n"/>
-      <c r="M72" s="19" t="n"/>
+      <c r="A72" s="20" t="n"/>
+      <c r="B72" s="20" t="n"/>
+      <c r="C72" s="20" t="n"/>
+      <c r="D72" s="20" t="n"/>
+      <c r="E72" s="20" t="n"/>
+      <c r="F72" s="20" t="n"/>
+      <c r="G72" s="20" t="n"/>
+      <c r="H72" s="20" t="n"/>
+      <c r="I72" s="20" t="n"/>
+      <c r="J72" s="20" t="n"/>
+      <c r="K72" s="20" t="n"/>
+      <c r="L72" s="20" t="n"/>
+      <c r="M72" s="20" t="n"/>
     </row>
     <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
+      <c r="A74" s="12" t="inlineStr">
         <is>
           <t>Bottes   (1)</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="12" t="inlineStr">
+      <c r="A75" s="13" t="inlineStr">
         <is>
           <t>Swift Boots</t>
         </is>
       </c>
-      <c r="B75" s="13" t="inlineStr">
+      <c r="B75" s="14" t="inlineStr">
         <is>
           <t>bottes-vives</t>
         </is>
       </c>
-      <c r="C75" s="17" t="inlineStr">
+      <c r="C75" s="18" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="D75" s="15" t="n">
+      <c r="D75" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E75" s="16" t="inlineStr">
+      <c r="E75" s="17" t="inlineStr">
         <is>
           <t>Quicken</t>
         </is>
       </c>
-      <c r="F75" s="15" t="n">
+      <c r="F75" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="G75" s="16" t="n"/>
-      <c r="H75" s="16" t="n"/>
-      <c r="I75" s="16" t="n"/>
-      <c r="J75" s="16" t="n"/>
-      <c r="K75" s="16" t="n"/>
-      <c r="L75" s="16" t="n"/>
-      <c r="M75" s="16" t="n"/>
+      <c r="G75" s="17" t="n"/>
+      <c r="H75" s="17" t="n"/>
+      <c r="I75" s="17" t="n"/>
+      <c r="J75" s="17" t="n"/>
+      <c r="K75" s="17" t="n"/>
+      <c r="L75" s="17" t="n"/>
+      <c r="M75" s="17" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="19" t="n"/>
-      <c r="B76" s="19" t="n"/>
-      <c r="C76" s="19" t="n"/>
-      <c r="D76" s="19" t="n"/>
-      <c r="E76" s="19" t="n"/>
-      <c r="F76" s="19" t="n"/>
-      <c r="G76" s="19" t="n"/>
-      <c r="H76" s="19" t="n"/>
-      <c r="I76" s="19" t="n"/>
-      <c r="J76" s="19" t="n"/>
-      <c r="K76" s="19" t="n"/>
-      <c r="L76" s="19" t="n"/>
-      <c r="M76" s="19" t="n"/>
+      <c r="A76" s="20" t="n"/>
+      <c r="B76" s="20" t="n"/>
+      <c r="C76" s="20" t="n"/>
+      <c r="D76" s="20" t="n"/>
+      <c r="E76" s="20" t="n"/>
+      <c r="F76" s="20" t="n"/>
+      <c r="G76" s="20" t="n"/>
+      <c r="H76" s="20" t="n"/>
+      <c r="I76" s="20" t="n"/>
+      <c r="J76" s="20" t="n"/>
+      <c r="K76" s="20" t="n"/>
+      <c r="L76" s="20" t="n"/>
+      <c r="M76" s="20" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="19" t="n"/>
-      <c r="B77" s="19" t="n"/>
-      <c r="C77" s="19" t="n"/>
-      <c r="D77" s="19" t="n"/>
-      <c r="E77" s="19" t="n"/>
-      <c r="F77" s="19" t="n"/>
-      <c r="G77" s="19" t="n"/>
-      <c r="H77" s="19" t="n"/>
-      <c r="I77" s="19" t="n"/>
-      <c r="J77" s="19" t="n"/>
-      <c r="K77" s="19" t="n"/>
-      <c r="L77" s="19" t="n"/>
-      <c r="M77" s="19" t="n"/>
+      <c r="A77" s="20" t="n"/>
+      <c r="B77" s="20" t="n"/>
+      <c r="C77" s="20" t="n"/>
+      <c r="D77" s="20" t="n"/>
+      <c r="E77" s="20" t="n"/>
+      <c r="F77" s="20" t="n"/>
+      <c r="G77" s="20" t="n"/>
+      <c r="H77" s="20" t="n"/>
+      <c r="I77" s="20" t="n"/>
+      <c r="J77" s="20" t="n"/>
+      <c r="K77" s="20" t="n"/>
+      <c r="L77" s="20" t="n"/>
+      <c r="M77" s="20" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="19" t="n"/>
-      <c r="B78" s="19" t="n"/>
-      <c r="C78" s="19" t="n"/>
-      <c r="D78" s="19" t="n"/>
-      <c r="E78" s="19" t="n"/>
-      <c r="F78" s="19" t="n"/>
-      <c r="G78" s="19" t="n"/>
-      <c r="H78" s="19" t="n"/>
-      <c r="I78" s="19" t="n"/>
-      <c r="J78" s="19" t="n"/>
-      <c r="K78" s="19" t="n"/>
-      <c r="L78" s="19" t="n"/>
-      <c r="M78" s="19" t="n"/>
+      <c r="A78" s="20" t="n"/>
+      <c r="B78" s="20" t="n"/>
+      <c r="C78" s="20" t="n"/>
+      <c r="D78" s="20" t="n"/>
+      <c r="E78" s="20" t="n"/>
+      <c r="F78" s="20" t="n"/>
+      <c r="G78" s="20" t="n"/>
+      <c r="H78" s="20" t="n"/>
+      <c r="I78" s="20" t="n"/>
+      <c r="J78" s="20" t="n"/>
+      <c r="K78" s="20" t="n"/>
+      <c r="L78" s="20" t="n"/>
+      <c r="M78" s="20" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="19" t="n"/>
-      <c r="B79" s="19" t="n"/>
-      <c r="C79" s="19" t="n"/>
-      <c r="D79" s="19" t="n"/>
-      <c r="E79" s="19" t="n"/>
-      <c r="F79" s="19" t="n"/>
-      <c r="G79" s="19" t="n"/>
-      <c r="H79" s="19" t="n"/>
-      <c r="I79" s="19" t="n"/>
-      <c r="J79" s="19" t="n"/>
-      <c r="K79" s="19" t="n"/>
-      <c r="L79" s="19" t="n"/>
-      <c r="M79" s="19" t="n"/>
+      <c r="A79" s="20" t="n"/>
+      <c r="B79" s="20" t="n"/>
+      <c r="C79" s="20" t="n"/>
+      <c r="D79" s="20" t="n"/>
+      <c r="E79" s="20" t="n"/>
+      <c r="F79" s="20" t="n"/>
+      <c r="G79" s="20" t="n"/>
+      <c r="H79" s="20" t="n"/>
+      <c r="I79" s="20" t="n"/>
+      <c r="J79" s="20" t="n"/>
+      <c r="K79" s="20" t="n"/>
+      <c r="L79" s="20" t="n"/>
+      <c r="M79" s="20" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="19" t="n"/>
-      <c r="B80" s="19" t="n"/>
-      <c r="C80" s="19" t="n"/>
-      <c r="D80" s="19" t="n"/>
-      <c r="E80" s="19" t="n"/>
-      <c r="F80" s="19" t="n"/>
-      <c r="G80" s="19" t="n"/>
-      <c r="H80" s="19" t="n"/>
-      <c r="I80" s="19" t="n"/>
-      <c r="J80" s="19" t="n"/>
-      <c r="K80" s="19" t="n"/>
-      <c r="L80" s="19" t="n"/>
-      <c r="M80" s="19" t="n"/>
+      <c r="A80" s="20" t="n"/>
+      <c r="B80" s="20" t="n"/>
+      <c r="C80" s="20" t="n"/>
+      <c r="D80" s="20" t="n"/>
+      <c r="E80" s="20" t="n"/>
+      <c r="F80" s="20" t="n"/>
+      <c r="G80" s="20" t="n"/>
+      <c r="H80" s="20" t="n"/>
+      <c r="I80" s="20" t="n"/>
+      <c r="J80" s="20" t="n"/>
+      <c r="K80" s="20" t="n"/>
+      <c r="L80" s="20" t="n"/>
+      <c r="M80" s="20" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="19" t="n"/>
-      <c r="B81" s="19" t="n"/>
-      <c r="C81" s="19" t="n"/>
-      <c r="D81" s="19" t="n"/>
-      <c r="E81" s="19" t="n"/>
-      <c r="F81" s="19" t="n"/>
-      <c r="G81" s="19" t="n"/>
-      <c r="H81" s="19" t="n"/>
-      <c r="I81" s="19" t="n"/>
-      <c r="J81" s="19" t="n"/>
-      <c r="K81" s="19" t="n"/>
-      <c r="L81" s="19" t="n"/>
-      <c r="M81" s="19" t="n"/>
+      <c r="A81" s="20" t="n"/>
+      <c r="B81" s="20" t="n"/>
+      <c r="C81" s="20" t="n"/>
+      <c r="D81" s="20" t="n"/>
+      <c r="E81" s="20" t="n"/>
+      <c r="F81" s="20" t="n"/>
+      <c r="G81" s="20" t="n"/>
+      <c r="H81" s="20" t="n"/>
+      <c r="I81" s="20" t="n"/>
+      <c r="J81" s="20" t="n"/>
+      <c r="K81" s="20" t="n"/>
+      <c r="L81" s="20" t="n"/>
+      <c r="M81" s="20" t="n"/>
     </row>
     <row r="83" ht="20" customHeight="1">
-      <c r="A83" s="11" t="inlineStr">
+      <c r="A83" s="12" t="inlineStr">
         <is>
           <t>Sacs   (1)</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="12" t="inlineStr">
+      <c r="A84" s="13" t="inlineStr">
         <is>
           <t>Leather Pouch</t>
         </is>
       </c>
-      <c r="B84" s="13" t="inlineStr">
+      <c r="B84" s="14" t="inlineStr">
         <is>
           <t>sac-en-cuir</t>
         </is>
       </c>
-      <c r="C84" s="14" t="inlineStr">
+      <c r="C84" s="15" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D84" s="15" t="n">
+      <c r="D84" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E84" s="16" t="n"/>
-      <c r="F84" s="16" t="n"/>
-      <c r="G84" s="16" t="n"/>
-      <c r="H84" s="16" t="n"/>
-      <c r="I84" s="16" t="n"/>
-      <c r="J84" s="16" t="n"/>
-      <c r="K84" s="16" t="n"/>
-      <c r="L84" s="16" t="n"/>
-      <c r="M84" s="16" t="n"/>
+      <c r="E84" s="17" t="n"/>
+      <c r="F84" s="17" t="n"/>
+      <c r="G84" s="17" t="n"/>
+      <c r="H84" s="17" t="n"/>
+      <c r="I84" s="17" t="n"/>
+      <c r="J84" s="17" t="n"/>
+      <c r="K84" s="17" t="n"/>
+      <c r="L84" s="17" t="n"/>
+      <c r="M84" s="17" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="19" t="n"/>
-      <c r="B85" s="19" t="n"/>
-      <c r="C85" s="19" t="n"/>
-      <c r="D85" s="19" t="n"/>
-      <c r="E85" s="19" t="n"/>
-      <c r="F85" s="19" t="n"/>
-      <c r="G85" s="19" t="n"/>
-      <c r="H85" s="19" t="n"/>
-      <c r="I85" s="19" t="n"/>
-      <c r="J85" s="19" t="n"/>
-      <c r="K85" s="19" t="n"/>
-      <c r="L85" s="19" t="n"/>
-      <c r="M85" s="19" t="n"/>
+      <c r="A85" s="20" t="n"/>
+      <c r="B85" s="20" t="n"/>
+      <c r="C85" s="20" t="n"/>
+      <c r="D85" s="20" t="n"/>
+      <c r="E85" s="20" t="n"/>
+      <c r="F85" s="20" t="n"/>
+      <c r="G85" s="20" t="n"/>
+      <c r="H85" s="20" t="n"/>
+      <c r="I85" s="20" t="n"/>
+      <c r="J85" s="20" t="n"/>
+      <c r="K85" s="20" t="n"/>
+      <c r="L85" s="20" t="n"/>
+      <c r="M85" s="20" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="19" t="n"/>
-      <c r="B86" s="19" t="n"/>
-      <c r="C86" s="19" t="n"/>
-      <c r="D86" s="19" t="n"/>
-      <c r="E86" s="19" t="n"/>
-      <c r="F86" s="19" t="n"/>
-      <c r="G86" s="19" t="n"/>
-      <c r="H86" s="19" t="n"/>
-      <c r="I86" s="19" t="n"/>
-      <c r="J86" s="19" t="n"/>
-      <c r="K86" s="19" t="n"/>
-      <c r="L86" s="19" t="n"/>
-      <c r="M86" s="19" t="n"/>
+      <c r="A86" s="20" t="n"/>
+      <c r="B86" s="20" t="n"/>
+      <c r="C86" s="20" t="n"/>
+      <c r="D86" s="20" t="n"/>
+      <c r="E86" s="20" t="n"/>
+      <c r="F86" s="20" t="n"/>
+      <c r="G86" s="20" t="n"/>
+      <c r="H86" s="20" t="n"/>
+      <c r="I86" s="20" t="n"/>
+      <c r="J86" s="20" t="n"/>
+      <c r="K86" s="20" t="n"/>
+      <c r="L86" s="20" t="n"/>
+      <c r="M86" s="20" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="19" t="n"/>
-      <c r="B87" s="19" t="n"/>
-      <c r="C87" s="19" t="n"/>
-      <c r="D87" s="19" t="n"/>
-      <c r="E87" s="19" t="n"/>
-      <c r="F87" s="19" t="n"/>
-      <c r="G87" s="19" t="n"/>
-      <c r="H87" s="19" t="n"/>
-      <c r="I87" s="19" t="n"/>
-      <c r="J87" s="19" t="n"/>
-      <c r="K87" s="19" t="n"/>
-      <c r="L87" s="19" t="n"/>
-      <c r="M87" s="19" t="n"/>
+      <c r="A87" s="20" t="n"/>
+      <c r="B87" s="20" t="n"/>
+      <c r="C87" s="20" t="n"/>
+      <c r="D87" s="20" t="n"/>
+      <c r="E87" s="20" t="n"/>
+      <c r="F87" s="20" t="n"/>
+      <c r="G87" s="20" t="n"/>
+      <c r="H87" s="20" t="n"/>
+      <c r="I87" s="20" t="n"/>
+      <c r="J87" s="20" t="n"/>
+      <c r="K87" s="20" t="n"/>
+      <c r="L87" s="20" t="n"/>
+      <c r="M87" s="20" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="19" t="n"/>
-      <c r="B88" s="19" t="n"/>
-      <c r="C88" s="19" t="n"/>
-      <c r="D88" s="19" t="n"/>
-      <c r="E88" s="19" t="n"/>
-      <c r="F88" s="19" t="n"/>
-      <c r="G88" s="19" t="n"/>
-      <c r="H88" s="19" t="n"/>
-      <c r="I88" s="19" t="n"/>
-      <c r="J88" s="19" t="n"/>
-      <c r="K88" s="19" t="n"/>
-      <c r="L88" s="19" t="n"/>
-      <c r="M88" s="19" t="n"/>
+      <c r="A88" s="20" t="n"/>
+      <c r="B88" s="20" t="n"/>
+      <c r="C88" s="20" t="n"/>
+      <c r="D88" s="20" t="n"/>
+      <c r="E88" s="20" t="n"/>
+      <c r="F88" s="20" t="n"/>
+      <c r="G88" s="20" t="n"/>
+      <c r="H88" s="20" t="n"/>
+      <c r="I88" s="20" t="n"/>
+      <c r="J88" s="20" t="n"/>
+      <c r="K88" s="20" t="n"/>
+      <c r="L88" s="20" t="n"/>
+      <c r="M88" s="20" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="19" t="n"/>
-      <c r="B89" s="19" t="n"/>
-      <c r="C89" s="19" t="n"/>
-      <c r="D89" s="19" t="n"/>
-      <c r="E89" s="19" t="n"/>
-      <c r="F89" s="19" t="n"/>
-      <c r="G89" s="19" t="n"/>
-      <c r="H89" s="19" t="n"/>
-      <c r="I89" s="19" t="n"/>
-      <c r="J89" s="19" t="n"/>
-      <c r="K89" s="19" t="n"/>
-      <c r="L89" s="19" t="n"/>
-      <c r="M89" s="19" t="n"/>
+      <c r="A89" s="20" t="n"/>
+      <c r="B89" s="20" t="n"/>
+      <c r="C89" s="20" t="n"/>
+      <c r="D89" s="20" t="n"/>
+      <c r="E89" s="20" t="n"/>
+      <c r="F89" s="20" t="n"/>
+      <c r="G89" s="20" t="n"/>
+      <c r="H89" s="20" t="n"/>
+      <c r="I89" s="20" t="n"/>
+      <c r="J89" s="20" t="n"/>
+      <c r="K89" s="20" t="n"/>
+      <c r="L89" s="20" t="n"/>
+      <c r="M89" s="20" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="19" t="n"/>
-      <c r="B90" s="19" t="n"/>
-      <c r="C90" s="19" t="n"/>
-      <c r="D90" s="19" t="n"/>
-      <c r="E90" s="19" t="n"/>
-      <c r="F90" s="19" t="n"/>
-      <c r="G90" s="19" t="n"/>
-      <c r="H90" s="19" t="n"/>
-      <c r="I90" s="19" t="n"/>
-      <c r="J90" s="19" t="n"/>
-      <c r="K90" s="19" t="n"/>
-      <c r="L90" s="19" t="n"/>
-      <c r="M90" s="19" t="n"/>
+      <c r="A90" s="20" t="n"/>
+      <c r="B90" s="20" t="n"/>
+      <c r="C90" s="20" t="n"/>
+      <c r="D90" s="20" t="n"/>
+      <c r="E90" s="20" t="n"/>
+      <c r="F90" s="20" t="n"/>
+      <c r="G90" s="20" t="n"/>
+      <c r="H90" s="20" t="n"/>
+      <c r="I90" s="20" t="n"/>
+      <c r="J90" s="20" t="n"/>
+      <c r="K90" s="20" t="n"/>
+      <c r="L90" s="20" t="n"/>
+      <c r="M90" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -2293,769 +2308,769 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>BRUTAL — Cartes existantes (référence pour composer des items)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Nom</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Coût (Chaleur)</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>AOE</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Donnée par</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>Effet</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Bloodletting</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>coup-de-sang</t>
         </is>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="D3" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E3" s="15" t="inlineStr"/>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr"/>
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>Blood Ring</t>
         </is>
       </c>
-      <c r="G3" s="16" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>Deal 2 damage. Apply 2 Bleed (heals you each tick).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Cleave</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>couper-en-deux</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr"/>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr"/>
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>War Axe</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>Deal 12 damage. If the target dies, deal 12 damage to the next enemy.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Dragon's Blaze</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>embrasement-dragon</t>
         </is>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="22" t="inlineStr">
+      <c r="D5" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>Onyx Guard Plate</t>
         </is>
       </c>
-      <c r="G5" s="16" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Forge Smash</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>ecrasement</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr"/>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr"/>
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>Forge Hammer</t>
         </is>
       </c>
-      <c r="G6" s="16" t="inlineStr">
+      <c r="G6" s="17" t="inlineStr">
         <is>
           <t>Deal 8 damage. Gain 3 Stone.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Frostbite</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>givre-lent</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="22" t="inlineStr">
+      <c r="D7" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr"/>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr"/>
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>Frost Ring</t>
         </is>
       </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>Deal 2 damage. Chill: -30% speed for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Giant Swing</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>giant-swing</t>
         </is>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="22" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>War Axe</t>
         </is>
       </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
         <is>
           <t>Deal 9 damage to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Lava Hammer</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>coup-de-lave</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="22" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr"/>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr"/>
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Magma Hammer</t>
         </is>
       </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>Deal 5 damage. Apply 4 Burning.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Onyx Breath</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>souffle-onyx</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="22" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>Onyx Guard Plate</t>
         </is>
       </c>
-      <c r="G10" s="16" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>Apply 8 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Pickaxe Jab</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>coup-de-pioche</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="22" t="inlineStr">
+      <c r="D11" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr"/>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr"/>
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Miner's Pick</t>
         </is>
       </c>
-      <c r="G11" s="16" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>Deal 3 damage twice.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Pommel Strike</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>coup-de-pommeau</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr"/>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr"/>
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>War Axe</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>Deal 4 damage. Stun the target for 1 turn.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Punch</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>coup-faible</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="22" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr"/>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr"/>
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>— (deck de base)</t>
         </is>
       </c>
-      <c r="G13" s="16" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>Deal 3 damage.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>Rusty Cleave</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>coup-de-hache</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="22" t="inlineStr">
+      <c r="D14" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr"/>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr"/>
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>Rusty Axe</t>
         </is>
       </c>
-      <c r="G14" s="16" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>Deal 12 damage.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Shield Bash</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>coup-de-bouclier</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="22" t="inlineStr">
+      <c r="D15" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr"/>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr"/>
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>Tower Shield</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>Deal 3 damage. Stun the enemy for 2 turns.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>frappe</t>
         </is>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="22" t="inlineStr">
+      <c r="D16" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr"/>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr"/>
+      <c r="F16" s="17" t="inlineStr">
         <is>
           <t>— (deck de base)</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
+      <c r="G16" s="17" t="inlineStr">
         <is>
           <t>Deal 6 damage.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Venom Stab</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>coup-venimeux</t>
         </is>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="C17" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="22" t="inlineStr">
+      <c r="D17" s="23" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr"/>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr"/>
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>Basilisk Fang</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>Deal 4 damage. Apply 4 Poison.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Guard</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>garde</t>
         </is>
       </c>
-      <c r="C18" s="15" t="n">
+      <c r="C18" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="23" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr"/>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="E18" s="16" t="inlineStr"/>
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>— (deck de base)</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Hand Guard</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>garde-faible</t>
         </is>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="C19" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="23" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr"/>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr"/>
+      <c r="F19" s="17" t="inlineStr">
         <is>
           <t>— (deck de base)</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>Gain 3 Stone.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Mail Armor</t>
         </is>
       </c>
-      <c r="B20" s="21" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>mail-armor</t>
         </is>
       </c>
-      <c r="C20" s="15" t="n">
+      <c r="C20" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D20" s="24" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr"/>
-      <c r="F20" s="16" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr"/>
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>Forgemaster's Mail</t>
         </is>
       </c>
-      <c r="G20" s="16" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Onyx Armor</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>onyx-armor</t>
         </is>
       </c>
-      <c r="C21" s="15" t="n">
+      <c r="C21" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr"/>
-      <c r="F21" s="16" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr"/>
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>Onyx Guard Plate</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>Gain 15 Stone.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>Quench</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>trempe</t>
         </is>
       </c>
-      <c r="C22" s="15" t="n">
+      <c r="C22" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="23" t="inlineStr">
+      <c r="D22" s="24" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr"/>
-      <c r="F22" s="16" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr"/>
+      <c r="F22" s="17" t="inlineStr">
         <is>
           <t>Forgemaster's Mail</t>
         </is>
       </c>
-      <c r="G22" s="16" t="inlineStr">
+      <c r="G22" s="17" t="inlineStr">
         <is>
           <t>Spend all Forge Heat. Gain 4 Stone per Heat spent.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>Shield Wall</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>mur-bouclier</t>
         </is>
       </c>
-      <c r="C23" s="15" t="n">
+      <c r="C23" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="23" t="inlineStr">
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr"/>
-      <c r="F23" s="16" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr"/>
+      <c r="F23" s="17" t="inlineStr">
         <is>
           <t>Tower Shield</t>
         </is>
       </c>
-      <c r="G23" s="16" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
         <is>
           <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>Quicken</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>celerite-vive</t>
         </is>
       </c>
-      <c r="C24" s="15" t="n">
+      <c r="C24" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="24" t="inlineStr">
+      <c r="D24" s="25" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr"/>
-      <c r="F24" s="16" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr"/>
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>Swift Boots</t>
         </is>
       </c>
-      <c r="G24" s="16" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
         <is>
           <t>Haste: +30% attack speed for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>Sapphire Surge</t>
         </is>
       </c>
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>surge-saphir</t>
         </is>
       </c>
-      <c r="C25" s="15" t="n">
+      <c r="C25" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="24" t="inlineStr">
+      <c r="D25" s="25" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr"/>
-      <c r="F25" s="16" t="inlineStr">
+      <c r="E25" s="16" t="inlineStr"/>
+      <c r="F25" s="17" t="inlineStr">
         <is>
           <t>Sapphire Amulet</t>
         </is>
       </c>
-      <c r="G25" s="16" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
         <is>
           <t>Gain 2 Forge Heat (energy).</t>
         </is>

</xml_diff>

<commit_message>
[technique] Catalogue : colonne Rareté des cartes (selon l'arme source)
Dans l'onglet « Cartes » du catalogue Excel, chaque carte affiche une
rareté colorée = celle de l'objet LE MOINS rare qui la débloque
(ex. Strike = Common, donnée par des armes communes). « — » pour les
cartes du deck de base. Calcul automatique, présent UNIQUEMENT dans le
catalogue (cette rareté n'existe pas dans le jeu). Lisez-moi mis à jour.
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +62,9 @@
     <font>
       <color rgb="00888888"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00888888"/>
     </font>
   </fonts>
   <fills count="14">
@@ -158,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -226,6 +229,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -600,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -704,156 +710,173 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Rareté des cartes (onglet « Cartes »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>La couleur de rareté d'une carte = celle de l'objet LE MOINS rare qui la débloque (ex. « Strike » est Common car des armes communes la donnent). Calculée automatiquement à la génération — c'est PUREMENT indicatif pour s'y retrouver, cette rareté n'existe pas dans le jeu. « — » = carte du deck de base (donnée par aucun objet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>Légende des raretés</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  Common  (commun)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Uncommon  (uncommon)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rare  (rare)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  Epic  (epique)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  Legendary  (legendaire)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Tableau de référence pour garder une certaine balance</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Rareté</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Nb de cartes</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Dégât / énergie</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Armure / énergie</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Legendary</t>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D30" s="2" t="n">
         <v>8</v>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Armes à deux mains : ×1,5 sur dégât et armure/énergie (moins de cartes), souvent via des sorts chers en énergie.</t>
         </is>
@@ -2854,16 +2877,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2896,15 +2920,20 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
+          <t>Rareté</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
           <t>AOE</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>Donnée par</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>Effet</t>
         </is>
@@ -2929,17 +2958,22 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>Magma Hammer</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>Apply 10 Burning to ALL enemies. Already-burning enemies take double, then their Burning is forged into Stone for you.</t>
         </is>
@@ -2964,13 +2998,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr"/>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr"/>
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Blood Ring</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
         </is>
@@ -2995,13 +3034,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr"/>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr"/>
+      <c r="G5" s="18" t="inlineStr">
         <is>
           <t>Onyx Glove</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>Discard your hand. For each card discarded, apply 3 Burning to a random enemy.</t>
         </is>
@@ -3026,13 +3070,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr"/>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr"/>
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>War Axe</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>Deal 20 damage. If the target dies, deal 15 damage to the next enemy.</t>
         </is>
@@ -3057,17 +3106,22 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
         <is>
           <t>Magma Hammer, Onyx Guard Plate</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="H7" s="18" t="inlineStr">
         <is>
           <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
         </is>
@@ -3092,13 +3146,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr"/>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr"/>
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>Magma Hammer</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>Deal 12 damage. Apply 3 Burning.</t>
         </is>
@@ -3123,13 +3182,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr"/>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr"/>
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>Onyx Boots</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>Move all Burning from the target to the enemy behind it.</t>
         </is>
@@ -3154,13 +3218,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr"/>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr"/>
+      <c r="G10" s="18" t="inlineStr">
         <is>
           <t>Forge Hammer</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="H10" s="18" t="inlineStr">
         <is>
           <t>Deal 10 damage. Gain 8 Stone.</t>
         </is>
@@ -3185,13 +3254,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr"/>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr"/>
+      <c r="G11" s="18" t="inlineStr">
         <is>
           <t>Frost Ring</t>
         </is>
       </c>
-      <c r="G11" s="18" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>Deal 2 damage. Chill: -30% speed for 3 turns.</t>
         </is>
@@ -3216,17 +3290,22 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="G12" s="18" t="inlineStr">
         <is>
           <t>War Axe</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
+      <c r="H12" s="18" t="inlineStr">
         <is>
           <t>Deal 16 damage to ALL enemies. Apply 2 Bleed to ALL enemies.</t>
         </is>
@@ -3251,17 +3330,22 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="G13" s="18" t="inlineStr">
         <is>
           <t>Big Onyx Sword</t>
         </is>
       </c>
-      <c r="G13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>Spend all Forge Heat. Apply 8 Burning per Heat spent to ALL enemies.</t>
         </is>
@@ -3286,13 +3370,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr"/>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr"/>
+      <c r="G14" s="18" t="inlineStr">
         <is>
           <t>Magma Hammer</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>Deal 28 damage. Apply 4 Burning.</t>
         </is>
@@ -3317,17 +3406,22 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E15" s="17" t="inlineStr">
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="G15" s="18" t="inlineStr">
         <is>
           <t>Onyx Guard Plate</t>
         </is>
       </c>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="H15" s="18" t="inlineStr">
         <is>
           <t>Apply 8 Burning to ALL enemies.</t>
         </is>
@@ -3352,13 +3446,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr"/>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr"/>
+      <c r="G16" s="18" t="inlineStr">
         <is>
           <t>Onyx Glove</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>Gain 5 Stone. Deal 2 damage and apply 1 Burning.</t>
         </is>
@@ -3383,17 +3482,22 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="G17" s="18" t="inlineStr">
         <is>
           <t>Big Onyx Sword</t>
         </is>
       </c>
-      <c r="G17" s="18" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>Apply 8 Burning to ALL enemies.</t>
         </is>
@@ -3418,13 +3522,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr"/>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr"/>
+      <c r="G18" s="18" t="inlineStr">
         <is>
           <t>Big Onyx Sword</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr">
+      <c r="H18" s="18" t="inlineStr">
         <is>
           <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
         </is>
@@ -3449,13 +3558,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E19" s="17" t="inlineStr"/>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr"/>
+      <c r="G19" s="18" t="inlineStr">
         <is>
           <t>Miner's Pick</t>
         </is>
       </c>
-      <c r="G19" s="18" t="inlineStr">
+      <c r="H19" s="18" t="inlineStr">
         <is>
           <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
         </is>
@@ -3480,17 +3594,22 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="G20" s="18" t="inlineStr">
         <is>
           <t>Basilisk Fang</t>
         </is>
       </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="H20" s="18" t="inlineStr">
         <is>
           <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
         </is>
@@ -3515,13 +3634,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E21" s="17" t="inlineStr"/>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr"/>
+      <c r="G21" s="18" t="inlineStr">
         <is>
           <t>War Axe</t>
         </is>
       </c>
-      <c r="G21" s="18" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr">
         <is>
           <t>Deal 16 damage. Stun the target for 2 turns.</t>
         </is>
@@ -3546,13 +3670,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr"/>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr"/>
+      <c r="G22" s="18" t="inlineStr">
         <is>
           <t>— (deck de base)</t>
         </is>
       </c>
-      <c r="G22" s="18" t="inlineStr">
+      <c r="H22" s="18" t="inlineStr">
         <is>
           <t>Deal 3 damage.</t>
         </is>
@@ -3577,13 +3706,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr"/>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr"/>
+      <c r="G23" s="18" t="inlineStr">
         <is>
           <t>Rusty Axe</t>
         </is>
       </c>
-      <c r="G23" s="18" t="inlineStr">
+      <c r="H23" s="18" t="inlineStr">
         <is>
           <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
         </is>
@@ -3608,13 +3742,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr"/>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr"/>
+      <c r="G24" s="18" t="inlineStr">
         <is>
           <t>Tower Shield</t>
         </is>
       </c>
-      <c r="G24" s="18" t="inlineStr">
+      <c r="H24" s="18" t="inlineStr">
         <is>
           <t>Deal 3 damage. Stun the enemy for 2 turns.</t>
         </is>
@@ -3639,13 +3778,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E25" s="17" t="inlineStr"/>
-      <c r="F25" s="18" t="inlineStr">
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr"/>
+      <c r="G25" s="18" t="inlineStr">
         <is>
           <t>Forge Hammer</t>
         </is>
       </c>
-      <c r="G25" s="18" t="inlineStr">
+      <c r="H25" s="18" t="inlineStr">
         <is>
           <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
         </is>
@@ -3670,13 +3814,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E26" s="17" t="inlineStr"/>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr"/>
+      <c r="G26" s="18" t="inlineStr">
         <is>
           <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
         </is>
       </c>
-      <c r="G26" s="18" t="inlineStr">
+      <c r="H26" s="18" t="inlineStr">
         <is>
           <t>Deal 6 damage.</t>
         </is>
@@ -3701,13 +3850,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E27" s="17" t="inlineStr"/>
-      <c r="F27" s="18" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr"/>
+      <c r="G27" s="18" t="inlineStr">
         <is>
           <t>Basilisk Fang</t>
         </is>
       </c>
-      <c r="G27" s="18" t="inlineStr">
+      <c r="H27" s="18" t="inlineStr">
         <is>
           <t>Deal 4 damage. Apply 4 Poison.</t>
         </is>
@@ -3732,13 +3886,18 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E28" s="17" t="inlineStr"/>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="inlineStr"/>
+      <c r="G28" s="18" t="inlineStr">
         <is>
           <t>Basilisk Fang</t>
         </is>
       </c>
-      <c r="G28" s="18" t="inlineStr">
+      <c r="H28" s="18" t="inlineStr">
         <is>
           <t>Deal 18 damage. Doubled if the target has a negative status.</t>
         </is>
@@ -3758,18 +3917,23 @@
       <c r="C29" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="27" t="inlineStr">
+      <c r="D29" s="28" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E29" s="17" t="inlineStr"/>
-      <c r="F29" s="18" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr"/>
+      <c r="G29" s="18" t="inlineStr">
         <is>
           <t>— (deck de base)</t>
         </is>
       </c>
-      <c r="G29" s="18" t="inlineStr">
+      <c r="H29" s="18" t="inlineStr">
         <is>
           <t>Gain 5 Stone.</t>
         </is>
@@ -3789,18 +3953,23 @@
       <c r="C30" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="27" t="inlineStr">
+      <c r="D30" s="28" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E30" s="17" t="inlineStr"/>
-      <c r="F30" s="18" t="inlineStr">
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr"/>
+      <c r="G30" s="18" t="inlineStr">
         <is>
           <t>— (deck de base)</t>
         </is>
       </c>
-      <c r="G30" s="18" t="inlineStr">
+      <c r="H30" s="18" t="inlineStr">
         <is>
           <t>Gain 3 Stone.</t>
         </is>
@@ -3820,18 +3989,23 @@
       <c r="C31" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="27" t="inlineStr">
+      <c r="D31" s="28" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E31" s="17" t="inlineStr"/>
-      <c r="F31" s="18" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="inlineStr"/>
+      <c r="G31" s="18" t="inlineStr">
         <is>
           <t>Forgemaster's Mail</t>
         </is>
       </c>
-      <c r="G31" s="18" t="inlineStr">
+      <c r="H31" s="18" t="inlineStr">
         <is>
           <t>Gain 5 Stone.</t>
         </is>
@@ -3851,18 +4025,23 @@
       <c r="C32" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D32" s="27" t="inlineStr">
+      <c r="D32" s="28" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E32" s="17" t="inlineStr"/>
-      <c r="F32" s="18" t="inlineStr">
+      <c r="E32" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr"/>
+      <c r="G32" s="18" t="inlineStr">
         <is>
           <t>Onyx Guard Plate</t>
         </is>
       </c>
-      <c r="G32" s="18" t="inlineStr">
+      <c r="H32" s="18" t="inlineStr">
         <is>
           <t>Gain 15 Stone.</t>
         </is>
@@ -3882,18 +4061,23 @@
       <c r="C33" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D33" s="27" t="inlineStr">
+      <c r="D33" s="28" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E33" s="17" t="inlineStr"/>
-      <c r="F33" s="18" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr"/>
+      <c r="G33" s="18" t="inlineStr">
         <is>
           <t>Forgemaster's Mail</t>
         </is>
       </c>
-      <c r="G33" s="18" t="inlineStr">
+      <c r="H33" s="18" t="inlineStr">
         <is>
           <t>Spend all Forge Heat. Gain 4 Stone per Heat spent.</t>
         </is>
@@ -3913,18 +4097,23 @@
       <c r="C34" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D34" s="27" t="inlineStr">
+      <c r="D34" s="28" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E34" s="17" t="inlineStr"/>
-      <c r="F34" s="18" t="inlineStr">
+      <c r="E34" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr"/>
+      <c r="G34" s="18" t="inlineStr">
         <is>
           <t>Tower Shield</t>
         </is>
       </c>
-      <c r="G34" s="18" t="inlineStr">
+      <c r="H34" s="18" t="inlineStr">
         <is>
           <t>Gain 5 Stone.</t>
         </is>
@@ -3944,18 +4133,23 @@
       <c r="C35" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="28" t="inlineStr">
+      <c r="D35" s="29" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E35" s="17" t="inlineStr"/>
-      <c r="F35" s="18" t="inlineStr">
+      <c r="E35" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr"/>
+      <c r="G35" s="18" t="inlineStr">
         <is>
           <t>Onyx Boots</t>
         </is>
       </c>
-      <c r="G35" s="18" t="inlineStr">
+      <c r="H35" s="18" t="inlineStr">
         <is>
           <t>Haste for as many turns as your current Forge Heat.</t>
         </is>
@@ -3975,18 +4169,23 @@
       <c r="C36" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D36" s="28" t="inlineStr">
+      <c r="D36" s="29" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E36" s="17" t="inlineStr"/>
-      <c r="F36" s="18" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr"/>
+      <c r="G36" s="18" t="inlineStr">
         <is>
           <t>Miner's Gloves</t>
         </is>
       </c>
-      <c r="G36" s="18" t="inlineStr">
+      <c r="H36" s="18" t="inlineStr">
         <is>
           <t>Draw 2 cards.</t>
         </is>
@@ -4006,18 +4205,23 @@
       <c r="C37" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D37" s="28" t="inlineStr">
+      <c r="D37" s="29" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E37" s="17" t="inlineStr"/>
-      <c r="F37" s="18" t="inlineStr">
+      <c r="E37" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr"/>
+      <c r="G37" s="18" t="inlineStr">
         <is>
           <t>Big Onyx Sword</t>
         </is>
       </c>
-      <c r="G37" s="18" t="inlineStr">
+      <c r="H37" s="18" t="inlineStr">
         <is>
           <t>Gain 5 Forge Heat (energy).</t>
         </is>
@@ -4037,18 +4241,23 @@
       <c r="C38" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="28" t="inlineStr">
+      <c r="D38" s="29" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E38" s="17" t="inlineStr"/>
-      <c r="F38" s="18" t="inlineStr">
+      <c r="E38" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr"/>
+      <c r="G38" s="18" t="inlineStr">
         <is>
           <t>Perfect Sapphire Amulet</t>
         </is>
       </c>
-      <c r="G38" s="18" t="inlineStr">
+      <c r="H38" s="18" t="inlineStr">
         <is>
           <t>Gain 3 Forge Heat (energy).</t>
         </is>
@@ -4068,18 +4277,23 @@
       <c r="C39" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="28" t="inlineStr">
+      <c r="D39" s="29" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E39" s="17" t="inlineStr"/>
-      <c r="F39" s="18" t="inlineStr">
+      <c r="E39" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr"/>
+      <c r="G39" s="18" t="inlineStr">
         <is>
           <t>Swift Boots</t>
         </is>
       </c>
-      <c r="G39" s="18" t="inlineStr">
+      <c r="H39" s="18" t="inlineStr">
         <is>
           <t>Haste: +30% attack speed for 3 turns.</t>
         </is>
@@ -4099,18 +4313,23 @@
       <c r="C40" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D40" s="28" t="inlineStr">
+      <c r="D40" s="29" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E40" s="17" t="inlineStr"/>
-      <c r="F40" s="18" t="inlineStr">
+      <c r="E40" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F40" s="17" t="inlineStr"/>
+      <c r="G40" s="18" t="inlineStr">
         <is>
           <t>Sapphire Amulet, Nice Sapphire Amulet</t>
         </is>
       </c>
-      <c r="G40" s="18" t="inlineStr">
+      <c r="H40" s="18" t="inlineStr">
         <is>
           <t>Gain 2 Forge Heat (energy).</t>
         </is>
@@ -4118,7 +4337,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[technique] Catalogue régénéré : 22 items, 43 cartes
Reflète toutes les modifications de l'Excel de Brioche :
- 5 nouvelles cartes (Light Armor, Free Movement, Stacking Shield,
  All Should Be Fire, Heavy Armor)
- Valeurs des cartes existantes mises à jour
- Listes de cartes des armures et du Tower Shield actualisées

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJcbumK5KWRfGozDrLY2Kn
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -1567,21 +1567,21 @@
           <t>bouclier-tour</t>
         </is>
       </c>
-      <c r="C28" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D28" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Shield Wall</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="n">
         <v>3</v>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Shield Wall</t>
-        </is>
-      </c>
-      <c r="F28" s="17" t="n">
-        <v>1</v>
       </c>
       <c r="G28" s="18" t="inlineStr">
         <is>
@@ -1591,8 +1591,14 @@
       <c r="H28" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I28" s="18" t="n"/>
-      <c r="J28" s="18" t="n"/>
+      <c r="I28" s="18" t="inlineStr">
+        <is>
+          <t>Stacking Shield</t>
+        </is>
+      </c>
+      <c r="J28" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="K28" s="18" t="n"/>
       <c r="L28" s="18" t="n"/>
       <c r="M28" s="19" t="inlineStr"/>
@@ -1718,12 +1724,24 @@
         </is>
       </c>
       <c r="D37" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="18" t="n"/>
-      <c r="H37" s="18" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="E37" s="18" t="inlineStr">
+        <is>
+          <t>Light Armor</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="18" t="inlineStr">
+        <is>
+          <t>Free Movement</t>
+        </is>
+      </c>
+      <c r="H37" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="I37" s="18" t="n"/>
       <c r="J37" s="18" t="n"/>
       <c r="K37" s="18" t="n"/>
@@ -1748,7 +1766,7 @@
         </is>
       </c>
       <c r="D38" s="17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E38" s="18" t="inlineStr">
         <is>
@@ -1756,7 +1774,7 @@
         </is>
       </c>
       <c r="F38" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G38" s="18" t="inlineStr">
         <is>
@@ -1764,7 +1782,7 @@
         </is>
       </c>
       <c r="H38" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I38" s="18" t="inlineStr">
         <is>
@@ -1774,11 +1792,17 @@
       <c r="J38" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="K38" s="18" t="n"/>
-      <c r="L38" s="18" t="n"/>
+      <c r="K38" s="18" t="inlineStr">
+        <is>
+          <t>All Should Be Fire</t>
+        </is>
+      </c>
+      <c r="L38" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="M38" s="19" t="inlineStr">
         <is>
-          <t>Défense 5  ·  Set : Onyx Set</t>
+          <t>Set : Onyx Set</t>
         </is>
       </c>
       <c r="N38" s="18" t="n"/>
@@ -1800,7 +1824,7 @@
         </is>
       </c>
       <c r="D39" s="17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E39" s="18" t="inlineStr">
         <is>
@@ -1818,15 +1842,17 @@
       <c r="H39" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I39" s="18" t="n"/>
-      <c r="J39" s="18" t="n"/>
+      <c r="I39" s="18" t="inlineStr">
+        <is>
+          <t>Heavy Armor</t>
+        </is>
+      </c>
+      <c r="J39" s="17" t="n">
+        <v>2</v>
+      </c>
       <c r="K39" s="18" t="n"/>
       <c r="L39" s="18" t="n"/>
-      <c r="M39" s="19" t="inlineStr">
-        <is>
-          <t>Défense 3</t>
-        </is>
-      </c>
+      <c r="M39" s="19" t="inlineStr"/>
       <c r="N39" s="18" t="n"/>
     </row>
     <row r="40">
@@ -2877,7 +2903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2942,16 +2968,16 @@
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>Armor Forging</t>
+          <t>All Should Be Fire</t>
         </is>
       </c>
       <c r="B3" s="25" t="inlineStr">
         <is>
-          <t>forgeage-d-armure</t>
+          <t>tout-en-feu</t>
         </is>
       </c>
       <c r="C3" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
@@ -2970,176 +2996,176 @@
       </c>
       <c r="G3" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H3" s="18" t="inlineStr">
         <is>
-          <t>Apply 10 Burning to ALL enemies. Already-burning enemies take double, then their Burning is forged into Stone for you.</t>
+          <t>Convert ALL enemy statuses (positive and negative) to Burning, then double the Burning.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="24" t="inlineStr">
         <is>
-          <t>Bloodletting</t>
+          <t>Armor Forging</t>
         </is>
       </c>
       <c r="B4" s="25" t="inlineStr">
         <is>
-          <t>coup-de-sang</t>
+          <t>forgeage-d-armure</t>
         </is>
       </c>
       <c r="C4" s="17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="F4" s="17" t="inlineStr"/>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G4" s="18" t="inlineStr">
         <is>
-          <t>Blood Ring</t>
+          <t>Magma Hammer</t>
         </is>
       </c>
       <c r="H4" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
+          <t>Apply 10 Burning to ALL enemies. Already-burning enemies take double, then their Burning is forged into Stone for you.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>Burning Hand</t>
+          <t>Bloodletting</t>
         </is>
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>main-brulante</t>
+          <t>coup-de-sang</t>
         </is>
       </c>
       <c r="C5" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E5" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Blood Ring</t>
         </is>
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
-          <t>Discard your hand. For each card discarded, apply 3 Burning to a random enemy.</t>
+          <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>Cleave</t>
+          <t>Burning Hand</t>
         </is>
       </c>
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>couper-en-deux</t>
+          <t>main-brulante</t>
         </is>
       </c>
       <c r="C6" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr"/>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Deal 20 damage. If the target dies, deal 15 damage to the next enemy.</t>
+          <t>Discard your hand. For each card discarded, apply 8 Burning to a random enemy.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>Dragon's Blaze</t>
+          <t>Cleave</t>
         </is>
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>embrasement-dragon</t>
+          <t>couper-en-deux</t>
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E7" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="F7" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr"/>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer, Onyx Guard Plate</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
+          <t>Deal 20 damage. If the target dies, deal 15 damage to the next enemy.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>Fire Strike</t>
+          <t>Dragon's Blaze</t>
         </is>
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>feu-frappe</t>
+          <t>embrasement-dragon</t>
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
@@ -3151,27 +3177,31 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr"/>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer</t>
+          <t>Magma Hammer, Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>Deal 12 damage. Apply 3 Burning.</t>
+          <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>Flaming Kick</t>
+          <t>Fire Strike</t>
         </is>
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>coup-de-pied-ardent</t>
+          <t>feu-frappe</t>
         </is>
       </c>
       <c r="C9" s="17" t="n">
@@ -3190,64 +3220,64 @@
       <c r="F9" s="17" t="inlineStr"/>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots</t>
+          <t>Magma Hammer</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>Move all Burning from the target to the enemy behind it.</t>
+          <t>Deal 12 damage. Apply 3 Burning.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>Forge Smash</t>
+          <t>Flaming Kick</t>
         </is>
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>ecrasement</t>
+          <t>coup-de-pied-ardent</t>
         </is>
       </c>
       <c r="C10" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F10" s="17" t="inlineStr"/>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>Forge Hammer</t>
+          <t>Onyx Boots</t>
         </is>
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>Deal 10 damage. Gain 8 Stone.</t>
+          <t>Move all Burning from the target to the enemy behind it.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>Frostbite</t>
+          <t>Forge Smash</t>
         </is>
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>givre-lent</t>
+          <t>ecrasement</t>
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
@@ -3262,77 +3292,73 @@
       <c r="F11" s="17" t="inlineStr"/>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>Frost Ring</t>
+          <t>Forge Hammer</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>Deal 2 damage. Chill: -30% speed for 3 turns.</t>
+          <t>Deal 10 damage. Gain 8 Stone.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>Giant Swing</t>
+          <t>Frostbite</t>
         </is>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>giant-swing</t>
+          <t>givre-lent</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="F12" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr"/>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>Frost Ring</t>
         </is>
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>Deal 16 damage to ALL enemies. Apply 2 Bleed to ALL enemies.</t>
+          <t>Deal 5 damage. Chill: -30% speed for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>Heat Rejection</t>
+          <t>Giant Swing</t>
         </is>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>rejet-chaleur</t>
+          <t>giant-swing</t>
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E13" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
@@ -3342,28 +3368,28 @@
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>Spend all Forge Heat. Apply 8 Burning per Heat spent to ALL enemies.</t>
+          <t>Deal 16 damage to ALL enemies. Apply 2 Bleed to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>Lava Hammer</t>
+          <t>Heat Rejection</t>
         </is>
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>coup-de-lave</t>
+          <t>rejet-chaleur</t>
         </is>
       </c>
       <c r="C14" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
@@ -3375,31 +3401,35 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F14" s="17" t="inlineStr"/>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H14" s="18" t="inlineStr">
         <is>
-          <t>Deal 28 damage. Apply 4 Burning.</t>
+          <t>Spend all Forge Heat. Apply 8 Burning per Heat spent to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>Onyx Breath</t>
+          <t>Lava Hammer</t>
         </is>
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>souffle-onyx</t>
+          <t>coup-de-lave</t>
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
@@ -3411,35 +3441,31 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F15" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="F15" s="17" t="inlineStr"/>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>Onyx Guard Plate</t>
+          <t>Magma Hammer</t>
         </is>
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>Apply 8 Burning to ALL enemies.</t>
+          <t>Deal 28 damage. Apply 4 Burning.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>Onyx Fist</t>
+          <t>Onyx Breath</t>
         </is>
       </c>
       <c r="B16" s="25" t="inlineStr">
         <is>
-          <t>poing-onyx</t>
+          <t>souffle-onyx</t>
         </is>
       </c>
       <c r="C16" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
@@ -3451,27 +3477,31 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F16" s="17" t="inlineStr"/>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H16" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone. Deal 2 damage and apply 1 Burning.</t>
+          <t>Apply 20 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>Onyx Radiance</t>
+          <t>Onyx Fist</t>
         </is>
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>onyx-radiance</t>
+          <t>poing-onyx</t>
         </is>
       </c>
       <c r="C17" s="17" t="n">
@@ -3487,35 +3517,31 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F17" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="F17" s="17" t="inlineStr"/>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>Apply 8 Burning to ALL enemies.</t>
+          <t>Gain 10 Stone. Deal 10 damage and apply 3 Burning.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>Onyx Slash</t>
+          <t>Onyx Radiance</t>
         </is>
       </c>
       <c r="B18" s="25" t="inlineStr">
         <is>
-          <t>onyx-slash</t>
+          <t>onyx-radiance</t>
         </is>
       </c>
       <c r="C18" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
@@ -3527,7 +3553,11 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F18" s="17" t="inlineStr"/>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
           <t>Big Onyx Sword</t>
@@ -3535,99 +3565,95 @@
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
+          <t>Apply 8 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>Pickaxe Jab</t>
+          <t>Onyx Slash</t>
         </is>
       </c>
       <c r="B19" s="25" t="inlineStr">
         <is>
-          <t>coup-de-pioche</t>
+          <t>onyx-slash</t>
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E19" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr"/>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Miner's Pick</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
+          <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>Poison Dance</t>
+          <t>Pickaxe Jab</t>
         </is>
       </c>
       <c r="B20" s="25" t="inlineStr">
         <is>
-          <t>danse-empoisonnee</t>
+          <t>coup-de-pioche</t>
         </is>
       </c>
       <c r="C20" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E20" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="F20" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr"/>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>Miner's Pick</t>
         </is>
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
+          <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>Pommel Strike</t>
+          <t>Poison Dance</t>
         </is>
       </c>
       <c r="B21" s="25" t="inlineStr">
         <is>
-          <t>coup-de-pommeau</t>
+          <t>danse-empoisonnee</t>
         </is>
       </c>
       <c r="C21" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
@@ -3639,99 +3665,103 @@
           <t>Rare</t>
         </is>
       </c>
-      <c r="F21" s="17" t="inlineStr"/>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
-          <t>Deal 16 damage. Stun the target for 2 turns.</t>
+          <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>Punch</t>
+          <t>Pommel Strike</t>
         </is>
       </c>
       <c r="B22" s="25" t="inlineStr">
         <is>
-          <t>coup-faible</t>
+          <t>coup-de-pommeau</t>
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E22" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr"/>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage.</t>
+          <t>Deal 16 damage. Stun the target for 2 turns.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>Rusty Cleave</t>
+          <t>Punch</t>
         </is>
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>coup-de-hache</t>
+          <t>coup-faible</t>
         </is>
       </c>
       <c r="C23" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr"/>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>Rusty Axe</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
+          <t>Deal 3 damage.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>Shield Bash</t>
+          <t>Rusty Cleave</t>
         </is>
       </c>
       <c r="B24" s="25" t="inlineStr">
         <is>
-          <t>coup-de-bouclier</t>
+          <t>coup-de-hache</t>
         </is>
       </c>
       <c r="C24" s="17" t="n">
@@ -3742,104 +3772,104 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr"/>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>Rusty Axe</t>
         </is>
       </c>
       <c r="H24" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage. Stun the enemy for 2 turns.</t>
+          <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>Splash Strike</t>
+          <t>Shield Bash</t>
         </is>
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>eclaboussure-de-frappe</t>
+          <t>coup-de-bouclier</t>
         </is>
       </c>
       <c r="C25" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E25" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E25" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr"/>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>Forge Hammer</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
+          <t>Deal 10 damage. Stun the enemy for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>Strike</t>
+          <t>Splash Strike</t>
         </is>
       </c>
       <c r="B26" s="25" t="inlineStr">
         <is>
-          <t>frappe</t>
+          <t>eclaboussure-de-frappe</t>
         </is>
       </c>
       <c r="C26" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D26" s="26" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F26" s="17" t="inlineStr"/>
       <c r="G26" s="18" t="inlineStr">
         <is>
-          <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
+          <t>Forge Hammer</t>
         </is>
       </c>
       <c r="H26" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage.</t>
+          <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>Venom Stab</t>
+          <t>Strike</t>
         </is>
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>coup-venimeux</t>
+          <t>frappe</t>
         </is>
       </c>
       <c r="C27" s="17" t="n">
@@ -3850,36 +3880,36 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr"/>
       <c r="G27" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
         </is>
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
-          <t>Deal 4 damage. Apply 4 Poison.</t>
+          <t>Deal 6 damage.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>Wound Opening</t>
+          <t>Venom Stab</t>
         </is>
       </c>
       <c r="B28" s="25" t="inlineStr">
         <is>
-          <t>ouverture-des-plaies</t>
+          <t>coup-venimeux</t>
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D28" s="26" t="inlineStr">
         <is>
@@ -3899,55 +3929,55 @@
       </c>
       <c r="H28" s="18" t="inlineStr">
         <is>
-          <t>Deal 18 damage. Doubled if the target has a negative status.</t>
+          <t>Deal 4 damage. Apply 4 Poison.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>Guard</t>
+          <t>Wound Opening</t>
         </is>
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>garde</t>
+          <t>ouverture-des-plaies</t>
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="28" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E29" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>2</v>
+      </c>
+      <c r="D29" s="26" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E29" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr"/>
       <c r="G29" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H29" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone.</t>
+          <t>Deal 18 damage. Doubled if the target has a negative status.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>Hand Guard</t>
+          <t>Guard</t>
         </is>
       </c>
       <c r="B30" s="25" t="inlineStr">
         <is>
-          <t>garde-faible</t>
+          <t>garde</t>
         </is>
       </c>
       <c r="C30" s="17" t="n">
@@ -3971,19 +4001,19 @@
       </c>
       <c r="H30" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Stone.</t>
+          <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>Mail Armor</t>
+          <t>Hand Guard</t>
         </is>
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>mail-armor</t>
+          <t>garde-faible</t>
         </is>
       </c>
       <c r="C31" s="17" t="n">
@@ -3994,32 +4024,32 @@
           <t>Défense</t>
         </is>
       </c>
-      <c r="E31" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E31" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="17" t="inlineStr"/>
       <c r="G31" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H31" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone.</t>
+          <t>Gain 3 Stone.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>Onyx Armor</t>
+          <t>Heavy Armor</t>
         </is>
       </c>
       <c r="B32" s="25" t="inlineStr">
         <is>
-          <t>onyx-armor</t>
+          <t>armure-lourde</t>
         </is>
       </c>
       <c r="C32" s="17" t="n">
@@ -4030,68 +4060,68 @@
           <t>Défense</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E32" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr"/>
       <c r="G32" s="18" t="inlineStr">
         <is>
-          <t>Onyx Guard Plate</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H32" s="18" t="inlineStr">
         <is>
-          <t>Gain 15 Stone.</t>
+          <t>Gain 20 Stone.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>Quench</t>
+          <t>Light Armor</t>
         </is>
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>trempe</t>
+          <t>armure-legere</t>
         </is>
       </c>
       <c r="C33" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" s="28" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F33" s="17" t="inlineStr"/>
       <c r="G33" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>Traveler's Garb</t>
         </is>
       </c>
       <c r="H33" s="18" t="inlineStr">
         <is>
-          <t>Spend all Forge Heat. Gain 4 Stone per Heat spent.</t>
+          <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>Shield Wall</t>
+          <t>Mail Armor</t>
         </is>
       </c>
       <c r="B34" s="25" t="inlineStr">
         <is>
-          <t>mur-bouclier</t>
+          <t>mail-armor</t>
         </is>
       </c>
       <c r="C34" s="17" t="n">
@@ -4102,40 +4132,40 @@
           <t>Défense</t>
         </is>
       </c>
-      <c r="E34" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E34" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F34" s="17" t="inlineStr"/>
       <c r="G34" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H34" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone.</t>
+          <t>Gain 7 Stone for every enemy still alive.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>Burning Run</t>
+          <t>Onyx Armor</t>
         </is>
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>course-ardente</t>
+          <t>onyx-armor</t>
         </is>
       </c>
       <c r="C35" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="29" t="inlineStr">
-        <is>
-          <t>Buff</t>
+      <c r="D35" s="28" t="inlineStr">
+        <is>
+          <t>Défense</t>
         </is>
       </c>
       <c r="E35" s="22" t="inlineStr">
@@ -4146,190 +4176,370 @@
       <c r="F35" s="17" t="inlineStr"/>
       <c r="G35" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H35" s="18" t="inlineStr">
         <is>
-          <t>Haste for as many turns as your current Forge Heat.</t>
+          <t>Gain 30 Stone.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>Master's Hand</t>
+          <t>Quench</t>
         </is>
       </c>
       <c r="B36" s="25" t="inlineStr">
         <is>
-          <t>main-de-maitre</t>
+          <t>trempe</t>
         </is>
       </c>
       <c r="C36" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="29" t="inlineStr">
-        <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E36" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+        <v>0</v>
+      </c>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E36" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr"/>
       <c r="G36" s="18" t="inlineStr">
         <is>
-          <t>Miner's Gloves</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H36" s="18" t="inlineStr">
         <is>
-          <t>Draw 2 cards.</t>
+          <t>Spend all Forge Heat. Gain 10 Stone per Heat spent.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>Onyx Overheat</t>
+          <t>Shield Wall</t>
         </is>
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>onyx-overheat</t>
+          <t>mur-bouclier</t>
         </is>
       </c>
       <c r="C37" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="29" t="inlineStr">
-        <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E37" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+        <v>1</v>
+      </c>
+      <c r="D37" s="28" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E37" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr"/>
       <c r="G37" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Forge Heat (energy).</t>
+          <t>Gain 10 Stone.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Surge</t>
+          <t>Stacking Shield</t>
         </is>
       </c>
       <c r="B38" s="25" t="inlineStr">
         <is>
-          <t>surge-saphir-parfait</t>
+          <t>bouclier-empilant</t>
         </is>
       </c>
       <c r="C38" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="29" t="inlineStr">
-        <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E38" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+        <v>4</v>
+      </c>
+      <c r="D38" s="28" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E38" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F38" s="17" t="inlineStr"/>
       <c r="G38" s="18" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Amulet</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H38" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Forge Heat (energy).</t>
+          <t>Double your current Stone.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>Quicken</t>
+          <t>Burning Run</t>
         </is>
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>celerite-vive</t>
+          <t>course-ardente</t>
         </is>
       </c>
       <c r="C39" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" s="29" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E39" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E39" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr"/>
       <c r="G39" s="18" t="inlineStr">
         <is>
-          <t>Swift Boots</t>
+          <t>Onyx Boots</t>
         </is>
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>Haste: +30% attack speed for 3 turns.</t>
+          <t>Haste for as many turns as your current Forge Heat.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>Sapphire Surge</t>
+          <t>Free Movement</t>
         </is>
       </c>
       <c r="B40" s="25" t="inlineStr">
         <is>
-          <t>surge-saphir</t>
+          <t>mouvement-degage</t>
         </is>
       </c>
       <c r="C40" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D40" s="29" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E40" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F40" s="17" t="inlineStr"/>
       <c r="G40" s="18" t="inlineStr">
         <is>
+          <t>Traveler's Garb</t>
+        </is>
+      </c>
+      <c r="H40" s="18" t="inlineStr">
+        <is>
+          <t>Haste for 5 of your turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>Master's Hand</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="inlineStr">
+        <is>
+          <t>main-de-maitre</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="29" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr"/>
+      <c r="G41" s="18" t="inlineStr">
+        <is>
+          <t>Miner's Gloves</t>
+        </is>
+      </c>
+      <c r="H41" s="18" t="inlineStr">
+        <is>
+          <t>Draw 2 cards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="24" t="inlineStr">
+        <is>
+          <t>Onyx Overheat</t>
+        </is>
+      </c>
+      <c r="B42" s="25" t="inlineStr">
+        <is>
+          <t>onyx-overheat</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="29" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F42" s="17" t="inlineStr"/>
+      <c r="G42" s="18" t="inlineStr">
+        <is>
+          <t>Big Onyx Sword</t>
+        </is>
+      </c>
+      <c r="H42" s="18" t="inlineStr">
+        <is>
+          <t>Gain 5 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="24" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Surge</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="inlineStr">
+        <is>
+          <t>surge-saphir-parfait</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="29" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E43" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F43" s="17" t="inlineStr"/>
+      <c r="G43" s="18" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Amulet</t>
+        </is>
+      </c>
+      <c r="H43" s="18" t="inlineStr">
+        <is>
+          <t>Gain 3 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="24" t="inlineStr">
+        <is>
+          <t>Quicken</t>
+        </is>
+      </c>
+      <c r="B44" s="25" t="inlineStr">
+        <is>
+          <t>celerite-vive</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="29" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E44" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F44" s="17" t="inlineStr"/>
+      <c r="G44" s="18" t="inlineStr">
+        <is>
+          <t>Swift Boots</t>
+        </is>
+      </c>
+      <c r="H44" s="18" t="inlineStr">
+        <is>
+          <t>Haste: +30% attack speed for 3 turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="24" t="inlineStr">
+        <is>
+          <t>Sapphire Surge</t>
+        </is>
+      </c>
+      <c r="B45" s="25" t="inlineStr">
+        <is>
+          <t>surge-saphir</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="29" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E45" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F45" s="17" t="inlineStr"/>
+      <c r="G45" s="18" t="inlineStr">
+        <is>
           <t>Sapphire Amulet, Nice Sapphire Amulet</t>
         </is>
       </c>
-      <c r="H40" s="18" t="inlineStr">
+      <c r="H45" s="18" t="inlineStr">
         <is>
           <t>Gain 2 Forge Heat (energy).</t>
         </is>

</xml_diff>

<commit_message>
[technique] Catalogue régénéré : 32 items, 57 cartes, 3 sets
- Libellé "En début de combat" ajouté pour le déclencheur debutCombat (Mail Set)
- Reflète tous les nouveaux items, cartes et sets

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJcbumK5KWRfGozDrLY2Kn
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -161,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -226,6 +226,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -894,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N96"/>
+  <dimension ref="A1:N106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1703,7 +1706,7 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>Armures   (3)</t>
+          <t>Armures   (4)</t>
         </is>
       </c>
     </row>
@@ -1852,24 +1855,64 @@
       </c>
       <c r="K39" s="18" t="n"/>
       <c r="L39" s="18" t="n"/>
-      <c r="M39" s="19" t="inlineStr"/>
+      <c r="M39" s="19" t="inlineStr">
+        <is>
+          <t>Set : Mail Set</t>
+        </is>
+      </c>
       <c r="N39" s="18" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="n"/>
-      <c r="B40" s="23" t="n"/>
-      <c r="C40" s="23" t="n"/>
-      <c r="D40" s="23" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
-      <c r="J40" s="23" t="n"/>
-      <c r="K40" s="23" t="n"/>
-      <c r="L40" s="23" t="n"/>
-      <c r="M40" s="23" t="n"/>
-      <c r="N40" s="23" t="n"/>
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Crusader Plate</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>plate-croise</t>
+        </is>
+      </c>
+      <c r="C40" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>Radiant Strike</t>
+        </is>
+      </c>
+      <c r="F40" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" s="18" t="inlineStr">
+        <is>
+          <t>Sacred Ground</t>
+        </is>
+      </c>
+      <c r="H40" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="I40" s="18" t="inlineStr">
+        <is>
+          <t>Blinding Flash</t>
+        </is>
+      </c>
+      <c r="J40" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="18" t="n"/>
+      <c r="L40" s="18" t="n"/>
+      <c r="M40" s="19" t="inlineStr">
+        <is>
+          <t>Set : Crusader Set</t>
+        </is>
+      </c>
+      <c r="N40" s="18" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="23" t="n"/>
@@ -1951,67 +1994,47 @@
       <c r="M45" s="23" t="n"/>
       <c r="N45" s="23" t="n"/>
     </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="23" t="n"/>
+      <c r="B46" s="23" t="n"/>
+      <c r="C46" s="23" t="n"/>
+      <c r="D46" s="23" t="n"/>
+      <c r="E46" s="23" t="n"/>
+      <c r="F46" s="23" t="n"/>
+      <c r="G46" s="23" t="n"/>
+      <c r="H46" s="23" t="n"/>
+      <c r="I46" s="23" t="n"/>
+      <c r="J46" s="23" t="n"/>
+      <c r="K46" s="23" t="n"/>
+      <c r="L46" s="23" t="n"/>
+      <c r="M46" s="23" t="n"/>
+      <c r="N46" s="23" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="13" t="inlineStr">
         <is>
           <t>Colliers   (3)</t>
         </is>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="14" t="inlineStr">
-        <is>
-          <t>Sapphire Amulet</t>
-        </is>
-      </c>
-      <c r="B48" s="15" t="inlineStr">
-        <is>
-          <t>collier-de-saphir</t>
-        </is>
-      </c>
-      <c r="C48" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="D48" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="18" t="inlineStr">
-        <is>
-          <t>Sapphire Surge</t>
-        </is>
-      </c>
-      <c r="F48" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="18" t="n"/>
-      <c r="H48" s="18" t="n"/>
-      <c r="I48" s="18" t="n"/>
-      <c r="J48" s="18" t="n"/>
-      <c r="K48" s="18" t="n"/>
-      <c r="L48" s="18" t="n"/>
-      <c r="M48" s="19" t="inlineStr"/>
-      <c r="N48" s="18" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
         <is>
-          <t>Nice Sapphire Amulet</t>
+          <t>Sapphire Amulet</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>collier-de-saphir-fin</t>
-        </is>
-      </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+          <t>collier-de-saphir</t>
+        </is>
+      </c>
+      <c r="C49" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="D49" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" s="18" t="inlineStr">
         <is>
@@ -2019,7 +2042,7 @@
         </is>
       </c>
       <c r="F49" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G49" s="18" t="n"/>
       <c r="H49" s="18" t="n"/>
@@ -2033,29 +2056,29 @@
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Amulet</t>
+          <t>Nice Sapphire Amulet</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>collier-de-saphir-parfait</t>
-        </is>
-      </c>
-      <c r="C50" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+          <t>collier-de-saphir-fin</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D50" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E50" s="18" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Surge</t>
+          <t>Sapphire Surge</t>
         </is>
       </c>
       <c r="F50" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G50" s="18" t="n"/>
       <c r="H50" s="18" t="n"/>
@@ -2067,20 +2090,40 @@
       <c r="N50" s="18" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="23" t="n"/>
-      <c r="B51" s="23" t="n"/>
-      <c r="C51" s="23" t="n"/>
-      <c r="D51" s="23" t="n"/>
-      <c r="E51" s="23" t="n"/>
-      <c r="F51" s="23" t="n"/>
-      <c r="G51" s="23" t="n"/>
-      <c r="H51" s="23" t="n"/>
-      <c r="I51" s="23" t="n"/>
-      <c r="J51" s="23" t="n"/>
-      <c r="K51" s="23" t="n"/>
-      <c r="L51" s="23" t="n"/>
-      <c r="M51" s="23" t="n"/>
-      <c r="N51" s="23" t="n"/>
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Amulet</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>collier-de-saphir-parfait</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Surge</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G51" s="18" t="n"/>
+      <c r="H51" s="18" t="n"/>
+      <c r="I51" s="18" t="n"/>
+      <c r="J51" s="18" t="n"/>
+      <c r="K51" s="18" t="n"/>
+      <c r="L51" s="18" t="n"/>
+      <c r="M51" s="19" t="inlineStr"/>
+      <c r="N51" s="18" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="23" t="n"/>
@@ -2162,58 +2205,38 @@
       <c r="M56" s="23" t="n"/>
       <c r="N56" s="23" t="n"/>
     </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>Bagues   (2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="14" t="inlineStr">
-        <is>
-          <t>Blood Ring</t>
-        </is>
-      </c>
-      <c r="B59" s="15" t="inlineStr">
-        <is>
-          <t>bague-de-sang</t>
-        </is>
-      </c>
-      <c r="C59" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="D59" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="E59" s="18" t="inlineStr">
-        <is>
-          <t>Bloodletting</t>
-        </is>
-      </c>
-      <c r="F59" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G59" s="18" t="n"/>
-      <c r="H59" s="18" t="n"/>
-      <c r="I59" s="18" t="n"/>
-      <c r="J59" s="18" t="n"/>
-      <c r="K59" s="18" t="n"/>
-      <c r="L59" s="18" t="n"/>
-      <c r="M59" s="19" t="inlineStr"/>
-      <c r="N59" s="18" t="n"/>
+    <row r="57">
+      <c r="A57" s="23" t="n"/>
+      <c r="B57" s="23" t="n"/>
+      <c r="C57" s="23" t="n"/>
+      <c r="D57" s="23" t="n"/>
+      <c r="E57" s="23" t="n"/>
+      <c r="F57" s="23" t="n"/>
+      <c r="G57" s="23" t="n"/>
+      <c r="H57" s="23" t="n"/>
+      <c r="I57" s="23" t="n"/>
+      <c r="J57" s="23" t="n"/>
+      <c r="K57" s="23" t="n"/>
+      <c r="L57" s="23" t="n"/>
+      <c r="M57" s="23" t="n"/>
+      <c r="N57" s="23" t="n"/>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>Bagues   (3)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>Frost Ring</t>
+          <t>Blood Ring</t>
         </is>
       </c>
       <c r="B60" s="15" t="inlineStr">
         <is>
-          <t>anneau-de-givre</t>
+          <t>bague-de-sang</t>
         </is>
       </c>
       <c r="C60" s="20" t="inlineStr">
@@ -2226,7 +2249,7 @@
       </c>
       <c r="E60" s="18" t="inlineStr">
         <is>
-          <t>Frostbite</t>
+          <t>Bloodletting</t>
         </is>
       </c>
       <c r="F60" s="17" t="n">
@@ -2242,36 +2265,76 @@
       <c r="N60" s="18" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="23" t="n"/>
-      <c r="B61" s="23" t="n"/>
-      <c r="C61" s="23" t="n"/>
-      <c r="D61" s="23" t="n"/>
-      <c r="E61" s="23" t="n"/>
-      <c r="F61" s="23" t="n"/>
-      <c r="G61" s="23" t="n"/>
-      <c r="H61" s="23" t="n"/>
-      <c r="I61" s="23" t="n"/>
-      <c r="J61" s="23" t="n"/>
-      <c r="K61" s="23" t="n"/>
-      <c r="L61" s="23" t="n"/>
-      <c r="M61" s="23" t="n"/>
-      <c r="N61" s="23" t="n"/>
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>Frost Ring</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>anneau-de-givre</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>Frostbite</t>
+        </is>
+      </c>
+      <c r="F61" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="18" t="n"/>
+      <c r="H61" s="18" t="n"/>
+      <c r="I61" s="18" t="n"/>
+      <c r="J61" s="18" t="n"/>
+      <c r="K61" s="18" t="n"/>
+      <c r="L61" s="18" t="n"/>
+      <c r="M61" s="19" t="inlineStr"/>
+      <c r="N61" s="18" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="23" t="n"/>
-      <c r="B62" s="23" t="n"/>
-      <c r="C62" s="23" t="n"/>
-      <c r="D62" s="23" t="n"/>
-      <c r="E62" s="23" t="n"/>
-      <c r="F62" s="23" t="n"/>
-      <c r="G62" s="23" t="n"/>
-      <c r="H62" s="23" t="n"/>
-      <c r="I62" s="23" t="n"/>
-      <c r="J62" s="23" t="n"/>
-      <c r="K62" s="23" t="n"/>
-      <c r="L62" s="23" t="n"/>
-      <c r="M62" s="23" t="n"/>
-      <c r="N62" s="23" t="n"/>
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Perfect Frost Ring</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>anneau-de-givre-parfait</t>
+        </is>
+      </c>
+      <c r="C62" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>Frost Cascade</t>
+        </is>
+      </c>
+      <c r="F62" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" s="18" t="n"/>
+      <c r="H62" s="18" t="n"/>
+      <c r="I62" s="18" t="n"/>
+      <c r="J62" s="18" t="n"/>
+      <c r="K62" s="18" t="n"/>
+      <c r="L62" s="18" t="n"/>
+      <c r="M62" s="19" t="inlineStr"/>
+      <c r="N62" s="18" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="23" t="n"/>
@@ -2337,158 +2400,230 @@
       <c r="M66" s="23" t="n"/>
       <c r="N66" s="23" t="n"/>
     </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="A68" s="13" t="inlineStr">
-        <is>
-          <t>Gants   (2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="14" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="23" t="n"/>
+      <c r="B67" s="23" t="n"/>
+      <c r="C67" s="23" t="n"/>
+      <c r="D67" s="23" t="n"/>
+      <c r="E67" s="23" t="n"/>
+      <c r="F67" s="23" t="n"/>
+      <c r="G67" s="23" t="n"/>
+      <c r="H67" s="23" t="n"/>
+      <c r="I67" s="23" t="n"/>
+      <c r="J67" s="23" t="n"/>
+      <c r="K67" s="23" t="n"/>
+      <c r="L67" s="23" t="n"/>
+      <c r="M67" s="23" t="n"/>
+      <c r="N67" s="23" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="23" t="n"/>
+      <c r="B68" s="23" t="n"/>
+      <c r="C68" s="23" t="n"/>
+      <c r="D68" s="23" t="n"/>
+      <c r="E68" s="23" t="n"/>
+      <c r="F68" s="23" t="n"/>
+      <c r="G68" s="23" t="n"/>
+      <c r="H68" s="23" t="n"/>
+      <c r="I68" s="23" t="n"/>
+      <c r="J68" s="23" t="n"/>
+      <c r="K68" s="23" t="n"/>
+      <c r="L68" s="23" t="n"/>
+      <c r="M68" s="23" t="n"/>
+      <c r="N68" s="23" t="n"/>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>Gants   (4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
         <is>
           <t>Miner's Gloves</t>
         </is>
       </c>
-      <c r="B69" s="15" t="inlineStr">
+      <c r="B71" s="15" t="inlineStr">
         <is>
           <t>gants-de-mineur</t>
         </is>
       </c>
-      <c r="C69" s="16" t="inlineStr">
+      <c r="C71" s="16" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="D69" s="17" t="n">
+      <c r="D71" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="E69" s="18" t="inlineStr">
+      <c r="E71" s="18" t="inlineStr">
         <is>
           <t>Master's Hand</t>
         </is>
       </c>
-      <c r="F69" s="17" t="n">
+      <c r="F71" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G69" s="18" t="n"/>
-      <c r="H69" s="18" t="n"/>
-      <c r="I69" s="18" t="n"/>
-      <c r="J69" s="18" t="n"/>
-      <c r="K69" s="18" t="n"/>
-      <c r="L69" s="18" t="n"/>
-      <c r="M69" s="19" t="inlineStr"/>
-      <c r="N69" s="18" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="14" t="inlineStr">
+      <c r="G71" s="18" t="n"/>
+      <c r="H71" s="18" t="n"/>
+      <c r="I71" s="18" t="n"/>
+      <c r="J71" s="18" t="n"/>
+      <c r="K71" s="18" t="n"/>
+      <c r="L71" s="18" t="n"/>
+      <c r="M71" s="19" t="inlineStr"/>
+      <c r="N71" s="18" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
         <is>
           <t>Onyx Glove</t>
         </is>
       </c>
-      <c r="B70" s="15" t="inlineStr">
+      <c r="B72" s="15" t="inlineStr">
         <is>
           <t>gants-onyx</t>
         </is>
       </c>
-      <c r="C70" s="22" t="inlineStr">
+      <c r="C72" s="22" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="D70" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="E70" s="18" t="inlineStr">
+      <c r="D72" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E72" s="18" t="inlineStr">
         <is>
           <t>Burning Hand</t>
         </is>
       </c>
-      <c r="F70" s="17" t="n">
+      <c r="F72" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G70" s="18" t="inlineStr">
+      <c r="G72" s="18" t="inlineStr">
         <is>
           <t>Onyx Fist</t>
         </is>
       </c>
-      <c r="H70" s="17" t="n">
+      <c r="H72" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I70" s="18" t="n"/>
-      <c r="J70" s="18" t="n"/>
-      <c r="K70" s="18" t="n"/>
-      <c r="L70" s="18" t="n"/>
-      <c r="M70" s="19" t="inlineStr">
+      <c r="I72" s="18" t="inlineStr">
+        <is>
+          <t>Forge from Ashes</t>
+        </is>
+      </c>
+      <c r="J72" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K72" s="18" t="n"/>
+      <c r="L72" s="18" t="n"/>
+      <c r="M72" s="19" t="inlineStr">
         <is>
           <t>Set : Onyx Set</t>
         </is>
       </c>
-      <c r="N70" s="18" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="23" t="n"/>
-      <c r="B71" s="23" t="n"/>
-      <c r="C71" s="23" t="n"/>
-      <c r="D71" s="23" t="n"/>
-      <c r="E71" s="23" t="n"/>
-      <c r="F71" s="23" t="n"/>
-      <c r="G71" s="23" t="n"/>
-      <c r="H71" s="23" t="n"/>
-      <c r="I71" s="23" t="n"/>
-      <c r="J71" s="23" t="n"/>
-      <c r="K71" s="23" t="n"/>
-      <c r="L71" s="23" t="n"/>
-      <c r="M71" s="23" t="n"/>
-      <c r="N71" s="23" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="23" t="n"/>
-      <c r="B72" s="23" t="n"/>
-      <c r="C72" s="23" t="n"/>
-      <c r="D72" s="23" t="n"/>
-      <c r="E72" s="23" t="n"/>
-      <c r="F72" s="23" t="n"/>
-      <c r="G72" s="23" t="n"/>
-      <c r="H72" s="23" t="n"/>
-      <c r="I72" s="23" t="n"/>
-      <c r="J72" s="23" t="n"/>
-      <c r="K72" s="23" t="n"/>
-      <c r="L72" s="23" t="n"/>
-      <c r="M72" s="23" t="n"/>
-      <c r="N72" s="23" t="n"/>
+      <c r="N72" s="18" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="23" t="n"/>
-      <c r="B73" s="23" t="n"/>
-      <c r="C73" s="23" t="n"/>
-      <c r="D73" s="23" t="n"/>
-      <c r="E73" s="23" t="n"/>
-      <c r="F73" s="23" t="n"/>
-      <c r="G73" s="23" t="n"/>
-      <c r="H73" s="23" t="n"/>
-      <c r="I73" s="23" t="n"/>
-      <c r="J73" s="23" t="n"/>
-      <c r="K73" s="23" t="n"/>
-      <c r="L73" s="23" t="n"/>
-      <c r="M73" s="23" t="n"/>
-      <c r="N73" s="23" t="n"/>
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>Mail Glove</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>gants-de-maille</t>
+        </is>
+      </c>
+      <c r="C73" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D73" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Master's Hand</t>
+        </is>
+      </c>
+      <c r="F73" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G73" s="18" t="inlineStr">
+        <is>
+          <t>Outnumbered</t>
+        </is>
+      </c>
+      <c r="H73" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I73" s="18" t="inlineStr">
+        <is>
+          <t>Mail Advantage</t>
+        </is>
+      </c>
+      <c r="J73" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K73" s="18" t="n"/>
+      <c r="L73" s="18" t="n"/>
+      <c r="M73" s="19" t="inlineStr">
+        <is>
+          <t>Set : Mail Set</t>
+        </is>
+      </c>
+      <c r="N73" s="18" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="23" t="n"/>
-      <c r="B74" s="23" t="n"/>
-      <c r="C74" s="23" t="n"/>
-      <c r="D74" s="23" t="n"/>
-      <c r="E74" s="23" t="n"/>
-      <c r="F74" s="23" t="n"/>
-      <c r="G74" s="23" t="n"/>
-      <c r="H74" s="23" t="n"/>
-      <c r="I74" s="23" t="n"/>
-      <c r="J74" s="23" t="n"/>
-      <c r="K74" s="23" t="n"/>
-      <c r="L74" s="23" t="n"/>
-      <c r="M74" s="23" t="n"/>
-      <c r="N74" s="23" t="n"/>
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t>Crusader Gauntlets</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>gants-croise</t>
+        </is>
+      </c>
+      <c r="C74" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D74" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>Lumen Jab</t>
+        </is>
+      </c>
+      <c r="F74" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G74" s="18" t="inlineStr">
+        <is>
+          <t>Halo Burst</t>
+        </is>
+      </c>
+      <c r="H74" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I74" s="18" t="n"/>
+      <c r="J74" s="18" t="n"/>
+      <c r="K74" s="18" t="n"/>
+      <c r="L74" s="18" t="n"/>
+      <c r="M74" s="19" t="inlineStr">
+        <is>
+          <t>Set : Crusader Set</t>
+        </is>
+      </c>
+      <c r="N74" s="18" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="23" t="n"/>
@@ -2522,265 +2657,338 @@
       <c r="M76" s="23" t="n"/>
       <c r="N76" s="23" t="n"/>
     </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="13" t="inlineStr">
-        <is>
-          <t>Bottes   (2)</t>
-        </is>
-      </c>
+    <row r="77">
+      <c r="A77" s="23" t="n"/>
+      <c r="B77" s="23" t="n"/>
+      <c r="C77" s="23" t="n"/>
+      <c r="D77" s="23" t="n"/>
+      <c r="E77" s="23" t="n"/>
+      <c r="F77" s="23" t="n"/>
+      <c r="G77" s="23" t="n"/>
+      <c r="H77" s="23" t="n"/>
+      <c r="I77" s="23" t="n"/>
+      <c r="J77" s="23" t="n"/>
+      <c r="K77" s="23" t="n"/>
+      <c r="L77" s="23" t="n"/>
+      <c r="M77" s="23" t="n"/>
+      <c r="N77" s="23" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="23" t="n"/>
+      <c r="B78" s="23" t="n"/>
+      <c r="C78" s="23" t="n"/>
+      <c r="D78" s="23" t="n"/>
+      <c r="E78" s="23" t="n"/>
+      <c r="F78" s="23" t="n"/>
+      <c r="G78" s="23" t="n"/>
+      <c r="H78" s="23" t="n"/>
+      <c r="I78" s="23" t="n"/>
+      <c r="J78" s="23" t="n"/>
+      <c r="K78" s="23" t="n"/>
+      <c r="L78" s="23" t="n"/>
+      <c r="M78" s="23" t="n"/>
+      <c r="N78" s="23" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="14" t="inlineStr">
+      <c r="A79" s="23" t="n"/>
+      <c r="B79" s="23" t="n"/>
+      <c r="C79" s="23" t="n"/>
+      <c r="D79" s="23" t="n"/>
+      <c r="E79" s="23" t="n"/>
+      <c r="F79" s="23" t="n"/>
+      <c r="G79" s="23" t="n"/>
+      <c r="H79" s="23" t="n"/>
+      <c r="I79" s="23" t="n"/>
+      <c r="J79" s="23" t="n"/>
+      <c r="K79" s="23" t="n"/>
+      <c r="L79" s="23" t="n"/>
+      <c r="M79" s="23" t="n"/>
+      <c r="N79" s="23" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="23" t="n"/>
+      <c r="B80" s="23" t="n"/>
+      <c r="C80" s="23" t="n"/>
+      <c r="D80" s="23" t="n"/>
+      <c r="E80" s="23" t="n"/>
+      <c r="F80" s="23" t="n"/>
+      <c r="G80" s="23" t="n"/>
+      <c r="H80" s="23" t="n"/>
+      <c r="I80" s="23" t="n"/>
+      <c r="J80" s="23" t="n"/>
+      <c r="K80" s="23" t="n"/>
+      <c r="L80" s="23" t="n"/>
+      <c r="M80" s="23" t="n"/>
+      <c r="N80" s="23" t="n"/>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>Bottes   (4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="inlineStr">
         <is>
           <t>Swift Boots</t>
         </is>
       </c>
-      <c r="B79" s="15" t="inlineStr">
+      <c r="B83" s="15" t="inlineStr">
         <is>
           <t>bottes-vives</t>
         </is>
       </c>
-      <c r="C79" s="21" t="inlineStr">
+      <c r="C83" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="D83" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Quicken</t>
+        </is>
+      </c>
+      <c r="F83" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G83" s="18" t="inlineStr">
+        <is>
+          <t>Second Wind</t>
+        </is>
+      </c>
+      <c r="H83" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I83" s="18" t="n"/>
+      <c r="J83" s="18" t="n"/>
+      <c r="K83" s="18" t="n"/>
+      <c r="L83" s="18" t="n"/>
+      <c r="M83" s="19" t="inlineStr"/>
+      <c r="N83" s="18" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>Onyx Boots</t>
+        </is>
+      </c>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>bottes-onyx</t>
+        </is>
+      </c>
+      <c r="C84" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D84" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Burning Run</t>
+        </is>
+      </c>
+      <c r="F84" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="18" t="inlineStr">
+        <is>
+          <t>Flaming Kick</t>
+        </is>
+      </c>
+      <c r="H84" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I84" s="18" t="inlineStr">
+        <is>
+          <t>Fire Boost</t>
+        </is>
+      </c>
+      <c r="J84" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K84" s="18" t="inlineStr">
+        <is>
+          <t>Boost</t>
+        </is>
+      </c>
+      <c r="L84" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M84" s="19" t="inlineStr">
+        <is>
+          <t>Set : Onyx Set</t>
+        </is>
+      </c>
+      <c r="N84" s="18" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>Mail Boots</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="inlineStr">
+        <is>
+          <t>bottes-de-maille</t>
+        </is>
+      </c>
+      <c r="C85" s="21" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="D79" s="17" t="n">
+      <c r="D85" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E85" s="18" t="inlineStr">
+        <is>
+          <t>Quicken</t>
+        </is>
+      </c>
+      <c r="F85" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="E79" s="18" t="inlineStr">
-        <is>
-          <t>Quicken</t>
-        </is>
-      </c>
-      <c r="F79" s="17" t="n">
+      <c r="G85" s="18" t="inlineStr">
+        <is>
+          <t>Mail Advantage</t>
+        </is>
+      </c>
+      <c r="H85" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I85" s="18" t="inlineStr">
+        <is>
+          <t>Boost</t>
+        </is>
+      </c>
+      <c r="J85" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G79" s="18" t="n"/>
-      <c r="H79" s="18" t="n"/>
-      <c r="I79" s="18" t="n"/>
-      <c r="J79" s="18" t="n"/>
-      <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
-      <c r="M79" s="19" t="inlineStr"/>
-      <c r="N79" s="18" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="14" t="inlineStr">
-        <is>
-          <t>Onyx Boots</t>
-        </is>
-      </c>
-      <c r="B80" s="15" t="inlineStr">
-        <is>
-          <t>bottes-onyx</t>
-        </is>
-      </c>
-      <c r="C80" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="D80" s="17" t="n">
+      <c r="K85" s="18" t="n"/>
+      <c r="L85" s="18" t="n"/>
+      <c r="M85" s="19" t="inlineStr">
+        <is>
+          <t>Set : Mail Set</t>
+        </is>
+      </c>
+      <c r="N85" s="18" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>Crusader Greaves</t>
+        </is>
+      </c>
+      <c r="B86" s="15" t="inlineStr">
+        <is>
+          <t>bottes-croise</t>
+        </is>
+      </c>
+      <c r="C86" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D86" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="E80" s="18" t="inlineStr">
-        <is>
-          <t>Burning Run</t>
-        </is>
-      </c>
-      <c r="F80" s="17" t="n">
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Crusader's Charge</t>
+        </is>
+      </c>
+      <c r="F86" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="G80" s="18" t="inlineStr">
-        <is>
-          <t>Flaming Kick</t>
-        </is>
-      </c>
-      <c r="H80" s="17" t="n">
+      <c r="G86" s="18" t="inlineStr">
+        <is>
+          <t>Dazzling Kick</t>
+        </is>
+      </c>
+      <c r="H86" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I80" s="18" t="n"/>
-      <c r="J80" s="18" t="n"/>
-      <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
-      <c r="M80" s="19" t="inlineStr">
-        <is>
-          <t>Set : Onyx Set</t>
-        </is>
-      </c>
-      <c r="N80" s="18" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="23" t="n"/>
-      <c r="B81" s="23" t="n"/>
-      <c r="C81" s="23" t="n"/>
-      <c r="D81" s="23" t="n"/>
-      <c r="E81" s="23" t="n"/>
-      <c r="F81" s="23" t="n"/>
-      <c r="G81" s="23" t="n"/>
-      <c r="H81" s="23" t="n"/>
-      <c r="I81" s="23" t="n"/>
-      <c r="J81" s="23" t="n"/>
-      <c r="K81" s="23" t="n"/>
-      <c r="L81" s="23" t="n"/>
-      <c r="M81" s="23" t="n"/>
-      <c r="N81" s="23" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="23" t="n"/>
-      <c r="B82" s="23" t="n"/>
-      <c r="C82" s="23" t="n"/>
-      <c r="D82" s="23" t="n"/>
-      <c r="E82" s="23" t="n"/>
-      <c r="F82" s="23" t="n"/>
-      <c r="G82" s="23" t="n"/>
-      <c r="H82" s="23" t="n"/>
-      <c r="I82" s="23" t="n"/>
-      <c r="J82" s="23" t="n"/>
-      <c r="K82" s="23" t="n"/>
-      <c r="L82" s="23" t="n"/>
-      <c r="M82" s="23" t="n"/>
-      <c r="N82" s="23" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="23" t="n"/>
-      <c r="B83" s="23" t="n"/>
-      <c r="C83" s="23" t="n"/>
-      <c r="D83" s="23" t="n"/>
-      <c r="E83" s="23" t="n"/>
-      <c r="F83" s="23" t="n"/>
-      <c r="G83" s="23" t="n"/>
-      <c r="H83" s="23" t="n"/>
-      <c r="I83" s="23" t="n"/>
-      <c r="J83" s="23" t="n"/>
-      <c r="K83" s="23" t="n"/>
-      <c r="L83" s="23" t="n"/>
-      <c r="M83" s="23" t="n"/>
-      <c r="N83" s="23" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="23" t="n"/>
-      <c r="B84" s="23" t="n"/>
-      <c r="C84" s="23" t="n"/>
-      <c r="D84" s="23" t="n"/>
-      <c r="E84" s="23" t="n"/>
-      <c r="F84" s="23" t="n"/>
-      <c r="G84" s="23" t="n"/>
-      <c r="H84" s="23" t="n"/>
-      <c r="I84" s="23" t="n"/>
-      <c r="J84" s="23" t="n"/>
-      <c r="K84" s="23" t="n"/>
-      <c r="L84" s="23" t="n"/>
-      <c r="M84" s="23" t="n"/>
-      <c r="N84" s="23" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="23" t="n"/>
-      <c r="B85" s="23" t="n"/>
-      <c r="C85" s="23" t="n"/>
-      <c r="D85" s="23" t="n"/>
-      <c r="E85" s="23" t="n"/>
-      <c r="F85" s="23" t="n"/>
-      <c r="G85" s="23" t="n"/>
-      <c r="H85" s="23" t="n"/>
-      <c r="I85" s="23" t="n"/>
-      <c r="J85" s="23" t="n"/>
-      <c r="K85" s="23" t="n"/>
-      <c r="L85" s="23" t="n"/>
-      <c r="M85" s="23" t="n"/>
-      <c r="N85" s="23" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="23" t="n"/>
-      <c r="B86" s="23" t="n"/>
-      <c r="C86" s="23" t="n"/>
-      <c r="D86" s="23" t="n"/>
-      <c r="E86" s="23" t="n"/>
-      <c r="F86" s="23" t="n"/>
-      <c r="G86" s="23" t="n"/>
-      <c r="H86" s="23" t="n"/>
-      <c r="I86" s="23" t="n"/>
-      <c r="J86" s="23" t="n"/>
-      <c r="K86" s="23" t="n"/>
-      <c r="L86" s="23" t="n"/>
-      <c r="M86" s="23" t="n"/>
-      <c r="N86" s="23" t="n"/>
-    </row>
-    <row r="88" ht="20" customHeight="1">
-      <c r="A88" s="13" t="inlineStr">
-        <is>
-          <t>Sacs   (2)</t>
-        </is>
-      </c>
+      <c r="I86" s="18" t="n"/>
+      <c r="J86" s="18" t="n"/>
+      <c r="K86" s="18" t="n"/>
+      <c r="L86" s="18" t="n"/>
+      <c r="M86" s="19" t="inlineStr">
+        <is>
+          <t>Set : Crusader Set</t>
+        </is>
+      </c>
+      <c r="N86" s="18" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="23" t="n"/>
+      <c r="B87" s="23" t="n"/>
+      <c r="C87" s="23" t="n"/>
+      <c r="D87" s="23" t="n"/>
+      <c r="E87" s="23" t="n"/>
+      <c r="F87" s="23" t="n"/>
+      <c r="G87" s="23" t="n"/>
+      <c r="H87" s="23" t="n"/>
+      <c r="I87" s="23" t="n"/>
+      <c r="J87" s="23" t="n"/>
+      <c r="K87" s="23" t="n"/>
+      <c r="L87" s="23" t="n"/>
+      <c r="M87" s="23" t="n"/>
+      <c r="N87" s="23" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="23" t="n"/>
+      <c r="B88" s="23" t="n"/>
+      <c r="C88" s="23" t="n"/>
+      <c r="D88" s="23" t="n"/>
+      <c r="E88" s="23" t="n"/>
+      <c r="F88" s="23" t="n"/>
+      <c r="G88" s="23" t="n"/>
+      <c r="H88" s="23" t="n"/>
+      <c r="I88" s="23" t="n"/>
+      <c r="J88" s="23" t="n"/>
+      <c r="K88" s="23" t="n"/>
+      <c r="L88" s="23" t="n"/>
+      <c r="M88" s="23" t="n"/>
+      <c r="N88" s="23" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="14" t="inlineStr">
-        <is>
-          <t>Leather Pouch</t>
-        </is>
-      </c>
-      <c r="B89" s="15" t="inlineStr">
-        <is>
-          <t>sac-en-cuir</t>
-        </is>
-      </c>
-      <c r="C89" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="D89" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E89" s="18" t="n"/>
-      <c r="F89" s="18" t="n"/>
-      <c r="G89" s="18" t="n"/>
-      <c r="H89" s="18" t="n"/>
-      <c r="I89" s="18" t="n"/>
-      <c r="J89" s="18" t="n"/>
-      <c r="K89" s="18" t="n"/>
-      <c r="L89" s="18" t="n"/>
-      <c r="M89" s="19" t="inlineStr">
-        <is>
-          <t>+2 rangées de sac</t>
-        </is>
-      </c>
-      <c r="N89" s="18" t="n"/>
+      <c r="A89" s="23" t="n"/>
+      <c r="B89" s="23" t="n"/>
+      <c r="C89" s="23" t="n"/>
+      <c r="D89" s="23" t="n"/>
+      <c r="E89" s="23" t="n"/>
+      <c r="F89" s="23" t="n"/>
+      <c r="G89" s="23" t="n"/>
+      <c r="H89" s="23" t="n"/>
+      <c r="I89" s="23" t="n"/>
+      <c r="J89" s="23" t="n"/>
+      <c r="K89" s="23" t="n"/>
+      <c r="L89" s="23" t="n"/>
+      <c r="M89" s="23" t="n"/>
+      <c r="N89" s="23" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="14" t="inlineStr">
-        <is>
-          <t>Big Leather Pouch</t>
-        </is>
-      </c>
-      <c r="B90" s="15" t="inlineStr">
-        <is>
-          <t>grand-sac-en-cuir</t>
-        </is>
-      </c>
-      <c r="C90" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="D90" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E90" s="18" t="n"/>
-      <c r="F90" s="18" t="n"/>
-      <c r="G90" s="18" t="n"/>
-      <c r="H90" s="18" t="n"/>
-      <c r="I90" s="18" t="n"/>
-      <c r="J90" s="18" t="n"/>
-      <c r="K90" s="18" t="n"/>
-      <c r="L90" s="18" t="n"/>
-      <c r="M90" s="19" t="inlineStr">
-        <is>
-          <t>+3 rangées de sac</t>
-        </is>
-      </c>
-      <c r="N90" s="18" t="n"/>
+      <c r="A90" s="23" t="n"/>
+      <c r="B90" s="23" t="n"/>
+      <c r="C90" s="23" t="n"/>
+      <c r="D90" s="23" t="n"/>
+      <c r="E90" s="23" t="n"/>
+      <c r="F90" s="23" t="n"/>
+      <c r="G90" s="23" t="n"/>
+      <c r="H90" s="23" t="n"/>
+      <c r="I90" s="23" t="n"/>
+      <c r="J90" s="23" t="n"/>
+      <c r="K90" s="23" t="n"/>
+      <c r="L90" s="23" t="n"/>
+      <c r="M90" s="23" t="n"/>
+      <c r="N90" s="23" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="23" t="n"/>
@@ -2814,82 +3022,325 @@
       <c r="M92" s="23" t="n"/>
       <c r="N92" s="23" t="n"/>
     </row>
-    <row r="93">
-      <c r="A93" s="23" t="n"/>
-      <c r="B93" s="23" t="n"/>
-      <c r="C93" s="23" t="n"/>
-      <c r="D93" s="23" t="n"/>
-      <c r="E93" s="23" t="n"/>
-      <c r="F93" s="23" t="n"/>
-      <c r="G93" s="23" t="n"/>
-      <c r="H93" s="23" t="n"/>
-      <c r="I93" s="23" t="n"/>
-      <c r="J93" s="23" t="n"/>
-      <c r="K93" s="23" t="n"/>
-      <c r="L93" s="23" t="n"/>
-      <c r="M93" s="23" t="n"/>
-      <c r="N93" s="23" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="23" t="n"/>
-      <c r="B94" s="23" t="n"/>
-      <c r="C94" s="23" t="n"/>
-      <c r="D94" s="23" t="n"/>
-      <c r="E94" s="23" t="n"/>
-      <c r="F94" s="23" t="n"/>
-      <c r="G94" s="23" t="n"/>
-      <c r="H94" s="23" t="n"/>
-      <c r="I94" s="23" t="n"/>
-      <c r="J94" s="23" t="n"/>
-      <c r="K94" s="23" t="n"/>
-      <c r="L94" s="23" t="n"/>
-      <c r="M94" s="23" t="n"/>
-      <c r="N94" s="23" t="n"/>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>Sacs   (6)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="23" t="n"/>
-      <c r="B95" s="23" t="n"/>
-      <c r="C95" s="23" t="n"/>
-      <c r="D95" s="23" t="n"/>
-      <c r="E95" s="23" t="n"/>
-      <c r="F95" s="23" t="n"/>
-      <c r="G95" s="23" t="n"/>
-      <c r="H95" s="23" t="n"/>
-      <c r="I95" s="23" t="n"/>
-      <c r="J95" s="23" t="n"/>
-      <c r="K95" s="23" t="n"/>
-      <c r="L95" s="23" t="n"/>
-      <c r="M95" s="23" t="n"/>
-      <c r="N95" s="23" t="n"/>
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>Leather Pouch</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="inlineStr">
+        <is>
+          <t>sac-en-cuir</t>
+        </is>
+      </c>
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="D95" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="18" t="n"/>
+      <c r="F95" s="18" t="n"/>
+      <c r="G95" s="18" t="n"/>
+      <c r="H95" s="18" t="n"/>
+      <c r="I95" s="18" t="n"/>
+      <c r="J95" s="18" t="n"/>
+      <c r="K95" s="18" t="n"/>
+      <c r="L95" s="18" t="n"/>
+      <c r="M95" s="19" t="inlineStr">
+        <is>
+          <t>+1 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N95" s="18" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="23" t="n"/>
-      <c r="B96" s="23" t="n"/>
-      <c r="C96" s="23" t="n"/>
-      <c r="D96" s="23" t="n"/>
-      <c r="E96" s="23" t="n"/>
-      <c r="F96" s="23" t="n"/>
-      <c r="G96" s="23" t="n"/>
-      <c r="H96" s="23" t="n"/>
-      <c r="I96" s="23" t="n"/>
-      <c r="J96" s="23" t="n"/>
-      <c r="K96" s="23" t="n"/>
-      <c r="L96" s="23" t="n"/>
-      <c r="M96" s="23" t="n"/>
-      <c r="N96" s="23" t="n"/>
+      <c r="A96" s="14" t="inlineStr">
+        <is>
+          <t>Big Leather Pouch</t>
+        </is>
+      </c>
+      <c r="B96" s="15" t="inlineStr">
+        <is>
+          <t>grand-sac-en-cuir</t>
+        </is>
+      </c>
+      <c r="C96" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="D96" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="18" t="n"/>
+      <c r="F96" s="18" t="n"/>
+      <c r="G96" s="18" t="n"/>
+      <c r="H96" s="18" t="n"/>
+      <c r="I96" s="18" t="n"/>
+      <c r="J96" s="18" t="n"/>
+      <c r="K96" s="18" t="n"/>
+      <c r="L96" s="18" t="n"/>
+      <c r="M96" s="19" t="inlineStr">
+        <is>
+          <t>+2 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N96" s="18" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>Huge Leather Pouch</t>
+        </is>
+      </c>
+      <c r="B97" s="15" t="inlineStr">
+        <is>
+          <t>enorme-sac-en-cuir</t>
+        </is>
+      </c>
+      <c r="C97" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D97" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="18" t="n"/>
+      <c r="F97" s="18" t="n"/>
+      <c r="G97" s="18" t="n"/>
+      <c r="H97" s="18" t="n"/>
+      <c r="I97" s="18" t="n"/>
+      <c r="J97" s="18" t="n"/>
+      <c r="K97" s="18" t="n"/>
+      <c r="L97" s="18" t="n"/>
+      <c r="M97" s="19" t="inlineStr">
+        <is>
+          <t>+3 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N97" s="18" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="inlineStr">
+        <is>
+          <t>Backpack</t>
+        </is>
+      </c>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>sac-a-dos</t>
+        </is>
+      </c>
+      <c r="C98" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D98" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="18" t="n"/>
+      <c r="F98" s="18" t="n"/>
+      <c r="G98" s="18" t="n"/>
+      <c r="H98" s="18" t="n"/>
+      <c r="I98" s="18" t="n"/>
+      <c r="J98" s="18" t="n"/>
+      <c r="K98" s="18" t="n"/>
+      <c r="L98" s="18" t="n"/>
+      <c r="M98" s="19" t="inlineStr">
+        <is>
+          <t>+4 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N98" s="18" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="14" t="inlineStr">
+        <is>
+          <t>Bottomless Bag</t>
+        </is>
+      </c>
+      <c r="B99" s="15" t="inlineStr">
+        <is>
+          <t>sac-sans-fond</t>
+        </is>
+      </c>
+      <c r="C99" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D99" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="18" t="n"/>
+      <c r="F99" s="18" t="n"/>
+      <c r="G99" s="18" t="n"/>
+      <c r="H99" s="18" t="n"/>
+      <c r="I99" s="18" t="n"/>
+      <c r="J99" s="18" t="n"/>
+      <c r="K99" s="18" t="n"/>
+      <c r="L99" s="18" t="n"/>
+      <c r="M99" s="19" t="inlineStr">
+        <is>
+          <t>+6 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N99" s="18" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="inlineStr">
+        <is>
+          <t>Master Miner's Bag</t>
+        </is>
+      </c>
+      <c r="B100" s="15" t="inlineStr">
+        <is>
+          <t>sac-maitre-mineur</t>
+        </is>
+      </c>
+      <c r="C100" s="24" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="D100" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="18" t="n"/>
+      <c r="F100" s="18" t="n"/>
+      <c r="G100" s="18" t="n"/>
+      <c r="H100" s="18" t="n"/>
+      <c r="I100" s="18" t="n"/>
+      <c r="J100" s="18" t="n"/>
+      <c r="K100" s="18" t="n"/>
+      <c r="L100" s="18" t="n"/>
+      <c r="M100" s="19" t="inlineStr">
+        <is>
+          <t>+10 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N100" s="18" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="23" t="n"/>
+      <c r="B101" s="23" t="n"/>
+      <c r="C101" s="23" t="n"/>
+      <c r="D101" s="23" t="n"/>
+      <c r="E101" s="23" t="n"/>
+      <c r="F101" s="23" t="n"/>
+      <c r="G101" s="23" t="n"/>
+      <c r="H101" s="23" t="n"/>
+      <c r="I101" s="23" t="n"/>
+      <c r="J101" s="23" t="n"/>
+      <c r="K101" s="23" t="n"/>
+      <c r="L101" s="23" t="n"/>
+      <c r="M101" s="23" t="n"/>
+      <c r="N101" s="23" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="23" t="n"/>
+      <c r="B102" s="23" t="n"/>
+      <c r="C102" s="23" t="n"/>
+      <c r="D102" s="23" t="n"/>
+      <c r="E102" s="23" t="n"/>
+      <c r="F102" s="23" t="n"/>
+      <c r="G102" s="23" t="n"/>
+      <c r="H102" s="23" t="n"/>
+      <c r="I102" s="23" t="n"/>
+      <c r="J102" s="23" t="n"/>
+      <c r="K102" s="23" t="n"/>
+      <c r="L102" s="23" t="n"/>
+      <c r="M102" s="23" t="n"/>
+      <c r="N102" s="23" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="23" t="n"/>
+      <c r="B103" s="23" t="n"/>
+      <c r="C103" s="23" t="n"/>
+      <c r="D103" s="23" t="n"/>
+      <c r="E103" s="23" t="n"/>
+      <c r="F103" s="23" t="n"/>
+      <c r="G103" s="23" t="n"/>
+      <c r="H103" s="23" t="n"/>
+      <c r="I103" s="23" t="n"/>
+      <c r="J103" s="23" t="n"/>
+      <c r="K103" s="23" t="n"/>
+      <c r="L103" s="23" t="n"/>
+      <c r="M103" s="23" t="n"/>
+      <c r="N103" s="23" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="23" t="n"/>
+      <c r="B104" s="23" t="n"/>
+      <c r="C104" s="23" t="n"/>
+      <c r="D104" s="23" t="n"/>
+      <c r="E104" s="23" t="n"/>
+      <c r="F104" s="23" t="n"/>
+      <c r="G104" s="23" t="n"/>
+      <c r="H104" s="23" t="n"/>
+      <c r="I104" s="23" t="n"/>
+      <c r="J104" s="23" t="n"/>
+      <c r="K104" s="23" t="n"/>
+      <c r="L104" s="23" t="n"/>
+      <c r="M104" s="23" t="n"/>
+      <c r="N104" s="23" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="23" t="n"/>
+      <c r="B105" s="23" t="n"/>
+      <c r="C105" s="23" t="n"/>
+      <c r="D105" s="23" t="n"/>
+      <c r="E105" s="23" t="n"/>
+      <c r="F105" s="23" t="n"/>
+      <c r="G105" s="23" t="n"/>
+      <c r="H105" s="23" t="n"/>
+      <c r="I105" s="23" t="n"/>
+      <c r="J105" s="23" t="n"/>
+      <c r="K105" s="23" t="n"/>
+      <c r="L105" s="23" t="n"/>
+      <c r="M105" s="23" t="n"/>
+      <c r="N105" s="23" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="23" t="n"/>
+      <c r="B106" s="23" t="n"/>
+      <c r="C106" s="23" t="n"/>
+      <c r="D106" s="23" t="n"/>
+      <c r="E106" s="23" t="n"/>
+      <c r="F106" s="23" t="n"/>
+      <c r="G106" s="23" t="n"/>
+      <c r="H106" s="23" t="n"/>
+      <c r="I106" s="23" t="n"/>
+      <c r="J106" s="23" t="n"/>
+      <c r="K106" s="23" t="n"/>
+      <c r="L106" s="23" t="n"/>
+      <c r="M106" s="23" t="n"/>
+      <c r="N106" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A17:N17"/>
+    <mergeCell ref="A70:N70"/>
     <mergeCell ref="A27:N27"/>
-    <mergeCell ref="A88:N88"/>
+    <mergeCell ref="A94:N94"/>
     <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A78:N78"/>
+    <mergeCell ref="A48:N48"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A68:N68"/>
-    <mergeCell ref="A47:N47"/>
+    <mergeCell ref="A59:N59"/>
+    <mergeCell ref="A82:N82"/>
     <mergeCell ref="A36:N36"/>
-    <mergeCell ref="A58:N58"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2903,7 +3354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2966,12 +3417,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>All Should Be Fire</t>
         </is>
       </c>
-      <c r="B3" s="25" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>tout-en-feu</t>
         </is>
@@ -2979,7 +3430,7 @@
       <c r="C3" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="26" t="inlineStr">
+      <c r="D3" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
@@ -3006,12 +3457,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Armor Forging</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>forgeage-d-armure</t>
         </is>
@@ -3019,7 +3470,7 @@
       <c r="C4" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
@@ -3046,518 +3497,518 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>Blinding Flash</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>eclair-aveuglant</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Crusader Plate</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Apply 2 Confusion to ALL enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Bloodletting</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>coup-de-sang</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C6" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D6" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="F5" s="17" t="inlineStr"/>
-      <c r="G5" s="18" t="inlineStr">
-        <is>
-          <t>Blood Ring</t>
-        </is>
-      </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>Burning Hand</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>main-brulante</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr"/>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Blood Ring</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Discard your hand. For each card discarded, apply 8 Burning to a random enemy.</t>
+          <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>Cleave</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>couper-en-deux</t>
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>Burning Hand</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>main-brulante</t>
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="26" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr"/>
       <c r="G7" s="18" t="inlineStr">
         <is>
+          <t>Onyx Glove</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>Discard your hand. For each card discarded, apply 8 Burning to a random enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>Cleave</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>couper-en-deux</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr"/>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
           <t>War Axe</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>Deal 20 damage. If the target dies, deal 15 damage to the next enemy.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>Dragon's Blaze</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="inlineStr">
-        <is>
-          <t>embrasement-dragon</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="26" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>Dazzling Kick</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>coup-eblouissant</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="inlineStr">
-        <is>
-          <t>Magma Hammer, Onyx Guard Plate</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="24" t="inlineStr">
-        <is>
-          <t>Fire Strike</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="inlineStr">
-        <is>
-          <t>feu-frappe</t>
-        </is>
-      </c>
-      <c r="C9" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="26" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
-      <c r="E9" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr"/>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer</t>
+          <t>Crusader Greaves</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>Deal 12 damage. Apply 3 Burning.</t>
+          <t>Deal 10 damage. Apply 3 Confusion.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>Flaming Kick</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="inlineStr">
-        <is>
-          <t>coup-de-pied-ardent</t>
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>Dragon's Blaze</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>embrasement-dragon</t>
         </is>
       </c>
       <c r="C10" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Magma Hammer, Onyx Guard Plate</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>Fire Strike</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>feu-frappe</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="26" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>Epic</t>
-        </is>
-      </c>
-      <c r="F10" s="17" t="inlineStr"/>
-      <c r="G10" s="18" t="inlineStr">
-        <is>
-          <t>Onyx Boots</t>
-        </is>
-      </c>
-      <c r="H10" s="18" t="inlineStr">
-        <is>
-          <t>Move all Burning from the target to the enemy behind it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>Forge Smash</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="inlineStr">
-        <is>
-          <t>ecrasement</t>
-        </is>
-      </c>
-      <c r="C11" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="26" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr"/>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>Forge Hammer</t>
+          <t>Magma Hammer</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>Deal 10 damage. Gain 8 Stone.</t>
+          <t>Deal 12 damage. Apply 3 Burning.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
-        <is>
-          <t>Frostbite</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="inlineStr">
-        <is>
-          <t>givre-lent</t>
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>Flaming Kick</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>coup-de-pied-ardent</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="26" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr"/>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>Frost Ring</t>
+          <t>Onyx Boots</t>
         </is>
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>Deal 5 damage. Chill: -30% speed for 3 turns.</t>
+          <t>Move all Burning from the target to the enemy behind it.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
-        <is>
-          <t>Giant Swing</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="inlineStr">
-        <is>
-          <t>giant-swing</t>
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>Forge Smash</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>ecrasement</t>
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="26" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E13" s="21" t="inlineStr">
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr"/>
+      <c r="G13" s="18" t="inlineStr">
+        <is>
+          <t>Forge Hammer</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>Deal 10 damage. Gain 8 Stone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>Frost Cascade</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>gel-cascade</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="G13" s="18" t="inlineStr">
-        <is>
-          <t>War Axe</t>
-        </is>
-      </c>
-      <c r="H13" s="18" t="inlineStr">
-        <is>
-          <t>Deal 16 damage to ALL enemies. Apply 2 Bleed to ALL enemies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Heat Rejection</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="inlineStr">
-        <is>
-          <t>rejet-chaleur</t>
-        </is>
-      </c>
-      <c r="C14" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr"/>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Perfect Frost Ring</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Deal 8 damage and apply 3 Chill. If the target was already chilled, cascade the same hit to the next enemy, and so on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>Frostbite</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>givre-lent</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="F14" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="G14" s="18" t="inlineStr">
-        <is>
-          <t>Big Onyx Sword</t>
-        </is>
-      </c>
-      <c r="H14" s="18" t="inlineStr">
-        <is>
-          <t>Spend all Forge Heat. Apply 8 Burning per Heat spent to ALL enemies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>Lava Hammer</t>
-        </is>
-      </c>
-      <c r="B15" s="25" t="inlineStr">
-        <is>
-          <t>coup-de-lave</t>
-        </is>
-      </c>
-      <c r="C15" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="26" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
-      <c r="E15" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr"/>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer</t>
+          <t>Frost Ring</t>
         </is>
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>Deal 28 damage. Apply 4 Burning.</t>
+          <t>Deal 5 damage. Chill: -30% speed for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>Onyx Breath</t>
-        </is>
-      </c>
-      <c r="B16" s="25" t="inlineStr">
-        <is>
-          <t>souffle-onyx</t>
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>Giant Swing</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>giant-swing</t>
         </is>
       </c>
       <c r="C16" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="26" t="inlineStr">
+      <c r="D16" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>War Axe</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>Deal 16 damage to ALL enemies. Apply 2 Bleed to ALL enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>Halo Burst</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>eclat-de-halo</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G17" s="18" t="inlineStr">
+        <is>
+          <t>Crusader Gauntlets</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>Deal 6 damage to ALL enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>Heat Rejection</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>rejet-chaleur</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="F16" s="17" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
-        <is>
-          <t>Onyx Guard Plate</t>
-        </is>
-      </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>Apply 20 Burning to ALL enemies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="24" t="inlineStr">
-        <is>
-          <t>Onyx Fist</t>
-        </is>
-      </c>
-      <c r="B17" s="25" t="inlineStr">
-        <is>
-          <t>poing-onyx</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="26" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
-      <c r="E17" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="F17" s="17" t="inlineStr"/>
-      <c r="G17" s="18" t="inlineStr">
-        <is>
-          <t>Onyx Glove</t>
-        </is>
-      </c>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>Gain 10 Stone. Deal 10 damage and apply 3 Burning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="24" t="inlineStr">
-        <is>
-          <t>Onyx Radiance</t>
-        </is>
-      </c>
-      <c r="B18" s="25" t="inlineStr">
-        <is>
-          <t>onyx-radiance</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="26" t="inlineStr">
-        <is>
-          <t>Attaque</t>
-        </is>
-      </c>
-      <c r="E18" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="F18" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
           <t>Big Onyx Sword</t>
@@ -3565,25 +4016,25 @@
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>Apply 8 Burning to ALL enemies.</t>
+          <t>Spend all Forge Heat. Apply 8 Burning per Heat spent to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="24" t="inlineStr">
-        <is>
-          <t>Onyx Slash</t>
-        </is>
-      </c>
-      <c r="B19" s="25" t="inlineStr">
-        <is>
-          <t>onyx-slash</t>
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>Lava Hammer</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>coup-de-lave</t>
         </is>
       </c>
       <c r="C19" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="26" t="inlineStr">
+      <c r="D19" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
@@ -3596,73 +4047,73 @@
       <c r="F19" s="17" t="inlineStr"/>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Magma Hammer</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
+          <t>Deal 28 damage. Apply 4 Burning.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>Pickaxe Jab</t>
-        </is>
-      </c>
-      <c r="B20" s="25" t="inlineStr">
-        <is>
-          <t>coup-de-pioche</t>
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>Lumen Jab</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>coup-de-lumiere</t>
         </is>
       </c>
       <c r="C20" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="26" t="inlineStr">
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F20" s="17" t="inlineStr"/>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>Miner's Pick</t>
+          <t>Crusader Gauntlets</t>
         </is>
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
+          <t>Deal 8 damage. Apply 1 Confusion.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>Poison Dance</t>
-        </is>
-      </c>
-      <c r="B21" s="25" t="inlineStr">
-        <is>
-          <t>danse-empoisonnee</t>
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>Onyx Breath</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>souffle-onyx</t>
         </is>
       </c>
       <c r="C21" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="D21" s="26" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E21" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -3672,282 +4123,290 @@
       </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
-          <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
+          <t>Apply 20 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="inlineStr">
-        <is>
-          <t>Pommel Strike</t>
-        </is>
-      </c>
-      <c r="B22" s="25" t="inlineStr">
-        <is>
-          <t>coup-de-pommeau</t>
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>Onyx Fist</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>poing-onyx</t>
         </is>
       </c>
       <c r="C22" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="26" t="inlineStr">
+      <c r="D22" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E22" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr"/>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>Deal 16 damage. Stun the target for 2 turns.</t>
+          <t>Gain 10 Stone. Deal 10 damage and apply 3 Burning.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="24" t="inlineStr">
-        <is>
-          <t>Punch</t>
-        </is>
-      </c>
-      <c r="B23" s="25" t="inlineStr">
-        <is>
-          <t>coup-faible</t>
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>Onyx Radiance</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>onyx-radiance</t>
         </is>
       </c>
       <c r="C23" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="26" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E23" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F23" s="17" t="inlineStr"/>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage.</t>
+          <t>Apply 8 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="24" t="inlineStr">
-        <is>
-          <t>Rusty Cleave</t>
-        </is>
-      </c>
-      <c r="B24" s="25" t="inlineStr">
-        <is>
-          <t>coup-de-hache</t>
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>Onyx Slash</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>onyx-slash</t>
         </is>
       </c>
       <c r="C24" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D24" s="26" t="inlineStr">
+      <c r="D24" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr"/>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>Rusty Axe</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H24" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
+          <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="24" t="inlineStr">
-        <is>
-          <t>Shield Bash</t>
-        </is>
-      </c>
-      <c r="B25" s="25" t="inlineStr">
-        <is>
-          <t>coup-de-bouclier</t>
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>Pickaxe Jab</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>coup-de-pioche</t>
         </is>
       </c>
       <c r="C25" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D25" s="26" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E25" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr"/>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>Miner's Pick</t>
         </is>
       </c>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>Deal 10 damage. Stun the enemy for 3 turns.</t>
+          <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="24" t="inlineStr">
-        <is>
-          <t>Splash Strike</t>
-        </is>
-      </c>
-      <c r="B26" s="25" t="inlineStr">
-        <is>
-          <t>eclaboussure-de-frappe</t>
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>Poison Dance</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>danse-empoisonnee</t>
         </is>
       </c>
       <c r="C26" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="D26" s="26" t="inlineStr">
+      <c r="D26" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="F26" s="17" t="inlineStr"/>
+      <c r="E26" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G26" s="18" t="inlineStr">
         <is>
-          <t>Forge Hammer</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H26" s="18" t="inlineStr">
         <is>
-          <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
+          <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>Strike</t>
-        </is>
-      </c>
-      <c r="B27" s="25" t="inlineStr">
-        <is>
-          <t>frappe</t>
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>Pommel Strike</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>coup-de-pommeau</t>
         </is>
       </c>
       <c r="C27" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="26" t="inlineStr">
+      <c r="D27" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E27" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr"/>
       <c r="G27" s="18" t="inlineStr">
         <is>
-          <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage.</t>
+          <t>Deal 16 damage. Stun the target for 2 turns.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="24" t="inlineStr">
-        <is>
-          <t>Venom Stab</t>
-        </is>
-      </c>
-      <c r="B28" s="25" t="inlineStr">
-        <is>
-          <t>coup-venimeux</t>
+      <c r="A28" s="25" t="inlineStr">
+        <is>
+          <t>Punch</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>coup-faible</t>
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="26" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E28" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E28" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr"/>
       <c r="G28" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H28" s="18" t="inlineStr">
         <is>
-          <t>Deal 4 damage. Apply 4 Poison.</t>
+          <t>Deal 3 damage.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="24" t="inlineStr">
-        <is>
-          <t>Wound Opening</t>
-        </is>
-      </c>
-      <c r="B29" s="25" t="inlineStr">
-        <is>
-          <t>ouverture-des-plaies</t>
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>Radiant Strike</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="inlineStr">
+        <is>
+          <t>frappe-radiante</t>
         </is>
       </c>
       <c r="C29" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D29" s="26" t="inlineStr">
+      <c r="D29" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
@@ -3960,140 +4419,140 @@
       <c r="F29" s="17" t="inlineStr"/>
       <c r="G29" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>Crusader Plate</t>
         </is>
       </c>
       <c r="H29" s="18" t="inlineStr">
         <is>
-          <t>Deal 18 damage. Doubled if the target has a negative status.</t>
+          <t>Deal 14 damage. Apply 2 Confusion.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="24" t="inlineStr">
-        <is>
-          <t>Guard</t>
-        </is>
-      </c>
-      <c r="B30" s="25" t="inlineStr">
-        <is>
-          <t>garde</t>
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>Rusty Cleave</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>coup-de-hache</t>
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="28" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E30" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>2</v>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F30" s="17" t="inlineStr"/>
       <c r="G30" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>Rusty Axe</t>
         </is>
       </c>
       <c r="H30" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone.</t>
+          <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="24" t="inlineStr">
-        <is>
-          <t>Hand Guard</t>
-        </is>
-      </c>
-      <c r="B31" s="25" t="inlineStr">
-        <is>
-          <t>garde-faible</t>
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>Shield Bash</t>
+        </is>
+      </c>
+      <c r="B31" s="26" t="inlineStr">
+        <is>
+          <t>coup-de-bouclier</t>
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="28" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E31" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>2</v>
+      </c>
+      <c r="D31" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E31" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F31" s="17" t="inlineStr"/>
       <c r="G31" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H31" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Stone.</t>
+          <t>Deal 10 damage. Stun the enemy for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="24" t="inlineStr">
-        <is>
-          <t>Heavy Armor</t>
-        </is>
-      </c>
-      <c r="B32" s="25" t="inlineStr">
-        <is>
-          <t>armure-lourde</t>
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>Splash Strike</t>
+        </is>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>eclaboussure-de-frappe</t>
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" s="28" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E32" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+        <v>3</v>
+      </c>
+      <c r="D32" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr"/>
       <c r="G32" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>Forge Hammer</t>
         </is>
       </c>
       <c r="H32" s="18" t="inlineStr">
         <is>
-          <t>Gain 20 Stone.</t>
+          <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="24" t="inlineStr">
-        <is>
-          <t>Light Armor</t>
-        </is>
-      </c>
-      <c r="B33" s="25" t="inlineStr">
-        <is>
-          <t>armure-legere</t>
+      <c r="A33" s="25" t="inlineStr">
+        <is>
+          <t>Strike</t>
+        </is>
+      </c>
+      <c r="B33" s="26" t="inlineStr">
+        <is>
+          <t>frappe</t>
         </is>
       </c>
       <c r="C33" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="28" t="inlineStr">
-        <is>
-          <t>Défense</t>
+      <c r="D33" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
         </is>
       </c>
       <c r="E33" s="16" t="inlineStr">
@@ -4104,32 +4563,32 @@
       <c r="F33" s="17" t="inlineStr"/>
       <c r="G33" s="18" t="inlineStr">
         <is>
-          <t>Traveler's Garb</t>
+          <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
         </is>
       </c>
       <c r="H33" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone.</t>
+          <t>Deal 6 damage.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>Mail Armor</t>
-        </is>
-      </c>
-      <c r="B34" s="25" t="inlineStr">
-        <is>
-          <t>mail-armor</t>
+      <c r="A34" s="25" t="inlineStr">
+        <is>
+          <t>Venom Stab</t>
+        </is>
+      </c>
+      <c r="B34" s="26" t="inlineStr">
+        <is>
+          <t>coup-venimeux</t>
         </is>
       </c>
       <c r="C34" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D34" s="28" t="inlineStr">
-        <is>
-          <t>Défense</t>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
         </is>
       </c>
       <c r="E34" s="21" t="inlineStr">
@@ -4140,138 +4599,138 @@
       <c r="F34" s="17" t="inlineStr"/>
       <c r="G34" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H34" s="18" t="inlineStr">
         <is>
-          <t>Gain 7 Stone for every enemy still alive.</t>
+          <t>Deal 4 damage. Apply 4 Poison.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>Onyx Armor</t>
-        </is>
-      </c>
-      <c r="B35" s="25" t="inlineStr">
-        <is>
-          <t>onyx-armor</t>
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>Wound Opening</t>
+        </is>
+      </c>
+      <c r="B35" s="26" t="inlineStr">
+        <is>
+          <t>ouverture-des-plaies</t>
         </is>
       </c>
       <c r="C35" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="28" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E35" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E35" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F35" s="17" t="inlineStr"/>
       <c r="G35" s="18" t="inlineStr">
         <is>
-          <t>Onyx Guard Plate</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H35" s="18" t="inlineStr">
         <is>
-          <t>Gain 30 Stone.</t>
+          <t>Deal 18 damage. Doubled if the target has a negative status.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>Quench</t>
-        </is>
-      </c>
-      <c r="B36" s="25" t="inlineStr">
-        <is>
-          <t>trempe</t>
+      <c r="A36" s="25" t="inlineStr">
+        <is>
+          <t>Guard</t>
+        </is>
+      </c>
+      <c r="B36" s="26" t="inlineStr">
+        <is>
+          <t>garde</t>
         </is>
       </c>
       <c r="C36" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="28" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="D36" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E36" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E36" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr"/>
       <c r="G36" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H36" s="18" t="inlineStr">
         <is>
-          <t>Spend all Forge Heat. Gain 10 Stone per Heat spent.</t>
+          <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="24" t="inlineStr">
-        <is>
-          <t>Shield Wall</t>
-        </is>
-      </c>
-      <c r="B37" s="25" t="inlineStr">
-        <is>
-          <t>mur-bouclier</t>
+      <c r="A37" s="25" t="inlineStr">
+        <is>
+          <t>Hand Guard</t>
+        </is>
+      </c>
+      <c r="B37" s="26" t="inlineStr">
+        <is>
+          <t>garde-faible</t>
         </is>
       </c>
       <c r="C37" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="28" t="inlineStr">
+      <c r="D37" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E37" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E37" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr"/>
       <c r="G37" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>Gain 10 Stone.</t>
+          <t>Gain 3 Stone.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="24" t="inlineStr">
-        <is>
-          <t>Stacking Shield</t>
-        </is>
-      </c>
-      <c r="B38" s="25" t="inlineStr">
-        <is>
-          <t>bouclier-empilant</t>
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>Heavy Armor</t>
+        </is>
+      </c>
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>armure-lourde</t>
         </is>
       </c>
       <c r="C38" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D38" s="28" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="D38" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
@@ -4284,132 +4743,132 @@
       <c r="F38" s="17" t="inlineStr"/>
       <c r="G38" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H38" s="18" t="inlineStr">
         <is>
-          <t>Double your current Stone.</t>
+          <t>Gain 20 Stone.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>Burning Run</t>
-        </is>
-      </c>
-      <c r="B39" s="25" t="inlineStr">
-        <is>
-          <t>course-ardente</t>
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>Light Armor</t>
+        </is>
+      </c>
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>armure-legere</t>
         </is>
       </c>
       <c r="C39" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" s="29" t="inlineStr">
         <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E39" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr"/>
       <c r="G39" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots</t>
+          <t>Traveler's Garb</t>
         </is>
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>Haste for as many turns as your current Forge Heat.</t>
+          <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="24" t="inlineStr">
-        <is>
-          <t>Free Movement</t>
-        </is>
-      </c>
-      <c r="B40" s="25" t="inlineStr">
-        <is>
-          <t>mouvement-degage</t>
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>Mail Armor</t>
+        </is>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>mail-armor</t>
         </is>
       </c>
       <c r="C40" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" s="29" t="inlineStr">
         <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E40" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E40" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F40" s="17" t="inlineStr"/>
       <c r="G40" s="18" t="inlineStr">
         <is>
-          <t>Traveler's Garb</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H40" s="18" t="inlineStr">
         <is>
-          <t>Haste for 5 of your turns.</t>
+          <t>Gain 7 Stone for every enemy still alive.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="24" t="inlineStr">
-        <is>
-          <t>Master's Hand</t>
-        </is>
-      </c>
-      <c r="B41" s="25" t="inlineStr">
-        <is>
-          <t>main-de-maitre</t>
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>Onyx Armor</t>
+        </is>
+      </c>
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>onyx-armor</t>
         </is>
       </c>
       <c r="C41" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" s="29" t="inlineStr">
         <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E41" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E41" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F41" s="17" t="inlineStr"/>
       <c r="G41" s="18" t="inlineStr">
         <is>
-          <t>Miner's Gloves</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H41" s="18" t="inlineStr">
         <is>
-          <t>Draw 2 cards.</t>
+          <t>Gain 30 Stone.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="24" t="inlineStr">
-        <is>
-          <t>Onyx Overheat</t>
-        </is>
-      </c>
-      <c r="B42" s="25" t="inlineStr">
-        <is>
-          <t>onyx-overheat</t>
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>Quench</t>
+        </is>
+      </c>
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>trempe</t>
         </is>
       </c>
       <c r="C42" s="17" t="n">
@@ -4417,71 +4876,71 @@
       </c>
       <c r="D42" s="29" t="inlineStr">
         <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E42" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E42" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F42" s="17" t="inlineStr"/>
       <c r="G42" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H42" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Forge Heat (energy).</t>
+          <t>Spend all Forge Heat. Gain 10 Stone per Heat spent.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="24" t="inlineStr">
-        <is>
-          <t>Perfect Sapphire Surge</t>
-        </is>
-      </c>
-      <c r="B43" s="25" t="inlineStr">
-        <is>
-          <t>surge-saphir-parfait</t>
+      <c r="A43" s="25" t="inlineStr">
+        <is>
+          <t>Sacred Ground</t>
+        </is>
+      </c>
+      <c r="B43" s="26" t="inlineStr">
+        <is>
+          <t>terre-sacree</t>
         </is>
       </c>
       <c r="C43" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D43" s="29" t="inlineStr">
         <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E43" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E43" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F43" s="17" t="inlineStr"/>
       <c r="G43" s="18" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Amulet</t>
+          <t>Crusader Plate</t>
         </is>
       </c>
       <c r="H43" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Forge Heat (energy).</t>
+          <t>Gain 18 Stone.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="24" t="inlineStr">
-        <is>
-          <t>Quicken</t>
-        </is>
-      </c>
-      <c r="B44" s="25" t="inlineStr">
-        <is>
-          <t>celerite-vive</t>
+      <c r="A44" s="25" t="inlineStr">
+        <is>
+          <t>Shield Wall</t>
+        </is>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>mur-bouclier</t>
         </is>
       </c>
       <c r="C44" s="17" t="n">
@@ -4489,7 +4948,7 @@
       </c>
       <c r="D44" s="29" t="inlineStr">
         <is>
-          <t>Buff</t>
+          <t>Défense</t>
         </is>
       </c>
       <c r="E44" s="21" t="inlineStr">
@@ -4500,48 +4959,552 @@
       <c r="F44" s="17" t="inlineStr"/>
       <c r="G44" s="18" t="inlineStr">
         <is>
-          <t>Swift Boots</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H44" s="18" t="inlineStr">
         <is>
-          <t>Haste: +30% attack speed for 3 turns.</t>
+          <t>Gain 10 Stone.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="24" t="inlineStr">
-        <is>
-          <t>Sapphire Surge</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="inlineStr">
-        <is>
-          <t>surge-saphir</t>
+      <c r="A45" s="25" t="inlineStr">
+        <is>
+          <t>Stacking Shield</t>
+        </is>
+      </c>
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>bouclier-empilant</t>
         </is>
       </c>
       <c r="C45" s="17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D45" s="29" t="inlineStr">
         <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E45" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E45" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F45" s="17" t="inlineStr"/>
       <c r="G45" s="18" t="inlineStr">
         <is>
+          <t>Tower Shield</t>
+        </is>
+      </c>
+      <c r="H45" s="18" t="inlineStr">
+        <is>
+          <t>Double your current Stone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="25" t="inlineStr">
+        <is>
+          <t>Boost</t>
+        </is>
+      </c>
+      <c r="B46" s="26" t="inlineStr">
+        <is>
+          <t>boost</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E46" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F46" s="17" t="inlineStr"/>
+      <c r="G46" s="18" t="inlineStr">
+        <is>
+          <t>Onyx Boots, Mail Boots</t>
+        </is>
+      </c>
+      <c r="H46" s="18" t="inlineStr">
+        <is>
+          <t>Gain 3 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>Burning Run</t>
+        </is>
+      </c>
+      <c r="B47" s="26" t="inlineStr">
+        <is>
+          <t>course-ardente</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F47" s="17" t="inlineStr"/>
+      <c r="G47" s="18" t="inlineStr">
+        <is>
+          <t>Onyx Boots</t>
+        </is>
+      </c>
+      <c r="H47" s="18" t="inlineStr">
+        <is>
+          <t>Haste for as many turns as your current Forge Heat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>Crusader's Charge</t>
+        </is>
+      </c>
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>charge-du-croise</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E48" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F48" s="17" t="inlineStr"/>
+      <c r="G48" s="18" t="inlineStr">
+        <is>
+          <t>Crusader Greaves</t>
+        </is>
+      </c>
+      <c r="H48" s="18" t="inlineStr">
+        <is>
+          <t>Haste: +30% attack speed for 3 turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>Fire Boost</t>
+        </is>
+      </c>
+      <c r="B49" s="26" t="inlineStr">
+        <is>
+          <t>boost-feu</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F49" s="17" t="inlineStr"/>
+      <c r="G49" s="18" t="inlineStr">
+        <is>
+          <t>Onyx Boots</t>
+        </is>
+      </c>
+      <c r="H49" s="18" t="inlineStr">
+        <is>
+          <t>Convert 4 of your own Burning into 2 Forge Heat. No effect below 4 Burning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>Forge from Ashes</t>
+        </is>
+      </c>
+      <c r="B50" s="26" t="inlineStr">
+        <is>
+          <t>forge-des-cendres</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F50" s="17" t="inlineStr"/>
+      <c r="G50" s="18" t="inlineStr">
+        <is>
+          <t>Onyx Glove</t>
+        </is>
+      </c>
+      <c r="H50" s="18" t="inlineStr">
+        <is>
+          <t>Discard your hand and draw that many cards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>Free Movement</t>
+        </is>
+      </c>
+      <c r="B51" s="26" t="inlineStr">
+        <is>
+          <t>mouvement-degage</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="inlineStr"/>
+      <c r="G51" s="18" t="inlineStr">
+        <is>
+          <t>Traveler's Garb</t>
+        </is>
+      </c>
+      <c r="H51" s="18" t="inlineStr">
+        <is>
+          <t>Haste for 5 of your turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="25" t="inlineStr">
+        <is>
+          <t>Mail Advantage</t>
+        </is>
+      </c>
+      <c r="B52" s="26" t="inlineStr">
+        <is>
+          <t>avantage-maille</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E52" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr"/>
+      <c r="G52" s="18" t="inlineStr">
+        <is>
+          <t>Mail Glove, Mail Boots</t>
+        </is>
+      </c>
+      <c r="H52" s="18" t="inlineStr">
+        <is>
+          <t>Gain 8 Stone and Haste for 2 turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="25" t="inlineStr">
+        <is>
+          <t>Master's Hand</t>
+        </is>
+      </c>
+      <c r="B53" s="26" t="inlineStr">
+        <is>
+          <t>main-de-maitre</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="inlineStr"/>
+      <c r="G53" s="18" t="inlineStr">
+        <is>
+          <t>Miner's Gloves, Mail Glove</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr">
+        <is>
+          <t>Draw 2 cards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="25" t="inlineStr">
+        <is>
+          <t>Onyx Overheat</t>
+        </is>
+      </c>
+      <c r="B54" s="26" t="inlineStr">
+        <is>
+          <t>onyx-overheat</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E54" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr"/>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>Big Onyx Sword</t>
+        </is>
+      </c>
+      <c r="H54" s="18" t="inlineStr">
+        <is>
+          <t>Gain 5 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>Outnumbered</t>
+        </is>
+      </c>
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>surnombre</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E55" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F55" s="17" t="inlineStr"/>
+      <c r="G55" s="18" t="inlineStr">
+        <is>
+          <t>Mail Glove</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr">
+        <is>
+          <t>Draw 1 card per living enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="25" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Surge</t>
+        </is>
+      </c>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>surge-saphir-parfait</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E56" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F56" s="17" t="inlineStr"/>
+      <c r="G56" s="18" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Amulet</t>
+        </is>
+      </c>
+      <c r="H56" s="18" t="inlineStr">
+        <is>
+          <t>Gain 3 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>Quicken</t>
+        </is>
+      </c>
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>celerite-vive</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F57" s="17" t="inlineStr"/>
+      <c r="G57" s="18" t="inlineStr">
+        <is>
+          <t>Swift Boots, Mail Boots</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr">
+        <is>
+          <t>Haste: +30% attack speed for 3 turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="25" t="inlineStr">
+        <is>
+          <t>Sapphire Surge</t>
+        </is>
+      </c>
+      <c r="B58" s="26" t="inlineStr">
+        <is>
+          <t>surge-saphir</t>
+        </is>
+      </c>
+      <c r="C58" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F58" s="17" t="inlineStr"/>
+      <c r="G58" s="18" t="inlineStr">
+        <is>
           <t>Sapphire Amulet, Nice Sapphire Amulet</t>
         </is>
       </c>
-      <c r="H45" s="18" t="inlineStr">
+      <c r="H58" s="18" t="inlineStr">
         <is>
           <t>Gain 2 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="25" t="inlineStr">
+        <is>
+          <t>Second Wind</t>
+        </is>
+      </c>
+      <c r="B59" s="26" t="inlineStr">
+        <is>
+          <t>second-souffle</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F59" s="17" t="inlineStr"/>
+      <c r="G59" s="18" t="inlineStr">
+        <is>
+          <t>Swift Boots</t>
+        </is>
+      </c>
+      <c r="H59" s="18" t="inlineStr">
+        <is>
+          <t>Trade 5 Haste turns for 3 Forge Heat. No effect below 5 Haste.</t>
         </is>
       </c>
     </row>
@@ -4560,7 +5523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4606,7 +5569,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Onyx Set</t>
         </is>
@@ -4628,16 +5591,48 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="23" t="n"/>
-      <c r="C5" s="23" t="n"/>
-      <c r="D5" s="23" t="n"/>
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>Mail Set</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Forgemaster's Mail  +  Mail Glove  +  Mail Boots</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>En début de combat</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>At the start of combat, gain 10 Stone per enemy faced.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="23" t="n"/>
-      <c r="C6" s="23" t="n"/>
-      <c r="D6" s="23" t="n"/>
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>Crusader Set</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Crusader Plate  +  Crusader Gauntlets  +  Crusader Greaves</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Quand le héros est frappé en mêlée</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>When hit by a melee attack, the attacker is Dazzled (1 Confusion).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="23" t="n"/>
@@ -4662,6 +5657,18 @@
       <c r="B10" s="23" t="n"/>
       <c r="C10" s="23" t="n"/>
       <c r="D10" s="23" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="23" t="n"/>
+      <c r="C11" s="23" t="n"/>
+      <c r="D11" s="23" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="23" t="n"/>
+      <c r="C12" s="23" t="n"/>
+      <c r="D12" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
[technique] Catalogue régénéré : 35 items, 64 cartes, 4 sets
Libellé du déclencheur "saignementCombo" ajouté pour le set de Sang.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJcbumK5KWRfGozDrLY2Kn
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -897,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1706,7 +1706,7 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>Armures   (4)</t>
+          <t>Armures   (5)</t>
         </is>
       </c>
     </row>
@@ -1915,20 +1915,56 @@
       <c r="N40" s="18" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="n"/>
-      <c r="B41" s="23" t="n"/>
-      <c r="C41" s="23" t="n"/>
-      <c r="D41" s="23" t="n"/>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="23" t="n"/>
-      <c r="G41" s="23" t="n"/>
-      <c r="H41" s="23" t="n"/>
-      <c r="I41" s="23" t="n"/>
-      <c r="J41" s="23" t="n"/>
-      <c r="K41" s="23" t="n"/>
-      <c r="L41" s="23" t="n"/>
-      <c r="M41" s="23" t="n"/>
-      <c r="N41" s="23" t="n"/>
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Blood Plate</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>plate-sang</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E41" s="18" t="inlineStr">
+        <is>
+          <t>Crimson Carve</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" s="18" t="inlineStr">
+        <is>
+          <t>Sanguine Guard</t>
+        </is>
+      </c>
+      <c r="H41" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" s="18" t="inlineStr">
+        <is>
+          <t>Bloodbath</t>
+        </is>
+      </c>
+      <c r="J41" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K41" s="18" t="n"/>
+      <c r="L41" s="18" t="n"/>
+      <c r="M41" s="19" t="inlineStr">
+        <is>
+          <t>Set : Blood Set</t>
+        </is>
+      </c>
+      <c r="N41" s="18" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="23" t="n"/>
@@ -2010,67 +2046,47 @@
       <c r="M46" s="23" t="n"/>
       <c r="N46" s="23" t="n"/>
     </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="23" t="n"/>
+      <c r="B47" s="23" t="n"/>
+      <c r="C47" s="23" t="n"/>
+      <c r="D47" s="23" t="n"/>
+      <c r="E47" s="23" t="n"/>
+      <c r="F47" s="23" t="n"/>
+      <c r="G47" s="23" t="n"/>
+      <c r="H47" s="23" t="n"/>
+      <c r="I47" s="23" t="n"/>
+      <c r="J47" s="23" t="n"/>
+      <c r="K47" s="23" t="n"/>
+      <c r="L47" s="23" t="n"/>
+      <c r="M47" s="23" t="n"/>
+      <c r="N47" s="23" t="n"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>Colliers   (3)</t>
         </is>
       </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
-          <t>Sapphire Amulet</t>
-        </is>
-      </c>
-      <c r="B49" s="15" t="inlineStr">
-        <is>
-          <t>collier-de-saphir</t>
-        </is>
-      </c>
-      <c r="C49" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="D49" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>Sapphire Surge</t>
-        </is>
-      </c>
-      <c r="F49" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" s="18" t="n"/>
-      <c r="H49" s="18" t="n"/>
-      <c r="I49" s="18" t="n"/>
-      <c r="J49" s="18" t="n"/>
-      <c r="K49" s="18" t="n"/>
-      <c r="L49" s="18" t="n"/>
-      <c r="M49" s="19" t="inlineStr"/>
-      <c r="N49" s="18" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>Nice Sapphire Amulet</t>
+          <t>Sapphire Amulet</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>collier-de-saphir-fin</t>
-        </is>
-      </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+          <t>collier-de-saphir</t>
+        </is>
+      </c>
+      <c r="C50" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="D50" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" s="18" t="inlineStr">
         <is>
@@ -2078,7 +2094,7 @@
         </is>
       </c>
       <c r="F50" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G50" s="18" t="n"/>
       <c r="H50" s="18" t="n"/>
@@ -2092,29 +2108,29 @@
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Amulet</t>
+          <t>Nice Sapphire Amulet</t>
         </is>
       </c>
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>collier-de-saphir-parfait</t>
-        </is>
-      </c>
-      <c r="C51" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+          <t>collier-de-saphir-fin</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D51" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E51" s="18" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Surge</t>
+          <t>Sapphire Surge</t>
         </is>
       </c>
       <c r="F51" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G51" s="18" t="n"/>
       <c r="H51" s="18" t="n"/>
@@ -2126,20 +2142,40 @@
       <c r="N51" s="18" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="23" t="n"/>
-      <c r="B52" s="23" t="n"/>
-      <c r="C52" s="23" t="n"/>
-      <c r="D52" s="23" t="n"/>
-      <c r="E52" s="23" t="n"/>
-      <c r="F52" s="23" t="n"/>
-      <c r="G52" s="23" t="n"/>
-      <c r="H52" s="23" t="n"/>
-      <c r="I52" s="23" t="n"/>
-      <c r="J52" s="23" t="n"/>
-      <c r="K52" s="23" t="n"/>
-      <c r="L52" s="23" t="n"/>
-      <c r="M52" s="23" t="n"/>
-      <c r="N52" s="23" t="n"/>
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Amulet</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>collier-de-saphir-parfait</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Surge</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" s="18" t="n"/>
+      <c r="H52" s="18" t="n"/>
+      <c r="I52" s="18" t="n"/>
+      <c r="J52" s="18" t="n"/>
+      <c r="K52" s="18" t="n"/>
+      <c r="L52" s="18" t="n"/>
+      <c r="M52" s="19" t="inlineStr"/>
+      <c r="N52" s="18" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="23" t="n"/>
@@ -2221,58 +2257,38 @@
       <c r="M57" s="23" t="n"/>
       <c r="N57" s="23" t="n"/>
     </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="13" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="23" t="n"/>
+      <c r="B58" s="23" t="n"/>
+      <c r="C58" s="23" t="n"/>
+      <c r="D58" s="23" t="n"/>
+      <c r="E58" s="23" t="n"/>
+      <c r="F58" s="23" t="n"/>
+      <c r="G58" s="23" t="n"/>
+      <c r="H58" s="23" t="n"/>
+      <c r="I58" s="23" t="n"/>
+      <c r="J58" s="23" t="n"/>
+      <c r="K58" s="23" t="n"/>
+      <c r="L58" s="23" t="n"/>
+      <c r="M58" s="23" t="n"/>
+      <c r="N58" s="23" t="n"/>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>Bagues   (3)</t>
         </is>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="14" t="inlineStr">
-        <is>
-          <t>Blood Ring</t>
-        </is>
-      </c>
-      <c r="B60" s="15" t="inlineStr">
-        <is>
-          <t>bague-de-sang</t>
-        </is>
-      </c>
-      <c r="C60" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="D60" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>Bloodletting</t>
-        </is>
-      </c>
-      <c r="F60" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G60" s="18" t="n"/>
-      <c r="H60" s="18" t="n"/>
-      <c r="I60" s="18" t="n"/>
-      <c r="J60" s="18" t="n"/>
-      <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
-      <c r="M60" s="19" t="inlineStr"/>
-      <c r="N60" s="18" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
         <is>
-          <t>Frost Ring</t>
+          <t>Blood Ring</t>
         </is>
       </c>
       <c r="B61" s="15" t="inlineStr">
         <is>
-          <t>anneau-de-givre</t>
+          <t>bague-de-sang</t>
         </is>
       </c>
       <c r="C61" s="20" t="inlineStr">
@@ -2285,7 +2301,7 @@
       </c>
       <c r="E61" s="18" t="inlineStr">
         <is>
-          <t>Frostbite</t>
+          <t>Bloodletting</t>
         </is>
       </c>
       <c r="F61" s="17" t="n">
@@ -2303,17 +2319,17 @@
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>Perfect Frost Ring</t>
+          <t>Frost Ring</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>anneau-de-givre-parfait</t>
-        </is>
-      </c>
-      <c r="C62" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+          <t>anneau-de-givre</t>
+        </is>
+      </c>
+      <c r="C62" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="D62" s="17" t="n">
@@ -2321,7 +2337,7 @@
       </c>
       <c r="E62" s="18" t="inlineStr">
         <is>
-          <t>Frost Cascade</t>
+          <t>Frostbite</t>
         </is>
       </c>
       <c r="F62" s="17" t="n">
@@ -2337,20 +2353,40 @@
       <c r="N62" s="18" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="23" t="n"/>
-      <c r="B63" s="23" t="n"/>
-      <c r="C63" s="23" t="n"/>
-      <c r="D63" s="23" t="n"/>
-      <c r="E63" s="23" t="n"/>
-      <c r="F63" s="23" t="n"/>
-      <c r="G63" s="23" t="n"/>
-      <c r="H63" s="23" t="n"/>
-      <c r="I63" s="23" t="n"/>
-      <c r="J63" s="23" t="n"/>
-      <c r="K63" s="23" t="n"/>
-      <c r="L63" s="23" t="n"/>
-      <c r="M63" s="23" t="n"/>
-      <c r="N63" s="23" t="n"/>
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>Perfect Frost Ring</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>anneau-de-givre-parfait</t>
+        </is>
+      </c>
+      <c r="C63" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Frost Cascade</t>
+        </is>
+      </c>
+      <c r="F63" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G63" s="18" t="n"/>
+      <c r="H63" s="18" t="n"/>
+      <c r="I63" s="18" t="n"/>
+      <c r="J63" s="18" t="n"/>
+      <c r="K63" s="18" t="n"/>
+      <c r="L63" s="18" t="n"/>
+      <c r="M63" s="19" t="inlineStr"/>
+      <c r="N63" s="18" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="23" t="n"/>
@@ -2432,123 +2468,87 @@
       <c r="M68" s="23" t="n"/>
       <c r="N68" s="23" t="n"/>
     </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="13" t="inlineStr">
-        <is>
-          <t>Gants   (4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="14" t="inlineStr">
-        <is>
-          <t>Miner's Gloves</t>
-        </is>
-      </c>
-      <c r="B71" s="15" t="inlineStr">
-        <is>
-          <t>gants-de-mineur</t>
-        </is>
-      </c>
-      <c r="C71" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="D71" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="E71" s="18" t="inlineStr">
-        <is>
-          <t>Master's Hand</t>
-        </is>
-      </c>
-      <c r="F71" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G71" s="18" t="n"/>
-      <c r="H71" s="18" t="n"/>
-      <c r="I71" s="18" t="n"/>
-      <c r="J71" s="18" t="n"/>
-      <c r="K71" s="18" t="n"/>
-      <c r="L71" s="18" t="n"/>
-      <c r="M71" s="19" t="inlineStr"/>
-      <c r="N71" s="18" t="n"/>
+    <row r="69">
+      <c r="A69" s="23" t="n"/>
+      <c r="B69" s="23" t="n"/>
+      <c r="C69" s="23" t="n"/>
+      <c r="D69" s="23" t="n"/>
+      <c r="E69" s="23" t="n"/>
+      <c r="F69" s="23" t="n"/>
+      <c r="G69" s="23" t="n"/>
+      <c r="H69" s="23" t="n"/>
+      <c r="I69" s="23" t="n"/>
+      <c r="J69" s="23" t="n"/>
+      <c r="K69" s="23" t="n"/>
+      <c r="L69" s="23" t="n"/>
+      <c r="M69" s="23" t="n"/>
+      <c r="N69" s="23" t="n"/>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>Gants   (5)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Miner's Gloves</t>
         </is>
       </c>
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>gants-onyx</t>
-        </is>
-      </c>
-      <c r="C72" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+          <t>gants-de-mineur</t>
+        </is>
+      </c>
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="D72" s="17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E72" s="18" t="inlineStr">
         <is>
-          <t>Burning Hand</t>
+          <t>Master's Hand</t>
         </is>
       </c>
       <c r="F72" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G72" s="18" t="inlineStr">
-        <is>
-          <t>Onyx Fist</t>
-        </is>
-      </c>
-      <c r="H72" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="I72" s="18" t="inlineStr">
-        <is>
-          <t>Forge from Ashes</t>
-        </is>
-      </c>
-      <c r="J72" s="17" t="n">
-        <v>2</v>
-      </c>
+      <c r="G72" s="18" t="n"/>
+      <c r="H72" s="18" t="n"/>
+      <c r="I72" s="18" t="n"/>
+      <c r="J72" s="18" t="n"/>
       <c r="K72" s="18" t="n"/>
       <c r="L72" s="18" t="n"/>
-      <c r="M72" s="19" t="inlineStr">
-        <is>
-          <t>Set : Onyx Set</t>
-        </is>
-      </c>
+      <c r="M72" s="19" t="inlineStr"/>
       <c r="N72" s="18" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
         <is>
-          <t>Mail Glove</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="B73" s="15" t="inlineStr">
         <is>
-          <t>gants-de-maille</t>
-        </is>
-      </c>
-      <c r="C73" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+          <t>gants-onyx</t>
+        </is>
+      </c>
+      <c r="C73" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="D73" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E73" s="18" t="inlineStr">
         <is>
-          <t>Master's Hand</t>
+          <t>Burning Hand</t>
         </is>
       </c>
       <c r="F73" s="17" t="n">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="G73" s="18" t="inlineStr">
         <is>
-          <t>Outnumbered</t>
+          <t>Onyx Fist</t>
         </is>
       </c>
       <c r="H73" s="17" t="n">
@@ -2564,17 +2564,17 @@
       </c>
       <c r="I73" s="18" t="inlineStr">
         <is>
-          <t>Mail Advantage</t>
+          <t>Forge from Ashes</t>
         </is>
       </c>
       <c r="J73" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" s="18" t="n"/>
       <c r="L73" s="18" t="n"/>
       <c r="M73" s="19" t="inlineStr">
         <is>
-          <t>Set : Mail Set</t>
+          <t>Set : Onyx Set</t>
         </is>
       </c>
       <c r="N73" s="18" t="n"/>
@@ -2582,12 +2582,12 @@
     <row r="74">
       <c r="A74" s="14" t="inlineStr">
         <is>
-          <t>Crusader Gauntlets</t>
+          <t>Mail Glove</t>
         </is>
       </c>
       <c r="B74" s="15" t="inlineStr">
         <is>
-          <t>gants-croise</t>
+          <t>gants-de-maille</t>
         </is>
       </c>
       <c r="C74" s="21" t="inlineStr">
@@ -2596,11 +2596,11 @@
         </is>
       </c>
       <c r="D74" s="17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E74" s="18" t="inlineStr">
         <is>
-          <t>Lumen Jab</t>
+          <t>Master's Hand</t>
         </is>
       </c>
       <c r="F74" s="17" t="n">
@@ -2608,54 +2608,120 @@
       </c>
       <c r="G74" s="18" t="inlineStr">
         <is>
-          <t>Halo Burst</t>
+          <t>Outnumbered</t>
         </is>
       </c>
       <c r="H74" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I74" s="18" t="inlineStr">
+        <is>
+          <t>Mail Advantage</t>
+        </is>
+      </c>
+      <c r="J74" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I74" s="18" t="n"/>
-      <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
       <c r="L74" s="18" t="n"/>
       <c r="M74" s="19" t="inlineStr">
         <is>
+          <t>Set : Mail Set</t>
+        </is>
+      </c>
+      <c r="N74" s="18" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>Crusader Gauntlets</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>gants-croise</t>
+        </is>
+      </c>
+      <c r="C75" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D75" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E75" s="18" t="inlineStr">
+        <is>
+          <t>Lumen Jab</t>
+        </is>
+      </c>
+      <c r="F75" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G75" s="18" t="inlineStr">
+        <is>
+          <t>Halo Burst</t>
+        </is>
+      </c>
+      <c r="H75" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I75" s="18" t="n"/>
+      <c r="J75" s="18" t="n"/>
+      <c r="K75" s="18" t="n"/>
+      <c r="L75" s="18" t="n"/>
+      <c r="M75" s="19" t="inlineStr">
+        <is>
           <t>Set : Crusader Set</t>
         </is>
       </c>
-      <c r="N74" s="18" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="23" t="n"/>
-      <c r="B75" s="23" t="n"/>
-      <c r="C75" s="23" t="n"/>
-      <c r="D75" s="23" t="n"/>
-      <c r="E75" s="23" t="n"/>
-      <c r="F75" s="23" t="n"/>
-      <c r="G75" s="23" t="n"/>
-      <c r="H75" s="23" t="n"/>
-      <c r="I75" s="23" t="n"/>
-      <c r="J75" s="23" t="n"/>
-      <c r="K75" s="23" t="n"/>
-      <c r="L75" s="23" t="n"/>
-      <c r="M75" s="23" t="n"/>
-      <c r="N75" s="23" t="n"/>
+      <c r="N75" s="18" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="23" t="n"/>
-      <c r="B76" s="23" t="n"/>
-      <c r="C76" s="23" t="n"/>
-      <c r="D76" s="23" t="n"/>
-      <c r="E76" s="23" t="n"/>
-      <c r="F76" s="23" t="n"/>
-      <c r="G76" s="23" t="n"/>
-      <c r="H76" s="23" t="n"/>
-      <c r="I76" s="23" t="n"/>
-      <c r="J76" s="23" t="n"/>
-      <c r="K76" s="23" t="n"/>
-      <c r="L76" s="23" t="n"/>
-      <c r="M76" s="23" t="n"/>
-      <c r="N76" s="23" t="n"/>
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>Blood Gauntlets</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>gants-sang</t>
+        </is>
+      </c>
+      <c r="C76" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D76" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E76" s="18" t="inlineStr">
+        <is>
+          <t>Open Veins</t>
+        </is>
+      </c>
+      <c r="F76" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G76" s="18" t="inlineStr">
+        <is>
+          <t>Contagion</t>
+        </is>
+      </c>
+      <c r="H76" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I76" s="18" t="n"/>
+      <c r="J76" s="18" t="n"/>
+      <c r="K76" s="18" t="n"/>
+      <c r="L76" s="18" t="n"/>
+      <c r="M76" s="19" t="inlineStr">
+        <is>
+          <t>Set : Blood Set</t>
+        </is>
+      </c>
+      <c r="N76" s="18" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="23" t="n"/>
@@ -2721,131 +2787,63 @@
       <c r="M80" s="23" t="n"/>
       <c r="N80" s="23" t="n"/>
     </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="13" t="inlineStr">
-        <is>
-          <t>Bottes   (4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="14" t="inlineStr">
-        <is>
-          <t>Swift Boots</t>
-        </is>
-      </c>
-      <c r="B83" s="15" t="inlineStr">
-        <is>
-          <t>bottes-vives</t>
-        </is>
-      </c>
-      <c r="C83" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="D83" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="E83" s="18" t="inlineStr">
-        <is>
-          <t>Quicken</t>
-        </is>
-      </c>
-      <c r="F83" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="G83" s="18" t="inlineStr">
-        <is>
-          <t>Second Wind</t>
-        </is>
-      </c>
-      <c r="H83" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I83" s="18" t="n"/>
-      <c r="J83" s="18" t="n"/>
-      <c r="K83" s="18" t="n"/>
-      <c r="L83" s="18" t="n"/>
-      <c r="M83" s="19" t="inlineStr"/>
-      <c r="N83" s="18" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="14" t="inlineStr">
-        <is>
-          <t>Onyx Boots</t>
-        </is>
-      </c>
-      <c r="B84" s="15" t="inlineStr">
-        <is>
-          <t>bottes-onyx</t>
-        </is>
-      </c>
-      <c r="C84" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="D84" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="E84" s="18" t="inlineStr">
-        <is>
-          <t>Burning Run</t>
-        </is>
-      </c>
-      <c r="F84" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G84" s="18" t="inlineStr">
-        <is>
-          <t>Flaming Kick</t>
-        </is>
-      </c>
-      <c r="H84" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I84" s="18" t="inlineStr">
-        <is>
-          <t>Fire Boost</t>
-        </is>
-      </c>
-      <c r="J84" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="K84" s="18" t="inlineStr">
-        <is>
-          <t>Boost</t>
-        </is>
-      </c>
-      <c r="L84" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="M84" s="19" t="inlineStr">
-        <is>
-          <t>Set : Onyx Set</t>
-        </is>
-      </c>
-      <c r="N84" s="18" t="n"/>
+    <row r="81">
+      <c r="A81" s="23" t="n"/>
+      <c r="B81" s="23" t="n"/>
+      <c r="C81" s="23" t="n"/>
+      <c r="D81" s="23" t="n"/>
+      <c r="E81" s="23" t="n"/>
+      <c r="F81" s="23" t="n"/>
+      <c r="G81" s="23" t="n"/>
+      <c r="H81" s="23" t="n"/>
+      <c r="I81" s="23" t="n"/>
+      <c r="J81" s="23" t="n"/>
+      <c r="K81" s="23" t="n"/>
+      <c r="L81" s="23" t="n"/>
+      <c r="M81" s="23" t="n"/>
+      <c r="N81" s="23" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="23" t="n"/>
+      <c r="B82" s="23" t="n"/>
+      <c r="C82" s="23" t="n"/>
+      <c r="D82" s="23" t="n"/>
+      <c r="E82" s="23" t="n"/>
+      <c r="F82" s="23" t="n"/>
+      <c r="G82" s="23" t="n"/>
+      <c r="H82" s="23" t="n"/>
+      <c r="I82" s="23" t="n"/>
+      <c r="J82" s="23" t="n"/>
+      <c r="K82" s="23" t="n"/>
+      <c r="L82" s="23" t="n"/>
+      <c r="M82" s="23" t="n"/>
+      <c r="N82" s="23" t="n"/>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>Bottes   (5)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>Mail Boots</t>
+          <t>Swift Boots</t>
         </is>
       </c>
       <c r="B85" s="15" t="inlineStr">
         <is>
-          <t>bottes-de-maille</t>
-        </is>
-      </c>
-      <c r="C85" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+          <t>bottes-vives</t>
+        </is>
+      </c>
+      <c r="C85" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="D85" s="17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E85" s="18" t="inlineStr">
         <is>
@@ -2853,55 +2851,45 @@
         </is>
       </c>
       <c r="F85" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G85" s="18" t="inlineStr">
         <is>
-          <t>Mail Advantage</t>
+          <t>Second Wind</t>
         </is>
       </c>
       <c r="H85" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I85" s="18" t="inlineStr">
-        <is>
-          <t>Boost</t>
-        </is>
-      </c>
-      <c r="J85" s="17" t="n">
-        <v>2</v>
-      </c>
+      <c r="I85" s="18" t="n"/>
+      <c r="J85" s="18" t="n"/>
       <c r="K85" s="18" t="n"/>
       <c r="L85" s="18" t="n"/>
-      <c r="M85" s="19" t="inlineStr">
-        <is>
-          <t>Set : Mail Set</t>
-        </is>
-      </c>
+      <c r="M85" s="19" t="inlineStr"/>
       <c r="N85" s="18" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>Crusader Greaves</t>
+          <t>Onyx Boots</t>
         </is>
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>bottes-croise</t>
-        </is>
-      </c>
-      <c r="C86" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+          <t>bottes-onyx</t>
+        </is>
+      </c>
+      <c r="C86" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="D86" s="17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E86" s="18" t="inlineStr">
         <is>
-          <t>Crusader's Charge</t>
+          <t>Burning Run</t>
         </is>
       </c>
       <c r="F86" s="17" t="n">
@@ -2909,70 +2897,178 @@
       </c>
       <c r="G86" s="18" t="inlineStr">
         <is>
+          <t>Flaming Kick</t>
+        </is>
+      </c>
+      <c r="H86" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I86" s="18" t="inlineStr">
+        <is>
+          <t>Fire Boost</t>
+        </is>
+      </c>
+      <c r="J86" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K86" s="18" t="inlineStr">
+        <is>
+          <t>Boost</t>
+        </is>
+      </c>
+      <c r="L86" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M86" s="19" t="inlineStr">
+        <is>
+          <t>Set : Onyx Set</t>
+        </is>
+      </c>
+      <c r="N86" s="18" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>Mail Boots</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="inlineStr">
+        <is>
+          <t>bottes-de-maille</t>
+        </is>
+      </c>
+      <c r="C87" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D87" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Quicken</t>
+        </is>
+      </c>
+      <c r="F87" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G87" s="18" t="inlineStr">
+        <is>
+          <t>Mail Advantage</t>
+        </is>
+      </c>
+      <c r="H87" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I87" s="18" t="inlineStr">
+        <is>
+          <t>Boost</t>
+        </is>
+      </c>
+      <c r="J87" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K87" s="18" t="n"/>
+      <c r="L87" s="18" t="n"/>
+      <c r="M87" s="19" t="inlineStr">
+        <is>
+          <t>Set : Mail Set</t>
+        </is>
+      </c>
+      <c r="N87" s="18" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>Crusader Greaves</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>bottes-croise</t>
+        </is>
+      </c>
+      <c r="C88" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D88" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Crusader's Charge</t>
+        </is>
+      </c>
+      <c r="F88" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="18" t="inlineStr">
+        <is>
           <t>Dazzling Kick</t>
         </is>
       </c>
-      <c r="H86" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="I86" s="18" t="n"/>
-      <c r="J86" s="18" t="n"/>
-      <c r="K86" s="18" t="n"/>
-      <c r="L86" s="18" t="n"/>
-      <c r="M86" s="19" t="inlineStr">
+      <c r="H88" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I88" s="18" t="n"/>
+      <c r="J88" s="18" t="n"/>
+      <c r="K88" s="18" t="n"/>
+      <c r="L88" s="18" t="n"/>
+      <c r="M88" s="19" t="inlineStr">
         <is>
           <t>Set : Crusader Set</t>
         </is>
       </c>
-      <c r="N86" s="18" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="23" t="n"/>
-      <c r="B87" s="23" t="n"/>
-      <c r="C87" s="23" t="n"/>
-      <c r="D87" s="23" t="n"/>
-      <c r="E87" s="23" t="n"/>
-      <c r="F87" s="23" t="n"/>
-      <c r="G87" s="23" t="n"/>
-      <c r="H87" s="23" t="n"/>
-      <c r="I87" s="23" t="n"/>
-      <c r="J87" s="23" t="n"/>
-      <c r="K87" s="23" t="n"/>
-      <c r="L87" s="23" t="n"/>
-      <c r="M87" s="23" t="n"/>
-      <c r="N87" s="23" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="23" t="n"/>
-      <c r="B88" s="23" t="n"/>
-      <c r="C88" s="23" t="n"/>
-      <c r="D88" s="23" t="n"/>
-      <c r="E88" s="23" t="n"/>
-      <c r="F88" s="23" t="n"/>
-      <c r="G88" s="23" t="n"/>
-      <c r="H88" s="23" t="n"/>
-      <c r="I88" s="23" t="n"/>
-      <c r="J88" s="23" t="n"/>
-      <c r="K88" s="23" t="n"/>
-      <c r="L88" s="23" t="n"/>
-      <c r="M88" s="23" t="n"/>
-      <c r="N88" s="23" t="n"/>
+      <c r="N88" s="18" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="23" t="n"/>
-      <c r="B89" s="23" t="n"/>
-      <c r="C89" s="23" t="n"/>
-      <c r="D89" s="23" t="n"/>
-      <c r="E89" s="23" t="n"/>
-      <c r="F89" s="23" t="n"/>
-      <c r="G89" s="23" t="n"/>
-      <c r="H89" s="23" t="n"/>
-      <c r="I89" s="23" t="n"/>
-      <c r="J89" s="23" t="n"/>
-      <c r="K89" s="23" t="n"/>
-      <c r="L89" s="23" t="n"/>
-      <c r="M89" s="23" t="n"/>
-      <c r="N89" s="23" t="n"/>
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>Blood Greaves</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>bottes-sang</t>
+        </is>
+      </c>
+      <c r="C89" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D89" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Hemorrhage</t>
+        </is>
+      </c>
+      <c r="F89" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G89" s="18" t="inlineStr">
+        <is>
+          <t>Blood Rush</t>
+        </is>
+      </c>
+      <c r="H89" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I89" s="18" t="n"/>
+      <c r="J89" s="18" t="n"/>
+      <c r="K89" s="18" t="n"/>
+      <c r="L89" s="18" t="n"/>
+      <c r="M89" s="19" t="inlineStr">
+        <is>
+          <t>Set : Blood Set</t>
+        </is>
+      </c>
+      <c r="N89" s="18" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="23" t="n"/>
@@ -3022,129 +3118,75 @@
       <c r="M92" s="23" t="n"/>
       <c r="N92" s="23" t="n"/>
     </row>
-    <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="13" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="23" t="n"/>
+      <c r="B93" s="23" t="n"/>
+      <c r="C93" s="23" t="n"/>
+      <c r="D93" s="23" t="n"/>
+      <c r="E93" s="23" t="n"/>
+      <c r="F93" s="23" t="n"/>
+      <c r="G93" s="23" t="n"/>
+      <c r="H93" s="23" t="n"/>
+      <c r="I93" s="23" t="n"/>
+      <c r="J93" s="23" t="n"/>
+      <c r="K93" s="23" t="n"/>
+      <c r="L93" s="23" t="n"/>
+      <c r="M93" s="23" t="n"/>
+      <c r="N93" s="23" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="23" t="n"/>
+      <c r="B94" s="23" t="n"/>
+      <c r="C94" s="23" t="n"/>
+      <c r="D94" s="23" t="n"/>
+      <c r="E94" s="23" t="n"/>
+      <c r="F94" s="23" t="n"/>
+      <c r="G94" s="23" t="n"/>
+      <c r="H94" s="23" t="n"/>
+      <c r="I94" s="23" t="n"/>
+      <c r="J94" s="23" t="n"/>
+      <c r="K94" s="23" t="n"/>
+      <c r="L94" s="23" t="n"/>
+      <c r="M94" s="23" t="n"/>
+      <c r="N94" s="23" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="23" t="n"/>
+      <c r="B95" s="23" t="n"/>
+      <c r="C95" s="23" t="n"/>
+      <c r="D95" s="23" t="n"/>
+      <c r="E95" s="23" t="n"/>
+      <c r="F95" s="23" t="n"/>
+      <c r="G95" s="23" t="n"/>
+      <c r="H95" s="23" t="n"/>
+      <c r="I95" s="23" t="n"/>
+      <c r="J95" s="23" t="n"/>
+      <c r="K95" s="23" t="n"/>
+      <c r="L95" s="23" t="n"/>
+      <c r="M95" s="23" t="n"/>
+      <c r="N95" s="23" t="n"/>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="13" t="inlineStr">
         <is>
           <t>Sacs   (6)</t>
         </is>
       </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="14" t="inlineStr">
-        <is>
-          <t>Leather Pouch</t>
-        </is>
-      </c>
-      <c r="B95" s="15" t="inlineStr">
-        <is>
-          <t>sac-en-cuir</t>
-        </is>
-      </c>
-      <c r="C95" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="D95" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E95" s="18" t="n"/>
-      <c r="F95" s="18" t="n"/>
-      <c r="G95" s="18" t="n"/>
-      <c r="H95" s="18" t="n"/>
-      <c r="I95" s="18" t="n"/>
-      <c r="J95" s="18" t="n"/>
-      <c r="K95" s="18" t="n"/>
-      <c r="L95" s="18" t="n"/>
-      <c r="M95" s="19" t="inlineStr">
-        <is>
-          <t>+1 rangées de sac</t>
-        </is>
-      </c>
-      <c r="N95" s="18" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="14" t="inlineStr">
-        <is>
-          <t>Big Leather Pouch</t>
-        </is>
-      </c>
-      <c r="B96" s="15" t="inlineStr">
-        <is>
-          <t>grand-sac-en-cuir</t>
-        </is>
-      </c>
-      <c r="C96" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="D96" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E96" s="18" t="n"/>
-      <c r="F96" s="18" t="n"/>
-      <c r="G96" s="18" t="n"/>
-      <c r="H96" s="18" t="n"/>
-      <c r="I96" s="18" t="n"/>
-      <c r="J96" s="18" t="n"/>
-      <c r="K96" s="18" t="n"/>
-      <c r="L96" s="18" t="n"/>
-      <c r="M96" s="19" t="inlineStr">
-        <is>
-          <t>+2 rangées de sac</t>
-        </is>
-      </c>
-      <c r="N96" s="18" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="14" t="inlineStr">
-        <is>
-          <t>Huge Leather Pouch</t>
-        </is>
-      </c>
-      <c r="B97" s="15" t="inlineStr">
-        <is>
-          <t>enorme-sac-en-cuir</t>
-        </is>
-      </c>
-      <c r="C97" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="D97" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E97" s="18" t="n"/>
-      <c r="F97" s="18" t="n"/>
-      <c r="G97" s="18" t="n"/>
-      <c r="H97" s="18" t="n"/>
-      <c r="I97" s="18" t="n"/>
-      <c r="J97" s="18" t="n"/>
-      <c r="K97" s="18" t="n"/>
-      <c r="L97" s="18" t="n"/>
-      <c r="M97" s="19" t="inlineStr">
-        <is>
-          <t>+3 rangées de sac</t>
-        </is>
-      </c>
-      <c r="N97" s="18" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>Backpack</t>
+          <t>Leather Pouch</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
         <is>
-          <t>sac-a-dos</t>
-        </is>
-      </c>
-      <c r="C98" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+          <t>sac-en-cuir</t>
+        </is>
+      </c>
+      <c r="C98" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="D98" s="17" t="n">
@@ -3160,7 +3202,7 @@
       <c r="L98" s="18" t="n"/>
       <c r="M98" s="19" t="inlineStr">
         <is>
-          <t>+4 rangées de sac</t>
+          <t>+1 rangées de sac</t>
         </is>
       </c>
       <c r="N98" s="18" t="n"/>
@@ -3168,17 +3210,17 @@
     <row r="99">
       <c r="A99" s="14" t="inlineStr">
         <is>
-          <t>Bottomless Bag</t>
+          <t>Big Leather Pouch</t>
         </is>
       </c>
       <c r="B99" s="15" t="inlineStr">
         <is>
-          <t>sac-sans-fond</t>
-        </is>
-      </c>
-      <c r="C99" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+          <t>grand-sac-en-cuir</t>
+        </is>
+      </c>
+      <c r="C99" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="D99" s="17" t="n">
@@ -3194,7 +3236,7 @@
       <c r="L99" s="18" t="n"/>
       <c r="M99" s="19" t="inlineStr">
         <is>
-          <t>+6 rangées de sac</t>
+          <t>+2 rangées de sac</t>
         </is>
       </c>
       <c r="N99" s="18" t="n"/>
@@ -3202,17 +3244,17 @@
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>Master Miner's Bag</t>
+          <t>Huge Leather Pouch</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
         <is>
-          <t>sac-maitre-mineur</t>
-        </is>
-      </c>
-      <c r="C100" s="24" t="inlineStr">
-        <is>
-          <t>Legendary</t>
+          <t>enorme-sac-en-cuir</t>
+        </is>
+      </c>
+      <c r="C100" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D100" s="17" t="n">
@@ -3228,58 +3270,112 @@
       <c r="L100" s="18" t="n"/>
       <c r="M100" s="19" t="inlineStr">
         <is>
+          <t>+3 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N100" s="18" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="14" t="inlineStr">
+        <is>
+          <t>Backpack</t>
+        </is>
+      </c>
+      <c r="B101" s="15" t="inlineStr">
+        <is>
+          <t>sac-a-dos</t>
+        </is>
+      </c>
+      <c r="C101" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D101" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="18" t="n"/>
+      <c r="F101" s="18" t="n"/>
+      <c r="G101" s="18" t="n"/>
+      <c r="H101" s="18" t="n"/>
+      <c r="I101" s="18" t="n"/>
+      <c r="J101" s="18" t="n"/>
+      <c r="K101" s="18" t="n"/>
+      <c r="L101" s="18" t="n"/>
+      <c r="M101" s="19" t="inlineStr">
+        <is>
+          <t>+4 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N101" s="18" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="inlineStr">
+        <is>
+          <t>Bottomless Bag</t>
+        </is>
+      </c>
+      <c r="B102" s="15" t="inlineStr">
+        <is>
+          <t>sac-sans-fond</t>
+        </is>
+      </c>
+      <c r="C102" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D102" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="18" t="n"/>
+      <c r="F102" s="18" t="n"/>
+      <c r="G102" s="18" t="n"/>
+      <c r="H102" s="18" t="n"/>
+      <c r="I102" s="18" t="n"/>
+      <c r="J102" s="18" t="n"/>
+      <c r="K102" s="18" t="n"/>
+      <c r="L102" s="18" t="n"/>
+      <c r="M102" s="19" t="inlineStr">
+        <is>
+          <t>+6 rangées de sac</t>
+        </is>
+      </c>
+      <c r="N102" s="18" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="14" t="inlineStr">
+        <is>
+          <t>Master Miner's Bag</t>
+        </is>
+      </c>
+      <c r="B103" s="15" t="inlineStr">
+        <is>
+          <t>sac-maitre-mineur</t>
+        </is>
+      </c>
+      <c r="C103" s="24" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="D103" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" s="18" t="n"/>
+      <c r="F103" s="18" t="n"/>
+      <c r="G103" s="18" t="n"/>
+      <c r="H103" s="18" t="n"/>
+      <c r="I103" s="18" t="n"/>
+      <c r="J103" s="18" t="n"/>
+      <c r="K103" s="18" t="n"/>
+      <c r="L103" s="18" t="n"/>
+      <c r="M103" s="19" t="inlineStr">
+        <is>
           <t>+10 rangées de sac</t>
         </is>
       </c>
-      <c r="N100" s="18" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="23" t="n"/>
-      <c r="B101" s="23" t="n"/>
-      <c r="C101" s="23" t="n"/>
-      <c r="D101" s="23" t="n"/>
-      <c r="E101" s="23" t="n"/>
-      <c r="F101" s="23" t="n"/>
-      <c r="G101" s="23" t="n"/>
-      <c r="H101" s="23" t="n"/>
-      <c r="I101" s="23" t="n"/>
-      <c r="J101" s="23" t="n"/>
-      <c r="K101" s="23" t="n"/>
-      <c r="L101" s="23" t="n"/>
-      <c r="M101" s="23" t="n"/>
-      <c r="N101" s="23" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="23" t="n"/>
-      <c r="B102" s="23" t="n"/>
-      <c r="C102" s="23" t="n"/>
-      <c r="D102" s="23" t="n"/>
-      <c r="E102" s="23" t="n"/>
-      <c r="F102" s="23" t="n"/>
-      <c r="G102" s="23" t="n"/>
-      <c r="H102" s="23" t="n"/>
-      <c r="I102" s="23" t="n"/>
-      <c r="J102" s="23" t="n"/>
-      <c r="K102" s="23" t="n"/>
-      <c r="L102" s="23" t="n"/>
-      <c r="M102" s="23" t="n"/>
-      <c r="N102" s="23" t="n"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="23" t="n"/>
-      <c r="B103" s="23" t="n"/>
-      <c r="C103" s="23" t="n"/>
-      <c r="D103" s="23" t="n"/>
-      <c r="E103" s="23" t="n"/>
-      <c r="F103" s="23" t="n"/>
-      <c r="G103" s="23" t="n"/>
-      <c r="H103" s="23" t="n"/>
-      <c r="I103" s="23" t="n"/>
-      <c r="J103" s="23" t="n"/>
-      <c r="K103" s="23" t="n"/>
-      <c r="L103" s="23" t="n"/>
-      <c r="M103" s="23" t="n"/>
-      <c r="N103" s="23" t="n"/>
+      <c r="N103" s="18" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="23" t="n"/>
@@ -3329,17 +3425,65 @@
       <c r="M106" s="23" t="n"/>
       <c r="N106" s="23" t="n"/>
     </row>
+    <row r="107">
+      <c r="A107" s="23" t="n"/>
+      <c r="B107" s="23" t="n"/>
+      <c r="C107" s="23" t="n"/>
+      <c r="D107" s="23" t="n"/>
+      <c r="E107" s="23" t="n"/>
+      <c r="F107" s="23" t="n"/>
+      <c r="G107" s="23" t="n"/>
+      <c r="H107" s="23" t="n"/>
+      <c r="I107" s="23" t="n"/>
+      <c r="J107" s="23" t="n"/>
+      <c r="K107" s="23" t="n"/>
+      <c r="L107" s="23" t="n"/>
+      <c r="M107" s="23" t="n"/>
+      <c r="N107" s="23" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="23" t="n"/>
+      <c r="B108" s="23" t="n"/>
+      <c r="C108" s="23" t="n"/>
+      <c r="D108" s="23" t="n"/>
+      <c r="E108" s="23" t="n"/>
+      <c r="F108" s="23" t="n"/>
+      <c r="G108" s="23" t="n"/>
+      <c r="H108" s="23" t="n"/>
+      <c r="I108" s="23" t="n"/>
+      <c r="J108" s="23" t="n"/>
+      <c r="K108" s="23" t="n"/>
+      <c r="L108" s="23" t="n"/>
+      <c r="M108" s="23" t="n"/>
+      <c r="N108" s="23" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="23" t="n"/>
+      <c r="B109" s="23" t="n"/>
+      <c r="C109" s="23" t="n"/>
+      <c r="D109" s="23" t="n"/>
+      <c r="E109" s="23" t="n"/>
+      <c r="F109" s="23" t="n"/>
+      <c r="G109" s="23" t="n"/>
+      <c r="H109" s="23" t="n"/>
+      <c r="I109" s="23" t="n"/>
+      <c r="J109" s="23" t="n"/>
+      <c r="K109" s="23" t="n"/>
+      <c r="L109" s="23" t="n"/>
+      <c r="M109" s="23" t="n"/>
+      <c r="N109" s="23" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A17:N17"/>
-    <mergeCell ref="A70:N70"/>
     <mergeCell ref="A27:N27"/>
-    <mergeCell ref="A94:N94"/>
     <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A48:N48"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A59:N59"/>
-    <mergeCell ref="A82:N82"/>
+    <mergeCell ref="A60:N60"/>
+    <mergeCell ref="A97:N97"/>
+    <mergeCell ref="A71:N71"/>
+    <mergeCell ref="A49:N49"/>
+    <mergeCell ref="A84:N84"/>
     <mergeCell ref="A36:N36"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3354,7 +3498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3539,120 +3683,124 @@
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>Bloodletting</t>
+          <t>Bloodbath</t>
         </is>
       </c>
       <c r="B6" s="26" t="inlineStr">
         <is>
-          <t>coup-de-sang</t>
+          <t>bain-de-sang</t>
         </is>
       </c>
       <c r="C6" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D6" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="F6" s="17" t="inlineStr"/>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Blood Ring</t>
+          <t>Blood Plate</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
+          <t>Apply 5 Bleed to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Burning Hand</t>
+          <t>Bloodletting</t>
         </is>
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>main-brulante</t>
+          <t>coup-de-sang</t>
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E7" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr"/>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Blood Ring</t>
         </is>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>Discard your hand. For each card discarded, apply 8 Burning to a random enemy.</t>
+          <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>Cleave</t>
+          <t>Burning Hand</t>
         </is>
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>couper-en-deux</t>
+          <t>main-brulante</t>
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr"/>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>Deal 20 damage. If the target dies, deal 15 damage to the next enemy.</t>
+          <t>Discard your hand. For each card discarded, apply 8 Burning to a random enemy.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>Dazzling Kick</t>
+          <t>Cleave</t>
         </is>
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>coup-eblouissant</t>
+          <t>couper-en-deux</t>
         </is>
       </c>
       <c r="C9" s="17" t="n">
@@ -3671,28 +3819,28 @@
       <c r="F9" s="17" t="inlineStr"/>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>Crusader Greaves</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>Deal 10 damage. Apply 3 Confusion.</t>
+          <t>Deal 20 damage. If the target dies, deal 15 damage to the next enemy.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Dragon's Blaze</t>
+          <t>Contagion</t>
         </is>
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>embrasement-dragon</t>
+          <t>contagion</t>
         </is>
       </c>
       <c r="C10" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
@@ -3704,35 +3852,31 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="F10" s="17" t="inlineStr"/>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer, Onyx Guard Plate</t>
+          <t>Blood Gauntlets</t>
         </is>
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
+          <t>Deal 6 damage. Both adjacent enemies gain Bleed equal to the target's Bleed.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Fire Strike</t>
+          <t>Crimson Carve</t>
         </is>
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>feu-frappe</t>
+          <t>carve-cramoisi</t>
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
@@ -3747,132 +3891,136 @@
       <c r="F11" s="17" t="inlineStr"/>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer</t>
+          <t>Blood Plate</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>Deal 12 damage. Apply 3 Burning.</t>
+          <t>Deal 12 damage. Apply 4 Bleed.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>Flaming Kick</t>
+          <t>Dazzling Kick</t>
         </is>
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>coup-de-pied-ardent</t>
+          <t>coup-eblouissant</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr"/>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots</t>
+          <t>Crusader Greaves</t>
         </is>
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>Move all Burning from the target to the enemy behind it.</t>
+          <t>Deal 10 damage. Apply 3 Confusion.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>Forge Smash</t>
+          <t>Dragon's Blaze</t>
         </is>
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>ecrasement</t>
+          <t>embrasement-dragon</t>
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="F13" s="17" t="inlineStr"/>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>Forge Hammer</t>
+          <t>Magma Hammer, Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>Deal 10 damage. Gain 8 Stone.</t>
+          <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>Frost Cascade</t>
+          <t>Fire Strike</t>
         </is>
       </c>
       <c r="B14" s="26" t="inlineStr">
         <is>
-          <t>gel-cascade</t>
+          <t>feu-frappe</t>
         </is>
       </c>
       <c r="C14" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E14" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr"/>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>Perfect Frost Ring</t>
+          <t>Magma Hammer</t>
         </is>
       </c>
       <c r="H14" s="18" t="inlineStr">
         <is>
-          <t>Deal 8 damage and apply 3 Chill. If the target was already chilled, cascade the same hit to the next enemy, and so on.</t>
+          <t>Deal 12 damage. Apply 3 Burning.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>Frostbite</t>
+          <t>Flaming Kick</t>
         </is>
       </c>
       <c r="B15" s="26" t="inlineStr">
         <is>
-          <t>givre-lent</t>
+          <t>coup-de-pied-ardent</t>
         </is>
       </c>
       <c r="C15" s="17" t="n">
@@ -3883,72 +4031,68 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr"/>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>Frost Ring</t>
+          <t>Onyx Boots</t>
         </is>
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>Deal 5 damage. Chill: -30% speed for 3 turns.</t>
+          <t>Move all Burning from the target to the enemy behind it.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t>Giant Swing</t>
+          <t>Forge Smash</t>
         </is>
       </c>
       <c r="B16" s="26" t="inlineStr">
         <is>
-          <t>giant-swing</t>
+          <t>ecrasement</t>
         </is>
       </c>
       <c r="C16" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E16" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="F16" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr"/>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>Forge Hammer</t>
         </is>
       </c>
       <c r="H16" s="18" t="inlineStr">
         <is>
-          <t>Deal 16 damage to ALL enemies. Apply 2 Bleed to ALL enemies.</t>
+          <t>Deal 10 damage. Gain 8 Stone.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>Halo Burst</t>
+          <t>Frost Cascade</t>
         </is>
       </c>
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>eclat-de-halo</t>
+          <t>gel-cascade</t>
         </is>
       </c>
       <c r="C17" s="17" t="n">
@@ -3964,111 +4108,107 @@
           <t>Rare</t>
         </is>
       </c>
-      <c r="F17" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="F17" s="17" t="inlineStr"/>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Crusader Gauntlets</t>
+          <t>Perfect Frost Ring</t>
         </is>
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage to ALL enemies.</t>
+          <t>Deal 8 damage and apply 3 Chill. If the target was already chilled, cascade the same hit to the next enemy, and so on.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>Heat Rejection</t>
+          <t>Frostbite</t>
         </is>
       </c>
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>rejet-chaleur</t>
+          <t>givre-lent</t>
         </is>
       </c>
       <c r="C18" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="F18" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr"/>
       <c r="G18" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Frost Ring</t>
         </is>
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>Spend all Forge Heat. Apply 8 Burning per Heat spent to ALL enemies.</t>
+          <t>Deal 5 damage. Chill: -30% speed for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>Lava Hammer</t>
+          <t>Giant Swing</t>
         </is>
       </c>
       <c r="B19" s="26" t="inlineStr">
         <is>
-          <t>coup-de-lave</t>
+          <t>giant-swing</t>
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E19" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="F19" s="17" t="inlineStr"/>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>Deal 28 damage. Apply 4 Burning.</t>
+          <t>Deal 16 damage to ALL enemies. Apply 2 Bleed to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>Lumen Jab</t>
+          <t>Halo Burst</t>
         </is>
       </c>
       <c r="B20" s="26" t="inlineStr">
         <is>
-          <t>coup-de-lumiere</t>
+          <t>eclat-de-halo</t>
         </is>
       </c>
       <c r="C20" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
@@ -4080,7 +4220,11 @@
           <t>Rare</t>
         </is>
       </c>
-      <c r="F20" s="17" t="inlineStr"/>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
           <t>Crusader Gauntlets</t>
@@ -4088,23 +4232,23 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Deal 8 damage. Apply 1 Confusion.</t>
+          <t>Deal 6 damage to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>Onyx Breath</t>
+          <t>Heat Rejection</t>
         </is>
       </c>
       <c r="B21" s="26" t="inlineStr">
         <is>
-          <t>souffle-onyx</t>
+          <t>rejet-chaleur</t>
         </is>
       </c>
       <c r="C21" s="17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D21" s="27" t="inlineStr">
         <is>
@@ -4123,28 +4267,28 @@
       </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>Onyx Guard Plate</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
-          <t>Apply 20 Burning to ALL enemies.</t>
+          <t>Spend all Forge Heat. Apply 8 Burning per Heat spent to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>Onyx Fist</t>
+          <t>Hemorrhage</t>
         </is>
       </c>
       <c r="B22" s="26" t="inlineStr">
         <is>
-          <t>poing-onyx</t>
+          <t>hemorragie</t>
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
@@ -4159,28 +4303,28 @@
       <c r="F22" s="17" t="inlineStr"/>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Blood Greaves</t>
         </is>
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>Gain 10 Stone. Deal 10 damage and apply 3 Burning.</t>
+          <t>Consume all the target's Bleed: deal 3 damage per Bleed consumed.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>Onyx Radiance</t>
+          <t>Lava Hammer</t>
         </is>
       </c>
       <c r="B23" s="26" t="inlineStr">
         <is>
-          <t>onyx-radiance</t>
+          <t>coup-de-lave</t>
         </is>
       </c>
       <c r="C23" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="27" t="inlineStr">
         <is>
@@ -4192,143 +4336,139 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="F23" s="17" t="inlineStr"/>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Magma Hammer</t>
         </is>
       </c>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>Apply 8 Burning to ALL enemies.</t>
+          <t>Deal 28 damage. Apply 4 Burning.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>Onyx Slash</t>
+          <t>Lumen Jab</t>
         </is>
       </c>
       <c r="B24" s="26" t="inlineStr">
         <is>
-          <t>onyx-slash</t>
+          <t>coup-de-lumiere</t>
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E24" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr"/>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Crusader Gauntlets</t>
         </is>
       </c>
       <c r="H24" s="18" t="inlineStr">
         <is>
-          <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
+          <t>Deal 8 damage. Apply 1 Confusion.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>Pickaxe Jab</t>
+          <t>Onyx Breath</t>
         </is>
       </c>
       <c r="B25" s="26" t="inlineStr">
         <is>
-          <t>coup-de-pioche</t>
+          <t>souffle-onyx</t>
         </is>
       </c>
       <c r="C25" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="F25" s="17" t="inlineStr"/>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>Miner's Pick</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
+          <t>Apply 20 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>Poison Dance</t>
+          <t>Onyx Fist</t>
         </is>
       </c>
       <c r="B26" s="26" t="inlineStr">
         <is>
-          <t>danse-empoisonnee</t>
+          <t>poing-onyx</t>
         </is>
       </c>
       <c r="C26" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E26" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="F26" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr"/>
       <c r="G26" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="H26" s="18" t="inlineStr">
         <is>
-          <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
+          <t>Gain 10 Stone. Deal 10 damage and apply 3 Burning.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>Pommel Strike</t>
+          <t>Onyx Radiance</t>
         </is>
       </c>
       <c r="B27" s="26" t="inlineStr">
         <is>
-          <t>coup-de-pommeau</t>
+          <t>onyx-radiance</t>
         </is>
       </c>
       <c r="C27" s="17" t="n">
@@ -4339,108 +4479,112 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="F27" s="17" t="inlineStr"/>
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G27" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
-          <t>Deal 16 damage. Stun the target for 2 turns.</t>
+          <t>Apply 8 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="25" t="inlineStr">
         <is>
-          <t>Punch</t>
+          <t>Onyx Slash</t>
         </is>
       </c>
       <c r="B28" s="26" t="inlineStr">
         <is>
-          <t>coup-faible</t>
+          <t>onyx-slash</t>
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E28" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr"/>
       <c r="G28" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H28" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage.</t>
+          <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="25" t="inlineStr">
         <is>
-          <t>Radiant Strike</t>
+          <t>Open Veins</t>
         </is>
       </c>
       <c r="B29" s="26" t="inlineStr">
         <is>
-          <t>frappe-radiante</t>
+          <t>ouvrir-les-veines</t>
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr"/>
       <c r="G29" s="18" t="inlineStr">
         <is>
-          <t>Crusader Plate</t>
+          <t>Blood Gauntlets</t>
         </is>
       </c>
       <c r="H29" s="18" t="inlineStr">
         <is>
-          <t>Deal 14 damage. Apply 2 Confusion.</t>
+          <t>Deal 4 damage. Apply 5 Bleed.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="25" t="inlineStr">
         <is>
-          <t>Rusty Cleave</t>
+          <t>Pickaxe Jab</t>
         </is>
       </c>
       <c r="B30" s="26" t="inlineStr">
         <is>
-          <t>coup-de-hache</t>
+          <t>coup-de-pioche</t>
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
@@ -4455,28 +4599,28 @@
       <c r="F30" s="17" t="inlineStr"/>
       <c r="G30" s="18" t="inlineStr">
         <is>
-          <t>Rusty Axe</t>
+          <t>Miner's Pick</t>
         </is>
       </c>
       <c r="H30" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
+          <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="25" t="inlineStr">
         <is>
-          <t>Shield Bash</t>
+          <t>Poison Dance</t>
         </is>
       </c>
       <c r="B31" s="26" t="inlineStr">
         <is>
-          <t>coup-de-bouclier</t>
+          <t>danse-empoisonnee</t>
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31" s="27" t="inlineStr">
         <is>
@@ -4488,103 +4632,107 @@
           <t>Rare</t>
         </is>
       </c>
-      <c r="F31" s="17" t="inlineStr"/>
+      <c r="F31" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G31" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H31" s="18" t="inlineStr">
         <is>
-          <t>Deal 10 damage. Stun the enemy for 3 turns.</t>
+          <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>Splash Strike</t>
+          <t>Pommel Strike</t>
         </is>
       </c>
       <c r="B32" s="26" t="inlineStr">
         <is>
-          <t>eclaboussure-de-frappe</t>
+          <t>coup-de-pommeau</t>
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E32" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E32" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr"/>
       <c r="G32" s="18" t="inlineStr">
         <is>
-          <t>Forge Hammer</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H32" s="18" t="inlineStr">
         <is>
-          <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
+          <t>Deal 16 damage. Stun the target for 2 turns.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="25" t="inlineStr">
         <is>
-          <t>Strike</t>
+          <t>Punch</t>
         </is>
       </c>
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>frappe</t>
+          <t>coup-faible</t>
         </is>
       </c>
       <c r="C33" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E33" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F33" s="17" t="inlineStr"/>
       <c r="G33" s="18" t="inlineStr">
         <is>
-          <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H33" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage.</t>
+          <t>Deal 3 damage.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="25" t="inlineStr">
         <is>
-          <t>Venom Stab</t>
+          <t>Radiant Strike</t>
         </is>
       </c>
       <c r="B34" s="26" t="inlineStr">
         <is>
-          <t>coup-venimeux</t>
+          <t>frappe-radiante</t>
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
@@ -4599,24 +4747,24 @@
       <c r="F34" s="17" t="inlineStr"/>
       <c r="G34" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>Crusader Plate</t>
         </is>
       </c>
       <c r="H34" s="18" t="inlineStr">
         <is>
-          <t>Deal 4 damage. Apply 4 Poison.</t>
+          <t>Deal 14 damage. Apply 2 Confusion.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="25" t="inlineStr">
         <is>
-          <t>Wound Opening</t>
+          <t>Rusty Cleave</t>
         </is>
       </c>
       <c r="B35" s="26" t="inlineStr">
         <is>
-          <t>ouverture-des-plaies</t>
+          <t>coup-de-hache</t>
         </is>
       </c>
       <c r="C35" s="17" t="n">
@@ -4627,184 +4775,184 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F35" s="17" t="inlineStr"/>
       <c r="G35" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>Rusty Axe</t>
         </is>
       </c>
       <c r="H35" s="18" t="inlineStr">
         <is>
-          <t>Deal 18 damage. Doubled if the target has a negative status.</t>
+          <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="25" t="inlineStr">
         <is>
-          <t>Guard</t>
+          <t>Shield Bash</t>
         </is>
       </c>
       <c r="B36" s="26" t="inlineStr">
         <is>
-          <t>garde</t>
+          <t>coup-de-bouclier</t>
         </is>
       </c>
       <c r="C36" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="29" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E36" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>2</v>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E36" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr"/>
       <c r="G36" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H36" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone.</t>
+          <t>Deal 10 damage. Stun the enemy for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="25" t="inlineStr">
         <is>
-          <t>Hand Guard</t>
+          <t>Splash Strike</t>
         </is>
       </c>
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t>garde-faible</t>
+          <t>eclaboussure-de-frappe</t>
         </is>
       </c>
       <c r="C37" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="29" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E37" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>3</v>
+      </c>
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E37" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr"/>
       <c r="G37" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>Forge Hammer</t>
         </is>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Stone.</t>
+          <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="25" t="inlineStr">
         <is>
-          <t>Heavy Armor</t>
+          <t>Strike</t>
         </is>
       </c>
       <c r="B38" s="26" t="inlineStr">
         <is>
-          <t>armure-lourde</t>
+          <t>frappe</t>
         </is>
       </c>
       <c r="C38" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" s="29" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E38" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+        <v>1</v>
+      </c>
+      <c r="D38" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F38" s="17" t="inlineStr"/>
       <c r="G38" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
         </is>
       </c>
       <c r="H38" s="18" t="inlineStr">
         <is>
-          <t>Gain 20 Stone.</t>
+          <t>Deal 6 damage.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>Light Armor</t>
+          <t>Venom Stab</t>
         </is>
       </c>
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t>armure-legere</t>
+          <t>coup-venimeux</t>
         </is>
       </c>
       <c r="C39" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="29" t="inlineStr">
-        <is>
-          <t>Défense</t>
-        </is>
-      </c>
-      <c r="E39" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="D39" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
+        </is>
+      </c>
+      <c r="E39" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr"/>
       <c r="G39" s="18" t="inlineStr">
         <is>
-          <t>Traveler's Garb</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone.</t>
+          <t>Deal 4 damage. Apply 4 Poison.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="25" t="inlineStr">
         <is>
-          <t>Mail Armor</t>
+          <t>Wound Opening</t>
         </is>
       </c>
       <c r="B40" s="26" t="inlineStr">
         <is>
-          <t>mail-armor</t>
+          <t>ouverture-des-plaies</t>
         </is>
       </c>
       <c r="C40" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="29" t="inlineStr">
-        <is>
-          <t>Défense</t>
+        <v>2</v>
+      </c>
+      <c r="D40" s="27" t="inlineStr">
+        <is>
+          <t>Attaque</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
@@ -4815,96 +4963,96 @@
       <c r="F40" s="17" t="inlineStr"/>
       <c r="G40" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H40" s="18" t="inlineStr">
         <is>
-          <t>Gain 7 Stone for every enemy still alive.</t>
+          <t>Deal 18 damage. Doubled if the target has a negative status.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="25" t="inlineStr">
         <is>
-          <t>Onyx Armor</t>
+          <t>Guard</t>
         </is>
       </c>
       <c r="B41" s="26" t="inlineStr">
         <is>
-          <t>onyx-armor</t>
+          <t>garde</t>
         </is>
       </c>
       <c r="C41" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E41" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="17" t="inlineStr"/>
       <c r="G41" s="18" t="inlineStr">
         <is>
-          <t>Onyx Guard Plate</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H41" s="18" t="inlineStr">
         <is>
-          <t>Gain 30 Stone.</t>
+          <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="25" t="inlineStr">
         <is>
-          <t>Quench</t>
+          <t>Hand Guard</t>
         </is>
       </c>
       <c r="B42" s="26" t="inlineStr">
         <is>
-          <t>trempe</t>
+          <t>garde-faible</t>
         </is>
       </c>
       <c r="C42" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E42" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E42" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F42" s="17" t="inlineStr"/>
       <c r="G42" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H42" s="18" t="inlineStr">
         <is>
-          <t>Spend all Forge Heat. Gain 10 Stone per Heat spent.</t>
+          <t>Gain 3 Stone.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="25" t="inlineStr">
         <is>
-          <t>Sacred Ground</t>
+          <t>Heavy Armor</t>
         </is>
       </c>
       <c r="B43" s="26" t="inlineStr">
         <is>
-          <t>terre-sacree</t>
+          <t>armure-lourde</t>
         </is>
       </c>
       <c r="C43" s="17" t="n">
@@ -4923,24 +5071,24 @@
       <c r="F43" s="17" t="inlineStr"/>
       <c r="G43" s="18" t="inlineStr">
         <is>
-          <t>Crusader Plate</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H43" s="18" t="inlineStr">
         <is>
-          <t>Gain 18 Stone.</t>
+          <t>Gain 20 Stone.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>Shield Wall</t>
+          <t>Light Armor</t>
         </is>
       </c>
       <c r="B44" s="26" t="inlineStr">
         <is>
-          <t>mur-bouclier</t>
+          <t>armure-legere</t>
         </is>
       </c>
       <c r="C44" s="17" t="n">
@@ -4951,36 +5099,36 @@
           <t>Défense</t>
         </is>
       </c>
-      <c r="E44" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F44" s="17" t="inlineStr"/>
       <c r="G44" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>Traveler's Garb</t>
         </is>
       </c>
       <c r="H44" s="18" t="inlineStr">
         <is>
-          <t>Gain 10 Stone.</t>
+          <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>Stacking Shield</t>
+          <t>Mail Armor</t>
         </is>
       </c>
       <c r="B45" s="26" t="inlineStr">
         <is>
-          <t>bouclier-empilant</t>
+          <t>mail-armor</t>
         </is>
       </c>
       <c r="C45" s="17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D45" s="29" t="inlineStr">
         <is>
@@ -4995,104 +5143,104 @@
       <c r="F45" s="17" t="inlineStr"/>
       <c r="G45" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
-          <t>Double your current Stone.</t>
+          <t>Gain 7 Stone for every enemy still alive.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>Boost</t>
+          <t>Onyx Armor</t>
         </is>
       </c>
       <c r="B46" s="26" t="inlineStr">
         <is>
-          <t>boost</t>
+          <t>onyx-armor</t>
         </is>
       </c>
       <c r="C46" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="30" t="inlineStr">
-        <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E46" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+        <v>2</v>
+      </c>
+      <c r="D46" s="29" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F46" s="17" t="inlineStr"/>
       <c r="G46" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots, Mail Boots</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H46" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Forge Heat (energy).</t>
+          <t>Gain 30 Stone.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>Burning Run</t>
+          <t>Quench</t>
         </is>
       </c>
       <c r="B47" s="26" t="inlineStr">
         <is>
-          <t>course-ardente</t>
+          <t>trempe</t>
         </is>
       </c>
       <c r="C47" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" s="30" t="inlineStr">
-        <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E47" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+        <v>0</v>
+      </c>
+      <c r="D47" s="29" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E47" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F47" s="17" t="inlineStr"/>
       <c r="G47" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>Haste for as many turns as your current Forge Heat.</t>
+          <t>Spend all Forge Heat. Gain 10 Stone per Heat spent.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>Crusader's Charge</t>
+          <t>Sacred Ground</t>
         </is>
       </c>
       <c r="B48" s="26" t="inlineStr">
         <is>
-          <t>charge-du-croise</t>
+          <t>terre-sacree</t>
         </is>
       </c>
       <c r="C48" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="30" t="inlineStr">
-        <is>
-          <t>Buff</t>
+        <v>2</v>
+      </c>
+      <c r="D48" s="29" t="inlineStr">
+        <is>
+          <t>Défense</t>
         </is>
       </c>
       <c r="E48" s="21" t="inlineStr">
@@ -5103,32 +5251,32 @@
       <c r="F48" s="17" t="inlineStr"/>
       <c r="G48" s="18" t="inlineStr">
         <is>
-          <t>Crusader Greaves</t>
+          <t>Crusader Plate</t>
         </is>
       </c>
       <c r="H48" s="18" t="inlineStr">
         <is>
-          <t>Haste: +30% attack speed for 3 turns.</t>
+          <t>Gain 18 Stone.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>Fire Boost</t>
+          <t>Sanguine Guard</t>
         </is>
       </c>
       <c r="B49" s="26" t="inlineStr">
         <is>
-          <t>boost-feu</t>
+          <t>garde-sanguine</t>
         </is>
       </c>
       <c r="C49" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="30" t="inlineStr">
-        <is>
-          <t>Buff</t>
+        <v>2</v>
+      </c>
+      <c r="D49" s="29" t="inlineStr">
+        <is>
+          <t>Défense</t>
         </is>
       </c>
       <c r="E49" s="22" t="inlineStr">
@@ -5139,96 +5287,96 @@
       <c r="F49" s="17" t="inlineStr"/>
       <c r="G49" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots</t>
+          <t>Blood Plate</t>
         </is>
       </c>
       <c r="H49" s="18" t="inlineStr">
         <is>
-          <t>Convert 4 of your own Burning into 2 Forge Heat. No effect below 4 Burning.</t>
+          <t>Gain 1 Stone per Bleed among ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>Forge from Ashes</t>
+          <t>Shield Wall</t>
         </is>
       </c>
       <c r="B50" s="26" t="inlineStr">
         <is>
-          <t>forge-des-cendres</t>
+          <t>mur-bouclier</t>
         </is>
       </c>
       <c r="C50" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D50" s="30" t="inlineStr">
-        <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E50" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+        <v>1</v>
+      </c>
+      <c r="D50" s="29" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E50" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F50" s="17" t="inlineStr"/>
       <c r="G50" s="18" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H50" s="18" t="inlineStr">
         <is>
-          <t>Discard your hand and draw that many cards.</t>
+          <t>Gain 10 Stone.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>Free Movement</t>
+          <t>Stacking Shield</t>
         </is>
       </c>
       <c r="B51" s="26" t="inlineStr">
         <is>
-          <t>mouvement-degage</t>
+          <t>bouclier-empilant</t>
         </is>
       </c>
       <c r="C51" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" s="30" t="inlineStr">
-        <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="E51" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+        <v>4</v>
+      </c>
+      <c r="D51" s="29" t="inlineStr">
+        <is>
+          <t>Défense</t>
+        </is>
+      </c>
+      <c r="E51" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F51" s="17" t="inlineStr"/>
       <c r="G51" s="18" t="inlineStr">
         <is>
-          <t>Traveler's Garb</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H51" s="18" t="inlineStr">
         <is>
-          <t>Haste for 5 of your turns.</t>
+          <t>Double your current Stone.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>Mail Advantage</t>
+          <t>Blood Rush</t>
         </is>
       </c>
       <c r="B52" s="26" t="inlineStr">
         <is>
-          <t>avantage-maille</t>
+          <t>ruee-de-sang</t>
         </is>
       </c>
       <c r="C52" s="17" t="n">
@@ -5239,72 +5387,72 @@
           <t>Buff</t>
         </is>
       </c>
-      <c r="E52" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E52" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F52" s="17" t="inlineStr"/>
       <c r="G52" s="18" t="inlineStr">
         <is>
-          <t>Mail Glove, Mail Boots</t>
+          <t>Blood Greaves</t>
         </is>
       </c>
       <c r="H52" s="18" t="inlineStr">
         <is>
-          <t>Gain 8 Stone and Haste for 2 turns.</t>
+          <t>Gain 1 Forge Heat per 4 Bleed among ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Master's Hand</t>
+          <t>Boost</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
         <is>
-          <t>main-de-maitre</t>
+          <t>boost</t>
         </is>
       </c>
       <c r="C53" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D53" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E53" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E53" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F53" s="17" t="inlineStr"/>
       <c r="G53" s="18" t="inlineStr">
         <is>
-          <t>Miner's Gloves, Mail Glove</t>
+          <t>Onyx Boots, Mail Boots</t>
         </is>
       </c>
       <c r="H53" s="18" t="inlineStr">
         <is>
-          <t>Draw 2 cards.</t>
+          <t>Gain 3 Forge Heat (energy).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>Onyx Overheat</t>
+          <t>Burning Run</t>
         </is>
       </c>
       <c r="B54" s="26" t="inlineStr">
         <is>
-          <t>onyx-overheat</t>
+          <t>course-ardente</t>
         </is>
       </c>
       <c r="C54" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D54" s="30" t="inlineStr">
         <is>
@@ -5319,28 +5467,28 @@
       <c r="F54" s="17" t="inlineStr"/>
       <c r="G54" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Onyx Boots</t>
         </is>
       </c>
       <c r="H54" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Forge Heat (energy).</t>
+          <t>Haste for as many turns as your current Forge Heat.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>Outnumbered</t>
+          <t>Crusader's Charge</t>
         </is>
       </c>
       <c r="B55" s="26" t="inlineStr">
         <is>
-          <t>surnombre</t>
+          <t>charge-du-croise</t>
         </is>
       </c>
       <c r="C55" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55" s="30" t="inlineStr">
         <is>
@@ -5355,28 +5503,28 @@
       <c r="F55" s="17" t="inlineStr"/>
       <c r="G55" s="18" t="inlineStr">
         <is>
-          <t>Mail Glove</t>
+          <t>Crusader Greaves</t>
         </is>
       </c>
       <c r="H55" s="18" t="inlineStr">
         <is>
-          <t>Draw 1 card per living enemy.</t>
+          <t>Haste: +30% attack speed for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Surge</t>
+          <t>Fire Boost</t>
         </is>
       </c>
       <c r="B56" s="26" t="inlineStr">
         <is>
-          <t>surge-saphir-parfait</t>
+          <t>boost-feu</t>
         </is>
       </c>
       <c r="C56" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D56" s="30" t="inlineStr">
         <is>
@@ -5391,118 +5539,370 @@
       <c r="F56" s="17" t="inlineStr"/>
       <c r="G56" s="18" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Amulet</t>
+          <t>Onyx Boots</t>
         </is>
       </c>
       <c r="H56" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Forge Heat (energy).</t>
+          <t>Convert 4 of your own Burning into 2 Forge Heat. No effect below 4 Burning.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>Quicken</t>
+          <t>Forge from Ashes</t>
         </is>
       </c>
       <c r="B57" s="26" t="inlineStr">
         <is>
-          <t>celerite-vive</t>
+          <t>forge-des-cendres</t>
         </is>
       </c>
       <c r="C57" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E57" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E57" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F57" s="17" t="inlineStr"/>
       <c r="G57" s="18" t="inlineStr">
         <is>
-          <t>Swift Boots, Mail Boots</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="H57" s="18" t="inlineStr">
         <is>
-          <t>Haste: +30% attack speed for 3 turns.</t>
+          <t>Discard your hand and draw that many cards.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>Sapphire Surge</t>
+          <t>Free Movement</t>
         </is>
       </c>
       <c r="B58" s="26" t="inlineStr">
         <is>
-          <t>surge-saphir</t>
+          <t>mouvement-degage</t>
         </is>
       </c>
       <c r="C58" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D58" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E58" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F58" s="17" t="inlineStr"/>
       <c r="G58" s="18" t="inlineStr">
         <is>
-          <t>Sapphire Amulet, Nice Sapphire Amulet</t>
+          <t>Traveler's Garb</t>
         </is>
       </c>
       <c r="H58" s="18" t="inlineStr">
         <is>
-          <t>Gain 2 Forge Heat (energy).</t>
+          <t>Haste for 5 of your turns.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>Second Wind</t>
+          <t>Mail Advantage</t>
         </is>
       </c>
       <c r="B59" s="26" t="inlineStr">
         <is>
-          <t>second-souffle</t>
+          <t>avantage-maille</t>
         </is>
       </c>
       <c r="C59" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D59" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E59" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E59" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F59" s="17" t="inlineStr"/>
       <c r="G59" s="18" t="inlineStr">
         <is>
+          <t>Mail Glove, Mail Boots</t>
+        </is>
+      </c>
+      <c r="H59" s="18" t="inlineStr">
+        <is>
+          <t>Gain 8 Stone and Haste for 2 turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="25" t="inlineStr">
+        <is>
+          <t>Master's Hand</t>
+        </is>
+      </c>
+      <c r="B60" s="26" t="inlineStr">
+        <is>
+          <t>main-de-maitre</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="F60" s="17" t="inlineStr"/>
+      <c r="G60" s="18" t="inlineStr">
+        <is>
+          <t>Miner's Gloves, Mail Glove</t>
+        </is>
+      </c>
+      <c r="H60" s="18" t="inlineStr">
+        <is>
+          <t>Draw 2 cards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
+          <t>Onyx Overheat</t>
+        </is>
+      </c>
+      <c r="B61" s="26" t="inlineStr">
+        <is>
+          <t>onyx-overheat</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E61" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F61" s="17" t="inlineStr"/>
+      <c r="G61" s="18" t="inlineStr">
+        <is>
+          <t>Big Onyx Sword</t>
+        </is>
+      </c>
+      <c r="H61" s="18" t="inlineStr">
+        <is>
+          <t>Gain 5 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>Outnumbered</t>
+        </is>
+      </c>
+      <c r="B62" s="26" t="inlineStr">
+        <is>
+          <t>surnombre</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E62" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F62" s="17" t="inlineStr"/>
+      <c r="G62" s="18" t="inlineStr">
+        <is>
+          <t>Mail Glove</t>
+        </is>
+      </c>
+      <c r="H62" s="18" t="inlineStr">
+        <is>
+          <t>Draw 1 card per living enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="25" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Surge</t>
+        </is>
+      </c>
+      <c r="B63" s="26" t="inlineStr">
+        <is>
+          <t>surge-saphir-parfait</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E63" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F63" s="17" t="inlineStr"/>
+      <c r="G63" s="18" t="inlineStr">
+        <is>
+          <t>Perfect Sapphire Amulet</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>Gain 3 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="25" t="inlineStr">
+        <is>
+          <t>Quicken</t>
+        </is>
+      </c>
+      <c r="B64" s="26" t="inlineStr">
+        <is>
+          <t>celerite-vive</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E64" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F64" s="17" t="inlineStr"/>
+      <c r="G64" s="18" t="inlineStr">
+        <is>
+          <t>Swift Boots, Mail Boots</t>
+        </is>
+      </c>
+      <c r="H64" s="18" t="inlineStr">
+        <is>
+          <t>Haste: +30% attack speed for 3 turns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t>Sapphire Surge</t>
+        </is>
+      </c>
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>surge-saphir</t>
+        </is>
+      </c>
+      <c r="C65" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E65" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F65" s="17" t="inlineStr"/>
+      <c r="G65" s="18" t="inlineStr">
+        <is>
+          <t>Sapphire Amulet, Nice Sapphire Amulet</t>
+        </is>
+      </c>
+      <c r="H65" s="18" t="inlineStr">
+        <is>
+          <t>Gain 2 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="25" t="inlineStr">
+        <is>
+          <t>Second Wind</t>
+        </is>
+      </c>
+      <c r="B66" s="26" t="inlineStr">
+        <is>
+          <t>second-souffle</t>
+        </is>
+      </c>
+      <c r="C66" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E66" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F66" s="17" t="inlineStr"/>
+      <c r="G66" s="18" t="inlineStr">
+        <is>
           <t>Swift Boots</t>
         </is>
       </c>
-      <c r="H59" s="18" t="inlineStr">
+      <c r="H66" s="18" t="inlineStr">
         <is>
           <t>Trade 5 Haste turns for 3 Forge Heat. No effect below 5 Haste.</t>
         </is>
@@ -5523,7 +5923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5635,10 +6035,26 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="23" t="n"/>
-      <c r="C7" s="23" t="n"/>
-      <c r="D7" s="23" t="n"/>
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>Blood Set</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Blood Plate  +  Blood Gauntlets  +  Blood Greaves</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Quand un combo de saignement inflige des dégâts bonus</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>When a Bleed combo deals bonus damage, heal the hero for that amount.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="23" t="n"/>
@@ -5669,6 +6085,12 @@
       <c r="B12" s="23" t="n"/>
       <c r="C12" s="23" t="n"/>
       <c r="D12" s="23" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="23" t="n"/>
+      <c r="C13" s="23" t="n"/>
+      <c r="D13" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
[équilibrage] Set de Sang : épique → uncommon
Rareté des 3 pièces passée à uncommon (build saignement accessible tôt).
Valeurs des cartes ramenées au palier uncommon :
- Crimson Carve 12/4 → 9/3 · Bloodbath 5 → 4 (AOE)
- Open Veins 4/5 → 3/4 · Contagion 6 → 5 dégâts
- Hemorrhage ×3 → ×2 par point · Blood Rush 1/4 → 1/5 saignement
- Blood Plate : +20 → +12 Pierre de départ, 7 → 6 cartes
Catalogue régénéré et concept.md mis à jour.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJcbumK5KWRfGozDrLY2Kn
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -1925,13 +1925,13 @@
           <t>plate-sang</t>
         </is>
       </c>
-      <c r="C41" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="C41" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="D41" s="17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E41" s="18" t="inlineStr">
         <is>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="J41" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K41" s="18" t="n"/>
       <c r="L41" s="18" t="n"/>
@@ -2688,9 +2688,9 @@
           <t>gants-sang</t>
         </is>
       </c>
-      <c r="C76" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="D76" s="17" t="n">
@@ -3035,9 +3035,9 @@
           <t>bottes-sang</t>
         </is>
       </c>
-      <c r="C89" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="D89" s="17" t="n">
@@ -3699,9 +3699,9 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Apply 5 Bleed to ALL enemies.</t>
+          <t>Apply 4 Bleed to ALL enemies.</t>
         </is>
       </c>
     </row>
@@ -3847,9 +3847,9 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F10" s="17" t="inlineStr"/>
@@ -3860,7 +3860,7 @@
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage. Both adjacent enemies gain Bleed equal to the target's Bleed.</t>
+          <t>Deal 5 damage. Both adjacent enemies gain Bleed equal to the target's Bleed.</t>
         </is>
       </c>
     </row>
@@ -3883,9 +3883,9 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E11" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr"/>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>Deal 12 damage. Apply 4 Bleed.</t>
+          <t>Deal 9 damage. Apply 3 Bleed.</t>
         </is>
       </c>
     </row>
@@ -4295,9 +4295,9 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr"/>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>Consume all the target's Bleed: deal 3 damage per Bleed consumed.</t>
+          <t>Consume all the target's Bleed: deal 2 damage per Bleed consumed.</t>
         </is>
       </c>
     </row>
@@ -4555,9 +4555,9 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E29" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E29" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr"/>
@@ -4568,7 +4568,7 @@
       </c>
       <c r="H29" s="18" t="inlineStr">
         <is>
-          <t>Deal 4 damage. Apply 5 Bleed.</t>
+          <t>Deal 3 damage. Apply 4 Bleed.</t>
         </is>
       </c>
     </row>
@@ -5279,9 +5279,9 @@
           <t>Défense</t>
         </is>
       </c>
-      <c r="E49" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F49" s="17" t="inlineStr"/>
@@ -5387,9 +5387,9 @@
           <t>Buff</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E52" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F52" s="17" t="inlineStr"/>
@@ -5400,7 +5400,7 @@
       </c>
       <c r="H52" s="18" t="inlineStr">
         <is>
-          <t>Gain 1 Forge Heat per 4 Bleed among ALL enemies.</t>
+          <t>Gain 1 Forge Heat per 5 Bleed among ALL enemies.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[technique] Catalogue : réafficher l'armure de départ et le passif des items
La colonne « Effet hors-carte » reportait l'appartenance au set mais avait
oublié armureDepart (armure de départ) et passifPropre. Réparé : chaque
armure réaffiche « Ajoute X d'armure en début de combat », et le Tower Shield
montre son passif. Permet de comparer les valeurs des armures pour équilibrer.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJcbumK5KWRfGozDrLY2Kn
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -672,14 +672,14 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Effets HORS carte (sac, deux mains, set d'armure)</t>
+          <t>Effets HORS carte (armure de départ, sac, deux mains, set d'armure)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>La colonne « Effet hors-carte » (onglet Items) décrit ce qu'un objet apporte EN DEHORS de ses cartes : rangées de sac, arme à deux mains, appartenance à un set. Pour un nouvel objet, écris ici son effet hors-carte (ex. « +4 rangées de sac »).</t>
+          <t>La colonne « Effet hors-carte » (onglet Items) décrit ce qu'un objet apporte EN DEHORS de ses cartes : armure (Pierre) donnée en début de combat, rangées de sac, arme à deux mains, passif propre, appartenance à un set. Pour un nouvel objet, écris ici son effet hors-carte (ex. « Ajoute 12 d'armure en début de combat », « +4 rangées de sac »).</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,11 @@
       </c>
       <c r="K28" s="18" t="n"/>
       <c r="L28" s="18" t="n"/>
-      <c r="M28" s="19" t="inlineStr"/>
+      <c r="M28" s="19" t="inlineStr">
+        <is>
+          <t>When hit by a melee attack, gain 2 Stone.</t>
+        </is>
+      </c>
       <c r="N28" s="18" t="n"/>
     </row>
     <row r="29">
@@ -1749,7 +1753,11 @@
       <c r="J37" s="18" t="n"/>
       <c r="K37" s="18" t="n"/>
       <c r="L37" s="18" t="n"/>
-      <c r="M37" s="19" t="inlineStr"/>
+      <c r="M37" s="19" t="inlineStr">
+        <is>
+          <t>Ajoute 8 d'armure en début de combat</t>
+        </is>
+      </c>
       <c r="N37" s="18" t="n"/>
     </row>
     <row r="38">
@@ -1805,7 +1813,7 @@
       </c>
       <c r="M38" s="19" t="inlineStr">
         <is>
-          <t>Set : Onyx Set</t>
+          <t>Ajoute 30 d'armure en début de combat  ·  Set : Onyx Set</t>
         </is>
       </c>
       <c r="N38" s="18" t="n"/>
@@ -1857,7 +1865,7 @@
       <c r="L39" s="18" t="n"/>
       <c r="M39" s="19" t="inlineStr">
         <is>
-          <t>Set : Mail Set</t>
+          <t>Ajoute 22 d'armure en début de combat  ·  Set : Mail Set</t>
         </is>
       </c>
       <c r="N39" s="18" t="n"/>
@@ -1909,7 +1917,7 @@
       <c r="L40" s="18" t="n"/>
       <c r="M40" s="19" t="inlineStr">
         <is>
-          <t>Set : Crusader Set</t>
+          <t>Ajoute 15 d'armure en début de combat  ·  Set : Crusader Set</t>
         </is>
       </c>
       <c r="N40" s="18" t="n"/>
@@ -1961,7 +1969,7 @@
       <c r="L41" s="18" t="n"/>
       <c r="M41" s="19" t="inlineStr">
         <is>
-          <t>Set : Blood Set</t>
+          <t>Ajoute 12 d'armure en début de combat  ·  Set : Blood Set</t>
         </is>
       </c>
       <c r="N41" s="18" t="n"/>

</xml_diff>

<commit_message>
[technique] Catalogue : vitesse des bottes + distinction carte non équipée
- Effet hors-carte affiche le bonus de vitesse des bottes (% + move speed)
- Cartes sans objet : « — (non équipée) » au lieu de « deck de base »
- Régénéré : 35 items, 65 cartes, 4 sets

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJcbumK5KWRfGozDrLY2Kn
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -1813,7 +1813,7 @@
       </c>
       <c r="M38" s="19" t="inlineStr">
         <is>
-          <t>Ajoute 30 d'armure en début de combat  ·  Set : Onyx Set</t>
+          <t>Ajoute 36 d'armure en début de combat  ·  Set : Onyx Set</t>
         </is>
       </c>
       <c r="N38" s="18" t="n"/>
@@ -1891,15 +1891,15 @@
       </c>
       <c r="E40" s="18" t="inlineStr">
         <is>
-          <t>Radiant Strike</t>
+          <t>Heavy Armor</t>
         </is>
       </c>
       <c r="F40" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40" s="18" t="inlineStr">
         <is>
-          <t>Sacred Ground</t>
+          <t>Armor of light</t>
         </is>
       </c>
       <c r="H40" s="17" t="n">
@@ -1913,11 +1913,17 @@
       <c r="J40" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="K40" s="18" t="n"/>
-      <c r="L40" s="18" t="n"/>
+      <c r="K40" s="18" t="inlineStr">
+        <is>
+          <t>Holy light</t>
+        </is>
+      </c>
+      <c r="L40" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="M40" s="19" t="inlineStr">
         <is>
-          <t>Ajoute 15 d'armure en début de combat  ·  Set : Crusader Set</t>
+          <t>Ajoute 30 d'armure en début de combat  ·  Set : Crusader Set</t>
         </is>
       </c>
       <c r="N40" s="18" t="n"/>
@@ -1933,9 +1939,9 @@
           <t>plate-sang</t>
         </is>
       </c>
-      <c r="C41" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="C41" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D41" s="17" t="n">
@@ -1943,11 +1949,11 @@
       </c>
       <c r="E41" s="18" t="inlineStr">
         <is>
-          <t>Crimson Carve</t>
+          <t>Heavy Armor</t>
         </is>
       </c>
       <c r="F41" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G41" s="18" t="inlineStr">
         <is>
@@ -1965,11 +1971,17 @@
       <c r="J41" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="K41" s="18" t="n"/>
-      <c r="L41" s="18" t="n"/>
+      <c r="K41" s="18" t="inlineStr">
+        <is>
+          <t>Drink blood</t>
+        </is>
+      </c>
+      <c r="L41" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="M41" s="19" t="inlineStr">
         <is>
-          <t>Ajoute 12 d'armure en début de combat  ·  Set : Blood Set</t>
+          <t>Ajoute 20 d'armure en début de combat  ·  Set : Blood Set</t>
         </is>
       </c>
       <c r="N41" s="18" t="n"/>
@@ -2656,11 +2668,11 @@
         </is>
       </c>
       <c r="D75" s="17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E75" s="18" t="inlineStr">
         <is>
-          <t>Lumen Jab</t>
+          <t>Master's Hand</t>
         </is>
       </c>
       <c r="F75" s="17" t="n">
@@ -2674,8 +2686,14 @@
       <c r="H75" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I75" s="18" t="n"/>
-      <c r="J75" s="18" t="n"/>
+      <c r="I75" s="18" t="inlineStr">
+        <is>
+          <t>Lay on Hands</t>
+        </is>
+      </c>
+      <c r="J75" s="17" t="n">
+        <v>2</v>
+      </c>
       <c r="K75" s="18" t="n"/>
       <c r="L75" s="18" t="n"/>
       <c r="M75" s="19" t="inlineStr">
@@ -2696,13 +2714,13 @@
           <t>gants-sang</t>
         </is>
       </c>
-      <c r="C76" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="C76" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D76" s="17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E76" s="18" t="inlineStr">
         <is>
@@ -2720,8 +2738,14 @@
       <c r="H76" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I76" s="18" t="n"/>
-      <c r="J76" s="18" t="n"/>
+      <c r="I76" s="18" t="inlineStr">
+        <is>
+          <t>Blood Absorption</t>
+        </is>
+      </c>
+      <c r="J76" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="K76" s="18" t="n"/>
       <c r="L76" s="18" t="n"/>
       <c r="M76" s="19" t="inlineStr">
@@ -2873,7 +2897,11 @@
       <c r="J85" s="18" t="n"/>
       <c r="K85" s="18" t="n"/>
       <c r="L85" s="18" t="n"/>
-      <c r="M85" s="19" t="inlineStr"/>
+      <c r="M85" s="19" t="inlineStr">
+        <is>
+          <t>+15% célérité, +3 move speed</t>
+        </is>
+      </c>
       <c r="N85" s="18" t="n"/>
     </row>
     <row r="86">
@@ -2929,7 +2957,7 @@
       </c>
       <c r="M86" s="19" t="inlineStr">
         <is>
-          <t>Set : Onyx Set</t>
+          <t>+30% célérité, +8 move speed  ·  Set : Onyx Set</t>
         </is>
       </c>
       <c r="N86" s="18" t="n"/>
@@ -2981,7 +3009,7 @@
       <c r="L87" s="18" t="n"/>
       <c r="M87" s="19" t="inlineStr">
         <is>
-          <t>Set : Mail Set</t>
+          <t>+20% célérité, +5 move speed  ·  Set : Mail Set</t>
         </is>
       </c>
       <c r="N87" s="18" t="n"/>
@@ -3003,11 +3031,11 @@
         </is>
       </c>
       <c r="D88" s="17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E88" s="18" t="inlineStr">
         <is>
-          <t>Crusader's Charge</t>
+          <t>Quicken</t>
         </is>
       </c>
       <c r="F88" s="17" t="n">
@@ -3015,19 +3043,25 @@
       </c>
       <c r="G88" s="18" t="inlineStr">
         <is>
-          <t>Dazzling Kick</t>
+          <t>Kick of light</t>
         </is>
       </c>
       <c r="H88" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I88" s="18" t="n"/>
-      <c r="J88" s="18" t="n"/>
+      <c r="I88" s="18" t="inlineStr">
+        <is>
+          <t>Boost</t>
+        </is>
+      </c>
+      <c r="J88" s="17" t="n">
+        <v>2</v>
+      </c>
       <c r="K88" s="18" t="n"/>
       <c r="L88" s="18" t="n"/>
       <c r="M88" s="19" t="inlineStr">
         <is>
-          <t>Set : Crusader Set</t>
+          <t>+20% célérité, +5 move speed  ·  Set : Crusader Set</t>
         </is>
       </c>
       <c r="N88" s="18" t="n"/>
@@ -3043,21 +3077,21 @@
           <t>bottes-sang</t>
         </is>
       </c>
-      <c r="C89" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="C89" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D89" s="17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E89" s="18" t="inlineStr">
         <is>
-          <t>Hemorrhage</t>
+          <t>Blood Slide</t>
         </is>
       </c>
       <c r="F89" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G89" s="18" t="inlineStr">
         <is>
@@ -3067,13 +3101,25 @@
       <c r="H89" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="I89" s="18" t="n"/>
-      <c r="J89" s="18" t="n"/>
-      <c r="K89" s="18" t="n"/>
-      <c r="L89" s="18" t="n"/>
+      <c r="I89" s="18" t="inlineStr">
+        <is>
+          <t>Quicken</t>
+        </is>
+      </c>
+      <c r="J89" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K89" s="18" t="inlineStr">
+        <is>
+          <t>Boost</t>
+        </is>
+      </c>
+      <c r="L89" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="M89" s="19" t="inlineStr">
         <is>
-          <t>Set : Blood Set</t>
+          <t>+20% célérité, +5 move speed  ·  Set : Blood Set</t>
         </is>
       </c>
       <c r="N89" s="18" t="n"/>
@@ -3506,7 +3552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3660,7 +3706,7 @@
         </is>
       </c>
       <c r="C5" s="17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D5" s="27" t="inlineStr">
         <is>
@@ -3691,25 +3737,25 @@
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>Bloodbath</t>
+          <t>Blood Slide</t>
         </is>
       </c>
       <c r="B6" s="26" t="inlineStr">
         <is>
-          <t>bain-de-sang</t>
+          <t>glissade-sur-sang</t>
         </is>
       </c>
       <c r="C6" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr">
@@ -3719,132 +3765,136 @@
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Blood Plate</t>
+          <t>Blood Greaves</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Apply 4 Bleed to ALL enemies.</t>
+          <t>Stun for 2 turns every enemy that has Bleed.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Bloodletting</t>
+          <t>Bloodbath</t>
         </is>
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>coup-de-sang</t>
+          <t>bain-de-sang</t>
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
-        </is>
-      </c>
-      <c r="F7" s="17" t="inlineStr"/>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>Blood Ring</t>
+          <t>Blood Plate</t>
         </is>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
+          <t>Take 10 damage. Apply 5 Bleed to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>Burning Hand</t>
+          <t>Bloodletting</t>
         </is>
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>main-brulante</t>
+          <t>coup-de-sang</t>
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr"/>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Blood Ring</t>
         </is>
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>Discard your hand. For each card discarded, apply 8 Burning to a random enemy.</t>
+          <t>Deal 3 damage + current Bleed stacks as bonus damage. Apply 3 Bleed (stacks don't reset).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>Cleave</t>
+          <t>Burning Hand</t>
         </is>
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>couper-en-deux</t>
+          <t>main-brulante</t>
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr"/>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>Deal 20 damage. If the target dies, deal 15 damage to the next enemy.</t>
+          <t>Discard your hand. For each card discarded, apply 8 Burning to a random enemy.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Contagion</t>
+          <t>Cleave</t>
         </is>
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>contagion</t>
+          <t>couper-en-deux</t>
         </is>
       </c>
       <c r="C10" s="17" t="n">
@@ -3855,32 +3905,32 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F10" s="17" t="inlineStr"/>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>Blood Gauntlets</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>Deal 5 damage. Both adjacent enemies gain Bleed equal to the target's Bleed.</t>
+          <t>Deal 20 damage. If the target dies, deal 15 damage to the next enemy.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Crimson Carve</t>
+          <t>Contagion</t>
         </is>
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>carve-cramoisi</t>
+          <t>contagion</t>
         </is>
       </c>
       <c r="C11" s="17" t="n">
@@ -3891,81 +3941,85 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr"/>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>Blood Plate</t>
+          <t>Blood Gauntlets</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>Deal 9 damage. Apply 3 Bleed.</t>
+          <t>Both adjacent enemies match the target's Bleed.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>Dazzling Kick</t>
+          <t>Dragon's Blaze</t>
         </is>
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>coup-eblouissant</t>
+          <t>embrasement-dragon</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="F12" s="17" t="inlineStr"/>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>Crusader Greaves</t>
+          <t>Magma Hammer, Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>Deal 10 damage. Apply 3 Confusion.</t>
+          <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>Dragon's Blaze</t>
+          <t>Drink blood</t>
         </is>
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>embrasement-dragon</t>
+          <t>boire-le-sang</t>
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E13" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
@@ -3975,12 +4029,12 @@
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>Magma Hammer, Onyx Guard Plate</t>
+          <t>Blood Plate</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
+          <t>Lose 20 HP. Deal 10 damage and 1 Bleed to ALL enemies. Heal 20 HP per enemy killed by this.</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4270,7 @@
         </is>
       </c>
       <c r="C20" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
@@ -4240,7 +4294,7 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage to ALL enemies.</t>
+          <t>Apply 1 more Confusion to each already-confused enemy.</t>
         </is>
       </c>
     </row>
@@ -4287,36 +4341,36 @@
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>Hemorrhage</t>
+          <t>Kick of light</t>
         </is>
       </c>
       <c r="B22" s="26" t="inlineStr">
         <is>
-          <t>hemorragie</t>
+          <t>coup-de-lumiere</t>
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr"/>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>Blood Greaves</t>
+          <t>Crusader Greaves</t>
         </is>
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>Consume all the target's Bleed: deal 2 damage per Bleed consumed.</t>
+          <t>Deal 6 damage. Apply 1 Confusion.</t>
         </is>
       </c>
     </row>
@@ -4359,52 +4413,56 @@
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>Lumen Jab</t>
+          <t>Onyx Breath</t>
         </is>
       </c>
       <c r="B24" s="26" t="inlineStr">
         <is>
-          <t>coup-de-lumiere</t>
+          <t>souffle-onyx</t>
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E24" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="F24" s="17" t="inlineStr"/>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>Crusader Gauntlets</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H24" s="18" t="inlineStr">
         <is>
-          <t>Deal 8 damage. Apply 1 Confusion.</t>
+          <t>Apply 20 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>Onyx Breath</t>
+          <t>Onyx Fist</t>
         </is>
       </c>
       <c r="B25" s="26" t="inlineStr">
         <is>
-          <t>souffle-onyx</t>
+          <t>poing-onyx</t>
         </is>
       </c>
       <c r="C25" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" s="27" t="inlineStr">
         <is>
@@ -4416,31 +4474,27 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F25" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="F25" s="17" t="inlineStr"/>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>Onyx Guard Plate</t>
+          <t>Onyx Glove</t>
         </is>
       </c>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>Apply 20 Burning to ALL enemies.</t>
+          <t>Gain 10 Stone. Deal 10 damage and apply 3 Burning.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>Onyx Fist</t>
+          <t>Onyx Radiance</t>
         </is>
       </c>
       <c r="B26" s="26" t="inlineStr">
         <is>
-          <t>poing-onyx</t>
+          <t>onyx-radiance</t>
         </is>
       </c>
       <c r="C26" s="17" t="n">
@@ -4456,31 +4510,35 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F26" s="17" t="inlineStr"/>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G26" s="18" t="inlineStr">
         <is>
-          <t>Onyx Glove</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H26" s="18" t="inlineStr">
         <is>
-          <t>Gain 10 Stone. Deal 10 damage and apply 3 Burning.</t>
+          <t>Apply 8 Burning to ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>Onyx Radiance</t>
+          <t>Onyx Slash</t>
         </is>
       </c>
       <c r="B27" s="26" t="inlineStr">
         <is>
-          <t>onyx-radiance</t>
+          <t>onyx-slash</t>
         </is>
       </c>
       <c r="C27" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="27" t="inlineStr">
         <is>
@@ -4492,11 +4550,7 @@
           <t>Epic</t>
         </is>
       </c>
-      <c r="F27" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="F27" s="17" t="inlineStr"/>
       <c r="G27" s="18" t="inlineStr">
         <is>
           <t>Big Onyx Sword</t>
@@ -4504,55 +4558,55 @@
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
-          <t>Apply 8 Burning to ALL enemies.</t>
+          <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="25" t="inlineStr">
         <is>
-          <t>Onyx Slash</t>
+          <t>Open Veins</t>
         </is>
       </c>
       <c r="B28" s="26" t="inlineStr">
         <is>
-          <t>onyx-slash</t>
+          <t>ouvrir-les-veines</t>
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E28" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr"/>
       <c r="G28" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Blood Gauntlets</t>
         </is>
       </c>
       <c r="H28" s="18" t="inlineStr">
         <is>
-          <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
+          <t>Take 10 damage. Apply 4 Bleed.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="25" t="inlineStr">
         <is>
-          <t>Open Veins</t>
+          <t>Pickaxe Jab</t>
         </is>
       </c>
       <c r="B29" s="26" t="inlineStr">
         <is>
-          <t>ouvrir-les-veines</t>
+          <t>coup-de-pioche</t>
         </is>
       </c>
       <c r="C29" s="17" t="n">
@@ -4563,72 +4617,76 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E29" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E29" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr"/>
       <c r="G29" s="18" t="inlineStr">
         <is>
-          <t>Blood Gauntlets</t>
+          <t>Miner's Pick</t>
         </is>
       </c>
       <c r="H29" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage. Apply 4 Bleed.</t>
+          <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="25" t="inlineStr">
         <is>
-          <t>Pickaxe Jab</t>
+          <t>Poison Dance</t>
         </is>
       </c>
       <c r="B30" s="26" t="inlineStr">
         <is>
-          <t>coup-de-pioche</t>
+          <t>danse-empoisonnee</t>
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E30" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="F30" s="17" t="inlineStr"/>
+      <c r="E30" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="G30" s="18" t="inlineStr">
         <is>
-          <t>Miner's Pick</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H30" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
+          <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="25" t="inlineStr">
         <is>
-          <t>Poison Dance</t>
+          <t>Pommel Strike</t>
         </is>
       </c>
       <c r="B31" s="26" t="inlineStr">
         <is>
-          <t>danse-empoisonnee</t>
+          <t>coup-de-pommeau</t>
         </is>
       </c>
       <c r="C31" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" s="27" t="inlineStr">
         <is>
@@ -4640,71 +4698,67 @@
           <t>Rare</t>
         </is>
       </c>
-      <c r="F31" s="17" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="F31" s="17" t="inlineStr"/>
       <c r="G31" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>War Axe</t>
         </is>
       </c>
       <c r="H31" s="18" t="inlineStr">
         <is>
-          <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
+          <t>Deal 16 damage. Stun the target for 2 turns.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>Pommel Strike</t>
+          <t>Punch</t>
         </is>
       </c>
       <c r="B32" s="26" t="inlineStr">
         <is>
-          <t>coup-de-pommeau</t>
+          <t>coup-faible</t>
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E32" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E32" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr"/>
       <c r="G32" s="18" t="inlineStr">
         <is>
-          <t>War Axe</t>
+          <t>— (deck de base)</t>
         </is>
       </c>
       <c r="H32" s="18" t="inlineStr">
         <is>
-          <t>Deal 16 damage. Stun the target for 2 turns.</t>
+          <t>Deal 3 damage.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="25" t="inlineStr">
         <is>
-          <t>Punch</t>
+          <t>Radiant Strike</t>
         </is>
       </c>
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>coup-faible</t>
+          <t>frappe-radiante</t>
         </is>
       </c>
       <c r="C33" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D33" s="27" t="inlineStr">
         <is>
@@ -4719,24 +4773,24 @@
       <c r="F33" s="17" t="inlineStr"/>
       <c r="G33" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>— (non équipée)</t>
         </is>
       </c>
       <c r="H33" s="18" t="inlineStr">
         <is>
-          <t>Deal 3 damage.</t>
+          <t>Deal 14 damage. Apply 2 Confusion.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="25" t="inlineStr">
         <is>
-          <t>Radiant Strike</t>
+          <t>Rusty Cleave</t>
         </is>
       </c>
       <c r="B34" s="26" t="inlineStr">
         <is>
-          <t>frappe-radiante</t>
+          <t>coup-de-hache</t>
         </is>
       </c>
       <c r="C34" s="17" t="n">
@@ -4747,32 +4801,32 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E34" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F34" s="17" t="inlineStr"/>
       <c r="G34" s="18" t="inlineStr">
         <is>
-          <t>Crusader Plate</t>
+          <t>Rusty Axe</t>
         </is>
       </c>
       <c r="H34" s="18" t="inlineStr">
         <is>
-          <t>Deal 14 damage. Apply 2 Confusion.</t>
+          <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="25" t="inlineStr">
         <is>
-          <t>Rusty Cleave</t>
+          <t>Shield Bash</t>
         </is>
       </c>
       <c r="B35" s="26" t="inlineStr">
         <is>
-          <t>coup-de-hache</t>
+          <t>coup-de-bouclier</t>
         </is>
       </c>
       <c r="C35" s="17" t="n">
@@ -4783,104 +4837,104 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E35" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F35" s="17" t="inlineStr"/>
       <c r="G35" s="18" t="inlineStr">
         <is>
-          <t>Rusty Axe</t>
+          <t>Tower Shield</t>
         </is>
       </c>
       <c r="H35" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
+          <t>Deal 10 damage. Stun the enemy for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="25" t="inlineStr">
         <is>
-          <t>Shield Bash</t>
+          <t>Splash Strike</t>
         </is>
       </c>
       <c r="B36" s="26" t="inlineStr">
         <is>
-          <t>coup-de-bouclier</t>
+          <t>eclaboussure-de-frappe</t>
         </is>
       </c>
       <c r="C36" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E36" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E36" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr"/>
       <c r="G36" s="18" t="inlineStr">
         <is>
-          <t>Tower Shield</t>
+          <t>Forge Hammer</t>
         </is>
       </c>
       <c r="H36" s="18" t="inlineStr">
         <is>
-          <t>Deal 10 damage. Stun the enemy for 3 turns.</t>
+          <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="25" t="inlineStr">
         <is>
-          <t>Splash Strike</t>
+          <t>Strike</t>
         </is>
       </c>
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t>eclaboussure-de-frappe</t>
+          <t>frappe</t>
         </is>
       </c>
       <c r="C37" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" s="27" t="inlineStr">
         <is>
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E37" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr"/>
       <c r="G37" s="18" t="inlineStr">
         <is>
-          <t>Forge Hammer</t>
+          <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
         </is>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
+          <t>Deal 6 damage.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="25" t="inlineStr">
         <is>
-          <t>Strike</t>
+          <t>Venom Stab</t>
         </is>
       </c>
       <c r="B38" s="26" t="inlineStr">
         <is>
-          <t>frappe</t>
+          <t>coup-venimeux</t>
         </is>
       </c>
       <c r="C38" s="17" t="n">
@@ -4891,36 +4945,36 @@
           <t>Attaque</t>
         </is>
       </c>
-      <c r="E38" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E38" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F38" s="17" t="inlineStr"/>
       <c r="G38" s="18" t="inlineStr">
         <is>
-          <t>Rusty Axe, Forge Hammer, Miner's Pick</t>
+          <t>Basilisk Fang</t>
         </is>
       </c>
       <c r="H38" s="18" t="inlineStr">
         <is>
-          <t>Deal 6 damage.</t>
+          <t>Deal 4 damage. Apply 4 Poison.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>Venom Stab</t>
+          <t>Wound Opening</t>
         </is>
       </c>
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t>coup-venimeux</t>
+          <t>ouverture-des-plaies</t>
         </is>
       </c>
       <c r="C39" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" s="27" t="inlineStr">
         <is>
@@ -4940,27 +4994,27 @@
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>Deal 4 damage. Apply 4 Poison.</t>
+          <t>Deal 18 damage. Doubled if the target has a negative status.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="25" t="inlineStr">
         <is>
-          <t>Wound Opening</t>
+          <t>Armor of light</t>
         </is>
       </c>
       <c r="B40" s="26" t="inlineStr">
         <is>
-          <t>ouverture-des-plaies</t>
+          <t>armure-de-lumiere</t>
         </is>
       </c>
       <c r="C40" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D40" s="27" t="inlineStr">
-        <is>
-          <t>Attaque</t>
+        <v>1</v>
+      </c>
+      <c r="D40" s="29" t="inlineStr">
+        <is>
+          <t>Défense</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
@@ -4971,12 +5025,12 @@
       <c r="F40" s="17" t="inlineStr"/>
       <c r="G40" s="18" t="inlineStr">
         <is>
-          <t>Basilisk Fang</t>
+          <t>Crusader Plate</t>
         </is>
       </c>
       <c r="H40" s="18" t="inlineStr">
         <is>
-          <t>Deal 18 damage. Doubled if the target has a negative status.</t>
+          <t>Gain 6 Stone. Dazzle the nearest enemy (2 Confusion).</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5061,7 @@
       <c r="F41" s="17" t="inlineStr"/>
       <c r="G41" s="18" t="inlineStr">
         <is>
-          <t>— (deck de base)</t>
+          <t>— (non équipée)</t>
         </is>
       </c>
       <c r="H41" s="18" t="inlineStr">
@@ -5079,7 +5133,7 @@
       <c r="F43" s="17" t="inlineStr"/>
       <c r="G43" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>Forgemaster's Mail, Crusader Plate, Blood Plate</t>
         </is>
       </c>
       <c r="H43" s="18" t="inlineStr">
@@ -5091,48 +5145,48 @@
     <row r="44">
       <c r="A44" s="25" t="inlineStr">
         <is>
-          <t>Light Armor</t>
+          <t>Holy light</t>
         </is>
       </c>
       <c r="B44" s="26" t="inlineStr">
         <is>
-          <t>armure-legere</t>
+          <t>lumiere-sacree</t>
         </is>
       </c>
       <c r="C44" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E44" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E44" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F44" s="17" t="inlineStr"/>
       <c r="G44" s="18" t="inlineStr">
         <is>
-          <t>Traveler's Garb</t>
+          <t>Crusader Plate</t>
         </is>
       </c>
       <c r="H44" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Stone.</t>
+          <t>Heal 30 HP.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>Mail Armor</t>
+          <t>Light Armor</t>
         </is>
       </c>
       <c r="B45" s="26" t="inlineStr">
         <is>
-          <t>mail-armor</t>
+          <t>armure-legere</t>
         </is>
       </c>
       <c r="C45" s="17" t="n">
@@ -5143,108 +5197,108 @@
           <t>Défense</t>
         </is>
       </c>
-      <c r="E45" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F45" s="17" t="inlineStr"/>
       <c r="G45" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>Traveler's Garb</t>
         </is>
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
-          <t>Gain 7 Stone for every enemy still alive.</t>
+          <t>Gain 5 Stone.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>Onyx Armor</t>
+          <t>Mail Armor</t>
         </is>
       </c>
       <c r="B46" s="26" t="inlineStr">
         <is>
-          <t>onyx-armor</t>
+          <t>mail-armor</t>
         </is>
       </c>
       <c r="C46" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D46" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E46" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F46" s="17" t="inlineStr"/>
       <c r="G46" s="18" t="inlineStr">
         <is>
-          <t>Onyx Guard Plate</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H46" s="18" t="inlineStr">
         <is>
-          <t>Gain 30 Stone.</t>
+          <t>Gain 7 Stone for every enemy still alive.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>Quench</t>
+          <t>Onyx Armor</t>
         </is>
       </c>
       <c r="B47" s="26" t="inlineStr">
         <is>
-          <t>trempe</t>
+          <t>onyx-armor</t>
         </is>
       </c>
       <c r="C47" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D47" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E47" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F47" s="17" t="inlineStr"/>
       <c r="G47" s="18" t="inlineStr">
         <is>
-          <t>Forgemaster's Mail</t>
+          <t>Onyx Guard Plate</t>
         </is>
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>Spend all Forge Heat. Gain 10 Stone per Heat spent.</t>
+          <t>Gain 30 Stone.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>Sacred Ground</t>
+          <t>Quench</t>
         </is>
       </c>
       <c r="B48" s="26" t="inlineStr">
         <is>
-          <t>terre-sacree</t>
+          <t>trempe</t>
         </is>
       </c>
       <c r="C48" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D48" s="29" t="inlineStr">
         <is>
@@ -5259,12 +5313,12 @@
       <c r="F48" s="17" t="inlineStr"/>
       <c r="G48" s="18" t="inlineStr">
         <is>
-          <t>Crusader Plate</t>
+          <t>Forgemaster's Mail</t>
         </is>
       </c>
       <c r="H48" s="18" t="inlineStr">
         <is>
-          <t>Gain 18 Stone.</t>
+          <t>Spend all Forge Heat. Gain 10 Stone per Heat spent.</t>
         </is>
       </c>
     </row>
@@ -5280,16 +5334,16 @@
         </is>
       </c>
       <c r="C49" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" s="29" t="inlineStr">
         <is>
           <t>Défense</t>
         </is>
       </c>
-      <c r="E49" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E49" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F49" s="17" t="inlineStr"/>
@@ -5300,7 +5354,7 @@
       </c>
       <c r="H49" s="18" t="inlineStr">
         <is>
-          <t>Gain 1 Stone per Bleed among ALL enemies.</t>
+          <t>Per Bleed among ALL enemies: gain 3 Stone and heal 2 HP.</t>
         </is>
       </c>
     </row>
@@ -5379,48 +5433,48 @@
     <row r="52">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>Blood Rush</t>
+          <t>Blood Absorption</t>
         </is>
       </c>
       <c r="B52" s="26" t="inlineStr">
         <is>
-          <t>ruee-de-sang</t>
+          <t>absorption-de-sang</t>
         </is>
       </c>
       <c r="C52" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D52" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E52" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E52" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F52" s="17" t="inlineStr"/>
       <c r="G52" s="18" t="inlineStr">
         <is>
-          <t>Blood Greaves</t>
+          <t>Blood Gauntlets</t>
         </is>
       </c>
       <c r="H52" s="18" t="inlineStr">
         <is>
-          <t>Gain 1 Forge Heat per 5 Bleed among ALL enemies.</t>
+          <t>Heal 5 HP per Bleed among ALL enemies, then remove all their Bleed.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>Boost</t>
+          <t>Blood Rush</t>
         </is>
       </c>
       <c r="B53" s="26" t="inlineStr">
         <is>
-          <t>boost</t>
+          <t>ruee-de-sang</t>
         </is>
       </c>
       <c r="C53" s="17" t="n">
@@ -5439,84 +5493,84 @@
       <c r="F53" s="17" t="inlineStr"/>
       <c r="G53" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots, Mail Boots</t>
+          <t>Blood Greaves</t>
         </is>
       </c>
       <c r="H53" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Forge Heat (energy).</t>
+          <t>Gain 1 Forge Heat per 5 Bleed among ALL enemies.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>Burning Run</t>
+          <t>Boost</t>
         </is>
       </c>
       <c r="B54" s="26" t="inlineStr">
         <is>
-          <t>course-ardente</t>
+          <t>boost</t>
         </is>
       </c>
       <c r="C54" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D54" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E54" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F54" s="17" t="inlineStr"/>
       <c r="G54" s="18" t="inlineStr">
         <is>
-          <t>Onyx Boots</t>
+          <t>Onyx Boots, Mail Boots, Crusader Greaves, Blood Greaves</t>
         </is>
       </c>
       <c r="H54" s="18" t="inlineStr">
         <is>
-          <t>Haste for as many turns as your current Forge Heat.</t>
+          <t>Gain 3 Forge Heat (energy).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>Crusader's Charge</t>
+          <t>Burning Run</t>
         </is>
       </c>
       <c r="B55" s="26" t="inlineStr">
         <is>
-          <t>charge-du-croise</t>
+          <t>course-ardente</t>
         </is>
       </c>
       <c r="C55" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D55" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E55" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E55" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F55" s="17" t="inlineStr"/>
       <c r="G55" s="18" t="inlineStr">
         <is>
-          <t>Crusader Greaves</t>
+          <t>Onyx Boots</t>
         </is>
       </c>
       <c r="H55" s="18" t="inlineStr">
         <is>
-          <t>Haste: +30% attack speed for 3 turns.</t>
+          <t>Haste for as many turns as your current Forge Heat.</t>
         </is>
       </c>
     </row>
@@ -5631,12 +5685,12 @@
     <row r="59">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>Mail Advantage</t>
+          <t>Lay on Hands</t>
         </is>
       </c>
       <c r="B59" s="26" t="inlineStr">
         <is>
-          <t>avantage-maille</t>
+          <t>imposition-des-mains</t>
         </is>
       </c>
       <c r="C59" s="17" t="n">
@@ -5655,24 +5709,24 @@
       <c r="F59" s="17" t="inlineStr"/>
       <c r="G59" s="18" t="inlineStr">
         <is>
-          <t>Mail Glove, Mail Boots</t>
+          <t>Crusader Gauntlets</t>
         </is>
       </c>
       <c r="H59" s="18" t="inlineStr">
         <is>
-          <t>Gain 8 Stone and Haste for 2 turns.</t>
+          <t>Remove one random negative status from the hero.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>Master's Hand</t>
+          <t>Mail Advantage</t>
         </is>
       </c>
       <c r="B60" s="26" t="inlineStr">
         <is>
-          <t>main-de-maitre</t>
+          <t>avantage-maille</t>
         </is>
       </c>
       <c r="C60" s="17" t="n">
@@ -5683,180 +5737,180 @@
           <t>Buff</t>
         </is>
       </c>
-      <c r="E60" s="16" t="inlineStr">
-        <is>
-          <t>Common</t>
+      <c r="E60" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F60" s="17" t="inlineStr"/>
       <c r="G60" s="18" t="inlineStr">
         <is>
-          <t>Miner's Gloves, Mail Glove</t>
+          <t>Mail Glove, Mail Boots</t>
         </is>
       </c>
       <c r="H60" s="18" t="inlineStr">
         <is>
-          <t>Draw 2 cards.</t>
+          <t>Gain 8 Stone and Haste for 2 turns.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>Onyx Overheat</t>
+          <t>Master's Hand</t>
         </is>
       </c>
       <c r="B61" s="26" t="inlineStr">
         <is>
-          <t>onyx-overheat</t>
+          <t>main-de-maitre</t>
         </is>
       </c>
       <c r="C61" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D61" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E61" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>Common</t>
         </is>
       </c>
       <c r="F61" s="17" t="inlineStr"/>
       <c r="G61" s="18" t="inlineStr">
         <is>
-          <t>Big Onyx Sword</t>
+          <t>Miner's Gloves, Mail Glove, Crusader Gauntlets</t>
         </is>
       </c>
       <c r="H61" s="18" t="inlineStr">
         <is>
-          <t>Gain 5 Forge Heat (energy).</t>
+          <t>Draw 2 cards.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>Outnumbered</t>
+          <t>Onyx Overheat</t>
         </is>
       </c>
       <c r="B62" s="26" t="inlineStr">
         <is>
-          <t>surnombre</t>
+          <t>onyx-overheat</t>
         </is>
       </c>
       <c r="C62" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D62" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E62" s="21" t="inlineStr">
-        <is>
-          <t>Rare</t>
+      <c r="E62" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F62" s="17" t="inlineStr"/>
       <c r="G62" s="18" t="inlineStr">
         <is>
-          <t>Mail Glove</t>
+          <t>Big Onyx Sword</t>
         </is>
       </c>
       <c r="H62" s="18" t="inlineStr">
         <is>
-          <t>Draw 1 card per living enemy.</t>
+          <t>Gain 5 Forge Heat (energy).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Surge</t>
+          <t>Outnumbered</t>
         </is>
       </c>
       <c r="B63" s="26" t="inlineStr">
         <is>
-          <t>surge-saphir-parfait</t>
+          <t>surnombre</t>
         </is>
       </c>
       <c r="C63" s="17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D63" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E63" s="22" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="E63" s="21" t="inlineStr">
+        <is>
+          <t>Rare</t>
         </is>
       </c>
       <c r="F63" s="17" t="inlineStr"/>
       <c r="G63" s="18" t="inlineStr">
         <is>
-          <t>Perfect Sapphire Amulet</t>
+          <t>Mail Glove</t>
         </is>
       </c>
       <c r="H63" s="18" t="inlineStr">
         <is>
-          <t>Gain 3 Forge Heat (energy).</t>
+          <t>Draw 1 card per living enemy.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="25" t="inlineStr">
         <is>
-          <t>Quicken</t>
+          <t>Perfect Sapphire Surge</t>
         </is>
       </c>
       <c r="B64" s="26" t="inlineStr">
         <is>
-          <t>celerite-vive</t>
+          <t>surge-saphir-parfait</t>
         </is>
       </c>
       <c r="C64" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D64" s="30" t="inlineStr">
         <is>
           <t>Buff</t>
         </is>
       </c>
-      <c r="E64" s="20" t="inlineStr">
-        <is>
-          <t>Uncommon</t>
+      <c r="E64" s="22" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="F64" s="17" t="inlineStr"/>
       <c r="G64" s="18" t="inlineStr">
         <is>
-          <t>Swift Boots, Mail Boots</t>
+          <t>Perfect Sapphire Amulet</t>
         </is>
       </c>
       <c r="H64" s="18" t="inlineStr">
         <is>
-          <t>Haste: +30% attack speed for 3 turns.</t>
+          <t>Gain 3 Forge Heat (energy).</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="25" t="inlineStr">
         <is>
-          <t>Sapphire Surge</t>
+          <t>Quicken</t>
         </is>
       </c>
       <c r="B65" s="26" t="inlineStr">
         <is>
-          <t>surge-saphir</t>
+          <t>celerite-vive</t>
         </is>
       </c>
       <c r="C65" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D65" s="30" t="inlineStr">
         <is>
@@ -5871,24 +5925,24 @@
       <c r="F65" s="17" t="inlineStr"/>
       <c r="G65" s="18" t="inlineStr">
         <is>
-          <t>Sapphire Amulet, Nice Sapphire Amulet</t>
+          <t>Swift Boots, Mail Boots, Crusader Greaves, Blood Greaves</t>
         </is>
       </c>
       <c r="H65" s="18" t="inlineStr">
         <is>
-          <t>Gain 2 Forge Heat (energy).</t>
+          <t>Haste: +30% attack speed for 3 turns.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="25" t="inlineStr">
         <is>
-          <t>Second Wind</t>
+          <t>Sapphire Surge</t>
         </is>
       </c>
       <c r="B66" s="26" t="inlineStr">
         <is>
-          <t>second-souffle</t>
+          <t>surge-saphir</t>
         </is>
       </c>
       <c r="C66" s="17" t="n">
@@ -5907,10 +5961,46 @@
       <c r="F66" s="17" t="inlineStr"/>
       <c r="G66" s="18" t="inlineStr">
         <is>
+          <t>Sapphire Amulet, Nice Sapphire Amulet</t>
+        </is>
+      </c>
+      <c r="H66" s="18" t="inlineStr">
+        <is>
+          <t>Gain 2 Forge Heat (energy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="25" t="inlineStr">
+        <is>
+          <t>Second Wind</t>
+        </is>
+      </c>
+      <c r="B67" s="26" t="inlineStr">
+        <is>
+          <t>second-souffle</t>
+        </is>
+      </c>
+      <c r="C67" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="E67" s="20" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="F67" s="17" t="inlineStr"/>
+      <c r="G67" s="18" t="inlineStr">
+        <is>
           <t>Swift Boots</t>
         </is>
       </c>
-      <c r="H66" s="18" t="inlineStr">
+      <c r="H67" s="18" t="inlineStr">
         <is>
           <t>Trade 5 Haste turns for 3 Forge Heat. No effect below 5 Haste.</t>
         </is>
@@ -6038,7 +6128,7 @@
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>When hit by a melee attack, the attacker is Dazzled (1 Confusion).</t>
+          <t>When hit by a melee attack, the attacker has a 50% chance to be Dazzled (1 Confusion).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[technique] Excel des cartes : IDs des 2 nouvelles cartes + Forge from Ashes a jour
Get ahead -> id prendre-l-avance ; Opening Wounds -> id ouvrir-les-plaies ;
Forge from Ashes : cout 1 + nouvel effet. Les 150 cartes du tableau ont
desormais toutes un ID.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -3608,10 +3608,14 @@
       </c>
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>Opening wounds</t>
-        </is>
-      </c>
-      <c r="C59" s="15" t="n"/>
+          <t>Opening Wounds</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>ouvrir-les-plaies</t>
+        </is>
+      </c>
       <c r="D59" s="15" t="n">
         <v>2</v>
       </c>
@@ -7523,7 +7527,11 @@
           <t>Get ahead</t>
         </is>
       </c>
-      <c r="C147" s="15" t="n"/>
+      <c r="C147" s="15" t="inlineStr">
+        <is>
+          <t>prendre-l-avance</t>
+        </is>
+      </c>
       <c r="D147" s="15" t="n">
         <v>2</v>
       </c>
@@ -7550,7 +7558,7 @@
       </c>
       <c r="J147" s="16" t="inlineStr">
         <is>
-          <t>Gagne 3 haste et stun l'ennemi selectioné pendant 3 tours</t>
+          <t>Gain 3 Haste. Stun the target for 3 turns.</t>
         </is>
       </c>
     </row>
@@ -8201,7 +8209,7 @@
         </is>
       </c>
       <c r="D163" s="21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E163" s="21" t="inlineStr">
         <is>
@@ -8226,7 +8234,7 @@
       </c>
       <c r="J163" s="22" t="inlineStr">
         <is>
-          <t>Discard your hand and draw that many cards.</t>
+          <t>Discard your hand and draw double the discarded cards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[technique] Excel des cartes : colonne 'Visuel' (case verte = illustration presente)
Nouvelle colonne K a cote des cartes : case VERTE (✔) quand l'illustration
existe deja, ROUGE (✗) quand elle manque. Check-list d'un coup d'oeil :
146 cartes ont leur visuel, 4 restent a faire (Opening Wounds + les 3 cartes
par defaut Exposed / Bare Hands / Bare Foot).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,8 +83,12 @@
       <color rgb="FF006B5E"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1B4D1B"/>
+    </font>
   </fonts>
-  <fills count="28">
+  <fills count="30">
     <fill>
       <patternFill/>
     </fill>
@@ -221,6 +225,16 @@
         <fgColor rgb="FF40E0D0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF63BE7B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF08080"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -249,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -358,6 +372,15 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1026,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J171"/>
+  <dimension ref="A1:K171"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="57" min="1" max="1"/>
@@ -1039,6 +1062,7 @@
     <col width="6" customWidth="1" style="57" min="8" max="8"/>
     <col width="42" customWidth="1" style="57" min="9" max="9"/>
     <col width="58" customWidth="1" style="57" min="10" max="10"/>
+    <col width="8" customWidth="1" style="57" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.95" customHeight="1" s="57">
@@ -1097,6 +1121,11 @@
       <c r="J2" s="10" t="inlineStr">
         <is>
           <t>Effet</t>
+        </is>
+      </c>
+      <c r="K2" s="58" t="inlineStr">
+        <is>
+          <t>Visuel</t>
         </is>
       </c>
     </row>
@@ -1115,6 +1144,7 @@
       <c r="H3" s="12" t="n"/>
       <c r="I3" s="12" t="n"/>
       <c r="J3" s="12" t="n"/>
+      <c r="K3" s="11" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="57">
       <c r="A4" s="13" t="inlineStr">
@@ -1161,6 +1191,11 @@
           <t>Deal 3 damage.</t>
         </is>
       </c>
+      <c r="K4" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="57">
       <c r="A5" s="13" t="inlineStr">
@@ -1207,6 +1242,11 @@
           <t>Deal 4 damage twice.</t>
         </is>
       </c>
+      <c r="K5" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="57">
       <c r="A6" s="13" t="inlineStr">
@@ -1253,6 +1293,11 @@
           <t>Deal 12 damage.</t>
         </is>
       </c>
+      <c r="K6" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="57">
       <c r="A7" s="13" t="inlineStr">
@@ -1299,6 +1344,11 @@
           <t>Deal 3 damage twice. If the target dies, hit a random other enemy for 3.</t>
         </is>
       </c>
+      <c r="K7" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="57">
       <c r="A8" s="13" t="inlineStr">
@@ -1345,6 +1395,11 @@
           <t>Deal 7 damage to the target and the enemy behind it.</t>
         </is>
       </c>
+      <c r="K8" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="57">
       <c r="A9" s="13" t="inlineStr">
@@ -1391,6 +1446,11 @@
           <t>Deal 6 damage to the target and 4 damage to each adjacent enemy.</t>
         </is>
       </c>
+      <c r="K9" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="57">
       <c r="A10" s="13" t="inlineStr">
@@ -1437,6 +1497,11 @@
           <t>Deal 8 damage.</t>
         </is>
       </c>
+      <c r="K10" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="57">
       <c r="A11" s="13" t="inlineStr">
@@ -1483,6 +1548,11 @@
           <t>Deal 20 damage.</t>
         </is>
       </c>
+      <c r="K11" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="57">
       <c r="A12" s="13" t="inlineStr">
@@ -1529,6 +1599,11 @@
           <t>Deal 6 damage.</t>
         </is>
       </c>
+      <c r="K12" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="57">
       <c r="A13" s="15" t="inlineStr">
@@ -1575,6 +1650,11 @@
           <t>Deal 20 damage.</t>
         </is>
       </c>
+      <c r="K13" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="57">
       <c r="A14" s="15" t="inlineStr">
@@ -1621,6 +1701,11 @@
           <t>Deal 9 damage.</t>
         </is>
       </c>
+      <c r="K14" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="57">
       <c r="A15" s="15" t="inlineStr">
@@ -1667,6 +1752,11 @@
           <t>Deal 18 damage. Doubled if you have 6+ Strength.</t>
         </is>
       </c>
+      <c r="K15" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="57">
       <c r="A16" s="15" t="inlineStr">
@@ -1713,6 +1803,11 @@
           <t>Deal 10 damage. Doubled if the target is below 50% HP.</t>
         </is>
       </c>
+      <c r="K16" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="57">
       <c r="A17" s="15" t="inlineStr">
@@ -1759,6 +1854,11 @@
           <t>Deal 3 damage three times.</t>
         </is>
       </c>
+      <c r="K17" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="57">
       <c r="A18" s="15" t="inlineStr">
@@ -1805,6 +1905,11 @@
           <t>Deal 12 damage to the target and the enemy behind it.</t>
         </is>
       </c>
+      <c r="K18" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="57">
       <c r="A19" s="15" t="inlineStr">
@@ -1851,6 +1956,11 @@
           <t>Deal 14 damage. Lose 4 HP.</t>
         </is>
       </c>
+      <c r="K19" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="57">
       <c r="A20" s="15" t="inlineStr">
@@ -1897,6 +2007,11 @@
           <t>Deal 5 damage three times.</t>
         </is>
       </c>
+      <c r="K20" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="57">
       <c r="A21" s="15" t="inlineStr">
@@ -1943,6 +2058,11 @@
           <t>Deal 14 damage to the target and 6 to each adjacent enemy.</t>
         </is>
       </c>
+      <c r="K21" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="57">
       <c r="A22" s="15" t="inlineStr">
@@ -1993,6 +2113,11 @@
           <t>Deal 8 damage to ALL enemies. Et ajoute 2 saignement</t>
         </is>
       </c>
+      <c r="K22" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="57">
       <c r="A23" s="17" t="inlineStr">
@@ -2039,6 +2164,11 @@
           <t>Deal 30 damage. If the target dies, deal 15 damage to the next enemy.</t>
         </is>
       </c>
+      <c r="K23" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="57">
       <c r="A24" s="17" t="inlineStr">
@@ -2085,6 +2215,11 @@
           <t>Deal 16 damage. Doubled if the target has a negative status.</t>
         </is>
       </c>
+      <c r="K24" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="17.1" customHeight="1" s="57">
       <c r="A25" s="21" t="inlineStr">
@@ -2129,6 +2264,11 @@
       <c r="J25" s="21" t="inlineStr">
         <is>
           <t>Deal 30 damage. Doubled if the target is below 50% HP.</t>
+        </is>
+      </c>
+      <c r="K25" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -2147,6 +2287,7 @@
       <c r="H26" s="20" t="n"/>
       <c r="I26" s="20" t="n"/>
       <c r="J26" s="20" t="n"/>
+      <c r="K26" s="19" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="57">
       <c r="A27" s="13" t="inlineStr">
@@ -2193,6 +2334,11 @@
           <t>Deal 4 damage. Apply 2 Burning.</t>
         </is>
       </c>
+      <c r="K27" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="57">
       <c r="A28" s="13" t="inlineStr">
@@ -2239,6 +2385,11 @@
           <t>Remove 3 Burning from yourself.</t>
         </is>
       </c>
+      <c r="K28" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="57">
       <c r="A29" s="15" t="inlineStr">
@@ -2289,6 +2440,11 @@
           <t>Deal 5 damage and apply 3 Burning to ALL enemies.</t>
         </is>
       </c>
+      <c r="K29" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="57">
       <c r="A30" s="15" t="inlineStr">
@@ -2335,6 +2491,11 @@
           <t>Deal 6 damage. Apply 3 Burning.</t>
         </is>
       </c>
+      <c r="K30" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="57">
       <c r="A31" s="15" t="inlineStr">
@@ -2381,6 +2542,11 @@
           <t>Deal 15 damage. Each adjacent enemy has a 50% chance to take 5 Burning.</t>
         </is>
       </c>
+      <c r="K31" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="57">
       <c r="A32" s="21" t="inlineStr">
@@ -2431,6 +2597,11 @@
           <t>Convert ALL enemy statuses (positive and negative) to Burning, then double the Burning.</t>
         </is>
       </c>
+      <c r="K32" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="57">
       <c r="A33" s="21" t="inlineStr">
@@ -2481,6 +2652,11 @@
           <t>Apply 10 Burning to ALL enemies. Already-burning enemies take double, then their Burning is forged into Stone for you.</t>
         </is>
       </c>
+      <c r="K33" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="57">
       <c r="A34" s="21" t="inlineStr">
@@ -2527,6 +2703,11 @@
           <t>Discard your hand. For each card discarded, apply 8 Burning to a random enemy.</t>
         </is>
       </c>
+      <c r="K34" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="57">
       <c r="A35" s="21" t="inlineStr">
@@ -2573,6 +2754,11 @@
           <t>Haste for as many turns as your current Forge Heat.</t>
         </is>
       </c>
+      <c r="K35" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="57">
       <c r="A36" s="21" t="inlineStr">
@@ -2623,6 +2809,11 @@
           <t>Detonate all Burning: deal 2 damage per Burning on ALL enemies.</t>
         </is>
       </c>
+      <c r="K36" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="57">
       <c r="A37" s="21" t="inlineStr">
@@ -2669,6 +2860,11 @@
           <t>Convert 4 of your own Burning into 2 Forge Heat. No effect below 4 Burning.</t>
         </is>
       </c>
+      <c r="K37" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="57">
       <c r="A38" s="21" t="inlineStr">
@@ -2715,6 +2911,11 @@
           <t>Deal 12 damage. Apply 3 Burning.</t>
         </is>
       </c>
+      <c r="K38" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="57">
       <c r="A39" s="21" t="inlineStr">
@@ -2761,6 +2962,11 @@
           <t>Move all Burning from the target to the enemy behind it.</t>
         </is>
       </c>
+      <c r="K39" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="57">
       <c r="A40" s="21" t="inlineStr">
@@ -2811,6 +3017,11 @@
           <t>Spend all Forge Heat. Apply 8 Burning per Heat spent to ALL enemies.</t>
         </is>
       </c>
+      <c r="K40" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="57">
       <c r="A41" s="21" t="inlineStr">
@@ -2857,6 +3068,11 @@
           <t>Deal 28 damage. Apply 4 Burning.</t>
         </is>
       </c>
+      <c r="K41" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="57">
       <c r="A42" s="21" t="inlineStr">
@@ -2907,6 +3123,11 @@
           <t>Apply 20 Burning to ALL enemies.</t>
         </is>
       </c>
+      <c r="K42" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="57">
       <c r="A43" s="21" t="inlineStr">
@@ -2953,6 +3174,11 @@
           <t>Gain 10 Stone. Deal 10 damage and apply 3 Burning.</t>
         </is>
       </c>
+      <c r="K43" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="57">
       <c r="A44" s="21" t="inlineStr">
@@ -3003,6 +3229,11 @@
           <t>Apply 8 Burning to ALL enemies.</t>
         </is>
       </c>
+      <c r="K44" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="17.1" customHeight="1" s="57">
       <c r="A45" s="21" t="inlineStr">
@@ -3047,6 +3278,11 @@
       <c r="J45" s="22" t="inlineStr">
         <is>
           <t>Deal 26 damage and 4 Burning. The enemy behind takes half (13 damage, 2 Burning).</t>
+        </is>
+      </c>
+      <c r="K45" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -3065,6 +3301,7 @@
       <c r="H46" s="24" t="n"/>
       <c r="I46" s="24" t="n"/>
       <c r="J46" s="24" t="n"/>
+      <c r="K46" s="23" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="57">
       <c r="A47" s="13" t="inlineStr">
@@ -3115,6 +3352,11 @@
           <t>Apply 2 Poison to ALL enemies.</t>
         </is>
       </c>
+      <c r="K47" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="57">
       <c r="A48" s="13" t="inlineStr">
@@ -3161,6 +3403,11 @@
           <t>Deal 3 damage. Apply 4 Poison.</t>
         </is>
       </c>
+      <c r="K48" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="57">
       <c r="A49" s="15" t="inlineStr">
@@ -3211,6 +3458,11 @@
           <t>Apply 6 Poison to ALL enemies.</t>
         </is>
       </c>
+      <c r="K49" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="57">
       <c r="A50" s="15" t="inlineStr">
@@ -3257,6 +3509,11 @@
           <t>Deal 5 damage. Apply 5 Poison.</t>
         </is>
       </c>
+      <c r="K50" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="57">
       <c r="A51" s="17" t="inlineStr">
@@ -3307,6 +3564,11 @@
           <t>Hit ALL enemies 3 times for 3 damage. Apply 1 Poison per hit (2 if the enemy was already poisoned).</t>
         </is>
       </c>
+      <c r="K51" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="57">
       <c r="A52" s="17" t="inlineStr">
@@ -3353,6 +3615,11 @@
           <t>Inflige autant de degat physique que de dose de poison active sur la cible et au ennemi adjacent a la cible. Ajoute 2 poison aux cibles touché par cette carte.</t>
         </is>
       </c>
+      <c r="K52" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="17.1" customHeight="1" s="57">
       <c r="A53" s="17" t="inlineStr">
@@ -3397,6 +3664,11 @@
       <c r="J53" s="18" t="inlineStr">
         <is>
           <t>Deal 6 damage. Apply 4 Poison.</t>
+        </is>
+      </c>
+      <c r="K53" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -3415,6 +3687,7 @@
       <c r="H54" s="26" t="n"/>
       <c r="I54" s="26" t="n"/>
       <c r="J54" s="26" t="n"/>
+      <c r="K54" s="25" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="57">
       <c r="A55" s="13" t="inlineStr">
@@ -3461,6 +3734,11 @@
           <t>Deal 5 damage. Apply 2 Bleed.</t>
         </is>
       </c>
+      <c r="K55" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="57">
       <c r="A56" s="15" t="inlineStr">
@@ -3507,6 +3785,11 @@
           <t>Deal 3 damage. Apply 3 Bleed (stacks don't reset).</t>
         </is>
       </c>
+      <c r="K56" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="57">
       <c r="A57" s="15" t="inlineStr">
@@ -3553,6 +3836,11 @@
           <t>Deal 5 damage, apply 3 Bleed, and heal 3 HP.</t>
         </is>
       </c>
+      <c r="K57" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="57">
       <c r="A58" s="15" t="inlineStr">
@@ -3599,6 +3887,11 @@
           <t>Deal 6 damage. Apply 4 Bleed.</t>
         </is>
       </c>
+      <c r="K58" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="57">
       <c r="A59" s="15" t="inlineStr">
@@ -3645,6 +3938,11 @@
           <t>Deal 15 damage. Apply 4 bleed.</t>
         </is>
       </c>
+      <c r="K59" s="60" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="57">
       <c r="A60" s="15" t="inlineStr">
@@ -3695,6 +3993,11 @@
           <t>Deal 6 damage and apply 2 Bleed to ALL enemies.</t>
         </is>
       </c>
+      <c r="K60" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="57">
       <c r="A61" s="17" t="inlineStr">
@@ -3741,6 +4044,11 @@
           <t>Heal 5 HP per Bleed among ALL enemies, then remove all their Bleed.</t>
         </is>
       </c>
+      <c r="K61" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="57">
       <c r="A62" s="17" t="inlineStr">
@@ -3787,6 +4095,11 @@
           <t>Gain 1 Forge Heat per 5 Bleed among ALL enemies.</t>
         </is>
       </c>
+      <c r="K62" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="57">
       <c r="A63" s="17" t="inlineStr">
@@ -3837,6 +4150,11 @@
           <t>Stun for 2 turns every enemy that has Bleed.</t>
         </is>
       </c>
+      <c r="K63" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="57">
       <c r="A64" s="17" t="inlineStr">
@@ -3887,6 +4205,11 @@
           <t>Take 10 damage. Apply 5 Bleed to ALL enemies.</t>
         </is>
       </c>
+      <c r="K64" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="57">
       <c r="A65" s="17" t="inlineStr">
@@ -3933,6 +4256,11 @@
           <t>Both adjacent enemies match the target's Bleed.</t>
         </is>
       </c>
+      <c r="K65" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="57">
       <c r="A66" s="17" t="inlineStr">
@@ -3983,6 +4311,11 @@
           <t>Lose 20 HP. Deal 10 damage and 1 Bleed to ALL enemies. Heal 20 HP per enemy killed by this.</t>
         </is>
       </c>
+      <c r="K66" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="57">
       <c r="A67" s="17" t="inlineStr">
@@ -4033,6 +4366,11 @@
           <t>Deal 16 damage to ALL enemies. Apply 2 Bleed to ALL enemies.</t>
         </is>
       </c>
+      <c r="K67" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="57">
       <c r="A68" s="17" t="inlineStr">
@@ -4079,6 +4417,11 @@
           <t>Take 10 damage. Apply 4 Bleed on an ennemi target.</t>
         </is>
       </c>
+      <c r="K68" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="57">
       <c r="A69" s="17" t="inlineStr">
@@ -4125,6 +4468,11 @@
           <t>Per Bleed among ALL enemies: gain 3 Stone and heal 2 HP.</t>
         </is>
       </c>
+      <c r="K69" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="57">
       <c r="A70" s="21" t="inlineStr">
@@ -4171,6 +4519,11 @@
           <t>Deal 14 damage. Apply 3 Bleed.</t>
         </is>
       </c>
+      <c r="K70" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="17.1" customHeight="1" s="57">
       <c r="A71" s="21" t="inlineStr">
@@ -4219,6 +4572,11 @@
       <c r="J71" s="21" t="inlineStr">
         <is>
           <t>Deal 20 damage and apply 3 Bleed to ALL enemies.</t>
+        </is>
+      </c>
+      <c r="K71" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -4237,6 +4595,7 @@
       <c r="H72" s="28" t="n"/>
       <c r="I72" s="28" t="n"/>
       <c r="J72" s="28" t="n"/>
+      <c r="K72" s="27" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" s="57">
       <c r="A73" s="13" t="inlineStr">
@@ -4283,6 +4642,11 @@
           <t>Deal 5 damage. Chill: -30% speed for 2 turns.</t>
         </is>
       </c>
+      <c r="K73" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="57">
       <c r="A74" s="15" t="inlineStr">
@@ -4333,6 +4697,11 @@
           <t>Chill ALL enemies (-30% speed for 3 turns).</t>
         </is>
       </c>
+      <c r="K74" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="57">
       <c r="A75" s="15" t="inlineStr">
@@ -4379,6 +4748,11 @@
           <t>Deal 5 damage. Chill: -30% speed for 3 turns.</t>
         </is>
       </c>
+      <c r="K75" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="57">
       <c r="A76" s="16" t="inlineStr">
@@ -4425,6 +4799,11 @@
           <t>Deal 10 damage. Chill: -30% speed for 2 turns.</t>
         </is>
       </c>
+      <c r="K76" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="57">
       <c r="A77" s="15" t="inlineStr">
@@ -4471,6 +4850,11 @@
           <t>Deal 8 damage, +5 more if the target is Chilled.</t>
         </is>
       </c>
+      <c r="K77" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="17.1" customHeight="1" s="57">
       <c r="A78" s="17" t="inlineStr">
@@ -4515,6 +4899,11 @@
       <c r="J78" s="18" t="inlineStr">
         <is>
           <t>Deal 8 damage and apply 3 Chill. If the target was already chilled, cascade the same hit to the next enemy, and so on.</t>
+        </is>
+      </c>
+      <c r="K78" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -4533,6 +4922,7 @@
       <c r="H79" s="30" t="n"/>
       <c r="I79" s="30" t="n"/>
       <c r="J79" s="30" t="n"/>
+      <c r="K79" s="29" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1" s="57">
       <c r="A80" s="13" t="inlineStr">
@@ -4579,6 +4969,11 @@
           <t>Deal 14 damage. Apply 2 Confusion.</t>
         </is>
       </c>
+      <c r="K80" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="57">
       <c r="A81" s="13" t="inlineStr">
@@ -4625,6 +5020,11 @@
           <t>Apply 2 Confusion to the target.</t>
         </is>
       </c>
+      <c r="K81" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="57">
       <c r="A82" s="15" t="inlineStr">
@@ -4671,6 +5071,11 @@
           <t>Steal a random buff from the target enemy and apply it to yourself.</t>
         </is>
       </c>
+      <c r="K82" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="57">
       <c r="A83" s="17" t="inlineStr">
@@ -4717,6 +5122,11 @@
           <t>Gain 6 Stone. Apply 2 confusion to the nearest enemy.</t>
         </is>
       </c>
+      <c r="K83" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="57">
       <c r="A84" s="17" t="inlineStr">
@@ -4767,6 +5177,11 @@
           <t>Apply 2 Confusion to ALL enemies.</t>
         </is>
       </c>
+      <c r="K84" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="57">
       <c r="A85" s="17" t="inlineStr">
@@ -4817,6 +5232,11 @@
           <t>Apply 1 more Confusion to each already-confused enemy.</t>
         </is>
       </c>
+      <c r="K85" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="57">
       <c r="A86" s="17" t="inlineStr">
@@ -4863,6 +5283,11 @@
           <t>Deal 10 damage. Apply 1 Confusion.</t>
         </is>
       </c>
+      <c r="K86" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="57">
       <c r="A87" s="17" t="inlineStr">
@@ -4909,6 +5334,11 @@
           <t>Deal 12 damage. Stun the target for 1 turns.</t>
         </is>
       </c>
+      <c r="K87" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="57">
       <c r="A88" s="17" t="inlineStr">
@@ -4955,6 +5385,11 @@
           <t>Deal 40 damage. Stun the target for 2 turn.</t>
         </is>
       </c>
+      <c r="K88" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="57">
       <c r="A89" s="17" t="inlineStr">
@@ -5001,6 +5436,11 @@
           <t>Deal 8 damage. Stun the enemy for 3 turns.</t>
         </is>
       </c>
+      <c r="K89" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="17.1" customHeight="1" s="57">
       <c r="A90" s="17" t="inlineStr">
@@ -5049,6 +5489,11 @@
       <c r="J90" s="18" t="inlineStr">
         <is>
           <t>Deal 10 damage to ALL enemies. If you have 20+ Stone, stun them all for 1 turn.</t>
+        </is>
+      </c>
+      <c r="K90" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -5067,6 +5512,7 @@
       <c r="H91" s="32" t="n"/>
       <c r="I91" s="32" t="n"/>
       <c r="J91" s="32" t="n"/>
+      <c r="K91" s="31" t="n"/>
     </row>
     <row r="92" ht="15" customHeight="1" s="57">
       <c r="A92" s="13" t="inlineStr">
@@ -5113,6 +5559,11 @@
           <t>Gain 3 Stone.</t>
         </is>
       </c>
+      <c r="K92" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="57">
       <c r="A93" s="13" t="inlineStr">
@@ -5159,6 +5610,11 @@
           <t>Gain 5 Stone.</t>
         </is>
       </c>
+      <c r="K93" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="57">
       <c r="A94" s="13" t="inlineStr">
@@ -5205,6 +5661,11 @@
           <t>Gain 8 Stone.</t>
         </is>
       </c>
+      <c r="K94" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="57">
       <c r="A95" s="13" t="inlineStr">
@@ -5251,6 +5712,11 @@
           <t>Gain 6 Stone.</t>
         </is>
       </c>
+      <c r="K95" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="57">
       <c r="A96" s="13" t="inlineStr">
@@ -5297,6 +5763,11 @@
           <t>Gain 9 Stone.</t>
         </is>
       </c>
+      <c r="K96" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="57">
       <c r="A97" s="15" t="inlineStr">
@@ -5343,6 +5814,11 @@
           <t>Gain 12 Stone and 3 Regen.</t>
         </is>
       </c>
+      <c r="K97" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="57">
       <c r="A98" s="15" t="inlineStr">
@@ -5389,6 +5865,11 @@
           <t>Gain 12 Stone.</t>
         </is>
       </c>
+      <c r="K98" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="57">
       <c r="A99" s="15" t="inlineStr">
@@ -5435,6 +5916,11 @@
           <t>Deal damage equal to your Stone, then gain 8 Stone.</t>
         </is>
       </c>
+      <c r="K99" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="57">
       <c r="A100" s="15" t="inlineStr">
@@ -5481,6 +5967,11 @@
           <t>Deal 10 damage. Gain 8 Stone.</t>
         </is>
       </c>
+      <c r="K100" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="57">
       <c r="A101" s="15" t="inlineStr">
@@ -5527,6 +6018,11 @@
           <t>Gain 18 Stone.</t>
         </is>
       </c>
+      <c r="K101" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="57">
       <c r="A102" s="15" t="inlineStr">
@@ -5573,6 +6069,11 @@
           <t>Gain 23 Stone. Counts as three Stone cards for Stone Age combos.</t>
         </is>
       </c>
+      <c r="K102" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="57">
       <c r="A103" s="15" t="inlineStr">
@@ -5619,6 +6120,11 @@
           <t>Gain 4 Riposte: reflect melee damage you take back to the attacker. Lose 1 per trigger.</t>
         </is>
       </c>
+      <c r="K103" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="57">
       <c r="A104" s="15" t="inlineStr">
@@ -5665,6 +6171,11 @@
           <t>Gain 10 Stone.</t>
         </is>
       </c>
+      <c r="K104" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="57">
       <c r="A105" s="15" t="inlineStr">
@@ -5711,6 +6222,11 @@
           <t>Gain 7 Stone.</t>
         </is>
       </c>
+      <c r="K105" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="57">
       <c r="A106" s="15" t="inlineStr">
@@ -5757,6 +6273,11 @@
           <t>Gain 1 Stone for each Stone card played this combat (Many Stone counts as 3).</t>
         </is>
       </c>
+      <c r="K106" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="57">
       <c r="A107" s="15" t="inlineStr">
@@ -5803,6 +6324,11 @@
           <t>Deal damage equal to your current Stone.</t>
         </is>
       </c>
+      <c r="K107" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="57">
       <c r="A108" s="15" t="inlineStr">
@@ -5849,6 +6375,11 @@
           <t xml:space="preserve">Gain 12 Stone. </t>
         </is>
       </c>
+      <c r="K108" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="57">
       <c r="A109" s="17" t="inlineStr">
@@ -5895,6 +6426,11 @@
           <t>Gain 22 Stone.</t>
         </is>
       </c>
+      <c r="K109" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="57">
       <c r="A110" s="17" t="inlineStr">
@@ -5941,6 +6477,11 @@
           <t>Gain 8 Stone and Haste for 2 turns.</t>
         </is>
       </c>
+      <c r="K110" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="57">
       <c r="A111" s="17" t="inlineStr">
@@ -5987,6 +6528,11 @@
           <t>Gain 7 Stone for every enemy still alive.</t>
         </is>
       </c>
+      <c r="K111" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="57">
       <c r="A112" s="17" t="inlineStr">
@@ -6033,6 +6579,11 @@
           <t>Spend all Forge Heat. Gain 10 Stone per Heat spent.</t>
         </is>
       </c>
+      <c r="K112" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="57">
       <c r="A113" s="17" t="inlineStr">
@@ -6079,6 +6630,11 @@
           <t>Double your current Stone.</t>
         </is>
       </c>
+      <c r="K113" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="57">
       <c r="A114" s="17" t="inlineStr">
@@ -6125,6 +6681,11 @@
           <t>Deal damage equal to your Stone, then gain 10 Stone.</t>
         </is>
       </c>
+      <c r="K114" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="17.1" customHeight="1" s="57">
       <c r="A115" s="21" t="inlineStr">
@@ -6171,6 +6732,11 @@
           <t>Gain 30 Stone.</t>
         </is>
       </c>
+      <c r="K115" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="57">
       <c r="A116" s="13" t="inlineStr">
@@ -6215,6 +6781,11 @@
       <c r="J116" s="14" t="inlineStr">
         <is>
           <t>Gain 2 Stone.</t>
+        </is>
+      </c>
+      <c r="K116" s="60" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -6233,6 +6804,7 @@
       <c r="H117" s="34" t="n"/>
       <c r="I117" s="34" t="n"/>
       <c r="J117" s="34" t="n"/>
+      <c r="K117" s="33" t="n"/>
     </row>
     <row r="118" ht="15" customHeight="1" s="57">
       <c r="A118" s="13" t="inlineStr">
@@ -6279,6 +6851,11 @@
           <t>Gain 3 Regen. Each turn: heal that many HP, then lose 1 Regen.</t>
         </is>
       </c>
+      <c r="K118" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="57">
       <c r="A119" s="15" t="inlineStr">
@@ -6325,6 +6902,11 @@
           <t>Consume the target's Bleed: heal that many HP. Gain 1 Forge Heat.</t>
         </is>
       </c>
+      <c r="K119" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="15" customHeight="1" s="57">
       <c r="A120" s="15" t="inlineStr">
@@ -6371,6 +6953,11 @@
           <t>Deal 12 damage. Remove a random buff from the target; if one was removed, gain 4 Regen.</t>
         </is>
       </c>
+      <c r="K120" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="15" customHeight="1" s="57">
       <c r="A121" s="15" t="inlineStr">
@@ -6421,6 +7008,11 @@
           <t>Deal 6 damage to ALL enemies. Heal 4 HP per enemy hit.</t>
         </is>
       </c>
+      <c r="K121" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="15" customHeight="1" s="57">
       <c r="A122" s="17" t="inlineStr">
@@ -6467,6 +7059,11 @@
           <t>Heal 30 HP.</t>
         </is>
       </c>
+      <c r="K122" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="57">
       <c r="A123" s="17" t="inlineStr">
@@ -6513,6 +7110,11 @@
           <t>Remove a random buff from the target. If one was removed, gain 4 Regen.</t>
         </is>
       </c>
+      <c r="K123" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="17.1" customHeight="1" s="57">
       <c r="A124" s="21" t="inlineStr">
@@ -6559,6 +7161,11 @@
           <t>Heal 10 HP per enemy that has Bleed.</t>
         </is>
       </c>
+      <c r="K124" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="15" customHeight="1" s="57">
       <c r="A125" s="21" t="inlineStr">
@@ -6603,6 +7210,11 @@
       <c r="J125" s="22" t="inlineStr">
         <is>
           <t>Deal 15 damage. If the target dies, gain 4 Strength and heal 20 HP.</t>
+        </is>
+      </c>
+      <c r="K125" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -6621,6 +7233,7 @@
       <c r="H126" s="36" t="n"/>
       <c r="I126" s="36" t="n"/>
       <c r="J126" s="36" t="n"/>
+      <c r="K126" s="35" t="n"/>
     </row>
     <row r="127" ht="15" customHeight="1" s="57">
       <c r="A127" s="13" t="inlineStr">
@@ -6667,6 +7280,11 @@
           <t>Gain 0 to 3 Forge Heat at random.</t>
         </is>
       </c>
+      <c r="K127" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="15" customHeight="1" s="57">
       <c r="A128" s="13" t="inlineStr">
@@ -6713,6 +7331,11 @@
           <t>Gain 1 Forge Heat (energy).</t>
         </is>
       </c>
+      <c r="K128" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="15" customHeight="1" s="57">
       <c r="A129" s="15" t="inlineStr">
@@ -6759,6 +7382,11 @@
           <t>Deal 6 damage. Gain 2 Forge Heat.</t>
         </is>
       </c>
+      <c r="K129" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="15" customHeight="1" s="57">
       <c r="A130" s="15" t="inlineStr">
@@ -6809,6 +7437,11 @@
           <t>Deal 4 damage to ALL enemies. Gain 2 Forge Heat.</t>
         </is>
       </c>
+      <c r="K130" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="15" customHeight="1" s="57">
       <c r="A131" s="15" t="inlineStr">
@@ -6855,6 +7488,11 @@
           <t>Gain 3 Forge Heat (energy).</t>
         </is>
       </c>
+      <c r="K131" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="15" customHeight="1" s="57">
       <c r="A132" s="15" t="inlineStr">
@@ -6901,6 +7539,11 @@
           <t>Draw 1 card. Gain 2 Forge Heat.</t>
         </is>
       </c>
+      <c r="K132" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="15" customHeight="1" s="57">
       <c r="A133" s="15" t="inlineStr">
@@ -6947,6 +7590,11 @@
           <t>Gain 1 Forge Heat per 8 Stone cards played this combat (min 1, max 6).</t>
         </is>
       </c>
+      <c r="K133" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="15" customHeight="1" s="57">
       <c r="A134" s="15" t="inlineStr">
@@ -6993,6 +7641,11 @@
           <t>Gain 4 Forge Heat (energy).</t>
         </is>
       </c>
+      <c r="K134" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="15" customHeight="1" s="57">
       <c r="A135" s="15" t="inlineStr">
@@ -7039,6 +7692,11 @@
           <t>Gain 1 to 5 Forge Heat at random.</t>
         </is>
       </c>
+      <c r="K135" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="15" customHeight="1" s="57">
       <c r="A136" s="15" t="inlineStr">
@@ -7085,6 +7743,11 @@
           <t>Gain 2 Forge Heat (energy).</t>
         </is>
       </c>
+      <c r="K136" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="15" customHeight="1" s="57">
       <c r="A137" s="15" t="inlineStr">
@@ -7131,6 +7794,11 @@
           <t>Trade 5 Haste turns for 3 Forge Heat. No effect below 5 Haste.</t>
         </is>
       </c>
+      <c r="K137" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="17.1" customHeight="1" s="57">
       <c r="A138" s="21" t="inlineStr">
@@ -7177,6 +7845,11 @@
           <t>Gain 5 Forge Heat (energy).</t>
         </is>
       </c>
+      <c r="K138" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="15" customHeight="1" s="57">
       <c r="A139" s="21" t="inlineStr">
@@ -7221,6 +7894,11 @@
       <c r="J139" s="22" t="inlineStr">
         <is>
           <t>Gain 3 Forge Heat (energy).</t>
+        </is>
+      </c>
+      <c r="K139" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -7239,6 +7917,7 @@
       <c r="H140" s="38" t="n"/>
       <c r="I140" s="38" t="n"/>
       <c r="J140" s="38" t="n"/>
+      <c r="K140" s="37" t="n"/>
     </row>
     <row r="141" ht="15" customHeight="1" s="57">
       <c r="A141" s="13" t="inlineStr">
@@ -7285,6 +7964,11 @@
           <t>Gain 2 Haste.</t>
         </is>
       </c>
+      <c r="K141" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="15" customHeight="1" s="57">
       <c r="A142" s="13" t="inlineStr">
@@ -7331,6 +8015,11 @@
           <t>Haste for 4 of your turns.</t>
         </is>
       </c>
+      <c r="K142" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="15" customHeight="1" s="57">
       <c r="A143" s="13" t="inlineStr">
@@ -7377,6 +8066,11 @@
           <t>Each of your turns, gain 1 permanent Haste (it builds up all combat). Stacks when replayed.</t>
         </is>
       </c>
+      <c r="K143" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="15" customHeight="1" s="57">
       <c r="A144" s="15" t="inlineStr">
@@ -7423,6 +8117,11 @@
           <t>Haste for 3 turns. Draw 1 card.</t>
         </is>
       </c>
+      <c r="K144" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="17.1" customHeight="1" s="57">
       <c r="A145" s="15" t="inlineStr">
@@ -7469,6 +8168,11 @@
           <t>Gain 4 Haste. Each stack: +5% speed. Lose 1 per turn.</t>
         </is>
       </c>
+      <c r="K145" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="17.1" customHeight="1" s="57">
       <c r="A146" s="15" t="inlineStr">
@@ -7515,6 +8219,11 @@
           <t>Take an extra turn right after this one.</t>
         </is>
       </c>
+      <c r="K146" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="15" customHeight="1" s="57">
       <c r="A147" s="15" t="inlineStr">
@@ -7561,6 +8270,11 @@
           <t>Gain 3 Haste. Stun the target for 3 turns.</t>
         </is>
       </c>
+      <c r="K147" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="15" customHeight="1" s="57">
       <c r="A148" s="13" t="inlineStr">
@@ -7605,6 +8319,11 @@
       <c r="J148" s="14" t="inlineStr">
         <is>
           <t>Gain 2 Haste.</t>
+        </is>
+      </c>
+      <c r="K148" s="60" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
     </row>
@@ -7623,6 +8342,7 @@
       <c r="H149" s="40" t="n"/>
       <c r="I149" s="40" t="n"/>
       <c r="J149" s="40" t="n"/>
+      <c r="K149" s="39" t="n"/>
     </row>
     <row r="150" ht="15" customHeight="1" s="57">
       <c r="A150" s="13" t="inlineStr">
@@ -7669,6 +8389,11 @@
           <t>Gain 2 Strength (+2 damage to every attack this combat).</t>
         </is>
       </c>
+      <c r="K150" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="15" customHeight="1" s="57">
       <c r="A151" s="15" t="inlineStr">
@@ -7715,6 +8440,11 @@
           <t>Gain 3 Strength.</t>
         </is>
       </c>
+      <c r="K151" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="15" customHeight="1" s="57">
       <c r="A152" s="15" t="inlineStr">
@@ -7761,6 +8491,11 @@
           <t>Deal 14 damage. Gain 3 Strength.</t>
         </is>
       </c>
+      <c r="K152" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="17.1" customHeight="1" s="57">
       <c r="A153" s="15" t="inlineStr">
@@ -7807,6 +8542,11 @@
           <t>Gain 4 Strength.</t>
         </is>
       </c>
+      <c r="K153" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="15" customHeight="1" s="57">
       <c r="A154" s="15" t="inlineStr">
@@ -7853,6 +8593,11 @@
           <t>Gain 4 Strength. Draw 2 cards.</t>
         </is>
       </c>
+      <c r="K154" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="15" customHeight="1" s="57">
       <c r="A155" s="15" t="inlineStr">
@@ -7897,6 +8642,11 @@
       <c r="J155" s="16" t="inlineStr">
         <is>
           <t>Gain 3 Strength. Draw 1 card.</t>
+        </is>
+      </c>
+      <c r="K155" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -7915,6 +8665,7 @@
       <c r="H156" s="42" t="n"/>
       <c r="I156" s="42" t="n"/>
       <c r="J156" s="42" t="n"/>
+      <c r="K156" s="41" t="n"/>
     </row>
     <row r="157" ht="15" customHeight="1" s="57">
       <c r="A157" s="13" t="inlineStr">
@@ -7961,6 +8712,11 @@
           <t>Draw 2 cards.</t>
         </is>
       </c>
+      <c r="K157" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="15" customHeight="1" s="57">
       <c r="A158" s="13" t="inlineStr">
@@ -8007,6 +8763,11 @@
           <t>Draw 1 card. Gain Stone equal to twice its cost.</t>
         </is>
       </c>
+      <c r="K158" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="15" customHeight="1" s="57">
       <c r="A159" s="15" t="inlineStr">
@@ -8053,6 +8814,11 @@
           <t>Draw 3 cards. Keep those costing less than 3 Forge Heat, discard the rest.</t>
         </is>
       </c>
+      <c r="K159" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="15" customHeight="1" s="57">
       <c r="A160" s="15" t="inlineStr">
@@ -8099,6 +8865,11 @@
           <t>Draw 1 card per 6 Stone cards played this combat (min 1, max 6).</t>
         </is>
       </c>
+      <c r="K160" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="15" customHeight="1" s="57">
       <c r="A161" s="15" t="inlineStr">
@@ -8145,6 +8916,11 @@
           <t>Draw 2 cards. Gain 1 Forge Heat.</t>
         </is>
       </c>
+      <c r="K161" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="15" customHeight="1" s="57">
       <c r="A162" s="17" t="inlineStr">
@@ -8191,6 +8967,11 @@
           <t>Draw 1 card per living enemy.</t>
         </is>
       </c>
+      <c r="K162" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="15" customHeight="1" s="57">
       <c r="A163" s="21" t="inlineStr">
@@ -8237,6 +9018,11 @@
           <t>Discard your hand and draw double the discarded cards.</t>
         </is>
       </c>
+      <c r="K163" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="15" customHeight="1" s="57">
       <c r="A164" s="13" t="inlineStr">
@@ -8281,6 +9067,11 @@
       <c r="J164" s="14" t="inlineStr">
         <is>
           <t>Discard 1 card, then draw 1.</t>
+        </is>
+      </c>
+      <c r="K164" s="60" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[visuel] Illustrations des 3 cartes par defaut optimisees + colonne Visuel a jour
exposed / bare-hands / bare-foot uploadees par Brioche, converties en WebP
(6 Mo -> 0,5 Mo). Les 3 cartes par defaut ont desormais leur illustration :
149/150 cartes ont un visuel, il ne reste qu'Opening Wounds. Colonne 'Visuel'
de l'Excel regeneree en consequence (3 cases passees au vert).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -6783,9 +6783,9 @@
           <t>Gain 2 Stone.</t>
         </is>
       </c>
-      <c r="K116" s="60" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="K116" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -8321,9 +8321,9 @@
           <t>Gain 2 Haste.</t>
         </is>
       </c>
-      <c r="K148" s="60" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="K148" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>
@@ -9069,9 +9069,9 @@
           <t>Discard 1 card, then draw 1.</t>
         </is>
       </c>
-      <c r="K164" s="60" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="K164" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[visuel] Opening Wounds : illustration optimisee (WebP) + colonne Visuel 150/150
Derniere illustration manquante uploadee par Brioche, convertie en WebP
(2 Mo -> 0,2 Mo) et liee a la carte. TOUTES les cartes ont desormais leur
visuel : la colonne 'Visuel' de l'Excel est entierement verte (150/150).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -3938,9 +3938,9 @@
           <t>Deal 15 damage. Apply 4 bleed.</t>
         </is>
       </c>
-      <c r="K59" s="60" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="K59" s="59" t="inlineStr">
+        <is>
+          <t>✔</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[technique] Table de valeur editable aussi pour les ressources
Meme workflow que la valeur des objets, applique aux ressources (minerais +
bois + cuir) : nouvel onglet « Ressources » dans le classeur -> VALEUR_RESSOURCE
dans jeu/data/valeurs.js, regenere par outils/importer_valeurs.py (l'importer
lit maintenant les DEUX onglets et ecrit VALEUR_OBJET + VALEUR_RESSOURCE).

prixBaseRessource() lit d'abord cette table, avec l'ancien bareme par rang en
secours. Les valeurs semees reprennent EXACTEMENT les prix actuels -> aucun
changement de balance, mais Brioche peut desormais ajuster le prix de base de
chaque ressource a la main dans l'Excel.

Verifie : les 19 prix de base ressource sont identiques a avant, page chargee
sans erreur JS. Docs a jour (concept.md, marche.md).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Effets" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Recettes" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Valeurs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Ressources" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -24538,4 +24539,405 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="57" min="1" max="1"/>
+    <col width="16" customWidth="1" style="57" min="2" max="2"/>
+    <col width="8" customWidth="1" style="57" min="3" max="3"/>
+    <col width="12" customWidth="1" style="57" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t>VALEUR DES RESSOURCES — SOURCE ÉDITABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="62" t="inlineStr">
+        <is>
+          <t>Édite la colonne « Valeur » (D), puis lance : python3 outils/importer_valeurs.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="62" t="inlineStr">
+        <is>
+          <t>Valeur = prix de BASE au marché (le marché la fait ensuite fluctuer). Ce sont les prix ACTUELS, à ajuster librement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="85" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B6" s="85" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="C6" s="85" t="inlineStr">
+        <is>
+          <t>Rang</t>
+        </is>
+      </c>
+      <c r="D6" s="85" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="86" t="inlineStr">
+        <is>
+          <t>pierre-taillee</t>
+        </is>
+      </c>
+      <c r="B7" s="87" t="inlineStr">
+        <is>
+          <t>Cut Stone</t>
+        </is>
+      </c>
+      <c r="C7" s="88" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="85" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="86" t="inlineStr">
+        <is>
+          <t>charbon</t>
+        </is>
+      </c>
+      <c r="B8" s="87" t="inlineStr">
+        <is>
+          <t>Coal</t>
+        </is>
+      </c>
+      <c r="C8" s="88" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="85" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="86" t="inlineStr">
+        <is>
+          <t>cuivre</t>
+        </is>
+      </c>
+      <c r="B9" s="87" t="inlineStr">
+        <is>
+          <t>Copper</t>
+        </is>
+      </c>
+      <c r="C9" s="88" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="85" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="86" t="inlineStr">
+        <is>
+          <t>fer</t>
+        </is>
+      </c>
+      <c r="B10" s="87" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="C10" s="88" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="85" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="86" t="inlineStr">
+        <is>
+          <t>argent</t>
+        </is>
+      </c>
+      <c r="B11" s="87" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="C11" s="89" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" s="85" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="86" t="inlineStr">
+        <is>
+          <t>or</t>
+        </is>
+      </c>
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C12" s="89" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" s="85" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="86" t="inlineStr">
+        <is>
+          <t>malachite</t>
+        </is>
+      </c>
+      <c r="B13" s="87" t="inlineStr">
+        <is>
+          <t>Malachite</t>
+        </is>
+      </c>
+      <c r="C13" s="90" t="n">
+        <v>7</v>
+      </c>
+      <c r="D13" s="85" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="86" t="inlineStr">
+        <is>
+          <t>lapis</t>
+        </is>
+      </c>
+      <c r="B14" s="87" t="inlineStr">
+        <is>
+          <t>Lapis Lazuli</t>
+        </is>
+      </c>
+      <c r="C14" s="90" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" s="85" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="86" t="inlineStr">
+        <is>
+          <t>amethyste</t>
+        </is>
+      </c>
+      <c r="B15" s="87" t="inlineStr">
+        <is>
+          <t>Amethyst</t>
+        </is>
+      </c>
+      <c r="C15" s="90" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="85" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="86" t="inlineStr">
+        <is>
+          <t>titane</t>
+        </is>
+      </c>
+      <c r="B16" s="87" t="inlineStr">
+        <is>
+          <t>Titanium</t>
+        </is>
+      </c>
+      <c r="C16" s="90" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="85" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="86" t="inlineStr">
+        <is>
+          <t>emeraude</t>
+        </is>
+      </c>
+      <c r="B17" s="87" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="C17" s="90" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" s="85" t="n">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="86" t="inlineStr">
+        <is>
+          <t>rubis</t>
+        </is>
+      </c>
+      <c r="B18" s="87" t="inlineStr">
+        <is>
+          <t>Ruby</t>
+        </is>
+      </c>
+      <c r="C18" s="90" t="n">
+        <v>9</v>
+      </c>
+      <c r="D18" s="85" t="n">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="86" t="inlineStr">
+        <is>
+          <t>saphir</t>
+        </is>
+      </c>
+      <c r="B19" s="87" t="inlineStr">
+        <is>
+          <t>Sapphire</t>
+        </is>
+      </c>
+      <c r="C19" s="91" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" s="85" t="n">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="86" t="inlineStr">
+        <is>
+          <t>diamant</t>
+        </is>
+      </c>
+      <c r="B20" s="87" t="inlineStr">
+        <is>
+          <t>Diamond</t>
+        </is>
+      </c>
+      <c r="C20" s="91" t="n">
+        <v>11</v>
+      </c>
+      <c r="D20" s="85" t="n">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="86" t="inlineStr">
+        <is>
+          <t>mithril</t>
+        </is>
+      </c>
+      <c r="B21" s="87" t="inlineStr">
+        <is>
+          <t>Mithril</t>
+        </is>
+      </c>
+      <c r="C21" s="91" t="n">
+        <v>11</v>
+      </c>
+      <c r="D21" s="85" t="n">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="86" t="inlineStr">
+        <is>
+          <t>onyx</t>
+        </is>
+      </c>
+      <c r="B22" s="87" t="inlineStr">
+        <is>
+          <t>Onyx</t>
+        </is>
+      </c>
+      <c r="C22" s="91" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="85" t="n">
+        <v>1928</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="86" t="inlineStr">
+        <is>
+          <t>pierre-solaire</t>
+        </is>
+      </c>
+      <c r="B23" s="87" t="inlineStr">
+        <is>
+          <t>Sunstone</t>
+        </is>
+      </c>
+      <c r="C23" s="91" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" s="85" t="n">
+        <v>1928</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="86" t="inlineStr">
+        <is>
+          <t>bois</t>
+        </is>
+      </c>
+      <c r="B24" s="87" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="C24" s="88" t="inlineStr"/>
+      <c r="D24" s="85" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="86" t="inlineStr">
+        <is>
+          <t>cuir</t>
+        </is>
+      </c>
+      <c r="B25" s="87" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="C25" s="88" t="inlineStr"/>
+      <c r="D25" s="85" t="n">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[gameplay] Trois paliers de bois et de cuir (commun / uncommon / rare)
Ajout des paliers superieurs pour les deux ressources de craft :
- Cuir : Leather (commun, existant) -> Thick Leather (uncommon) -> Strange
  Leather (rare).
- Bois : Wood (commun, existant) -> Dark Wood (uncommon) -> Enchanted Wood
  (rare).

Nouvelles ressources dans data/items.js (categorie ressource, meme famille
cuir/bois, hors MINERAIS donc jamais dans les veines). Valeurs de base ajoutees
a l'onglet « Ressources » du classeur -> valeurs.js (Thick Leather 40, Strange
Leather 130, Dark Wood 35, Enchanted Wood 120), editables comme le reste.

Pretes a etre utilisees dans les recettes et les tables de butin par famille
selon la rarete de l'objet. Verifie : prix corrects, hors pool de minerai, page
chargee sans erreur JS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -24547,7 +24547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="57" min="1" max="1"/>
@@ -24937,6 +24937,70 @@
         <v>7</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="86" t="inlineStr">
+        <is>
+          <t>cuir-epais</t>
+        </is>
+      </c>
+      <c r="B26" s="87" t="inlineStr">
+        <is>
+          <t>Thick Leather</t>
+        </is>
+      </c>
+      <c r="C26" s="89" t="inlineStr"/>
+      <c r="D26" s="85" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="86" t="inlineStr">
+        <is>
+          <t>cuir-etrange</t>
+        </is>
+      </c>
+      <c r="B27" s="87" t="inlineStr">
+        <is>
+          <t>Strange Leather</t>
+        </is>
+      </c>
+      <c r="C27" s="90" t="inlineStr"/>
+      <c r="D27" s="85" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="86" t="inlineStr">
+        <is>
+          <t>bois-sombre</t>
+        </is>
+      </c>
+      <c r="B28" s="87" t="inlineStr">
+        <is>
+          <t>Dark Wood</t>
+        </is>
+      </c>
+      <c r="C28" s="89" t="inlineStr"/>
+      <c r="D28" s="85" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="86" t="inlineStr">
+        <is>
+          <t>bois-enchante</t>
+        </is>
+      </c>
+      <c r="B29" s="87" t="inlineStr">
+        <is>
+          <t>Enchanted Wood</t>
+        </is>
+      </c>
+      <c r="C29" s="90" t="inlineStr"/>
+      <c r="D29" s="85" t="n">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[gameplay] Loot de profondeur « Depth Portal » : garantit une porte de descente sur l'étage
Nouveau butin de run (🕳 Depth Portal, effet « porte ») dans le pool de choix : au
lieu d'un buff chiffré, il GARANTIT un passage `>` vers l'étage suivant sur l'étage
courant — posé au runtime sur une case sol libre (loin du départ) si l'étage n'en
avait pas. Complète le talent Deep Experience (chance) par une garantie ponctuelle.

- Excel « Profondeurs » + importer (effet « porte » autorisé) → data/profondeur.js.
- ui/profondeur.js : libellé « Guaranteed passage ».
- principal.js : garantirPorteCourante() + branche « porte » dans le choix (n'accumule
  pas, action unique). Idempotent (ne double pas une porte existante).

Vérifié : loot présent (~20% des choix), mutation pose bien une porte, 2e appel ne
double pas.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -25190,7 +25190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="57" min="1" max="1"/>
@@ -25391,6 +25391,37 @@
         <v>50</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>portail-profondeur</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Depth Portal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>porte</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>#5fd08a</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[technique] Stats des monstres éditables dans l'Excel (onglet « Monstres »)
Nouvel onglet « Monstres » (pv, attaque, xp, vitesse, niveau, famille + une
colonne d'actions spéciales « type:valeur:poids ») + outils/importer_monstres.py
qui régénère le bloc STATS_MONSTRES de data/ennemis.js. Ces stats REMPLACENT les
valeurs de secours du code : Brioche règle l'équilibrage dans l'Excel sans toucher
au code (l'art/technique du monstre, lui, reste dans le code).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Recettes" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Profondeurs" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Profondeurs-chances" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Monstres" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="60">
+  <fills count="61">
     <fill>
       <patternFill/>
     </fill>
@@ -414,6 +420,11 @@
         <fgColor rgb="002E2A22"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -456,7 +467,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -673,6 +684,8 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="59" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="60" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1402,6 +1415,258 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="57" min="1" max="1"/>
+    <col width="20" customWidth="1" style="57" min="2" max="2"/>
+    <col width="8" customWidth="1" style="57" min="3" max="3"/>
+    <col width="12" customWidth="1" style="57" min="4" max="4"/>
+    <col width="7" customWidth="1" style="57" min="5" max="5"/>
+    <col width="9" customWidth="1" style="57" min="6" max="6"/>
+    <col width="7" customWidth="1" style="57" min="7" max="7"/>
+    <col width="9" customWidth="1" style="57" min="8" max="8"/>
+    <col width="52" customWidth="1" style="57" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="100" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="100" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="C1" s="100" t="inlineStr">
+        <is>
+          <t>niveau</t>
+        </is>
+      </c>
+      <c r="D1" s="100" t="inlineStr">
+        <is>
+          <t>famille</t>
+        </is>
+      </c>
+      <c r="E1" s="100" t="inlineStr">
+        <is>
+          <t>pv</t>
+        </is>
+      </c>
+      <c r="F1" s="100" t="inlineStr">
+        <is>
+          <t>attaque</t>
+        </is>
+      </c>
+      <c r="G1" s="100" t="inlineStr">
+        <is>
+          <t>xp</t>
+        </is>
+      </c>
+      <c r="H1" s="100" t="inlineStr">
+        <is>
+          <t>vitesse</t>
+        </is>
+      </c>
+      <c r="I1" s="100" t="inlineStr">
+        <is>
+          <t>actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="101" t="inlineStr">
+        <is>
+          <t>identifiant (ne pas changer)</t>
+        </is>
+      </c>
+      <c r="B2" s="101" t="inlineStr">
+        <is>
+          <t>nom affiché (anglais)</t>
+        </is>
+      </c>
+      <c r="C2" s="101" t="inlineStr">
+        <is>
+          <t>niveau (→ or lâché)</t>
+        </is>
+      </c>
+      <c r="D2" s="101" t="inlineStr">
+        <is>
+          <t>gobelin / animal / (vide)</t>
+        </is>
+      </c>
+      <c r="E2" s="101" t="inlineStr">
+        <is>
+          <t>points de vie</t>
+        </is>
+      </c>
+      <c r="F2" s="101" t="inlineStr">
+        <is>
+          <t>dégâts par coup</t>
+        </is>
+      </c>
+      <c r="G2" s="101" t="inlineStr">
+        <is>
+          <t>XP donnée à la mort</t>
+        </is>
+      </c>
+      <c r="H2" s="101" t="inlineStr">
+        <is>
+          <t>vitesse d'initiative ET d'animation (grand = rapide)</t>
+        </is>
+      </c>
+      <c r="I2" s="101" t="inlineStr">
+        <is>
+          <t>actions spéciales : type:valeur:poids séparés par | (types: attaque, soigner, haste-allie). Vide = attaque simple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cave Goblin</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>24</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>gobelin-vif</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Goblin Skirmisher</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H4" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>gobelin-chaman</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Goblin Shaman</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>soigner:10:50 | haste-allie:2:30 | attaque:2:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ogre-masque</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Masked Ogre</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>58</v>
+      </c>
+      <c r="F6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>24</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
[technique] Stats de base du héros éditables dans l'Excel (onglet « Héros »)
Nouvel onglet « Héros » (vie, vitesse de marche, vitesse de combat, Chaleur de
forge, main max) + outils/importer_heros.py qui régénère data/heros_base.js.
Les constantes de base de talents.js, combat.js et heros.js pointent désormais
sur cette source unique : Brioche règle les stats de base sans toucher au code.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Profondeurs" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Profondeurs-chances" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Monstres" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Héros" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1667,6 +1668,162 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="57" min="1" max="1"/>
+    <col width="9" customWidth="1" style="57" min="2" max="2"/>
+    <col width="54" customWidth="1" style="57" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="100" t="inlineStr">
+        <is>
+          <t>clé</t>
+        </is>
+      </c>
+      <c r="B1" s="100" t="inlineStr">
+        <is>
+          <t>valeur</t>
+        </is>
+      </c>
+      <c r="C1" s="100" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>pv</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Vie de base (avant talents/équipement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>vitesseMarche</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>160</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Vitesse de déplacement en exploration (pixels/seconde)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>vitesseCombat</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Vitesse d'initiative en combat (ATB, agilité de base)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>chaleurDepart</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Chaleur de forge au début d'un combat</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>chaleurRecharge</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Chaleur regagnée à chaque tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>chaleurSeuil</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Seuil de surchauffe de la forge</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>chaleurMax</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Chaleur maximale</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>mainMax</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Nombre maximum de cartes en main</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
[gameplay] Grands monstres : occupent 2 places, plus gros, pop plus rare (ogre)
Nouvelle mécanique générique pilotée par un flag Excel « grand » (colonne J de
l'onglet Monstres) :
- un GRAND monstre occupe 2 emplacements du groupe et se CENTRE dessus (affiché
  plus gros, toujours à l'avant) ;
- il n'apparaît que s'il reste >=2 places libres ;
- il pop plus rarement (poids x GRAND_RARETE=0,5, en plus de la pondération niveau).
Règle commune à tous les grands monstres. Testé sur l'ogre masqué (agrandi à
280 px, ~6 % des groupes). Importer + concept.md mis à jour.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -1422,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="57" min="1" max="1"/>
@@ -1434,6 +1434,7 @@
     <col width="7" customWidth="1" style="57" min="7" max="7"/>
     <col width="9" customWidth="1" style="57" min="8" max="8"/>
     <col width="52" customWidth="1" style="57" min="9" max="9"/>
+    <col width="42" customWidth="1" style="57" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1482,6 +1483,11 @@
           <t>actions</t>
         </is>
       </c>
+      <c r="J1" s="100" t="inlineStr">
+        <is>
+          <t>grand</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="101" t="inlineStr">
@@ -1529,6 +1535,11 @@
           <t>actions spéciales : type:valeur:poids séparés par | (types: attaque, soigner, haste-allie). Vide = attaque simple.</t>
         </is>
       </c>
+      <c r="J2" s="101" t="inlineStr">
+        <is>
+          <t>met 1 si le monstre est GRAND (occupe 2 places, pop plus rare). Vide = normal.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1661,6 +1672,9 @@
       </c>
       <c r="H6" t="n">
         <v>6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[technique] Excel items : colonne « Total visé (barème) » — dégâts/armure totaux par item
L'outil outils/resumer_cartes.py résume aussi l'onglet « Items » : pour chaque
arme/armure, somme des cibles de ses cartes × quantité (dégâts pour une arme,
armure pour une armure) + nombre de cartes vs la cible de cartes de la rareté.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -788,6 +788,23 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>BRUTAL</author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Total que les cartes de l'item devraient fournir (outils/resumer_cartes.py) :
+somme des cibles de chaque carte × sa quantité — dégâts pour une arme, armure
+pour une armure. Entre parenthèses : nb de cartes de l'item vs cible de la rareté.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1870,7 +1887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L171"/>
+  <dimension ref="A1:M171"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="100" min="1" max="1"/>
@@ -10751,7 +10768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:H141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="100" min="1" max="1"/>
@@ -10759,6 +10776,7 @@
     <col width="11" customWidth="1" style="100" min="4" max="4"/>
     <col width="71.5703125" customWidth="1" style="100" min="5" max="5"/>
     <col width="52" customWidth="1" style="100" min="6" max="6"/>
+    <col width="30" customWidth="1" style="100" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.95" customHeight="1" s="100">
@@ -10790,6 +10808,11 @@
       <c r="F1" s="10" t="inlineStr">
         <is>
           <t>Effet hors-carte / spécial</t>
+        </is>
+      </c>
+      <c r="G1" s="101" t="inlineStr">
+        <is>
+          <t>Total visé (barème)</t>
         </is>
       </c>
     </row>
@@ -10832,6 +10855,11 @@
         </is>
       </c>
       <c r="F3" s="14" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>≈ 25 dégâts  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="100">
       <c r="A4" s="13" t="inlineStr">
@@ -10860,6 +10888,11 @@
         </is>
       </c>
       <c r="F4" s="14" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>≈ 20 dégâts  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="100">
       <c r="A5" s="13" t="inlineStr">
@@ -10888,6 +10921,11 @@
         </is>
       </c>
       <c r="F5" s="14" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>≈ 20 dégâts  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="100">
       <c r="A6" s="13" t="inlineStr">
@@ -10916,6 +10954,11 @@
         </is>
       </c>
       <c r="F6" s="14" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>≈ 35 dégâts  ·  ≈ 6 armure  (5 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="100">
       <c r="A7" s="13" t="inlineStr">
@@ -10944,6 +10987,11 @@
         </is>
       </c>
       <c r="F7" s="14" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>≈ 25 dégâts  (5 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="100">
       <c r="A8" s="13" t="inlineStr">
@@ -10972,6 +11020,11 @@
         </is>
       </c>
       <c r="F8" s="14" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>≈ 25 dégâts  ·  ≈ 3 armure  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="100">
       <c r="A9" s="13" t="inlineStr">
@@ -11000,6 +11053,11 @@
         </is>
       </c>
       <c r="F9" s="14" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>≈ 10 dégâts  ·  ≈ 6 armure  (5 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="100">
       <c r="A10" s="13" t="inlineStr">
@@ -11028,6 +11086,11 @@
         </is>
       </c>
       <c r="F10" s="14" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>≈ 35 dégâts  (5 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="100">
       <c r="A11" s="13" t="inlineStr">
@@ -11056,6 +11119,11 @@
         </is>
       </c>
       <c r="F11" s="14" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>≈ 20 dégâts  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="100">
       <c r="A12" s="13" t="inlineStr">
@@ -11084,6 +11152,11 @@
         </is>
       </c>
       <c r="F12" s="14" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>≈ 20 dégâts  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="100">
       <c r="A13" s="13" t="inlineStr">
@@ -11112,6 +11185,11 @@
         </is>
       </c>
       <c r="F13" s="14" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>≈ 20 dégâts  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="100">
       <c r="A14" s="13" t="inlineStr">
@@ -11140,6 +11218,11 @@
         </is>
       </c>
       <c r="F14" s="14" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>≈ 25 dégâts  (5 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="100">
       <c r="A15" s="13" t="inlineStr">
@@ -11168,6 +11251,11 @@
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>≈ 35 dégâts  (5 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="100">
       <c r="A16" s="13" t="inlineStr">
@@ -11196,6 +11284,11 @@
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>≈ 20 dégâts  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="100">
       <c r="A17" s="13" t="inlineStr">
@@ -11224,6 +11317,11 @@
         </is>
       </c>
       <c r="F17" s="14" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>≈ 15 dégâts  (4 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="100">
       <c r="A18" s="13" t="inlineStr">
@@ -11252,6 +11350,11 @@
         </is>
       </c>
       <c r="F18" s="14" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>≈ 25 dégâts  ·  ≈ 3 armure  (5 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="100">
       <c r="A19" s="15" t="inlineStr">
@@ -11280,6 +11383,11 @@
         </is>
       </c>
       <c r="F19" s="16" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>≈ 29 dégâts  (5 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="100">
       <c r="A20" s="16" t="inlineStr">
@@ -11312,6 +11420,11 @@
           <t>Deux mains</t>
         </is>
       </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>≈ 72 dégâts  (8 cartes/6 visées · 3 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="100">
       <c r="A21" s="15" t="inlineStr">
@@ -11340,6 +11453,11 @@
         </is>
       </c>
       <c r="F21" s="16" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>≈ 24 dégâts  (4 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="100">
       <c r="A22" s="15" t="inlineStr">
@@ -11368,6 +11486,11 @@
         </is>
       </c>
       <c r="F22" s="16" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>≈ 23 dégâts  (4 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="100">
       <c r="A23" s="15" t="inlineStr">
@@ -11396,6 +11519,11 @@
         </is>
       </c>
       <c r="F23" s="16" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>≈ 55 dégâts  (5 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="100">
       <c r="A24" s="15" t="inlineStr">
@@ -11424,6 +11552,11 @@
         </is>
       </c>
       <c r="F24" s="16" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>≈ 82 dégâts  (6 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="100">
       <c r="A25" s="15" t="inlineStr">
@@ -11452,6 +11585,11 @@
         </is>
       </c>
       <c r="F25" s="16" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>≈ 31 dégâts  (4 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="100">
       <c r="A26" s="15" t="inlineStr">
@@ -11484,6 +11622,11 @@
           <t>Deux mains</t>
         </is>
       </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>≈ 132 dégâts  ·  ≈ 7,5 armure  (9 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="100">
       <c r="A27" s="15" t="inlineStr">
@@ -11512,6 +11655,11 @@
         </is>
       </c>
       <c r="F27" s="16" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>≈ 42 dégâts  (5 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="100">
       <c r="A28" s="15" t="inlineStr">
@@ -11540,6 +11688,11 @@
         </is>
       </c>
       <c r="F28" s="16" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>≈ 23 dégâts  (4 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="100">
       <c r="A29" s="15" t="inlineStr">
@@ -11568,6 +11721,11 @@
         </is>
       </c>
       <c r="F29" s="16" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>≈ 53 dégâts  (5 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="100">
       <c r="A30" s="15" t="inlineStr">
@@ -11596,6 +11754,11 @@
         </is>
       </c>
       <c r="F30" s="16" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>≈ 40 dégâts  ·  ≈ 6 armure  (5 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="100">
       <c r="A31" s="15" t="inlineStr">
@@ -11628,6 +11791,11 @@
           <t>Combo: Twin combo: +3 permanent Strength if the same Twin Daggers are in your off-hand.</t>
         </is>
       </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>≈ 37 dégâts  (5 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="100">
       <c r="A32" s="15" t="inlineStr">
@@ -11656,6 +11824,11 @@
         </is>
       </c>
       <c r="F32" s="16" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>≈ 23 dégâts  (4 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="100">
       <c r="A33" s="15" t="inlineStr">
@@ -11684,6 +11857,11 @@
         </is>
       </c>
       <c r="F33" s="16" t="n"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>≈ 48 dégâts  ·  ≈ 6 armure  (5 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="100">
       <c r="A34" s="17" t="inlineStr">
@@ -11716,6 +11894,11 @@
           <t>Combo: Twin fang: +5 permanent Strength if another dagger is in your off-hand.</t>
         </is>
       </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>≈ 168 dégâts  (10 cartes/6 visées · 1 non listée)</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="100">
       <c r="A35" s="17" t="inlineStr">
@@ -11748,6 +11931,11 @@
           <t>Deux mains, Bonsu passif de 2 stone par tours (permanent tant que l'arme est équipée).</t>
         </is>
       </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>≈ 306 dégâts  ·  ≈ 24 armure  (8 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="100">
       <c r="A36" s="17" t="inlineStr">
@@ -11780,6 +11968,11 @@
           <t>Deux mains</t>
         </is>
       </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>≈ 252 dégâts  (6 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="100">
       <c r="A37" s="21" t="inlineStr">
@@ -11812,6 +12005,11 @@
           <t>Deux mains</t>
         </is>
       </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>≈ 204 dégâts  (7 cartes/7 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="100">
       <c r="A38" s="53" t="inlineStr">
@@ -11844,6 +12042,11 @@
           <t>Deux mains</t>
         </is>
       </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>≈ 357 dégâts  (8 cartes/7 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="100">
       <c r="A39" s="21" t="inlineStr">
@@ -11872,6 +12075,11 @@
         </is>
       </c>
       <c r="F39" s="22" t="n"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>≈ 272 dégâts  (7 cartes/7 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="17.1" customHeight="1" s="100">
       <c r="A40" s="47" t="inlineStr">
@@ -11912,6 +12120,11 @@
         </is>
       </c>
       <c r="F41" s="14" t="n"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="100">
       <c r="A42" s="13" t="inlineStr">
@@ -11940,6 +12153,11 @@
         </is>
       </c>
       <c r="F42" s="14" t="n"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>≈ 3 armure  (2 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="100">
       <c r="A43" s="13" t="inlineStr">
@@ -11968,6 +12186,11 @@
         </is>
       </c>
       <c r="F43" s="14" t="n"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>≈ 20 dégâts  (3 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="100">
       <c r="A44" s="13" t="inlineStr">
@@ -11996,6 +12219,11 @@
         </is>
       </c>
       <c r="F44" s="14" t="n"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (3 cartes/5 visées · 3 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="100">
       <c r="A45" s="13" t="inlineStr">
@@ -12024,6 +12252,11 @@
         </is>
       </c>
       <c r="F45" s="14" t="n"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="100">
       <c r="A46" s="13" t="inlineStr">
@@ -12052,6 +12285,11 @@
         </is>
       </c>
       <c r="F46" s="14" t="n"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>≈ 9 armure  (3 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="100">
       <c r="A47" s="15" t="inlineStr">
@@ -12080,6 +12318,11 @@
         </is>
       </c>
       <c r="F47" s="16" t="n"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>≈ 26 dégâts  (3 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="100">
       <c r="A48" s="15" t="inlineStr">
@@ -12108,6 +12351,11 @@
         </is>
       </c>
       <c r="F48" s="16" t="n"/>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>≈ 14 armure  (4 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="100">
       <c r="A49" s="15" t="inlineStr">
@@ -12136,6 +12384,11 @@
         </is>
       </c>
       <c r="F49" s="16" t="n"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="100">
       <c r="A50" s="15" t="inlineStr">
@@ -12164,6 +12417,11 @@
         </is>
       </c>
       <c r="F50" s="16" t="n"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>≈ 16 dégâts  (3 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="100">
       <c r="A51" s="15" t="inlineStr">
@@ -12196,6 +12454,11 @@
           <t>When hit by a melee attack, the attacker takes 2 damage.</t>
         </is>
       </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>≈ 16 armure  (3 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="100">
       <c r="A52" s="17" t="inlineStr">
@@ -12226,6 +12489,11 @@
       <c r="F52" s="18" t="inlineStr">
         <is>
           <t>When hit by a melee attack, gain 2 Stone.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>≈ 48 dégâts  ·  ≈ 47 armure  (6 cartes/6 visées)</t>
         </is>
       </c>
     </row>
@@ -12272,6 +12540,11 @@
           <t>Armure début: 8</t>
         </is>
       </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>≈ 14 armure  (4 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="100">
       <c r="A55" s="13" t="inlineStr">
@@ -12304,6 +12577,11 @@
           <t>Armure début: 6</t>
         </is>
       </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>≈ 3 armure  (2 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="100">
       <c r="A56" s="13" t="inlineStr">
@@ -12336,6 +12614,11 @@
           <t>Armure début: 6</t>
         </is>
       </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>≈ 9 armure  (3 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="100">
       <c r="A57" s="13" t="inlineStr">
@@ -12368,6 +12651,11 @@
           <t>Armure début: 6</t>
         </is>
       </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>≈ 6 armure  (4 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="100">
       <c r="A58" s="13" t="inlineStr">
@@ -12400,6 +12688,11 @@
           <t>Armure début: 8</t>
         </is>
       </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>≈ 9 armure  (4 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="100">
       <c r="A59" s="15" t="inlineStr">
@@ -12432,6 +12725,11 @@
           <t>Armure début: 15</t>
         </is>
       </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>≈ 30 armure  (4 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="100">
       <c r="A60" s="15" t="inlineStr">
@@ -12464,6 +12762,11 @@
           <t>Armure début: 4</t>
         </is>
       </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>≈ 5 armure  (4 cartes/6 visées · 3 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="100">
       <c r="A61" s="15" t="inlineStr">
@@ -12496,6 +12799,11 @@
           <t>Armure début: 10  ·  When hit by a melee attack, the attacker takes 2 damage.</t>
         </is>
       </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>≈ 25 armure  (4 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="100">
       <c r="A62" s="15" t="inlineStr">
@@ -12528,6 +12836,11 @@
           <t>Armure début: 12  ·  Set: Stone Age Set</t>
         </is>
       </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>≈ 85 armure  (10 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="100">
       <c r="A63" s="17" t="inlineStr">
@@ -12560,6 +12873,11 @@
           <t>Armure début: 20 - +4 stone a chaque tour (permanent)  ·  Set: Blood Set</t>
         </is>
       </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>≈ 60 dégâts  ·  ≈ 48 armure  (6 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="100">
       <c r="A64" s="17" t="inlineStr">
@@ -12592,6 +12910,11 @@
           <t>Armure début: 30 - +6 stone a chaque tour (permanent)  ·  Set: Crusader Set</t>
         </is>
       </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>≈ 60 dégâts  ·  ≈ 56 armure  (6 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="100">
       <c r="A65" s="17" t="inlineStr">
@@ -12624,6 +12947,11 @@
           <t>Armure début: 22 - +5 stone a chaque tour (permanent)  ·  Set: Mail Set</t>
         </is>
       </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>≈ 56 armure  (6 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="100">
       <c r="A66" s="21" t="inlineStr">
@@ -12654,6 +12982,11 @@
       <c r="F66" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Armure début: 36 - +10 stone a chaque tour (permanent) ·  Set: Onyx Set </t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>≈ 204 dégâts  ·  ≈ 72 armure  (7 cartes/7 visées)</t>
         </is>
       </c>
     </row>
@@ -12696,6 +13029,11 @@
         </is>
       </c>
       <c r="F68" s="14" t="n"/>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>≈ 10 dégâts  (2 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="100">
       <c r="A69" s="13" t="inlineStr">
@@ -12724,6 +13062,11 @@
         </is>
       </c>
       <c r="F69" s="14" t="n"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (1 carte/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="100">
       <c r="A70" s="13" t="inlineStr">
@@ -12752,6 +13095,11 @@
         </is>
       </c>
       <c r="F70" s="14" t="n"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="100">
       <c r="A71" s="13" t="inlineStr">
@@ -12780,6 +13128,11 @@
         </is>
       </c>
       <c r="F71" s="14" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="100">
       <c r="A72" s="13" t="inlineStr">
@@ -12808,6 +13161,11 @@
         </is>
       </c>
       <c r="F72" s="14" t="n"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>≈ 5 dégâts  (2 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="100">
       <c r="A73" s="15" t="inlineStr">
@@ -12836,6 +13194,11 @@
         </is>
       </c>
       <c r="F73" s="16" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="100">
       <c r="A74" s="15" t="inlineStr">
@@ -12864,6 +13227,11 @@
         </is>
       </c>
       <c r="F74" s="16" t="n"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="100">
       <c r="A75" s="15" t="inlineStr">
@@ -12892,6 +13260,11 @@
         </is>
       </c>
       <c r="F75" s="16" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (1 carte/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="100">
       <c r="A76" s="15" t="inlineStr">
@@ -12920,6 +13293,11 @@
         </is>
       </c>
       <c r="F76" s="16" t="n"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>≈ 13 dégâts  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="100">
       <c r="A77" s="17" t="inlineStr">
@@ -12948,6 +13326,11 @@
         </is>
       </c>
       <c r="F77" s="18" t="n"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="100">
       <c r="A78" s="21" t="inlineStr">
@@ -12976,6 +13359,11 @@
         </is>
       </c>
       <c r="F78" s="22" t="n"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (3 cartes/7 visées · 3 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="17.1" customHeight="1" s="100">
       <c r="A79" s="47" t="inlineStr">
@@ -13016,6 +13404,11 @@
         </is>
       </c>
       <c r="F80" s="14" t="n"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>≈ 10 dégâts  (2 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="100">
       <c r="A81" s="13" t="inlineStr">
@@ -13044,6 +13437,11 @@
         </is>
       </c>
       <c r="F81" s="14" t="n"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>≈ 10 dégâts  (2 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="100">
       <c r="A82" s="13" t="inlineStr">
@@ -13072,6 +13470,11 @@
         </is>
       </c>
       <c r="F82" s="14" t="n"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>≈ 10 dégâts  (2 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="100">
       <c r="A83" s="13" t="inlineStr">
@@ -13100,6 +13503,11 @@
         </is>
       </c>
       <c r="F83" s="14" t="n"/>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="100">
       <c r="A84" s="13" t="inlineStr">
@@ -13128,6 +13536,11 @@
         </is>
       </c>
       <c r="F84" s="14" t="n"/>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="100">
       <c r="A85" s="13" t="inlineStr">
@@ -13156,6 +13569,11 @@
         </is>
       </c>
       <c r="F85" s="14" t="n"/>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="100">
       <c r="A86" s="13" t="inlineStr">
@@ -13184,6 +13602,11 @@
         </is>
       </c>
       <c r="F86" s="14" t="n"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>≈ 6 armure  (2 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="100">
       <c r="A87" s="13" t="inlineStr">
@@ -13212,6 +13635,11 @@
         </is>
       </c>
       <c r="F87" s="14" t="n"/>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>≈ 10 dégâts  (2 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="100">
       <c r="A88" s="13" t="inlineStr">
@@ -13240,6 +13668,11 @@
         </is>
       </c>
       <c r="F88" s="14" t="n"/>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>≈ 3 armure  (2 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="100">
       <c r="A89" s="15" t="inlineStr">
@@ -13268,6 +13701,11 @@
         </is>
       </c>
       <c r="F89" s="16" t="n"/>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>≈ 16 dégâts  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="100">
       <c r="A90" s="15" t="inlineStr">
@@ -13296,6 +13734,11 @@
         </is>
       </c>
       <c r="F90" s="16" t="n"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>≈ 13 dégâts  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="100">
       <c r="A91" s="15" t="inlineStr">
@@ -13324,6 +13767,11 @@
         </is>
       </c>
       <c r="F91" s="16" t="n"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="100">
       <c r="A92" s="15" t="inlineStr">
@@ -13352,6 +13800,11 @@
         </is>
       </c>
       <c r="F92" s="16" t="n"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>≈ 16 dégâts  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="100">
       <c r="A93" s="15" t="inlineStr">
@@ -13380,6 +13833,11 @@
         </is>
       </c>
       <c r="F93" s="16" t="n"/>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>≈ 21 dégâts  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="100">
       <c r="A94" s="15" t="inlineStr">
@@ -13408,6 +13866,11 @@
         </is>
       </c>
       <c r="F94" s="16" t="n"/>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>≈ 6 armure  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="100">
       <c r="A95" s="15" t="inlineStr">
@@ -13436,6 +13899,11 @@
         </is>
       </c>
       <c r="F95" s="16" t="n"/>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="100">
       <c r="A96" s="15" t="inlineStr">
@@ -13464,6 +13932,11 @@
         </is>
       </c>
       <c r="F96" s="16" t="n"/>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>≈ 21 dégâts  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="100">
       <c r="A97" s="17" t="inlineStr">
@@ -13492,6 +13965,11 @@
         </is>
       </c>
       <c r="F97" s="18" t="n"/>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>≈ 48 dégâts  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="17.1" customHeight="1" s="100">
       <c r="A98" s="47" t="inlineStr">
@@ -13532,6 +14010,11 @@
         </is>
       </c>
       <c r="F99" s="14" t="n"/>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="100">
       <c r="A100" s="13" t="inlineStr">
@@ -13560,6 +14043,11 @@
         </is>
       </c>
       <c r="F100" s="14" t="n"/>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>≈ 3 armure  (2 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="100">
       <c r="A101" s="13" t="inlineStr">
@@ -13588,6 +14076,11 @@
         </is>
       </c>
       <c r="F101" s="14" t="n"/>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="100">
       <c r="A102" s="13" t="inlineStr">
@@ -13616,6 +14109,11 @@
         </is>
       </c>
       <c r="F102" s="14" t="n"/>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>≈ 10 dégâts  (2 cartes/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="100">
       <c r="A103" s="13" t="inlineStr">
@@ -13644,6 +14142,11 @@
         </is>
       </c>
       <c r="F103" s="14" t="n"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>≈ 5 dégâts  (2 cartes/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="100">
       <c r="A104" s="15" t="inlineStr">
@@ -13672,6 +14175,11 @@
         </is>
       </c>
       <c r="F104" s="16" t="n"/>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>≈ 16 dégâts  ·  ≈ 3 armure  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="100">
       <c r="A105" s="15" t="inlineStr">
@@ -13700,6 +14208,11 @@
         </is>
       </c>
       <c r="F105" s="16" t="n"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (3 cartes/6 visées · 3 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="100">
       <c r="A106" s="15" t="inlineStr">
@@ -13732,6 +14245,11 @@
           <t>Set: Stone Age Set</t>
         </is>
       </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>≈ 30 armure  (5 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="100">
       <c r="A107" s="15" t="inlineStr">
@@ -13760,6 +14278,11 @@
         </is>
       </c>
       <c r="F107" s="16" t="n"/>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="100">
       <c r="A108" s="15" t="inlineStr">
@@ -13788,6 +14311,11 @@
         </is>
       </c>
       <c r="F108" s="16" t="n"/>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>≈ 10 dégâts  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="100">
       <c r="A109" s="17" t="inlineStr">
@@ -13820,6 +14348,11 @@
           <t>Set: Blood Set</t>
         </is>
       </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>≈ 72 dégâts  (5 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="100">
       <c r="A110" s="17" t="inlineStr">
@@ -13852,6 +14385,11 @@
           <t>Set: Crusader Set</t>
         </is>
       </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>≈ 12 dégâts  (5 cartes/6 visées · 4 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="100">
       <c r="A111" s="17" t="inlineStr">
@@ -13884,6 +14422,11 @@
           <t>Set: Mail Set</t>
         </is>
       </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (5 cartes/6 visées · 5 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="100">
       <c r="A112" s="21" t="inlineStr">
@@ -13914,6 +14457,11 @@
       <c r="F112" s="22" t="inlineStr">
         <is>
           <t>Set: Onyx Set</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>≈ 34 dégâts  (6 cartes/7 visées · 4 buff)</t>
         </is>
       </c>
     </row>
@@ -13960,6 +14508,11 @@
           <t>+3 Agilité  ·  +10% déplacement</t>
         </is>
       </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="100">
       <c r="A115" s="13" t="inlineStr">
@@ -13992,6 +14545,11 @@
           <t>+2 Agilité  ·  +8% déplacement</t>
         </is>
       </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="100">
       <c r="A116" s="13" t="inlineStr">
@@ -14024,6 +14582,11 @@
           <t>+3 Agilité  ·  +15% déplacement</t>
         </is>
       </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/5 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="100">
       <c r="A117" s="13" t="inlineStr">
@@ -14056,6 +14619,11 @@
           <t>+1 Agilité  ·  +5% déplacement</t>
         </is>
       </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (1 carte/5 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="100">
       <c r="A118" s="15" t="inlineStr">
@@ -14088,6 +14656,11 @@
           <t>+6 Agilité  ·  +15% déplacement</t>
         </is>
       </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>≈ 5 dégâts  (2 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="100">
       <c r="A119" s="15" t="inlineStr">
@@ -14120,6 +14693,11 @@
           <t>+3 Agilité  ·  +6% déplacement  ·  Set: Stone Age Set</t>
         </is>
       </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>≈ 30 armure  (5 cartes/6 visées · 1 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="15" customHeight="1" s="100">
       <c r="A120" s="15" t="inlineStr">
@@ -14152,6 +14730,11 @@
           <t>+4 Agilité  ·  +8% déplacement</t>
         </is>
       </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>≈ 24 dégâts  ·  ≈ 3 armure  (2 cartes/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="15" customHeight="1" s="100">
       <c r="A121" s="15" t="inlineStr">
@@ -14184,6 +14767,11 @@
           <t>+7 Agilité  ·  +20% déplacement</t>
         </is>
       </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (4 cartes/6 visées · 4 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="15" customHeight="1" s="100">
       <c r="A122" s="15" t="inlineStr">
@@ -14216,6 +14804,11 @@
           <t>+8 Agilité  ·  +30% déplacement</t>
         </is>
       </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (2 cartes/6 visées · 2 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="100">
       <c r="A123" s="17" t="inlineStr">
@@ -14248,6 +14841,11 @@
           <t>+12 Agilité  ·  +25% déplacement  ·  Set: Blood Set</t>
         </is>
       </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>≈ 24 dégâts  (5 cartes/6 visées · 4 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="15" customHeight="1" s="100">
       <c r="A124" s="17" t="inlineStr">
@@ -14280,6 +14878,11 @@
           <t>+12 Agilité  ·  +25% déplacement  ·  Set: Crusader Set</t>
         </is>
       </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>≈ 24 dégâts  (5 cartes/6 visées · 3 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="15" customHeight="1" s="100">
       <c r="A125" s="17" t="inlineStr">
@@ -14312,6 +14915,11 @@
           <t>+10 Agilité  ·  +15% déplacement  ·  Set: Mail Set</t>
         </is>
       </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (5 cartes/6 visées · 5 buff)</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="15" customHeight="1" s="100">
       <c r="A126" s="21" t="inlineStr">
@@ -14342,6 +14950,11 @@
       <c r="F126" s="22" t="inlineStr">
         <is>
           <t>+18 Agilité  ·  +50% déplacement  ·  Set: Onyx Set</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>≈ 17 dégâts  (6 cartes/7 visées · 5 buff)</t>
         </is>
       </c>
     </row>
@@ -14388,6 +15001,11 @@
           <t>+1 rangées de sac</t>
         </is>
       </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (0 carte/5 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="15" customHeight="1" s="100">
       <c r="A129" s="15" t="inlineStr">
@@ -14420,6 +15038,11 @@
           <t>+2 rangées de sac</t>
         </is>
       </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (0 carte/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="15" customHeight="1" s="100">
       <c r="A130" s="17" t="inlineStr">
@@ -14452,6 +15075,11 @@
           <t>+4 rangées de sac</t>
         </is>
       </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (0 carte/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="15" customHeight="1" s="100">
       <c r="A131" s="17" t="inlineStr">
@@ -14484,6 +15112,11 @@
           <t>+3 rangées de sac</t>
         </is>
       </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (0 carte/6 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="15" customHeight="1" s="100">
       <c r="A132" s="21" t="inlineStr">
@@ -14516,6 +15149,11 @@
           <t>+6 rangées de sac</t>
         </is>
       </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (0 carte/7 visées)</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="15" customHeight="1" s="100">
       <c r="A133" s="49" t="inlineStr">
@@ -14546,6 +15184,11 @@
       <c r="F133" s="50" t="inlineStr">
         <is>
           <t>+10 rangées de sac</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>aucun dégât/armure  (0 carte/8 visées)</t>
         </is>
       </c>
     </row>
@@ -14615,6 +15258,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
[technique] Excel Monstres : +12 nouveaux monstres de profondeur + colonne « zone de pop » ; concept.md à jour
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -1278,7 +1278,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
@@ -1473,7 +1472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="102" min="1" max="1"/>
@@ -1486,6 +1485,7 @@
     <col width="9" customWidth="1" style="102" min="8" max="8"/>
     <col width="52" customWidth="1" style="102" min="9" max="9"/>
     <col width="42" customWidth="1" style="102" min="10" max="10"/>
+    <col width="26" customWidth="1" style="102" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1539,6 +1539,11 @@
           <t>grand</t>
         </is>
       </c>
+      <c r="K1" s="103" t="inlineStr">
+        <is>
+          <t>zone de pop</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="98" t="inlineStr">
@@ -1591,6 +1596,11 @@
           <t>met 1 si le monstre est GRAND (occupe 2 places, pop plus rare). Vide = normal.</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>où le monstre apparaît : « Eastern + profondeur » (surface est + mine) ou « Profondeur » (mine uniquement, étage 2+)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1623,6 +1633,11 @@
       <c r="H3" t="n">
         <v>6</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Eastern + profondeur</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1662,6 +1677,11 @@
           <t>applique 1 poisson par attaque (2x attaque = 2 poisons)</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Eastern + profondeur</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1699,6 +1719,11 @@
           <t>soigner:10:50 | haste-allie:2:30 | attaque:2:20</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Eastern + profondeur</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1733,6 +1758,503 @@
       </c>
       <c r="J6" t="n">
         <v>1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Eastern + profondeur</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>orc-rodeur</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Orc Rogue</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>40</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>22</v>
+      </c>
+      <c r="H7" t="n">
+        <v>15</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>frappe 2× par tour (attaqueHits 2)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>orc-guerrier</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Orc Warrior</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>75</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>orc-guerriere</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Orc Warmaiden</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F9" t="n">
+        <v>16</v>
+      </c>
+      <c r="G9" t="n">
+        <v>34</v>
+      </c>
+      <c r="H9" t="n">
+        <v>9</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>orc-brute</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Orc Berserker</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>95</v>
+      </c>
+      <c r="F10" t="n">
+        <v>20</v>
+      </c>
+      <c r="G10" t="n">
+        <v>44</v>
+      </c>
+      <c r="H10" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>orc-chamane</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Orc Shaman</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>45</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" t="n">
+        <v>36</v>
+      </c>
+      <c r="H11" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>soigner:12:45 | haste-allie:2:30 | attaque:6:25</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>blob-vert</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Green Slime</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>blob</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>55</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8</v>
+      </c>
+      <c r="G12" t="n">
+        <v>24</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1 poison par coup</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>blob-jaune</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ochre Slime</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>blob</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>50</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" t="n">
+        <v>24</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>poison par coup (acide, 3)</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>blob-rouge</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Crimson Slime</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>blob</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>80</v>
+      </c>
+      <c r="F14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>tanky</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>blob-bleu</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Azure Slime</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>blob</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>65</v>
+      </c>
+      <c r="F15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G15" t="n">
+        <v>30</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>piquants</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>molosse</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Dire Hound</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>40</v>
+      </c>
+      <c r="F16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" t="n">
+        <v>22</v>
+      </c>
+      <c r="H16" t="n">
+        <v>16</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>rapide</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>molosse-feu</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ember Hound</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>45</v>
+      </c>
+      <c r="F17" t="n">
+        <v>12</v>
+      </c>
+      <c r="G17" t="n">
+        <v>28</v>
+      </c>
+      <c r="H17" t="n">
+        <v>15</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>rapide, feu</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>molosse-sombre</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Shadow Hound</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>42</v>
+      </c>
+      <c r="F18" t="n">
+        <v>11</v>
+      </c>
+      <c r="G18" t="n">
+        <v>26</v>
+      </c>
+      <c r="H18" t="n">
+        <v>17</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>rapide</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1902,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M171"/>
+  <dimension ref="A1:L171"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="102" min="1" max="1"/>
@@ -10783,7 +11305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H141"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="102" min="1" max="1"/>

</xml_diff>

<commit_message>
[technique] Excel « Monstres » réorganisé + lisible (catégories, tri par niveau, NxM, actions en liste %)
Onglet « Monstres » rangé : sections colorées PAR CATÉGORIE (gobelins, orcs, blobs,
animaux, champignons, lapin), triées PAR NIVEAU. Les attaques multiples s'écrivent
« NxM » dans la colonne attaque (2x2, 6x2, 7x2…). Les attaques spéciales sont en LISTE
VERTICALE lisible « Libellé valeur (chance%) ». Nouvelle colonne « passif / note » pour
la saveur (poison par coup, en meute…), non lue par l'importer.

importer_monstres.py adapté : lit « NxM » (→ attaque + attaqueHits) et le format lisible
des actions (Soin / Hâte alliés / Attaque), en plus de l'ancien format. STATS_MONSTRES
régénéré ; stats effectives strictement inchangées (vérifié).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -164,8 +164,13 @@
       <b val="1"/>
       <color rgb="001F3864"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="62">
+  <fills count="68">
     <fill>
       <patternFill/>
     </fill>
@@ -472,8 +477,38 @@
         <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006E8B3D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007A4A2B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003E7C7C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008A5A2B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007A5AA0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A03030"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -525,11 +560,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -766,6 +815,30 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="60" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="62" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="62" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="63" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="63" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="64" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="64" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="65" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="65" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="66" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="66" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="67" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="67" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1536,1283 +1609,1490 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="102" min="1" max="1"/>
+    <col width="24" customWidth="1" style="102" min="1" max="1"/>
     <col width="20" customWidth="1" style="102" min="2" max="2"/>
     <col width="8" customWidth="1" style="102" min="3" max="3"/>
-    <col width="12" customWidth="1" style="102" min="4" max="4"/>
+    <col width="11" customWidth="1" style="102" min="4" max="4"/>
     <col width="7" customWidth="1" style="102" min="5" max="5"/>
-    <col width="9" customWidth="1" style="102" min="6" max="6"/>
+    <col width="10" customWidth="1" style="102" min="6" max="6"/>
     <col width="7" customWidth="1" style="102" min="7" max="7"/>
     <col width="9" customWidth="1" style="102" min="8" max="8"/>
-    <col width="52" customWidth="1" style="102" min="9" max="9"/>
-    <col width="42" customWidth="1" style="102" min="10" max="10"/>
-    <col width="26" customWidth="1" style="102" min="11" max="11"/>
+    <col width="26" customWidth="1" style="102" min="9" max="9"/>
+    <col width="8" customWidth="1" style="102" min="10" max="10"/>
+    <col width="30" customWidth="1" style="102" min="11" max="11"/>
+    <col width="34" customWidth="1" style="102" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="97" t="inlineStr">
+      <c r="A1" s="112" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="97" t="inlineStr">
+      <c r="B1" s="112" t="inlineStr">
         <is>
           <t>nom</t>
         </is>
       </c>
-      <c r="C1" s="97" t="inlineStr">
+      <c r="C1" s="112" t="inlineStr">
         <is>
           <t>niveau</t>
         </is>
       </c>
-      <c r="D1" s="97" t="inlineStr">
+      <c r="D1" s="112" t="inlineStr">
         <is>
           <t>famille</t>
         </is>
       </c>
-      <c r="E1" s="97" t="inlineStr">
+      <c r="E1" s="112" t="inlineStr">
         <is>
           <t>pv</t>
         </is>
       </c>
-      <c r="F1" s="97" t="inlineStr">
+      <c r="F1" s="112" t="inlineStr">
         <is>
           <t>attaque</t>
         </is>
       </c>
-      <c r="G1" s="97" t="inlineStr">
+      <c r="G1" s="112" t="inlineStr">
         <is>
           <t>xp</t>
         </is>
       </c>
-      <c r="H1" s="97" t="inlineStr">
+      <c r="H1" s="112" t="inlineStr">
         <is>
           <t>vitesse</t>
         </is>
       </c>
-      <c r="I1" s="97" t="inlineStr">
-        <is>
-          <t>actions</t>
-        </is>
-      </c>
-      <c r="J1" s="97" t="inlineStr">
+      <c r="I1" s="112" t="inlineStr">
+        <is>
+          <t>actions spéciales</t>
+        </is>
+      </c>
+      <c r="J1" s="112" t="inlineStr">
         <is>
           <t>grand</t>
         </is>
       </c>
-      <c r="K1" s="103" t="inlineStr">
+      <c r="K1" s="112" t="inlineStr">
         <is>
           <t>zone de pop</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="98" t="inlineStr">
+      <c r="L1" s="112" t="inlineStr">
+        <is>
+          <t>passif / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="54" customHeight="1" s="102">
+      <c r="A2" s="113" t="inlineStr">
         <is>
           <t>identifiant (ne pas changer)</t>
         </is>
       </c>
-      <c r="B2" s="98" t="inlineStr">
+      <c r="B2" s="113" t="inlineStr">
         <is>
           <t>nom affiché (anglais)</t>
         </is>
       </c>
-      <c r="C2" s="98" t="inlineStr">
+      <c r="C2" s="113" t="inlineStr">
         <is>
           <t>niveau (→ or lâché)</t>
         </is>
       </c>
-      <c r="D2" s="98" t="inlineStr">
-        <is>
-          <t>gobelin / animal / (vide)</t>
-        </is>
-      </c>
-      <c r="E2" s="98" t="inlineStr">
+      <c r="D2" s="113" t="inlineStr">
+        <is>
+          <t>gobelin / orc / blob / animal / mushroom / lapin</t>
+        </is>
+      </c>
+      <c r="E2" s="113" t="inlineStr">
         <is>
           <t>points de vie</t>
         </is>
       </c>
-      <c r="F2" s="98" t="inlineStr">
-        <is>
-          <t>dégâts par coup</t>
-        </is>
-      </c>
-      <c r="G2" s="98" t="inlineStr">
-        <is>
-          <t>XP donnée à la mort</t>
-        </is>
-      </c>
-      <c r="H2" s="98" t="inlineStr">
-        <is>
-          <t>vitesse d'initiative ET d'animation (grand = rapide)</t>
-        </is>
-      </c>
-      <c r="I2" s="98" t="inlineStr">
-        <is>
-          <t>actions spéciales : type:valeur:poids séparés par | (types: attaque, soigner, haste-allie). Vide = attaque simple.</t>
-        </is>
-      </c>
-      <c r="J2" s="98" t="inlineStr">
-        <is>
-          <t>met 1 si le monstre est GRAND (occupe 2 places, pop plus rare). Vide = normal.</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>où le monstre apparaît : « Eastern + profondeur » (surface est + mine) ou « Profondeur » (mine uniquement, étage 2+)</t>
+      <c r="F2" s="113" t="inlineStr">
+        <is>
+          <t>dégâts par coup. Multi-coups : « NxM » = N dégâts × M coups (ex. 2x2)</t>
+        </is>
+      </c>
+      <c r="G2" s="113" t="inlineStr">
+        <is>
+          <t>XP à la mort</t>
+        </is>
+      </c>
+      <c r="H2" s="113" t="inlineStr">
+        <is>
+          <t>vitesse d'initiative ET d'animation</t>
+        </is>
+      </c>
+      <c r="I2" s="113" t="inlineStr">
+        <is>
+          <t>attaques spéciales, UNE PAR LIGNE : « Libellé valeur (chance%) ». Libellés : Soin, Hâte alliés, Attaque. Les % somment à 100. Vide = attaque simple.</t>
+        </is>
+      </c>
+      <c r="J2" s="113" t="inlineStr">
+        <is>
+          <t>1 si GRAND (occupe 2 places, pop plus rare)</t>
+        </is>
+      </c>
+      <c r="K2" s="113" t="inlineStr">
+        <is>
+          <t>où il apparaît</t>
+        </is>
+      </c>
+      <c r="L2" s="113" t="inlineStr">
+        <is>
+          <t>passif / mémo (poison, meute…) — NON lu par l'importer, purement informatif</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="114" t="inlineStr">
+        <is>
+          <t>▸ GOBELINS</t>
+        </is>
+      </c>
+      <c r="B3" s="115" t="n"/>
+      <c r="C3" s="115" t="n"/>
+      <c r="D3" s="115" t="n"/>
+      <c r="E3" s="115" t="n"/>
+      <c r="F3" s="115" t="n"/>
+      <c r="G3" s="115" t="n"/>
+      <c r="H3" s="115" t="n"/>
+      <c r="I3" s="115" t="n"/>
+      <c r="J3" s="115" t="n"/>
+      <c r="K3" s="115" t="n"/>
+      <c r="L3" s="115" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="116" t="inlineStr">
+        <is>
+          <t>gobelin-vif</t>
+        </is>
+      </c>
+      <c r="B4" s="116" t="inlineStr">
+        <is>
+          <t>Goblin Skirmisher</t>
+        </is>
+      </c>
+      <c r="C4" s="117" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="116" t="inlineStr">
         <is>
           <t>gobelin</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="E4" s="117" t="n">
+        <v>16</v>
+      </c>
+      <c r="F4" s="117" t="inlineStr">
+        <is>
+          <t>2x2</t>
+        </is>
+      </c>
+      <c r="G4" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="H4" s="117" t="n">
+        <v>11</v>
+      </c>
+      <c r="I4" s="116" t="inlineStr"/>
+      <c r="J4" s="117" t="n"/>
+      <c r="K4" s="116" t="inlineStr">
+        <is>
+          <t>Eastern + profondeur</t>
+        </is>
+      </c>
+      <c r="L4" s="116" t="inlineStr">
+        <is>
+          <t>1 poison par coup</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="116" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="B5" s="116" t="inlineStr">
         <is>
           <t>Cave Goblin</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C5" s="117" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D5" s="116" t="inlineStr">
         <is>
           <t>gobelin</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E5" s="117" t="n">
         <v>24</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F5" s="117" t="n">
         <v>5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G5" s="117" t="n">
         <v>6</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H5" s="117" t="n">
         <v>6</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="I5" s="116" t="inlineStr"/>
+      <c r="J5" s="117" t="n"/>
+      <c r="K5" s="116" t="inlineStr">
         <is>
           <t>Eastern + profondeur</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>gobelin-vif</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Goblin Skirmisher</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+      <c r="L5" s="116" t="inlineStr"/>
+    </row>
+    <row r="6" ht="59" customHeight="1" s="102">
+      <c r="A6" s="116" t="inlineStr">
+        <is>
+          <t>gobelin-chaman</t>
+        </is>
+      </c>
+      <c r="B6" s="116" t="inlineStr">
+        <is>
+          <t>Goblin Shaman</t>
+        </is>
+      </c>
+      <c r="C6" s="117" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="116" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="E6" s="117" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="117" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" s="117" t="n">
+        <v>7</v>
+      </c>
+      <c r="I6" s="116" t="inlineStr">
+        <is>
+          <t>Soin 10 (50%)
+Hâte alliés 2 (30%)
+Attaque 2 (20%)</t>
+        </is>
+      </c>
+      <c r="J6" s="117" t="n"/>
+      <c r="K6" s="116" t="inlineStr">
+        <is>
+          <t>Eastern + profondeur</t>
+        </is>
+      </c>
+      <c r="L6" s="116" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="118" t="inlineStr">
+        <is>
+          <t>▸ ORCS</t>
+        </is>
+      </c>
+      <c r="B7" s="119" t="n"/>
+      <c r="C7" s="119" t="n"/>
+      <c r="D7" s="119" t="n"/>
+      <c r="E7" s="119" t="n"/>
+      <c r="F7" s="119" t="n"/>
+      <c r="G7" s="119" t="n"/>
+      <c r="H7" s="119" t="n"/>
+      <c r="I7" s="119" t="n"/>
+      <c r="J7" s="119" t="n"/>
+      <c r="K7" s="119" t="n"/>
+      <c r="L7" s="119" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="116" t="inlineStr">
+        <is>
+          <t>orc-rodeur</t>
+        </is>
+      </c>
+      <c r="B8" s="116" t="inlineStr">
+        <is>
+          <t>Orc Rogue</t>
+        </is>
+      </c>
+      <c r="C8" s="117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="116" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E8" s="117" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" s="117" t="inlineStr">
+        <is>
+          <t>6x2</t>
+        </is>
+      </c>
+      <c r="G8" s="117" t="n">
+        <v>22</v>
+      </c>
+      <c r="H8" s="117" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="116" t="inlineStr"/>
+      <c r="J8" s="117" t="n"/>
+      <c r="K8" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L8" s="116" t="inlineStr"/>
+    </row>
+    <row r="9" ht="59" customHeight="1" s="102">
+      <c r="A9" s="116" t="inlineStr">
+        <is>
+          <t>orc-chamane</t>
+        </is>
+      </c>
+      <c r="B9" s="116" t="inlineStr">
+        <is>
+          <t>Orc Shaman</t>
+        </is>
+      </c>
+      <c r="C9" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="116" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E9" s="117" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" s="117" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="117" t="n">
+        <v>36</v>
+      </c>
+      <c r="H9" s="117" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" s="116" t="inlineStr">
+        <is>
+          <t>Soin 12 (45%)
+Hâte alliés 2 (30%)
+Attaque 6 (25%)</t>
+        </is>
+      </c>
+      <c r="J9" s="117" t="n"/>
+      <c r="K9" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L9" s="116" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="116" t="inlineStr">
+        <is>
+          <t>orc-guerriere</t>
+        </is>
+      </c>
+      <c r="B10" s="116" t="inlineStr">
+        <is>
+          <t>Orc Warmaiden</t>
+        </is>
+      </c>
+      <c r="C10" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="116" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E10" s="117" t="n">
+        <v>60</v>
+      </c>
+      <c r="F10" s="117" t="n">
+        <v>16</v>
+      </c>
+      <c r="G10" s="117" t="n">
+        <v>34</v>
+      </c>
+      <c r="H10" s="117" t="n">
+        <v>9</v>
+      </c>
+      <c r="I10" s="116" t="inlineStr"/>
+      <c r="J10" s="117" t="n"/>
+      <c r="K10" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L10" s="116" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="116" t="inlineStr">
+        <is>
+          <t>orc-guerrier</t>
+        </is>
+      </c>
+      <c r="B11" s="116" t="inlineStr">
+        <is>
+          <t>Orc Warrior</t>
+        </is>
+      </c>
+      <c r="C11" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="116" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E11" s="117" t="n">
+        <v>75</v>
+      </c>
+      <c r="F11" s="117" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" s="117" t="n">
+        <v>30</v>
+      </c>
+      <c r="H11" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="I11" s="116" t="inlineStr"/>
+      <c r="J11" s="117" t="n"/>
+      <c r="K11" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L11" s="116" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="116" t="inlineStr">
+        <is>
+          <t>orc-brute</t>
+        </is>
+      </c>
+      <c r="B12" s="116" t="inlineStr">
+        <is>
+          <t>Orc Berserker</t>
+        </is>
+      </c>
+      <c r="C12" s="117" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="116" t="inlineStr">
+        <is>
+          <t>orc</t>
+        </is>
+      </c>
+      <c r="E12" s="117" t="n">
+        <v>95</v>
+      </c>
+      <c r="F12" s="117" t="n">
+        <v>20</v>
+      </c>
+      <c r="G12" s="117" t="n">
+        <v>44</v>
+      </c>
+      <c r="H12" s="117" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" s="116" t="inlineStr"/>
+      <c r="J12" s="117" t="n">
         <v>1</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>gobelin</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
+      <c r="K12" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L12" s="116" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="120" t="inlineStr">
+        <is>
+          <t>▸ BLOBS (limons)</t>
+        </is>
+      </c>
+      <c r="B13" s="121" t="n"/>
+      <c r="C13" s="121" t="n"/>
+      <c r="D13" s="121" t="n"/>
+      <c r="E13" s="121" t="n"/>
+      <c r="F13" s="121" t="n"/>
+      <c r="G13" s="121" t="n"/>
+      <c r="H13" s="121" t="n"/>
+      <c r="I13" s="121" t="n"/>
+      <c r="J13" s="121" t="n"/>
+      <c r="K13" s="121" t="n"/>
+      <c r="L13" s="121" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="116" t="inlineStr">
+        <is>
+          <t>blob-jaune</t>
+        </is>
+      </c>
+      <c r="B14" s="116" t="inlineStr">
+        <is>
+          <t>Ochre Slime</t>
+        </is>
+      </c>
+      <c r="C14" s="117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="116" t="inlineStr">
+        <is>
+          <t>blob</t>
+        </is>
+      </c>
+      <c r="E14" s="117" t="n">
+        <v>50</v>
+      </c>
+      <c r="F14" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" s="117" t="n">
+        <v>24</v>
+      </c>
+      <c r="H14" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" s="116" t="inlineStr"/>
+      <c r="J14" s="117" t="n"/>
+      <c r="K14" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L14" s="116" t="inlineStr">
+        <is>
+          <t>3 poison par coup (acide)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="116" t="inlineStr">
+        <is>
+          <t>blob-vert</t>
+        </is>
+      </c>
+      <c r="B15" s="116" t="inlineStr">
+        <is>
+          <t>Green Slime</t>
+        </is>
+      </c>
+      <c r="C15" s="117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="116" t="inlineStr">
+        <is>
+          <t>blob</t>
+        </is>
+      </c>
+      <c r="E15" s="117" t="n">
+        <v>55</v>
+      </c>
+      <c r="F15" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="117" t="n">
+        <v>24</v>
+      </c>
+      <c r="H15" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" s="116" t="inlineStr"/>
+      <c r="J15" s="117" t="n"/>
+      <c r="K15" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L15" s="116" t="inlineStr">
+        <is>
+          <t>2 poison par coup</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="116" t="inlineStr">
+        <is>
+          <t>blob-bleu</t>
+        </is>
+      </c>
+      <c r="B16" s="116" t="inlineStr">
+        <is>
+          <t>Azure Slime</t>
+        </is>
+      </c>
+      <c r="C16" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" s="116" t="inlineStr">
+        <is>
+          <t>blob</t>
+        </is>
+      </c>
+      <c r="E16" s="117" t="n">
+        <v>65</v>
+      </c>
+      <c r="F16" s="117" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" s="117" t="n">
+        <v>30</v>
+      </c>
+      <c r="H16" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" s="116" t="inlineStr"/>
+      <c r="J16" s="117" t="n"/>
+      <c r="K16" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L16" s="116" t="inlineStr">
+        <is>
+          <t>piquants</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="116" t="inlineStr">
+        <is>
+          <t>blob-rouge</t>
+        </is>
+      </c>
+      <c r="B17" s="116" t="inlineStr">
+        <is>
+          <t>Crimson Slime</t>
+        </is>
+      </c>
+      <c r="C17" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="116" t="inlineStr">
+        <is>
+          <t>blob</t>
+        </is>
+      </c>
+      <c r="E17" s="117" t="n">
+        <v>80</v>
+      </c>
+      <c r="F17" s="117" t="n">
+        <v>10</v>
+      </c>
+      <c r="G17" s="117" t="n">
+        <v>30</v>
+      </c>
+      <c r="H17" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" s="116" t="inlineStr"/>
+      <c r="J17" s="117" t="n"/>
+      <c r="K17" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L17" s="116" t="inlineStr">
+        <is>
+          <t>très résistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="122" t="inlineStr">
+        <is>
+          <t>▸ ANIMAUX (bêtes — lâchent du cuir)</t>
+        </is>
+      </c>
+      <c r="B18" s="123" t="n"/>
+      <c r="C18" s="123" t="n"/>
+      <c r="D18" s="123" t="n"/>
+      <c r="E18" s="123" t="n"/>
+      <c r="F18" s="123" t="n"/>
+      <c r="G18" s="123" t="n"/>
+      <c r="H18" s="123" t="n"/>
+      <c r="I18" s="123" t="n"/>
+      <c r="J18" s="123" t="n"/>
+      <c r="K18" s="123" t="n"/>
+      <c r="L18" s="123" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="116" t="inlineStr">
+        <is>
+          <t>molosse</t>
+        </is>
+      </c>
+      <c r="B19" s="116" t="inlineStr">
+        <is>
+          <t>Dire Hound</t>
+        </is>
+      </c>
+      <c r="C19" s="117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" s="116" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E19" s="117" t="n">
+        <v>40</v>
+      </c>
+      <c r="F19" s="117" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" s="117" t="n">
+        <v>22</v>
+      </c>
+      <c r="H19" s="117" t="n">
         <v>16</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2x2</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
+      <c r="I19" s="116" t="inlineStr"/>
+      <c r="J19" s="117" t="n"/>
+      <c r="K19" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L19" s="116" t="inlineStr">
+        <is>
+          <t>rapide ; en meute</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="116" t="inlineStr">
+        <is>
+          <t>ogre-masque</t>
+        </is>
+      </c>
+      <c r="B20" s="116" t="inlineStr">
+        <is>
+          <t>Masked Ogre</t>
+        </is>
+      </c>
+      <c r="C20" s="117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="116" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E20" s="117" t="n">
+        <v>80</v>
+      </c>
+      <c r="F20" s="117" t="n">
+        <v>30</v>
+      </c>
+      <c r="G20" s="117" t="n">
+        <v>60</v>
+      </c>
+      <c r="H20" s="117" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="116" t="inlineStr"/>
+      <c r="J20" s="117" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="116" t="inlineStr">
+        <is>
+          <t>Eastern + profondeur</t>
+        </is>
+      </c>
+      <c r="L20" s="116" t="inlineStr">
+        <is>
+          <t>pic de difficulté</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="116" t="inlineStr">
+        <is>
+          <t>molosse-sombre</t>
+        </is>
+      </c>
+      <c r="B21" s="116" t="inlineStr">
+        <is>
+          <t>Shadow Hound</t>
+        </is>
+      </c>
+      <c r="C21" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="116" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E21" s="117" t="n">
+        <v>42</v>
+      </c>
+      <c r="F21" s="117" t="n">
+        <v>11</v>
+      </c>
+      <c r="G21" s="117" t="n">
+        <v>26</v>
+      </c>
+      <c r="H21" s="117" t="n">
+        <v>17</v>
+      </c>
+      <c r="I21" s="116" t="inlineStr"/>
+      <c r="J21" s="117" t="n"/>
+      <c r="K21" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L21" s="116" t="inlineStr">
+        <is>
+          <t>rapide ; en meute</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="116" t="inlineStr">
+        <is>
+          <t>molosse-feu</t>
+        </is>
+      </c>
+      <c r="B22" s="116" t="inlineStr">
+        <is>
+          <t>Ember Hound</t>
+        </is>
+      </c>
+      <c r="C22" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" s="116" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E22" s="117" t="n">
+        <v>45</v>
+      </c>
+      <c r="F22" s="117" t="n">
+        <v>12</v>
+      </c>
+      <c r="G22" s="117" t="n">
+        <v>28</v>
+      </c>
+      <c r="H22" s="117" t="n">
+        <v>15</v>
+      </c>
+      <c r="I22" s="116" t="inlineStr"/>
+      <c r="J22" s="117" t="n"/>
+      <c r="K22" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L22" s="116" t="inlineStr">
+        <is>
+          <t>rapide, feu ; en meute</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="116" t="inlineStr">
+        <is>
+          <t>bear</t>
+        </is>
+      </c>
+      <c r="B23" s="116" t="inlineStr">
+        <is>
+          <t>Cave Bear</t>
+        </is>
+      </c>
+      <c r="C23" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" s="116" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E23" s="117" t="n">
+        <v>90</v>
+      </c>
+      <c r="F23" s="117" t="n">
+        <v>14</v>
+      </c>
+      <c r="G23" s="117" t="n">
+        <v>32</v>
+      </c>
+      <c r="H23" s="117" t="n">
         <v>8</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I23" s="116" t="inlineStr"/>
+      <c r="J23" s="117" t="n"/>
+      <c r="K23" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L23" s="116" t="inlineStr">
+        <is>
+          <t>en meute avec les molosses</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="116" t="inlineStr">
+        <is>
+          <t>bones-bear</t>
+        </is>
+      </c>
+      <c r="B24" s="116" t="inlineStr">
+        <is>
+          <t>Bonehide Bear</t>
+        </is>
+      </c>
+      <c r="C24" s="117" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" s="116" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E24" s="117" t="n">
+        <v>100</v>
+      </c>
+      <c r="F24" s="117" t="n">
+        <v>16</v>
+      </c>
+      <c r="G24" s="117" t="n">
+        <v>44</v>
+      </c>
+      <c r="H24" s="117" t="n">
+        <v>9</v>
+      </c>
+      <c r="I24" s="116" t="inlineStr"/>
+      <c r="J24" s="117" t="n"/>
+      <c r="K24" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L24" s="116" t="inlineStr">
+        <is>
+          <t>en meute avec les molosses</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="116" t="inlineStr">
+        <is>
+          <t>armor-bear</t>
+        </is>
+      </c>
+      <c r="B25" s="116" t="inlineStr">
+        <is>
+          <t>Armored War-Bear</t>
+        </is>
+      </c>
+      <c r="C25" s="117" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" s="116" t="inlineStr">
+        <is>
+          <t>animal</t>
+        </is>
+      </c>
+      <c r="E25" s="117" t="n">
+        <v>150</v>
+      </c>
+      <c r="F25" s="117" t="n">
+        <v>20</v>
+      </c>
+      <c r="G25" s="117" t="n">
+        <v>60</v>
+      </c>
+      <c r="H25" s="117" t="n">
+        <v>6</v>
+      </c>
+      <c r="I25" s="116" t="inlineStr"/>
+      <c r="J25" s="117" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L25" s="116" t="inlineStr">
+        <is>
+          <t>en meute avec les molosses</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="124" t="inlineStr">
+        <is>
+          <t>▸ CHAMPIGNONS</t>
+        </is>
+      </c>
+      <c r="B26" s="125" t="n"/>
+      <c r="C26" s="125" t="n"/>
+      <c r="D26" s="125" t="n"/>
+      <c r="E26" s="125" t="n"/>
+      <c r="F26" s="125" t="n"/>
+      <c r="G26" s="125" t="n"/>
+      <c r="H26" s="125" t="n"/>
+      <c r="I26" s="125" t="n"/>
+      <c r="J26" s="125" t="n"/>
+      <c r="K26" s="125" t="n"/>
+      <c r="L26" s="125" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="116" t="inlineStr">
+        <is>
+          <t>warrior-mushroom1</t>
+        </is>
+      </c>
+      <c r="B27" s="116" t="inlineStr">
+        <is>
+          <t>Toadstool Lancer</t>
+        </is>
+      </c>
+      <c r="C27" s="117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="116" t="inlineStr">
+        <is>
+          <t>mushroom</t>
+        </is>
+      </c>
+      <c r="E27" s="117" t="n">
+        <v>50</v>
+      </c>
+      <c r="F27" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="G27" s="117" t="n">
+        <v>22</v>
+      </c>
+      <c r="H27" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="I27" s="116" t="inlineStr"/>
+      <c r="J27" s="117" t="n"/>
+      <c r="K27" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L27" s="116" t="inlineStr"/>
+    </row>
+    <row r="28" ht="59" customHeight="1" s="102">
+      <c r="A28" s="116" t="inlineStr">
+        <is>
+          <t>mage-mushroom</t>
+        </is>
+      </c>
+      <c r="B28" s="116" t="inlineStr">
+        <is>
+          <t>Myconid Sage</t>
+        </is>
+      </c>
+      <c r="C28" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" s="116" t="inlineStr">
+        <is>
+          <t>mushroom</t>
+        </is>
+      </c>
+      <c r="E28" s="117" t="n">
+        <v>40</v>
+      </c>
+      <c r="F28" s="117" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" s="117" t="n">
+        <v>34</v>
+      </c>
+      <c r="H28" s="117" t="n">
+        <v>7</v>
+      </c>
+      <c r="I28" s="116" t="inlineStr">
+        <is>
+          <t>Soin 12 (45%)
+Hâte alliés 2 (30%)
+Attaque 5 (25%)</t>
+        </is>
+      </c>
+      <c r="J28" s="117" t="n"/>
+      <c r="K28" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L28" s="116" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="116" t="inlineStr">
+        <is>
+          <t>white-katana-mushroom</t>
+        </is>
+      </c>
+      <c r="B29" s="116" t="inlineStr">
+        <is>
+          <t>Myconid Ronin</t>
+        </is>
+      </c>
+      <c r="C29" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" s="116" t="inlineStr">
+        <is>
+          <t>mushroom</t>
+        </is>
+      </c>
+      <c r="E29" s="117" t="n">
+        <v>45</v>
+      </c>
+      <c r="F29" s="117" t="inlineStr">
+        <is>
+          <t>7x2</t>
+        </is>
+      </c>
+      <c r="G29" s="117" t="n">
+        <v>30</v>
+      </c>
+      <c r="H29" s="117" t="n">
+        <v>18</v>
+      </c>
+      <c r="I29" s="116" t="inlineStr"/>
+      <c r="J29" s="117" t="n"/>
+      <c r="K29" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L29" s="116" t="inlineStr">
+        <is>
+          <t>deux katanas</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="116" t="inlineStr">
+        <is>
+          <t>warrior-mushroom2</t>
+        </is>
+      </c>
+      <c r="B30" s="116" t="inlineStr">
+        <is>
+          <t>Fungal Knight</t>
+        </is>
+      </c>
+      <c r="C30" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="116" t="inlineStr">
+        <is>
+          <t>mushroom</t>
+        </is>
+      </c>
+      <c r="E30" s="117" t="n">
+        <v>85</v>
+      </c>
+      <c r="F30" s="117" t="n">
         <v>11</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>applique 1 poisson par attaque (2x attaque = 2 poisons)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Eastern + profondeur</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>gobelin-chaman</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Goblin Shaman</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>gobelin</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
+      <c r="G30" s="117" t="n">
+        <v>30</v>
+      </c>
+      <c r="H30" s="117" t="n">
+        <v>7</v>
+      </c>
+      <c r="I30" s="116" t="inlineStr"/>
+      <c r="J30" s="117" t="n"/>
+      <c r="K30" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L30" s="116" t="inlineStr">
+        <is>
+          <t>épée + bouclier</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="116" t="inlineStr">
+        <is>
+          <t>black-mushroom-specialist</t>
+        </is>
+      </c>
+      <c r="B31" s="116" t="inlineStr">
+        <is>
+          <t>Deathcap Reaper</t>
+        </is>
+      </c>
+      <c r="C31" s="117" t="n">
+        <v>5</v>
+      </c>
+      <c r="D31" s="116" t="inlineStr">
+        <is>
+          <t>mushroom</t>
+        </is>
+      </c>
+      <c r="E31" s="117" t="n">
+        <v>90</v>
+      </c>
+      <c r="F31" s="117" t="n">
+        <v>18</v>
+      </c>
+      <c r="G31" s="117" t="n">
+        <v>44</v>
+      </c>
+      <c r="H31" s="117" t="n">
+        <v>9</v>
+      </c>
+      <c r="I31" s="116" t="inlineStr"/>
+      <c r="J31" s="117" t="n"/>
+      <c r="K31" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L31" s="116" t="inlineStr">
+        <is>
+          <t>grosse hallebarde</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="59" customHeight="1" s="102">
+      <c r="A32" s="116" t="inlineStr">
+        <is>
+          <t>king-mushroom</t>
+        </is>
+      </c>
+      <c r="B32" s="116" t="inlineStr">
+        <is>
+          <t>Mushroom King</t>
+        </is>
+      </c>
+      <c r="C32" s="117" t="n">
+        <v>6</v>
+      </c>
+      <c r="D32" s="116" t="inlineStr">
+        <is>
+          <t>mushroom</t>
+        </is>
+      </c>
+      <c r="E32" s="117" t="n">
+        <v>140</v>
+      </c>
+      <c r="F32" s="117" t="n">
+        <v>16</v>
+      </c>
+      <c r="G32" s="117" t="n">
+        <v>70</v>
+      </c>
+      <c r="H32" s="117" t="n">
+        <v>6</v>
+      </c>
+      <c r="I32" s="116" t="inlineStr">
+        <is>
+          <t>Soin 18 (40%)
+Hâte alliés 2 (30%)
+Attaque 16 (30%)</t>
+        </is>
+      </c>
+      <c r="J32" s="117" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="116" t="inlineStr">
+        <is>
+          <t>Profondeur (mine, étage 2+)</t>
+        </is>
+      </c>
+      <c r="L32" s="116" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="126" t="inlineStr">
+        <is>
+          <t>▸ LAPIN BLANC (rencontre spéciale, évolutif)</t>
+        </is>
+      </c>
+      <c r="B33" s="127" t="n"/>
+      <c r="C33" s="127" t="n"/>
+      <c r="D33" s="127" t="n"/>
+      <c r="E33" s="127" t="n"/>
+      <c r="F33" s="127" t="n"/>
+      <c r="G33" s="127" t="n"/>
+      <c r="H33" s="127" t="n"/>
+      <c r="I33" s="127" t="n"/>
+      <c r="J33" s="127" t="n"/>
+      <c r="K33" s="127" t="n"/>
+      <c r="L33" s="127" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="116" t="inlineStr">
+        <is>
+          <t>lapin-stage1</t>
+        </is>
+      </c>
+      <c r="B34" s="116" t="inlineStr">
+        <is>
+          <t>White Rabbit</t>
+        </is>
+      </c>
+      <c r="C34" s="117" t="n">
+        <v>7</v>
+      </c>
+      <c r="D34" s="116" t="inlineStr">
+        <is>
+          <t>lapin</t>
+        </is>
+      </c>
+      <c r="E34" s="117" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="117" t="n">
+        <v>13</v>
+      </c>
+      <c r="I34" s="116" t="inlineStr"/>
+      <c r="J34" s="117" t="n"/>
+      <c r="K34" s="116" t="inlineStr">
+        <is>
+          <t>Rencontre spéciale rare (mine, étage 4+, seul/entre lapins)</t>
+        </is>
+      </c>
+      <c r="L34" s="116" t="inlineStr">
+        <is>
+          <t>stade 1 GENTIL : n'attaque pas ; le tuer le fait ÉVOLUER</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="116" t="inlineStr">
+        <is>
+          <t>lapin-stage2</t>
+        </is>
+      </c>
+      <c r="B35" s="116" t="inlineStr">
+        <is>
+          <t>Feral Hare</t>
+        </is>
+      </c>
+      <c r="C35" s="117" t="n">
+        <v>7</v>
+      </c>
+      <c r="D35" s="116" t="inlineStr">
+        <is>
+          <t>lapin</t>
+        </is>
+      </c>
+      <c r="E35" s="117" t="n">
+        <v>55</v>
+      </c>
+      <c r="F35" s="117" t="inlineStr">
+        <is>
+          <t>9x2</t>
+        </is>
+      </c>
+      <c r="G35" s="117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="117" t="n">
         <v>20</v>
       </c>
-      <c r="F5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G5" t="n">
-        <v>20</v>
-      </c>
-      <c r="H5" t="n">
-        <v>7</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>soigner:10:50 | haste-allie:2:30 | attaque:2:20</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Eastern + profondeur</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ogre-masque</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Masked Ogre</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>animal</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>80</v>
-      </c>
-      <c r="F6" t="n">
-        <v>30</v>
-      </c>
-      <c r="G6" t="n">
-        <v>60</v>
-      </c>
-      <c r="H6" t="n">
-        <v>5</v>
-      </c>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Eastern + profondeur</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>orc-rodeur</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Orc Rogue</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>orc</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>40</v>
-      </c>
-      <c r="F7" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" t="n">
-        <v>22</v>
-      </c>
-      <c r="H7" t="n">
-        <v>15</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>frappe 2× par tour (attaqueHits 2)</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>orc-guerrier</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Orc Warrior</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>orc</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>75</v>
-      </c>
-      <c r="F8" t="n">
-        <v>12</v>
-      </c>
-      <c r="G8" t="n">
-        <v>30</v>
-      </c>
-      <c r="H8" t="n">
-        <v>8</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>orc-guerriere</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Orc Warmaiden</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>orc</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>60</v>
-      </c>
-      <c r="F9" t="n">
-        <v>16</v>
-      </c>
-      <c r="G9" t="n">
-        <v>34</v>
-      </c>
-      <c r="H9" t="n">
-        <v>9</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>orc-brute</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Orc Berserker</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>5</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>orc</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>95</v>
-      </c>
-      <c r="F10" t="n">
-        <v>20</v>
-      </c>
-      <c r="G10" t="n">
-        <v>44</v>
-      </c>
-      <c r="H10" t="n">
-        <v>6</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>orc-chamane</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Orc Shaman</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>orc</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>45</v>
-      </c>
-      <c r="F11" t="n">
-        <v>6</v>
-      </c>
-      <c r="G11" t="n">
-        <v>36</v>
-      </c>
-      <c r="H11" t="n">
-        <v>7</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>soigner:12:45 | haste-allie:2:30 | attaque:6:25</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>blob-vert</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Green Slime</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>blob</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>55</v>
-      </c>
-      <c r="F12" t="n">
-        <v>8</v>
-      </c>
-      <c r="G12" t="n">
-        <v>24</v>
-      </c>
-      <c r="H12" t="n">
-        <v>4</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>1 poison par coup</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>blob-jaune</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Ochre Slime</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>blob</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>50</v>
-      </c>
-      <c r="F13" t="n">
-        <v>8</v>
-      </c>
-      <c r="G13" t="n">
-        <v>24</v>
-      </c>
-      <c r="H13" t="n">
-        <v>4</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>poison par coup (acide, 3)</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>blob-rouge</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Crimson Slime</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>blob</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>80</v>
-      </c>
-      <c r="F14" t="n">
+      <c r="I35" s="116" t="inlineStr"/>
+      <c r="J35" s="117" t="n"/>
+      <c r="K35" s="116" t="inlineStr">
+        <is>
+          <t>Rencontre spéciale (évolution)</t>
+        </is>
+      </c>
+      <c r="L35" s="116" t="inlineStr">
+        <is>
+          <t>stade 2 : évolue en stade 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="116" t="inlineStr">
+        <is>
+          <t>lapin-stage3</t>
+        </is>
+      </c>
+      <c r="B36" s="116" t="inlineStr">
+        <is>
+          <t>Bloodfang Horror</t>
+        </is>
+      </c>
+      <c r="C36" s="117" t="n">
         <v>10</v>
       </c>
-      <c r="G14" t="n">
-        <v>30</v>
-      </c>
-      <c r="H14" t="n">
-        <v>4</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>tanky</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>blob-bleu</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Azure Slime</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>4</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>blob</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>65</v>
-      </c>
-      <c r="F15" t="n">
-        <v>10</v>
-      </c>
-      <c r="G15" t="n">
-        <v>30</v>
-      </c>
-      <c r="H15" t="n">
-        <v>4</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>piquants</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>molosse</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Dire Hound</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>animal</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>40</v>
-      </c>
-      <c r="F16" t="n">
-        <v>10</v>
-      </c>
-      <c r="G16" t="n">
-        <v>22</v>
-      </c>
-      <c r="H16" t="n">
-        <v>16</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>rapide</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>molosse-feu</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Ember Hound</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>animal</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>45</v>
-      </c>
-      <c r="F17" t="n">
-        <v>12</v>
-      </c>
-      <c r="G17" t="n">
-        <v>28</v>
-      </c>
-      <c r="H17" t="n">
-        <v>15</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>rapide, feu</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>molosse-sombre</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Shadow Hound</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>4</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>animal</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>42</v>
-      </c>
-      <c r="F18" t="n">
-        <v>11</v>
-      </c>
-      <c r="G18" t="n">
+      <c r="D36" s="116" t="inlineStr">
+        <is>
+          <t>lapin</t>
+        </is>
+      </c>
+      <c r="E36" s="117" t="n">
+        <v>150</v>
+      </c>
+      <c r="F36" s="117" t="inlineStr">
+        <is>
+          <t>17x2</t>
+        </is>
+      </c>
+      <c r="G36" s="117" t="n">
+        <v>130</v>
+      </c>
+      <c r="H36" s="117" t="n">
         <v>26</v>
       </c>
-      <c r="H18" t="n">
-        <v>17</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>rapide</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>warrior-mushroom1</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Toadstool Lancer</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>3</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>mushroom</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>50</v>
-      </c>
-      <c r="F19" t="n">
-        <v>8</v>
-      </c>
-      <c r="G19" t="n">
-        <v>22</v>
-      </c>
-      <c r="H19" t="n">
-        <v>8</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>warrior-mushroom2</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Fungal Knight</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>4</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>mushroom</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>85</v>
-      </c>
-      <c r="F20" t="n">
-        <v>11</v>
-      </c>
-      <c r="G20" t="n">
-        <v>30</v>
-      </c>
-      <c r="H20" t="n">
-        <v>7</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>white-katana-mushroom</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Myconid Ronin</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>4</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>mushroom</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>45</v>
-      </c>
-      <c r="F21" t="n">
-        <v>7</v>
-      </c>
-      <c r="G21" t="n">
-        <v>30</v>
-      </c>
-      <c r="H21" t="n">
-        <v>18</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>frappe 2× par tour (attaqueHits 2)</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>black-mushroom-specialist</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Deathcap Reaper</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>5</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>mushroom</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>90</v>
-      </c>
-      <c r="F22" t="n">
-        <v>18</v>
-      </c>
-      <c r="G22" t="n">
-        <v>44</v>
-      </c>
-      <c r="H22" t="n">
-        <v>9</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>mage-mushroom</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Myconid Sage</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>4</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>mushroom</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>40</v>
-      </c>
-      <c r="F23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G23" t="n">
-        <v>34</v>
-      </c>
-      <c r="H23" t="n">
-        <v>7</v>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>soigner:12:45 | haste-allie:2:30 | attaque:5:25</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>king-mushroom</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Mushroom King</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>6</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>mushroom</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>140</v>
-      </c>
-      <c r="F24" t="n">
-        <v>16</v>
-      </c>
-      <c r="G24" t="n">
-        <v>70</v>
-      </c>
-      <c r="H24" t="n">
-        <v>6</v>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>soigner:18:40 | haste-allie:2:30 | attaque:16:30</t>
-        </is>
-      </c>
-      <c r="J24" t="n">
-        <v>1</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>bear</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Cave Bear</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>4</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>animal</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>90</v>
-      </c>
-      <c r="F25" t="n">
-        <v>14</v>
-      </c>
-      <c r="G25" t="n">
-        <v>32</v>
-      </c>
-      <c r="H25" t="n">
-        <v>8</v>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>en meute avec les molosses</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>bones-bear</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Bonehide Bear</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>5</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>animal</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>100</v>
-      </c>
-      <c r="F26" t="n">
-        <v>16</v>
-      </c>
-      <c r="G26" t="n">
-        <v>44</v>
-      </c>
-      <c r="H26" t="n">
-        <v>9</v>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>en meute avec les molosses</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>armor-bear</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Armored War-Bear</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>6</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>animal</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>150</v>
-      </c>
-      <c r="F27" t="n">
-        <v>20</v>
-      </c>
-      <c r="G27" t="n">
-        <v>60</v>
-      </c>
-      <c r="H27" t="n">
-        <v>6</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>en meute avec les molosses</t>
-        </is>
-      </c>
-      <c r="J27" t="n">
-        <v>1</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Profondeur (mine, étage 2+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>lapin-stage1</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>White Rabbit</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>7</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>lapin</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" t="n">
-        <v>13</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>stade 1 GENTIL : n'attaque pas ; le tuer le fait ÉVOLUER (pas dans l'Excel : voir code)</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Rencontre spéciale rare (mine, étage 4+, seul)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>lapin-stage2</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Feral Hare</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>7</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>lapin</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>55</v>
-      </c>
-      <c r="F29" t="n">
-        <v>9</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" t="n">
-        <v>20</v>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>stade 2 : frappe 2× (attaqueHits 2) ; évolue en stade 3</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Rencontre spéciale (évolution)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>lapin-stage3</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Bloodfang Horror</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>10</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>lapin</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>150</v>
-      </c>
-      <c r="F30" t="n">
-        <v>17</v>
-      </c>
-      <c r="G30" t="n">
-        <v>130</v>
-      </c>
-      <c r="H30" t="n">
-        <v>26</v>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>stade 3 : frappe 2× ; gros or (niv 10) + 2% Ring of Luck</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
+      <c r="I36" s="116" t="inlineStr"/>
+      <c r="J36" s="117" t="n"/>
+      <c r="K36" s="116" t="inlineStr">
         <is>
           <t>Rencontre spéciale (stade final)</t>
+        </is>
+      </c>
+      <c r="L36" s="116" t="inlineStr">
+        <is>
+          <t>stade 3 : gros or (niv 10) + 2% Ring of Luck</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[technique] Excel « Général » : réglages de taille de pile de minerai (base 5, talent Ore Hauler +5/rang)
Tient l'onglet « Général » à jour (règle de la Bible) avec les nouveaux réglages
d'équilibrage introduits par le talent « Ore Hauler ».

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -3263,7 +3263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="102" min="1" max="1"/>
@@ -3287,6 +3287,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="107" t="inlineStr">
         <is>
@@ -3753,69 +3754,69 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="108" t="inlineStr">
-        <is>
-          <t>LUCKY DELVER (talent forge — caverne de chance)</t>
-        </is>
-      </c>
-      <c r="B23" s="109" t="n"/>
-      <c r="C23" s="109" t="n"/>
-      <c r="D23" s="109" t="n"/>
-      <c r="E23" s="109" t="n"/>
+      <c r="A23" s="110" t="inlineStr">
+        <is>
+          <t>Minage</t>
+        </is>
+      </c>
+      <c r="B23" s="110" t="inlineStr">
+        <is>
+          <t>Taille de pile de base</t>
+        </is>
+      </c>
+      <c r="C23" s="111" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D23" s="110" t="inlineStr">
+        <is>
+          <t>Nombre max de minerais par pile SANS talent (avant : 10).</t>
+        </is>
+      </c>
+      <c r="E23" s="110" t="inlineStr">
+        <is>
+          <t>data/items.js + inventaire.js</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="110" t="inlineStr">
         <is>
-          <t>Caverne</t>
+          <t>Minage</t>
         </is>
       </c>
       <c r="B24" s="110" t="inlineStr">
         <is>
-          <t>Chance d'apparition</t>
+          <t>Talent « Ore Hauler » (par rang)</t>
         </is>
       </c>
       <c r="C24" s="111" t="inlineStr">
         <is>
-          <t>22 %</t>
+          <t>+5 (×5 rangs → 30)</t>
         </is>
       </c>
       <c r="D24" s="110" t="inlineStr">
         <is>
-          <t>Proba, par descente éligible (étage 3+), de tomber sur une caverne de chance.</t>
+          <t>Chaque rang du talent forge agrandit les piles de +5 (5 rangs → 30/pile).</t>
         </is>
       </c>
       <c r="E24" s="110" t="inlineStr">
         <is>
-          <t>principal.js</t>
+          <t>data/talents.js</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="110" t="inlineStr">
-        <is>
-          <t>Caverne</t>
-        </is>
-      </c>
-      <c r="B25" s="110" t="inlineStr">
-        <is>
-          <t>Bonus de minerais</t>
-        </is>
-      </c>
-      <c r="C25" s="111" t="inlineStr">
-        <is>
-          <t>+220 %</t>
-        </is>
-      </c>
-      <c r="D25" s="110" t="inlineStr">
-        <is>
-          <t>Boost du nombre de veines dans une caverne de chance.</t>
-        </is>
-      </c>
-      <c r="E25" s="110" t="inlineStr">
-        <is>
-          <t>principal.js</t>
-        </is>
-      </c>
+      <c r="A25" s="108" t="inlineStr">
+        <is>
+          <t>LUCKY DELVER (talent forge — caverne de chance)</t>
+        </is>
+      </c>
+      <c r="B25" s="109" t="n"/>
+      <c r="C25" s="109" t="n"/>
+      <c r="D25" s="109" t="n"/>
+      <c r="E25" s="109" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="110" t="inlineStr">
@@ -3825,17 +3826,17 @@
       </c>
       <c r="B26" s="110" t="inlineStr">
         <is>
-          <t>Taux de rencontre</t>
+          <t>Chance d'apparition</t>
         </is>
       </c>
       <c r="C26" s="111" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>22 %</t>
         </is>
       </c>
       <c r="D26" s="110" t="inlineStr">
         <is>
-          <t>Fréquence des combats dans une caverne (vs 0.3 normal → quasi zéro monstre).</t>
+          <t>Proba, par descente éligible (étage 3+), de tomber sur une caverne de chance.</t>
         </is>
       </c>
       <c r="E26" s="110" t="inlineStr">
@@ -3845,47 +3846,63 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="108" t="inlineStr">
-        <is>
-          <t>BANQUE</t>
-        </is>
-      </c>
-      <c r="B27" s="109" t="n"/>
-      <c r="C27" s="109" t="n"/>
-      <c r="D27" s="109" t="n"/>
-      <c r="E27" s="109" t="n"/>
+      <c r="A27" s="110" t="inlineStr">
+        <is>
+          <t>Caverne</t>
+        </is>
+      </c>
+      <c r="B27" s="110" t="inlineStr">
+        <is>
+          <t>Bonus de minerais</t>
+        </is>
+      </c>
+      <c r="C27" s="111" t="inlineStr">
+        <is>
+          <t>+220 %</t>
+        </is>
+      </c>
+      <c r="D27" s="110" t="inlineStr">
+        <is>
+          <t>Boost du nombre de veines dans une caverne de chance.</t>
+        </is>
+      </c>
+      <c r="E27" s="110" t="inlineStr">
+        <is>
+          <t>principal.js</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="110" t="inlineStr">
         <is>
-          <t>Banque</t>
+          <t>Caverne</t>
         </is>
       </c>
       <c r="B28" s="110" t="inlineStr">
         <is>
-          <t>Rendement du coffre-fort</t>
+          <t>Taux de rencontre</t>
         </is>
       </c>
       <c r="C28" s="111" t="inlineStr">
         <is>
-          <t>0.2 % / jour</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="D28" s="110" t="inlineStr">
         <is>
-          <t>Intérêt composé du dépôt SÛR (par jour de jeu).</t>
+          <t>Fréquence des combats dans une caverne (vs 0.3 normal → quasi zéro monstre).</t>
         </is>
       </c>
       <c r="E28" s="110" t="inlineStr">
         <is>
-          <t>data/banque.js</t>
+          <t>principal.js</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="108" t="inlineStr">
         <is>
-          <t>RENCONTRES &amp; GROUPES DE MONSTRES</t>
+          <t>BANQUE</t>
         </is>
       </c>
       <c r="B29" s="109" t="n"/>
@@ -3896,56 +3913,40 @@
     <row r="30">
       <c r="A30" s="110" t="inlineStr">
         <is>
-          <t>Mine</t>
+          <t>Banque</t>
         </is>
       </c>
       <c r="B30" s="110" t="inlineStr">
         <is>
-          <t>Taux de rencontre</t>
+          <t>Rendement du coffre-fort</t>
         </is>
       </c>
       <c r="C30" s="111" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.2 % / jour</t>
         </is>
       </c>
       <c r="D30" s="110" t="inlineStr">
         <is>
-          <t>Fréquence de base des combats en explorant une mine.</t>
+          <t>Intérêt composé du dépôt SÛR (par jour de jeu).</t>
         </is>
       </c>
       <c r="E30" s="110" t="inlineStr">
         <is>
-          <t>world/mine.js</t>
+          <t>data/banque.js</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="110" t="inlineStr">
-        <is>
-          <t>Mine</t>
-        </is>
-      </c>
-      <c r="B31" s="110" t="inlineStr">
-        <is>
-          <t>Étage « monstres profonds »</t>
-        </is>
-      </c>
-      <c r="C31" s="111" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D31" s="110" t="inlineStr">
-        <is>
-          <t>Étage mini où apparaissent orcs / blobs / molosses / ours / champignons.</t>
-        </is>
-      </c>
-      <c r="E31" s="110" t="inlineStr">
-        <is>
-          <t>world/mine.js</t>
-        </is>
-      </c>
+      <c r="A31" s="108" t="inlineStr">
+        <is>
+          <t>RENCONTRES &amp; GROUPES DE MONSTRES</t>
+        </is>
+      </c>
+      <c r="B31" s="109" t="n"/>
+      <c r="C31" s="109" t="n"/>
+      <c r="D31" s="109" t="n"/>
+      <c r="E31" s="109" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="110" t="inlineStr">
@@ -3955,17 +3956,17 @@
       </c>
       <c r="B32" s="110" t="inlineStr">
         <is>
-          <t>Chance de biome (thème)</t>
+          <t>Taux de rencontre</t>
         </is>
       </c>
       <c r="C32" s="111" t="inlineStr">
         <is>
-          <t>40 %</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="D32" s="110" t="inlineStr">
         <is>
-          <t>Proba qu'un étage éligible soit à thème (cristal / glace / lave…).</t>
+          <t>Fréquence de base des combats en explorant une mine.</t>
         </is>
       </c>
       <c r="E32" s="110" t="inlineStr">
@@ -3977,54 +3978,54 @@
     <row r="33">
       <c r="A33" s="110" t="inlineStr">
         <is>
-          <t>Groupes</t>
+          <t>Mine</t>
         </is>
       </c>
       <c r="B33" s="110" t="inlineStr">
         <is>
-          <t>Taille des groupes</t>
+          <t>Étage « monstres profonds »</t>
         </is>
       </c>
       <c r="C33" s="111" t="inlineStr">
         <is>
-          <t>30 / 30 / 20 / 15 / 5 %</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D33" s="110" t="inlineStr">
         <is>
-          <t>Proba d'un groupe de 1 / 2 / 3 / 4 / 5 emplacements.</t>
+          <t>Étage mini où apparaissent orcs / blobs / molosses / ours / champignons.</t>
         </is>
       </c>
       <c r="E33" s="110" t="inlineStr">
         <is>
-          <t>data/ennemis.js</t>
+          <t>world/mine.js</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="110" t="inlineStr">
         <is>
-          <t>Groupes</t>
+          <t>Mine</t>
         </is>
       </c>
       <c r="B34" s="110" t="inlineStr">
         <is>
-          <t>Facteur de niveau</t>
+          <t>Chance de biome (thème)</t>
         </is>
       </c>
       <c r="C34" s="111" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>40 %</t>
         </is>
       </c>
       <c r="D34" s="110" t="inlineStr">
         <is>
-          <t>Un niveau de monstre en plus = ~2× plus rare dans le tirage.</t>
+          <t>Proba qu'un étage éligible soit à thème (cristal / glace / lave…).</t>
         </is>
       </c>
       <c r="E34" s="110" t="inlineStr">
         <is>
-          <t>data/ennemis.js</t>
+          <t>world/mine.js</t>
         </is>
       </c>
     </row>
@@ -4036,17 +4037,17 @@
       </c>
       <c r="B35" s="110" t="inlineStr">
         <is>
-          <t>Rareté d'un « grand » (petit grp)</t>
+          <t>Taille des groupes</t>
         </is>
       </c>
       <c r="C35" s="111" t="inlineStr">
         <is>
-          <t>×0.5</t>
+          <t>30 / 30 / 20 / 15 / 5 %</t>
         </is>
       </c>
       <c r="D35" s="110" t="inlineStr">
         <is>
-          <t>Poids d'un grand monstre dans un petit groupe (plus rare).</t>
+          <t>Proba d'un groupe de 1 / 2 / 3 / 4 / 5 emplacements.</t>
         </is>
       </c>
       <c r="E35" s="110" t="inlineStr">
@@ -4063,17 +4064,17 @@
       </c>
       <c r="B36" s="110" t="inlineStr">
         <is>
-          <t>Bonus d'un « grand » (gros grp)</t>
+          <t>Facteur de niveau</t>
         </is>
       </c>
       <c r="C36" s="111" t="inlineStr">
         <is>
-          <t>×3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D36" s="110" t="inlineStr">
         <is>
-          <t>Poids d'un grand dans un gros groupe (favorisé).</t>
+          <t>Un niveau de monstre en plus = ~2× plus rare dans le tirage.</t>
         </is>
       </c>
       <c r="E36" s="110" t="inlineStr">
@@ -4085,25 +4086,79 @@
     <row r="37">
       <c r="A37" s="110" t="inlineStr">
         <is>
+          <t>Groupes</t>
+        </is>
+      </c>
+      <c r="B37" s="110" t="inlineStr">
+        <is>
+          <t>Rareté d'un « grand » (petit grp)</t>
+        </is>
+      </c>
+      <c r="C37" s="111" t="inlineStr">
+        <is>
+          <t>×0.5</t>
+        </is>
+      </c>
+      <c r="D37" s="110" t="inlineStr">
+        <is>
+          <t>Poids d'un grand monstre dans un petit groupe (plus rare).</t>
+        </is>
+      </c>
+      <c r="E37" s="110" t="inlineStr">
+        <is>
+          <t>data/ennemis.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="110" t="inlineStr">
+        <is>
+          <t>Groupes</t>
+        </is>
+      </c>
+      <c r="B38" s="110" t="inlineStr">
+        <is>
+          <t>Bonus d'un « grand » (gros grp)</t>
+        </is>
+      </c>
+      <c r="C38" s="111" t="inlineStr">
+        <is>
+          <t>×3</t>
+        </is>
+      </c>
+      <c r="D38" s="110" t="inlineStr">
+        <is>
+          <t>Poids d'un grand dans un gros groupe (favorisé).</t>
+        </is>
+      </c>
+      <c r="E38" s="110" t="inlineStr">
+        <is>
+          <t>data/ennemis.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="110" t="inlineStr">
+        <is>
           <t>Combat</t>
         </is>
       </c>
-      <c r="B37" s="110" t="inlineStr">
+      <c r="B39" s="110" t="inlineStr">
         <is>
           <t>Fuite selon nb d'ennemis</t>
         </is>
       </c>
-      <c r="C37" s="111" t="inlineStr">
+      <c r="C39" s="111" t="inlineStr">
         <is>
           <t>50 / 33 / 25 / 25 / 20 %</t>
         </is>
       </c>
-      <c r="D37" s="110" t="inlineStr">
+      <c r="D39" s="110" t="inlineStr">
         <is>
           <t>Chance de fuir un combat normal selon le nombre d'ennemis (1 à 5).</t>
         </is>
       </c>
-      <c r="E37" s="110" t="inlineStr">
+      <c r="E39" s="110" t="inlineStr">
         <is>
           <t>ui/combat.js</t>
         </is>

</xml_diff>

<commit_message>
[équilibrage] Tour de siège : chiffres dans l'Excel + doc concept
Ajoute les 4 monstres de la tour de siège à l'onglet « Monstres » du classeur
d'équilibrage (nouvelle section « Tour de siège »), pour que la base de
référence reste complète : la tour + son équipage (Kaboom, 3 de siège,
porte-étendard). L'importer sait désormais lire l'action « buff-allie »
(libellé « Bannière ») du porte-étendard ; le bloc auto de data/ennemis.js est
régénéré depuis l'Excel (les champs art/tech — dislocation, mèche, buff dégâts —
restent en code).

Documente aussi le boss dans docs/concept.md (mécanisme de dislocation
splitEnMort, mèche du Kaboom, buff du porte-étendard, drapeau spawnOnly).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -1609,7 +1609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="102" min="1" max="1"/>
@@ -3093,6 +3093,206 @@
       <c r="L36" s="116" t="inlineStr">
         <is>
           <t>stade 3 : gros or (niv 10) + 2% Ring of Luck</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="126" t="inlineStr">
+        <is>
+          <t>▸ TOUR DE SIÈGE (boss unique + son équipage, spawnOnly)</t>
+        </is>
+      </c>
+      <c r="B37" s="127" t="n"/>
+      <c r="C37" s="127" t="n"/>
+      <c r="D37" s="127" t="n"/>
+      <c r="E37" s="127" t="n"/>
+      <c r="F37" s="127" t="n"/>
+      <c r="G37" s="127" t="n"/>
+      <c r="H37" s="127" t="n"/>
+      <c r="I37" s="127" t="n"/>
+      <c r="J37" s="127" t="n"/>
+      <c r="K37" s="127" t="n"/>
+      <c r="L37" s="127" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="116" t="inlineStr">
+        <is>
+          <t>tour-de-siege-gobeline</t>
+        </is>
+      </c>
+      <c r="B38" s="116" t="inlineStr">
+        <is>
+          <t>Goblin Siege Tower</t>
+        </is>
+      </c>
+      <c r="C38" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="D38" s="116" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="E38" s="117" t="n">
+        <v>220</v>
+      </c>
+      <c r="F38" s="117" t="n">
+        <v>16</v>
+      </c>
+      <c r="G38" s="117" t="n">
+        <v>120</v>
+      </c>
+      <c r="H38" s="117" t="n">
+        <v>5</v>
+      </c>
+      <c r="I38" s="116" t="n"/>
+      <c r="J38" s="117" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" s="116" t="inlineStr">
+        <is>
+          <t>Rencontre spéciale (mine, étage 5+, TOUJOURS seule)</t>
+        </is>
+      </c>
+      <c r="L38" s="116" t="inlineStr">
+        <is>
+          <t>boss unique ; à sa mort se DISLOQUE en son équipage (Kaboom + 3 de siège + porte-étendard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="116" t="inlineStr">
+        <is>
+          <t>gobelin-kaboom</t>
+        </is>
+      </c>
+      <c r="B39" s="116" t="inlineStr">
+        <is>
+          <t>Goblin Kaboom</t>
+        </is>
+      </c>
+      <c r="C39" s="117" t="n">
+        <v>6</v>
+      </c>
+      <c r="D39" s="116" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="E39" s="117" t="n">
+        <v>20</v>
+      </c>
+      <c r="F39" s="117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="117" t="n">
+        <v>20</v>
+      </c>
+      <c r="H39" s="117" t="n">
+        <v>4</v>
+      </c>
+      <c r="I39" s="116" t="n"/>
+      <c r="J39" s="117" t="n"/>
+      <c r="K39" s="116" t="inlineStr">
+        <is>
+          <t>Équipage de la tour (n'apparaît QUE de sa mort)</t>
+        </is>
+      </c>
+      <c r="L39" s="116" t="inlineStr">
+        <is>
+          <t>longue mèche (2 tours) puis EXPLOSE pour 100 et meurt — dégâts en code (explose)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="116" t="inlineStr">
+        <is>
+          <t>gobelin-de-siege</t>
+        </is>
+      </c>
+      <c r="B40" s="116" t="inlineStr">
+        <is>
+          <t>Siege Goblin</t>
+        </is>
+      </c>
+      <c r="C40" s="117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="116" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="E40" s="117" t="n">
+        <v>24</v>
+      </c>
+      <c r="F40" s="117" t="n">
+        <v>7</v>
+      </c>
+      <c r="G40" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="H40" s="117" t="n">
+        <v>9</v>
+      </c>
+      <c r="I40" s="116" t="n"/>
+      <c r="J40" s="117" t="n"/>
+      <c r="K40" s="116" t="inlineStr">
+        <is>
+          <t>Équipage de la tour (n'apparaît QUE de sa mort)</t>
+        </is>
+      </c>
+      <c r="L40" s="116" t="inlineStr">
+        <is>
+          <t>juste son épée ; rapide mais fragile</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="116" t="inlineStr">
+        <is>
+          <t>gobelin-de-siege-etandart</t>
+        </is>
+      </c>
+      <c r="B41" s="116" t="inlineStr">
+        <is>
+          <t>Siege Standard-Bearer</t>
+        </is>
+      </c>
+      <c r="C41" s="117" t="n">
+        <v>6</v>
+      </c>
+      <c r="D41" s="116" t="inlineStr">
+        <is>
+          <t>gobelin</t>
+        </is>
+      </c>
+      <c r="E41" s="117" t="n">
+        <v>55</v>
+      </c>
+      <c r="F41" s="117" t="n">
+        <v>5</v>
+      </c>
+      <c r="G41" s="117" t="n">
+        <v>24</v>
+      </c>
+      <c r="H41" s="117" t="n">
+        <v>7</v>
+      </c>
+      <c r="I41" s="116" t="inlineStr">
+        <is>
+          <t>Bannière 2 (100%)</t>
+        </is>
+      </c>
+      <c r="J41" s="117" t="n"/>
+      <c r="K41" s="116" t="inlineStr">
+        <is>
+          <t>Équipage de la tour (n'apparaît QUE de sa mort)</t>
+        </is>
+      </c>
+      <c r="L41" s="116" t="inlineStr">
+        <is>
+          <t>buffe les alliés : +2 Hâte ET +2 dégâts par tour (le +dégâts est en code : buffDegats)</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3487,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="107" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
[gameplay] Le Fou du roi : rencontre-énigme des profondeurs (marché, tour unique, butin garanti)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -1609,7 +1609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="102" min="1" max="1"/>
@@ -3453,6 +3453,53 @@
       <c r="L45" s="116" t="inlineStr">
         <is>
           <t>DÉFENSEUR : 15 de bouclier perso (cf. Général) + donne du bouclier aux alliés chaque tour. À gauche. Synergie tank + dégâts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>fou-du-roi</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>The King's Fool</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>10</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>fou</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>100</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>200</v>
+      </c>
+      <c r="H46" t="n">
+        <v>14</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Marché (500/2000/10000 🪙) ; fuite après 1 tour du héros ; vol 200 🪙 si touché</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>TOUTES les profondeurs — 0,1 % par rencontre (tirage dédié, hors pool de zone)</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Rencontre-énigme : ne frappe jamais. Tué = butin garanti (5000 🪙 + 10 rubis/émeraude/saphir/diamant + 1 onyx + 1 sunstone) et ne revient plus. 3e paiement = cadeau (50000 XP, 10 onyx, 10 sunstone, 20 bois enchanté, 20 cuir étrange).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[gameplay] Fou du roi : la rencontre d'après le cadeau devient un vrai combat (il ne fuit plus, 60 de dégâts)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZD9AfytCUWGMcS4VfpH7V
</commit_message>
<xml_diff>
--- a/docs/BRUTAL-items-et-cartes.xlsx
+++ b/docs/BRUTAL-items-et-cartes.xlsx
@@ -3489,7 +3489,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Marché (500/2000/10000 🪙) ; fuite après 1 tour du héros ; vol 200 🪙 si touché</t>
+          <t>Marché (500/2000/10000 🪙) ; fuit après 1 tour du héros ; vol 200 🪙 si touché ; RANCUNE (après cadeau) : ne fuit plus et frappe à 60</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Rencontre-énigme : ne frappe jamais. Tué = butin garanti (5000 🪙 + 10 rubis/émeraude/saphir/diamant + 1 onyx + 1 sunstone) et ne revient plus. 3e paiement = cadeau (50000 XP, 10 onyx, 10 sunstone, 20 bois enchanté, 20 cuir étrange).</t>
+          <t>Rencontre-énigme : ne frappe JAMAIS tant qu'il marchande (il fuit avant). SEULE exception, la rancune (rencontre d'après le cadeau) : il reste et attaque à 60. Tué = butin garanti (5000 🪙 + 10 rubis/émeraude/saphir/diamant + 1 onyx + 1 sunstone) et ne revient plus. 3e paiement = cadeau (50000 XP, 10 onyx, 10 sunstone, 20 bois enchanté, 20 cuir étrange).</t>
         </is>
       </c>
     </row>

</xml_diff>